<commit_message>
Fix Best Chemistry ranking eligibility and remove padding
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F179"/>
+  <dimension ref="A1:F172"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -635,16 +635,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="str">
-        <v>分手的99個理由</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D12" t="str">
-        <v>胡咪老師</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E12">
-        <v>9.16</v>
+        <v>9.31</v>
       </c>
       <c r="F12" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 兩位主持人互動自然，接話流暢，笑聲同步率高，展現良好默契。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人默契極佳，對話流暢自然，能互相接話並適時加入幽默感，共同營造出引人入勝的節目氛圍。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契，接話流暢，插話頻率適中，彼此的幽默感與共鳴笑聲自然，共同營造出輕鬆愉快的對話氛圍。</v>
+        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
       </c>
     </row>
     <row r="13">
@@ -655,16 +655,16 @@
         <v>2</v>
       </c>
       <c r="C13" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D13" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E13">
-        <v>8.89</v>
+        <v>9.16</v>
       </c>
       <c r="F13" t="str">
-        <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
+        <v>[S4.EP4｜性平教育20年，...] 兩位主持人互動自然，接話流暢，笑聲同步率高，展現良好默契。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人默契極佳，對話流暢自然，能互相接話並適時加入幽默感，共同營造出引人入勝的節目氛圍。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契，接話流暢，插話頻率適中，彼此的幽默感與共鳴笑聲自然，共同營造出輕鬆愉快的對話氛圍。</v>
       </c>
     </row>
     <row r="14">
@@ -675,16 +675,16 @@
         <v>3</v>
       </c>
       <c r="C14" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D14" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E14">
         <v>8.89</v>
       </c>
       <c r="F14" t="str">
-        <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
+        <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
       </c>
     </row>
     <row r="15">
@@ -695,16 +695,16 @@
         <v>4</v>
       </c>
       <c r="C15" t="str">
-        <v>能量黑客</v>
+        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
       <c r="D15" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E15">
-        <v>8.73</v>
+        <v>8.89</v>
       </c>
       <c r="F15" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人互動自然，接話流暢，彼此間的幽默感和笑聲也增加了節目的親和力。女主持人興奮時的插話，男主持人也能很好地承接。 | [別人眼中的高光時刻，卻是我最耗...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高��尤其在幽默解釋「麻場」和「鐵軌」時，默契十足。 | [別急著振作！高能量的人允許自己...] 雙主持人Hank與Vicky之間的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現了良好的默契與引導能力。</v>
+        <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
       </c>
     </row>
     <row r="16">
@@ -715,16 +715,16 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <v>粉紅地獄辛辣麵</v>
+        <v>能量黑客</v>
       </c>
       <c r="D16" t="str">
-        <v>Vito大叔</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E16">
         <v>8.73</v>
       </c>
       <c r="F16" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] Vito和品希作為雙人主持，展現了良好的默契。他們接話流暢，很少出現互相打斷的情況，品希的提問常帶有女性的細膩與同理心，Vito則負責更宏觀的引導與專業提問。兩人的笑聲自然，共同營造了輕鬆愉快的對談氛圍。 | [S6EP19. 沐樂MOReL...] Vito與品希之間展現了極佳的默契，對話流暢自然，常有幽默的插科打諢和同步的笑聲，互動感強烈。 | [S6EP4. 放飛。萬哩露｜村...] 雙主持與來賓互動自然，接話流暢，笑聲同步率高，尤其在幽默對話時默契十足，��節目增添了活力。</v>
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人互動自然，接話流暢，彼此間的幽默感和笑聲也增加了節目的親和力。女主持人興奮時的插話，男主持人也能很好地承接。 | [別人眼中的高光時刻，卻是我最耗...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高��尤其在幽默解釋「麻場」和「鐵軌」時，默契十足。 | [別急著振作！高能量的人允許自己...] 雙主持人Hank與Vicky之間的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現了良好的默契與引導能力。</v>
       </c>
     </row>
     <row r="17">
@@ -735,13 +735,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="str">
-        <v>財富餐車不打烊</v>
+        <v>粉紅地獄辛辣麵</v>
       </c>
       <c r="D17" t="str">
-        <v>30節約男子</v>
+        <v>Vito大叔</v>
+      </c>
+      <c r="E17">
+        <v>8.73</v>
       </c>
       <c r="F17" t="str">
-        <v>單人主持節目，歸屬於單人男/女播音獎，不適用此雙人默契獎項。</v>
+        <v>[S6EP30. 我到日本當漁夫...] Vito和品希作為雙人主持，展現了良好的默契。他們接話流暢，很少出現互相打斷的情況，品希的提問常帶有女性的細膩與同理心，Vito則負責更宏觀的引導與專業提問。兩人的笑聲自然，共同營造了輕鬆愉快的對談氛圍。 | [S6EP19. 沐樂MOReL...] Vito與品希之間展現了極佳的默契，對話流暢自然，常有幽默的插科打諢和同步的笑聲，互動感強烈。 | [S6EP4. 放飛。萬哩露｜村...] 雙主持與來賓互動自然，接話流暢，笑聲同步率高，尤其在幽默對話時默契十足，��節目增添了活力。</v>
       </c>
     </row>
     <row r="18">
@@ -752,64 +755,76 @@
         <v>7</v>
       </c>
       <c r="C18" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D18" t="str">
-        <v>丁菱娟</v>
+        <v>無所不試無樂不作</v>
+      </c>
+      <c r="E18">
+        <v>8.57</v>
       </c>
       <c r="F18" t="str">
-        <v>單人主持節目，歸屬於單人男/女播音獎，不適用此雙人默契獎項。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 主持人與來賓之間的對話流暢自然，接話得體，沒有明顯的搶話或插話，展現了良好的互動默契。 | [【中年，正在試】把世界走成一本...] Norman和Summer的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現良好默契。</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>最佳默契獎</v>
+        <v>最神單元企劃獎</v>
       </c>
       <c r="B19">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C19" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>五吉郎</v>
       </c>
       <c r="D19" t="str">
-        <v>人生啊！小歐</v>
+        <v>五吉郎</v>
+      </c>
+      <c r="E19">
+        <v>10</v>
       </c>
       <c r="F19" t="str">
-        <v>單人主持節目，歸屬於單人男/女播音獎，不適用此雙人默契獎項。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 選題新穎，結合個人IP變現與美業轉型，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [EP174｜越省反而越窮？別把...] 選題結合心理學與財富自由，觀點新穎且具深度，案例生動，內容含金量高。 | [EP164｜滑短影音是在浪費時...] 選題新穎且具深度，圍繞來賓新書的核心理念展開，提供了許多關於閱讀與自我成長的實用觀點與啟發，內容含金量極高。</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>最佳默契獎</v>
+        <v>最神單元企劃獎</v>
       </c>
       <c r="B20">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C20" t="str">
-        <v>下半場人生陪談師</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D20" t="str">
-        <v>下半場人生事務有限公司</v>
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="E20">
+        <v>9.99</v>
       </c>
       <c r="F20" t="str">
-        <v>單人主持節目，歸屬於單人男/女播音獎，不適用此雙人默契獎項。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 選題非常新穎且具時事性，從藥物機制到社會政策的討論深度極高，內容含金量豐富。 | [《財富自由心理學》：賺錢，只是...] 選題「財富自由心理學」新穎且具深度，透過個人故事與哲學思辨，將財富議題提升至心靈層次，內容含金量高，案例生動具啟發性。 | [手總是停不下來？那是焦慮在尋找...] 選題新穎且具深度，深入探討身體重複行為的心理學面向，案例生動且內容含金量極高。</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>最佳默契獎</v>
+        <v>最神單元企劃獎</v>
       </c>
       <c r="B21">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C21" t="str">
-        <v>小思大維</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D21" t="str">
-        <v>小思大維｜雪柔</v>
+        <v>梁哲維</v>
+      </c>
+      <c r="E21">
+        <v>9.82</v>
       </c>
       <c r="F21" t="str">
-        <v>單人主持節目，歸屬於單人男/女播音獎，不適用此雙人默契獎項。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目以一本關於「好感影響力」的書為引子，邀請書中提及的創業家來分享故事，選題獨特且具深度。來賓的70年滷味傳承與公益行動，提供了豐富的內容含金量和啟發性。 | [【EP302 把命盤變成行動藍...] 選題新穎，結合「九紫離火運」與AI、全球局勢、個人發展等多元面向，案例生動且內容含金量極高。 | [【EP312《超越我執的生活》...] 選題「超越我執」具備深度與啟發性，結合心理學與靈性成長，內容含金量高，案例（如內在聲音、吃飯專注）生動且具體，展現了優秀的單元企劃能力。</v>
       </c>
     </row>
     <row r="22">
@@ -817,19 +832,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" t="str">
-        <v>五吉郎</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D22" t="str">
-        <v>五吉郎</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E22">
-        <v>10</v>
+        <v>9.76</v>
       </c>
       <c r="F22" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 選題新穎，結合個人IP變現與美業轉型，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [EP174｜越省反而越窮？別把...] 選題結合心理學與財富自由，觀點新穎且具深度，案例生動，內容含金量高。 | [EP164｜滑短影音是在浪費時...] 選題新穎且具深度，圍繞來賓新書的核心理念展開，提供了許多關於閱讀與自我成長的實用觀點與啟發，內容含金量極高。</v>
+        <v>[#801 市場震盪 17000...] 選題緊扣時事（股市下跌），並結合個人財務規劃與情緒管理，案例生動且內容含金量極高。 | [#809  買股票還在到處問明...] 選題「獲利加速系統」具備高度實用性與深度，結合AI工具的應用，內容含金量極高，企劃新穎。 | [#798 害怕投資賠錢？不用天...] 選題新穎且具備深度，聚焦於媽媽族群的投資教育與心態建立，內容含金量高，並透過生動的比喻（如游泳、無印良品櫃子）提升理解度。</v>
       </c>
     </row>
     <row r="23">
@@ -837,19 +852,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" t="str">
-        <v>哇賽心理學</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D23" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E23">
-        <v>9.99</v>
+        <v>9.74</v>
       </c>
       <c r="F23" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 選題非常新穎且具時事性，從藥物機制到社會政策的討論深度極高，內容含金量豐富。 | [《財富自由心理學》：賺錢，只是...] 選題「財富自由心理學」新穎且具深度，透過個人故事與哲學思辨，將財富議題提升至心靈層次，內容含金量高，案例生動具啟發性。 | [手總是停不下來？那是焦慮在尋找...] 選題新穎且具深度，深入探討身體重複行為的心理學面向，案例生動且內容含金量極高。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
       </c>
     </row>
     <row r="24">
@@ -857,19 +872,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C24" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D24" t="str">
-        <v>梁哲維</v>
+        <v>蕭邦</v>
       </c>
       <c r="E24">
-        <v>9.82</v>
+        <v>9.74</v>
       </c>
       <c r="F24" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目以一本關於「好感影響力」的書為引子，邀請書中提及的創業家來分享故事，選題獨特且具深度。來賓的70年滷味傳承與公益行動，提供了豐富的內容含金量和啟發性。 | [【EP302 把命盤變成行動藍...] 選題新穎，結合「九紫離火運」與AI、全球局勢、個人發展等多元面向，案例生動且內容含金量極高。 | [【EP312《超越我執的生活》...] 選題「超越我執」具備深度與啟發性，結合心理學與靈性成長，內容含金量高，案例（如內在聲音、吃飯專注）生動且具體，展現了優秀的單元企劃能力。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
       </c>
     </row>
     <row r="25">
@@ -877,19 +892,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C25" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D25" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E25">
-        <v>9.76</v>
+        <v>9.72</v>
       </c>
       <c r="F25" t="str">
-        <v>[#801 市場震盪 17000...] 選題緊扣時事（股市下跌），並結合個人財務規劃與情緒管理，案例生動且內容含金量極高。 | [#809  買股票還在到處問明...] 選題「獲利加速系統」具備高度實用性與深度，結合AI工具的應用，內容含金量極高，企劃新穎。 | [#798 害怕投資賠錢？不用天...] 選題新穎且具備深度，聚焦於媽媽族群的投資教育與心態建立，內容含金量高，並透過生動的比喻（如游泳、無印良品櫃子）提升理解度。</v>
+        <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
       </c>
     </row>
     <row r="26">
@@ -897,19 +912,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B26">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C26" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D26" t="str">
-        <v>莫菲穿搭</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E26">
-        <v>9.74</v>
+        <v>9.68</v>
       </c>
       <c r="F26" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
+        <v>[[EP0063] 50+Con...] 選題新穎，結合「第三人生大學」與「大嬸陪聊」概念，案例生動且含金量極高，具備深度思考與社會連結。 | [[EP0071] 50+Con...] 選題新穎且具深度，聚焦於二代接班與職涯轉型，來賓的個人案例生動且含金量極高，提供了獨特的視角和實用建議。 | [[EP0045] 50+Con...] 選題深入探討紫微斗數的「四化」與「殺破狼」命格，不僅新穎且具備高度的專業含金量。來賓的案例分享與對社會現象的連結，讓內容更具啟發性與實用價值。</v>
       </c>
     </row>
     <row r="27">
@@ -917,19 +932,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B27">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C27" t="str">
-        <v>蕭邦相談室</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D27" t="str">
-        <v>蕭邦</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E27">
-        <v>9.74</v>
+        <v>9.66</v>
       </c>
       <c r="F27" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
+        <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
       </c>
     </row>
     <row r="28">
@@ -937,79 +952,79 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B28">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C28" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>宋家小館</v>
       </c>
       <c r="D28" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E28">
-        <v>9.72</v>
+        <v>9.65</v>
       </c>
       <c r="F28" t="str">
-        <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
+        <v>[EP162 | 從房地產到Ma...] 選題新穎，結合來賓的獨特職涯與創業經驗，案例生動且內容含金量極高，具備深度思考與利基選題。 | [EP191 | 《我到日本當漁...] 選題新穎且具備高度利基性，探討台灣人赴日擔任漁夫的獨特經歷，結合家族養殖業歷史，內容含金量高且引人入勝。 | [EP182 | 聽見身體的聲音...] 選題新穎且具深度，將頌缽音療的歷史、科學原理、身心影���及實際應用解釋得非常透徹，內容含金量高。</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>最神單元企劃獎</v>
+        <v>最佳男播音員獎</v>
       </c>
       <c r="B29">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C29" t="str">
-        <v>我的動齡限量版</v>
+        <v>五吉郎</v>
       </c>
       <c r="D29" t="str">
-        <v>我的動齡限量版</v>
+        <v>五吉郎</v>
       </c>
       <c r="E29">
-        <v>9.68</v>
+        <v>9.55</v>
       </c>
       <c r="F29" t="str">
-        <v>[[EP0063] 50+Con...] 選題新穎，結合「第三人生大學」與「大嬸陪聊」概念，案例生動且含金量極高，具備深度思考與社會連結。 | [[EP0071] 50+Con...] 選題新穎且具深度，聚焦於二代接班與職涯轉型，來賓的個人案例生動且含金量極高，提供了獨特的視角和實用建議。 | [[EP0045] 50+Con...] 選題深入探討紫微斗數的「四化」與「殺破狼」命格，不僅新穎且具備高度的專業含金量。來賓的案例分享與對社會現象的連結，讓內容更具啟發性與實用價值。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 男主持人聲音清晰、有活力，中低音共鳴感佳，語速穩定度高，但口頭禪「就是」和「然後」出現頻率稍高。 | [EP174｜越省反而越窮？別把...] Andy的聲音溫暖清晰，語速穩定。好哥和蔡宇哲老師的聲音也很有特色，整體男聲表現優異。 | [EP164｜滑短影音是在浪費時...] 兩位男主持人的聲音皆具備良好的中低音共鳴。主主持人Andy口條流暢，語速穩定，但偶有口頭禪；來賓好哥的聲音則更為沉穩且富有磁性，整體播音表現優異。</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>最神單元企劃獎</v>
+        <v>最佳男播音員獎</v>
       </c>
       <c r="B30">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C30" t="str">
-        <v>下一本讀什麼？</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D30" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E30">
-        <v>9.66</v>
+        <v>9.49</v>
       </c>
       <c r="F30" t="str">
-        <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 男來賓（蔡醫師）口條流暢，聲音專業且具說服力，解釋複雜概念清晰易懂，語速雖快但穩定。 | [《財富自由心理學》：賺錢，只是...] 兩位男主持人皆表現出色。主講人雨哲口條流暢，聲音清晰溫和，語速穩定。來賓好哥聲線低沉有磁性，論述力強。整體播音實力優異。</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>最神單元企劃獎</v>
+        <v>最佳男播音員獎</v>
       </c>
       <c r="B31">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C31" t="str">
-        <v>宋家小館</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D31" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>梁哲維</v>
       </c>
       <c r="E31">
-        <v>9.65</v>
+        <v>9.32</v>
       </c>
       <c r="F31" t="str">
-        <v>[EP162 | 從房地產到Ma...] 選題新穎，結合來賓的獨特職涯與創業經驗，案例生動且內容含金量極高，具備深度思考與利基選題。 | [EP191 | 《我到日本當漁...] 選題新穎且具備高度利基性，探討台灣人赴日擔任漁夫的獨特經歷，結合家族養殖業歷史，內容含金量高且引人入勝。 | [EP182 | 聽見身體的聲音...] 選題新穎且具深度，將頌缽音療的歷史、科學原理、身心影���及實際應用解釋得非常透徹，內容含金量高。</v>
+        <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
       </c>
     </row>
     <row r="32">
@@ -1017,19 +1032,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C32" t="str">
-        <v>五吉郎</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D32" t="str">
-        <v>五吉郎</v>
+        <v>蕭邦</v>
       </c>
       <c r="E32">
-        <v>9.55</v>
+        <v>9.24</v>
       </c>
       <c r="F32" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 男主持人聲音清晰、有活力，中低音共鳴感佳，語速穩定度高，但口頭禪「就是」和「然後」出現頻率稍高。 | [EP174｜越省反而越窮？別把...] Andy的聲音溫暖清晰，語速穩定。好哥和蔡宇哲老師的聲音也很有特色，整體男聲表現優異。 | [EP164｜滑短影音是在浪費時...] 兩位男主持人的聲音皆具備良好的中低音共鳴。主主持人Andy口條流暢，語速穩定，但偶有口頭禪；來賓好哥的聲音則更為沉穩且富有磁性，整體播音表現優異。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
       </c>
     </row>
     <row r="33">
@@ -1037,19 +1052,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C33" t="str">
-        <v>哇賽心理學</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D33" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E33">
-        <v>9.49</v>
+        <v>9.21</v>
       </c>
       <c r="F33" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 男來賓（蔡醫師）口條流暢，聲音專業且具說服力，解釋複雜概念清晰易懂，語速雖快但穩定。 | [《財富自由心理學》：賺錢，只是...] 兩位男主持人皆表現出色。主講人雨哲口條流暢，聲音清晰溫和，語速穩定。來賓好哥聲線低沉有磁性，論述力強。整體播音實力優異。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
       </c>
     </row>
     <row r="34">
@@ -1057,19 +1072,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B34">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C34" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D34" t="str">
-        <v>梁哲維</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E34">
-        <v>9.32</v>
+        <v>9.16</v>
       </c>
       <c r="F34" t="str">
-        <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
+        <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
       </c>
     </row>
     <row r="35">
@@ -1077,19 +1092,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B35">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C35" t="str">
-        <v>蕭邦相談室</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D35" t="str">
-        <v>蕭邦</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E35">
-        <v>9.24</v>
+        <v>9.09</v>
       </c>
       <c r="F35" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
       </c>
     </row>
     <row r="36">
@@ -1097,19 +1112,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B36">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C36" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>財富餐車不打烊</v>
       </c>
       <c r="D36" t="str">
-        <v>GK爸爸</v>
+        <v>30節約男子</v>
       </c>
       <c r="E36">
-        <v>9.21</v>
+        <v>9.07</v>
       </c>
       <c r="F36" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
+        <v>[【EP39】矽谷阿雅｜貸款七百...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，但口頭禪「就是」和「然後」出現頻率稍高。 | [【EP51】胡咪＆Vito大叔...] Vito大叔的口條流暢，聲音低沉有磁性，語速穩定，能有效傳達情感。偶爾的口頭禪「就是」略多但不影響整體表現。 | [【EP36】明白｜父母雙亡，獨...] 男主持人聲音厚實有共鳴，語速雖快但咬字清晰，表達流暢。口頭禪「然後」、「就是」出現頻率稍高，但整體不影響專業度。</v>
       </c>
     </row>
     <row r="37">
@@ -1117,19 +1132,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B37">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C37" t="str">
-        <v>下一本讀什麼？</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D37" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E37">
-        <v>9.16</v>
+        <v>9.06</v>
       </c>
       <c r="F37" t="str">
-        <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
+        <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
       </c>
     </row>
     <row r="38">
@@ -1137,79 +1152,79 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B38">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C38" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D38" t="str">
-        <v>人生啊！小歐</v>
+        <v>張忘形</v>
       </c>
       <c r="E38">
-        <v>9.09</v>
+        <v>9.03</v>
       </c>
       <c r="F38" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
+        <v>[EP61｜為什麼越努力經營，反...] 男主持人聲音清晰、能量高，中低音共鳴感良好，語速雖快但仍能保持清晰度。情緒感染力強，但口頭禪「就是」出現頻率稍高。 | [EP50｜看到什麼都東西都想拍...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰，情感表達豐富。但口頭禪「就是」和「然後」出現頻率稍高，略影響流暢度。 | [EP65｜ 對方因為小事就對你...] 男主持人聲音厚實有共鳴，語速偏快但清晰度高，情感表達豐富。然而，「就是」和「那」等口頭禪出現頻率較高，略影響流暢度。</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>最佳男播音員獎</v>
+        <v>最佳女播音員獎</v>
       </c>
       <c r="B39">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C39" t="str">
-        <v>財富餐車不打烊</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D39" t="str">
-        <v>30節約男子</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E39">
-        <v>9.07</v>
+        <v>9.43</v>
       </c>
       <c r="F39" t="str">
-        <v>[【EP39】矽谷阿雅｜貸款七百...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，但口頭禪「就是」和「然後」出現頻率稍高。 | [【EP51】胡咪＆Vito大叔...] Vito大叔的口條流暢，聲音低沉有磁性，語速穩定，能有效傳達情感。偶爾的口頭禪「就是」略多但不影響整體表現。 | [【EP36】明白｜父母雙亡，獨...] 男主持人聲音厚實有共鳴，語速雖快但咬字清晰，表達流暢。口頭禪「然後」、「就是」出現頻率稍高，但整體不影響專業度。</v>
+        <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>最佳男播音員獎</v>
+        <v>最佳女播音員獎</v>
       </c>
       <c r="B40">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C40" t="str">
-        <v>夢想家說股事</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D40" t="str">
-        <v>美股夢想家</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E40">
-        <v>9.06</v>
+        <v>9.41</v>
       </c>
       <c r="F40" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>最佳男播音員獎</v>
+        <v>最佳女播音員獎</v>
       </c>
       <c r="B41">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C41" t="str">
-        <v>人類行為研究社</v>
+        <v>宋家小館</v>
       </c>
       <c r="D41" t="str">
-        <v>張忘形</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E41">
-        <v>9.03</v>
+        <v>9.32</v>
       </c>
       <c r="F41" t="str">
-        <v>[EP61｜為什麼越努力經營，反...] 男主持人聲音清晰、能量高，中低音共鳴感良好，語速雖快但仍能保持清晰度。情緒感染力強，但口頭禪「就是」出現頻率稍高。 | [EP50｜看到什麼都東西都想拍...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰，情感表達豐富。但口頭禪「就是」和「然後」出現頻率稍高，略影響流暢度。 | [EP65｜ 對方因為小事就對你...] 男主持人聲音厚實有共鳴，語速偏快但清晰度高，情感表達豐富。然而，「就是」和「那」等口頭禪出現頻率較高，略影響流暢度。</v>
+        <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
       </c>
     </row>
     <row r="42">
@@ -1217,19 +1232,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B42">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C42" t="str">
-        <v>布姐的沙發</v>
+        <v>說話人聲</v>
       </c>
       <c r="D42" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>聲音表達講師林依柔</v>
       </c>
       <c r="E42">
-        <v>9.43</v>
+        <v>9.31</v>
       </c>
       <c r="F42" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
+        <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
       </c>
     </row>
     <row r="43">
@@ -1237,19 +1252,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C43" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D43" t="str">
-        <v>莫菲穿搭</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E43">
-        <v>9.41</v>
+        <v>9.31</v>
       </c>
       <c r="F43" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
       </c>
     </row>
     <row r="44">
@@ -1257,19 +1272,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B44">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C44" t="str">
-        <v>宋家小館</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D44" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E44">
-        <v>9.32</v>
+        <v>9.26</v>
       </c>
       <c r="F44" t="str">
-        <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
+        <v>[#801 市場震盪 17000...] 女主持人聲音清晰、溫暖且具共鳴，語速穩定舒適，情緒感染��佳，但偶有贅字。 | [#809  買股票還在到處問明...] Cindy2聲音圓潤清晰，語速適中，語調親和，具備溫馨陪伴感，引導能力強。 | [#798 害怕投資賠錢？不用天...] 兩位女主持人聲音清晰、語速快但穩定，高音域圓潤且具備溫馨陪伴感，無刺耳爆音。主講人Sandy的語速較快，但整體表現優異。</v>
       </c>
     </row>
     <row r="45">
@@ -1277,19 +1292,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B45">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C45" t="str">
-        <v>楊肉盧</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D45" t="str">
-        <v>楊月娥（楊肉爐）</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E45">
-        <v>9.31</v>
+        <v>9.23</v>
       </c>
       <c r="F45" t="str">
-        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人聲音清晰，語速穩定，楊月娥的聲音富有感染力，小真的聲音溫和具陪伴感，整體播音實力優異。 | [EP142｜【母女鍋】你的大頭...] 兩位女主持人的口條皆非常流暢，發音清晰，語速穩定且舒適。楊月娥的聲音溫暖具陪伴感，路妍蓁則充滿活力與分析力，兩者相得益彰。 | [EP139｜【全家鍋】開始運動...] 女主持人語速較快，但發音清晰，語調充滿活力與感染力，能有效帶動節目氣氛。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
       </c>
     </row>
     <row r="46">
@@ -1297,19 +1312,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B46">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C46" t="str">
-        <v>說話人聲</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D46" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E46">
-        <v>9.31</v>
+        <v>9.18</v>
       </c>
       <c r="F46" t="str">
-        <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
+        <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
       </c>
     </row>
     <row r="47">
@@ -1317,19 +1332,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B47">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C47" t="str">
-        <v>蘇心時光</v>
+        <v>美業幹什麼</v>
       </c>
       <c r="D47" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="E47">
-        <v>9.31</v>
+        <v>9.07</v>
       </c>
       <c r="F47" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
+        <v>[EP199-別再相信快速致富：...] 女主持人阿莉口條流暢，聲音清晰且富有感染力，語速雖快但穩定，高音域圓潤，具備溫馨陪伴感。 | [EP192-當貴人還沒出現時，...] 女主持人阿令的聲音明亮清晰，高音域圓潤且富有親和力，語速偏快但咬字清晰，情感表達真誠，具有良好的播音魅力。 | [EP210-會做不一定會贏｜表...] 女主持人阿林口條流暢，聲音清晰，語速穩定，高音域圓潤且具陪伴感，但偶有贅字。</v>
       </c>
     </row>
     <row r="48">
@@ -1337,79 +1352,79 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B48">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C48" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D48" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E48">
-        <v>9.26</v>
+        <v>9.01</v>
       </c>
       <c r="F48" t="str">
-        <v>[#801 市場震盪 17000...] 女主持人聲音清晰、溫暖且具共鳴，語速穩定舒適，情緒感染��佳，但偶有贅字。 | [#809  買股票還在到處問明...] Cindy2聲音圓潤清晰，語速適中，語調親和，具備溫馨陪伴感，引導能力強。 | [#798 害怕投資賠錢？不用天...] 兩位女主持人聲音清晰、語速快但穩定，高音域圓潤且具備溫馨陪伴感，無刺耳爆音。主講人Sandy的語速較快，但整體表現優異。</v>
+        <v>[EP.322 流量破百萬卻賺不...] 女主持人聲音清晰、溫暖且富有感染力，語速較快但口條流暢，能有效傳達資訊與情感。 | [EP.318 行銷不是方法，是...] 女主持人聲音清晰、溫暖，語速穩定舒適，高音域圓潤，具備溫馨陪伴感，播音實力優異。 | [EP.316 與其等流量，不如...] 主講人Nico聲音清晰、語速穩定且富有活力，高音域圓潤，雖有口頭禪但整體播音品質優良。</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>最佳女播音員獎</v>
+        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B49">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C49" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>五吉郎</v>
       </c>
       <c r="D49" t="str">
-        <v>丁菱娟</v>
+        <v>五吉郎</v>
       </c>
       <c r="E49">
-        <v>9.23</v>
+        <v>8.88</v>
       </c>
       <c r="F49" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 結尾有明確呼籲聽眾行動，力道足夠，能有效催化聽眾實踐。 | [EP174｜越省反而越窮？別把...] 結尾有明確的行動呼籲，鼓勵聽眾訂閱、留言、並嘗試微小行動，力道足夠。 | [EP164｜滑短影音是在浪費時...] 節目中多次提及來賓的新書，並在結尾有明確的行動呼籲，但力道尚可加強，未達到極強的催化效果。</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>最佳女播音員獎</v>
+        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B50">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C50" t="str">
-        <v>我的動齡限量版</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D50" t="str">
-        <v>我的動齡限量版</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E50">
-        <v>9.18</v>
+        <v>8.83</v>
       </c>
       <c r="F50" t="str">
-        <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>最佳女播音員獎</v>
+        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B51">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C51" t="str">
-        <v>美業幹什麼</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D51" t="str">
-        <v>美業幹什麼｜蔡佩陵</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E51">
-        <v>9.07</v>
+        <v>8.76</v>
       </c>
       <c r="F51" t="str">
-        <v>[EP199-別再相信快速致富：...] 女主持人阿莉口條流暢，聲音清晰且富有感染力，語速雖快但穩定，高音域圓潤，具備溫馨陪伴感。 | [EP192-當貴人還沒出現時，...] 女主持人阿令的聲音明亮清晰，高音域圓潤且富有親和力，語速偏快但咬字清晰，情感表達真誠，具有良好的播音魅力。 | [EP210-會做不一定會贏｜表...] 女主持人阿林口條流暢，聲音清晰，語速穩定，高音域圓潤且具陪伴感，但偶有贅字。</v>
+        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
       </c>
     </row>
     <row r="52">
@@ -1417,19 +1432,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C52" t="str">
-        <v>五吉郎</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D52" t="str">
-        <v>五吉郎</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E52">
-        <v>8.88</v>
+        <v>8.72</v>
       </c>
       <c r="F52" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 結尾有明確呼籲聽眾行動，力道足夠，能有效催化聽眾實踐。 | [EP174｜越省反而越窮？別把...] 結尾有明確的行動呼籲，鼓勵聽眾訂閱、留言、並嘗試微小行動，力道足夠。 | [EP164｜滑短影音是在浪費時...] 節目中多次提及來賓的新書，並在結尾有明確的行動呼籲，但力道尚可加強，未達到極強的催化效果。</v>
+        <v>[EP225：【非典家庭CEO】...] 結尾有明確的行動呼籲，鼓勵聽眾點擊連結或撥打專線了解寄養家庭資訊，力道足夠且具體。 | [EP218：愛自己｜放下完美執...] 節目結尾的行動呼籲明確，針對線上課程提供了專屬優惠碼，具體且有吸引力，能有效促使聽眾採取行動。 | [EP219：【非典家庭CEO】...] 結尾有明確呼籲聽眾行動，力道足夠，鼓勵聽眾參與動物音樂會。</v>
       </c>
     </row>
     <row r="53">
@@ -1437,19 +1452,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B53">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C53" t="str">
-        <v>哇賽心理學</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D53" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E53">
-        <v>8.83</v>
+        <v>8.66</v>
       </c>
       <c r="F53" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
+        <v>[EP.617 《無限機器》讀後...] 結尾有明確呼籲聽眾訂閱電子報與節目，行動呼籲力道足夠且自然。 | [EP.573 從 0 到 10...] 結尾有明確呼籲聽眾填寫問卷和分享電子報，力道足夠且具體。 | [EP.607 《AI Firs...] 節目開頭與結尾都有明確且具說服力的行動呼籲，引導聽眾參與社群或閱讀書籍，催化力道足夠。</v>
       </c>
     </row>
     <row r="54">
@@ -1457,19 +1472,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B54">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C54" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D54" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>梁哲維</v>
       </c>
       <c r="E54">
-        <v>8.76</v>
+        <v>8.66</v>
       </c>
       <c r="F54" t="str">
-        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
       </c>
     </row>
     <row r="55">
@@ -1477,19 +1492,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B55">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C55" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D55" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E55">
-        <v>8.72</v>
+        <v>8.55</v>
       </c>
       <c r="F55" t="str">
-        <v>[EP225：【非典家庭CEO】...] 結尾有明確的行動呼籲，鼓勵聽眾點擊連結或撥打專線了解寄養家庭資訊，力道足夠且具體。 | [EP218：愛自己｜放下完美執...] 節目結尾的行動呼籲明確，針對線上課程提供了專屬優惠碼，具體且有吸引力，能有效促使聽眾採取行動。 | [EP219：【非典家庭CEO】...] 結尾有明確呼籲聽眾行動，力道足夠，鼓勵聽眾參與動物音樂會。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
       </c>
     </row>
     <row r="56">
@@ -1497,19 +1512,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B56">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C56" t="str">
-        <v>下一本讀什麼？</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D56" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E56">
-        <v>8.66</v>
+        <v>8.54</v>
       </c>
       <c r="F56" t="str">
-        <v>[EP.617 《無限機器》讀後...] 結尾有明確呼籲聽眾訂閱電子報與節目，行動呼籲力道足夠且自然。 | [EP.573 從 0 到 10...] 結尾有明確呼籲聽眾填寫問卷和分享電子報，力道足夠且具體。 | [EP.607 《AI Firs...] 節目開頭與結尾都有明確且具說服力的行動呼籲，引導聽眾參與社群或閱讀書籍，催化力道足夠。</v>
+        <v>[EP611 00998A(主動...] 結尾有明確呼籲聽眾查詢ETF資訊並諮詢營業員，行動呼籲清晰但力道中等。 | [EP628昇陽半導體(8028...] 結尾有明確呼籲聽眾參與其課程，行動呼籲力道足夠且資訊完整。 | [EP621《富媽媽 窮媽媽》第...] 結尾明確呼籲聽眾購買書籍以獲取更多資訊，並分享節目，行動呼籲清晰且具體。</v>
       </c>
     </row>
     <row r="57">
@@ -1517,19 +1532,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B57">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C57" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D57" t="str">
-        <v>梁哲維</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E57">
-        <v>8.66</v>
+        <v>8.51</v>
       </c>
       <c r="F57" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
+        <v>[EP.322 流量破百萬卻賺不...] 節目中段與結尾皆有明確的行動呼籲，引導聽眾訂閱、諮詢或了解更多資訊，力道足夠且具體。 | [EP.318 行銷不是方法，是...] 在節目中段和結尾都有明確且具說服力的行動呼籲，力道足夠，能有效催化聽眾實踐。 | [EP.316 與其等流量，不如...] 結尾行動呼籲明確，針對線上課程提供折扣碼與期限，具備足夠的催化力。</v>
       </c>
     </row>
     <row r="58">
@@ -1537,79 +1552,79 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B58">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C58" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D58" t="str">
-        <v>GK爸爸</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E58">
-        <v>8.55</v>
+        <v>8.49</v>
       </c>
       <c r="F58" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
+        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
+        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B59">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C59" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D59" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E59">
-        <v>8.54</v>
+        <v>9.22</v>
       </c>
       <c r="F59" t="str">
-        <v>[EP611 00998A(主動...] 結尾有明確呼籲聽眾查詢ETF資訊並諮詢營業員，行動呼籲清晰但力道中等。 | [EP628昇陽半導體(8028...] 結尾有明確呼籲聽眾參與其課程，行動呼籲力道足夠且資訊完整。 | [EP621《富媽媽 窮媽媽》第...] 結尾明確呼籲聽眾購買書籍以獲取更多資訊，並分享節目，行動呼籲清晰且具體。</v>
+        <v>[EP225：【非典家庭CEO】...] 寄養家庭議題雖然非絕對冷門，但節目深入探討其背後的挑戰、家庭動員與個人成長，提供了獨特的視角和豐富的細節，論述完整且具深度。 | [EP218：愛自己｜放下完美執...] 人類圖本身即為利基市場，本集更深入探討流日、閘門與關係互動等細節，論述完整且具專業度，滿足了特定聽眾群的深度需求。 | [EP219：【非典家庭CEO】...] 雖然育兒是廣泛議題，但從專業音樂家角度切入，並結合獨特的動物音樂會推廣，使其具備高度利基市場價值。</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
+        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B60">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C60" t="str">
-        <v>尼可這樣說</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D60" t="str">
-        <v>尼可這樣說</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E60">
-        <v>8.51</v>
+        <v>9.16</v>
       </c>
       <c r="F60" t="str">
-        <v>[EP.322 流量破百萬卻賺不...] 節目中段與結尾皆有明確的行動呼籲，引導聽眾訂閱、諮詢或了解更多資訊，力道足夠且具體。 | [EP.318 行銷不是方法，是...] 在節目中段和結尾都有明確且具說服力的行動呼籲，力道足夠，能有效催化聽眾實踐。 | [EP.316 與其等流量，不如...] 結尾行動呼籲明確，針對線上課程提供折扣碼與期限，具備足夠的催化力。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
+        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B61">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C61" t="str">
-        <v>分手的99個理由</v>
+        <v>宋家小館</v>
       </c>
       <c r="D61" t="str">
-        <v>胡咪老師</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E61">
-        <v>8.49</v>
+        <v>8.99</v>
       </c>
       <c r="F61" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
+        <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
       </c>
     </row>
     <row r="62">
@@ -1617,19 +1632,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B62">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C62" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D62" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E62">
-        <v>9.22</v>
+        <v>8.9</v>
       </c>
       <c r="F62" t="str">
-        <v>[EP225：【非典家庭CEO】...] 寄養家庭議題雖然非絕對冷門，但節目深入探討其背後的挑戰、家庭動員與個人成長，提供了獨特的視角和豐富的細節，論述完整且具深度。 | [EP218：愛自己｜放下完美執...] 人類圖本身即為利基市場，本集更深入探討流日、閘門與關係互動等細節，論述完整且具專業度，滿足了特定聽眾群的深度需求。 | [EP219：【非典家庭CEO】...] 雖然育兒是廣泛議題，但從專業音樂家角度切入，並結合獨特的動物音樂會推廣，使其具備高度利基市場價值。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
       </c>
     </row>
     <row r="63">
@@ -1637,19 +1652,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C63" t="str">
-        <v>哇賽心理學</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D63" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>蕭邦</v>
       </c>
       <c r="E63">
-        <v>9.16</v>
+        <v>8.74</v>
       </c>
       <c r="F63" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
       </c>
     </row>
     <row r="64">
@@ -1657,19 +1672,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B64">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C64" t="str">
-        <v>宋家小館</v>
+        <v>教出你的路</v>
       </c>
       <c r="D64" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>治療師瑪奇</v>
       </c>
       <c r="E64">
-        <v>8.99</v>
+        <v>8.66</v>
       </c>
       <c r="F64" t="str">
-        <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
+        <v>[EP47 有團隊的感覺如何？教...] 解剖學結合運動教學是一個相對利基的市場，主持人以獨特視角切入，論述完整且具深度，不易被取代。 | [EP31 為了愛移民，她打造 ...] 以植物性飲食為核心，並強調非卡路里導向的理念，在健康飲食領域中具備獨特的利基市場視角。 | [EP35 為什麼堅持開「解剖學...] 「應用解剖運動學」是一個相對專業且具利基性的市場，主持人對此議題的論述深入且完整，有效觸及目標受眾的需求。</v>
       </c>
     </row>
     <row r="65">
@@ -1677,19 +1692,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B65">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C65" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D65" t="str">
-        <v>無所不試無樂不作</v>
+        <v>梁哲維</v>
       </c>
       <c r="E65">
-        <v>8.9</v>
+        <v>8.66</v>
       </c>
       <c r="F65" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
+        <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
       </c>
     </row>
     <row r="66">
@@ -1697,19 +1712,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B66">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C66" t="str">
-        <v>蕭邦相談室</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D66" t="str">
-        <v>蕭邦</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E66">
-        <v>8.74</v>
+        <v>8.64</v>
       </c>
       <c r="F66" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
       </c>
     </row>
     <row r="67">
@@ -1717,19 +1732,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B67">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C67" t="str">
-        <v>教出你的路</v>
+        <v>財富餐車不打烊</v>
       </c>
       <c r="D67" t="str">
-        <v>治療師瑪奇</v>
+        <v>30節約男子</v>
       </c>
       <c r="E67">
-        <v>8.66</v>
+        <v>8.57</v>
       </c>
       <c r="F67" t="str">
-        <v>[EP47 有團隊的感覺如何？教...] 解剖學結合運動教學是一個相對利基的市場，主持人以獨特視角切入，論述完整且具深度，不易被取代。 | [EP31 為了愛移民，她打造 ...] 以植物性飲食為核心，並強調非卡路里導向的理念，在健康飲食領域中具備獨特的利基市場視角。 | [EP35 為什麼堅持開「解剖學...] 「應用解剖運動學」是一個相對專業且具利基性的市場，主持人對此議題的論述深入且完整，有效觸及目標受眾的需求。</v>
+        <v>[【EP39】矽谷阿雅｜貸款七百...] AI驅動的男士時尚租賃服務是一個非常具體的利基市場，節目對其論述完整且深入。 | [【EP51】胡咪＆Vito大叔...] 理財主題雖廣泛，但結合來賓的「30節約男」個人故事和「斷捨離」等具體實踐，使其在同類節目中具有一定的獨特性。 | [【EP36】明白｜父母雙亡，獨...] 議題稀有度高，將「獨生女」概念延伸至人生獨自面對挑戰的普遍性，論述完整且具啟發性。</v>
       </c>
     </row>
     <row r="68">
@@ -1737,27 +1752,27 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B68">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C68" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D68" t="str">
-        <v>梁哲維</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E68">
-        <v>8.66</v>
+        <v>8.57</v>
       </c>
       <c r="F68" t="str">
-        <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 議題聚焦台灣科技產業的供應鏈與產業分析，雖非極度冷門，但論述深度與專業性使其在利基市場中表現突出。 | [ep11. Z世代難搞嗎？用對...] Z世代議題雖非極度冷門，但節目從職場管理、品牌行銷等多維度深入剖析，並結合實務經驗，提供了獨特的觀點與論述，使其在同類議題中具備差異化。 | [ep23. 主動出擊的力量有多...] 議題雖非極度冷門，但以「搭訕」為切入點，並將其應用於廣泛的生活層面，論述獨特且完整。</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
+        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B69">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C69" t="str">
         <v>蘇心時光</v>
@@ -1766,50 +1781,50 @@
         <v>蘇絢慧分享空間</v>
       </c>
       <c r="E69">
-        <v>8.64</v>
+        <v>9.31</v>
       </c>
       <c r="F69" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
+        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B70">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C70" t="str">
-        <v>財富餐車不打烊</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D70" t="str">
-        <v>30節約男子</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E70">
-        <v>8.57</v>
+        <v>9.06</v>
       </c>
       <c r="F70" t="str">
-        <v>[【EP39】矽谷阿雅｜貸款七百...] AI驅動的男士時尚租賃服務是一個非常具體的利基市場，節目對其論述完整且深入。 | [【EP51】胡咪＆Vito大叔...] 理財主題雖廣泛，但結合來賓的「30節約男」個人故事和「斷捨離」等具體實踐，使其在同類節目中具有一定的獨特性。 | [【EP36】明白｜父母雙亡，獨...] 議題稀有度高，將「獨生女」概念延伸至人生獨自面對挑戰的普遍性，論述完整且具啟發性。</v>
+        <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
+        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B71">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C71" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>宋家小館</v>
       </c>
       <c r="D71" t="str">
-        <v>丁菱娟</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E71">
-        <v>8.57</v>
+        <v>8.99</v>
       </c>
       <c r="F71" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 議題聚焦台灣科技產業的供應鏈與產業分析，雖非極度冷門，但論述深度與專業性使其在利基市場中表現突出。 | [ep11. Z世代難搞嗎？用對...] Z世代議題雖非極度冷門，但節目從職場管理、品牌行銷等多維度深入剖析，並結合實務經驗，提供了獨特的觀點與論述，使其在同類議題中具備差異化。 | [ep23. 主動出擊的力量有多...] 議題雖非極度冷門，但以「搭訕」為切入點，並將其應用於廣泛的生活層面，論述獨特且完整。</v>
+        <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
       </c>
     </row>
     <row r="72">
@@ -1817,19 +1832,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B72">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C72" t="str">
-        <v>蘇心時光</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D72" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E72">
-        <v>9.31</v>
+        <v>8.99</v>
       </c>
       <c r="F72" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
+        <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
       </c>
     </row>
     <row r="73">
@@ -1837,19 +1852,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B73">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C73" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D73" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E73">
-        <v>9.06</v>
+        <v>8.93</v>
       </c>
       <c r="F73" t="str">
-        <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
+        <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
       </c>
     </row>
     <row r="74">
@@ -1857,19 +1872,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B74">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C74" t="str">
-        <v>宋家小館</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D74" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E74">
-        <v>8.99</v>
+        <v>8.9</v>
       </c>
       <c r="F74" t="str">
-        <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="75">
@@ -1877,19 +1892,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B75">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C75" t="str">
-        <v>分手的99個理由</v>
+        <v>五吉郎</v>
       </c>
       <c r="D75" t="str">
-        <v>胡咪老師</v>
+        <v>五吉郎</v>
       </c>
       <c r="E75">
-        <v>8.99</v>
+        <v>8.88</v>
       </c>
       <c r="F75" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 整體語調平穩溫和，適合深夜靜聽，但部分討論較為熱情，略有起伏。 | [EP174｜越省反而越窮？別把...] 聲音平穩，語調溫和，適合深夜聆聽，無突兀尖銳音。 | [EP164｜滑短影音是在浪費時...] 節目氛圍沉穩且具思考性，兩位主持人的語調平穩溫和，適合聽眾在夜晚靜心聆聽與反思，無突兀尖銳音效。</v>
       </c>
     </row>
     <row r="76">
@@ -1897,19 +1912,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B76">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C76" t="str">
-        <v>布姐的沙發</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D76" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E76">
-        <v>8.93</v>
+        <v>8.88</v>
       </c>
       <c r="F76" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="77">
@@ -1917,19 +1932,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B77">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C77" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>下半場人生陪談師</v>
       </c>
       <c r="D77" t="str">
-        <v>無所不試無樂不作</v>
+        <v>下半場人生事務有限公司</v>
       </c>
       <c r="E77">
-        <v>8.9</v>
+        <v>8.86</v>
       </c>
       <c r="F77" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
+        <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="78">
@@ -1937,79 +1952,79 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B78">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C78" t="str">
-        <v>五吉郎</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D78" t="str">
-        <v>五吉郎</v>
+        <v>梁哲維</v>
       </c>
       <c r="E78">
-        <v>8.88</v>
+        <v>8.82</v>
       </c>
       <c r="F78" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 整體語調平穩溫和，適合深夜靜聽，但部分討論較為熱情，略有起伏。 | [EP174｜越省反而越窮？別把...] 聲音平穩，語調溫和，適合深夜聆聽，無突兀尖銳音。 | [EP164｜滑短影音是在浪費時...] 節目氛圍沉穩且具思考性，兩位主持人的語調平穩溫和，適合聽眾在夜晚靜心聆聽與反思，無突兀尖銳音效。</v>
+        <v>[【EP330 帶著善意行動，最...] 聲音平穩溫和，談話內容有深度，適合深夜靜聽與思考。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的語調溫和穩定，聲音品質優良，適合在深夜時段放鬆聆聽，具有陪伴治癒感。 | [【EP312《超越我執的生活》...] 主持人語調溫和穩定，聲音沉穩，內容具備深度思考，無突兀尖銳爆音，非常適合深夜聆聽，能帶來陪伴與沉靜感。</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
+        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B79">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C79" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>五吉郎</v>
       </c>
       <c r="D79" t="str">
-        <v>GK爸爸</v>
+        <v>五吉郎</v>
       </c>
       <c r="E79">
-        <v>8.88</v>
+        <v>9.22</v>
       </c>
       <c r="F79" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
+        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B80">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C80" t="str">
-        <v>下半場人生陪談師</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D80" t="str">
-        <v>下半場人生事務有限公司</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E80">
-        <v>8.86</v>
+        <v>9.16</v>
       </c>
       <c r="F80" t="str">
-        <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
+        <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
+        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B81">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C81" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D81" t="str">
-        <v>梁哲維</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E81">
-        <v>8.82</v>
+        <v>9.16</v>
       </c>
       <c r="F81" t="str">
-        <v>[【EP330 帶著善意行動，最...] 聲音平穩溫和，談話內容有深度，適合深夜靜聽與思考。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的語調溫和穩定，聲音品質優良，適合在深夜時段放鬆聆聽，具有陪伴治癒感。 | [【EP312《超越我執的生活》...] 主持人語調溫和穩定，聲音沉穩，內容具備深度思考，無突兀尖銳爆音，非常適合深夜聆聽，能帶來陪伴與沉靜感。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
       </c>
     </row>
     <row r="82">
@@ -2017,19 +2032,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B82">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C82" t="str">
-        <v>五吉郎</v>
+        <v>郝聲音</v>
       </c>
       <c r="D82" t="str">
-        <v>五吉郎</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E82">
-        <v>9.22</v>
+        <v>9.09</v>
       </c>
       <c r="F82" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
+        <v>[郝聲音：（下） 莊鈞涵（Car...] 節奏明快，主持人與來賓充滿朝氣，內容實用且具激勵性，適合通勤時提神醒腦。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目節奏明快，開頭活力十足，內容實用且具啟發性，適合通勤時提神醒腦與獲取新知。 | [郝聲音：成為人生更自由的「精銳...] 節奏明快，語調朝氣蓬勃，內容具啟發性，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="83">
@@ -2037,19 +2052,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B83">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C83" t="str">
-        <v>下一本讀什麼？</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D83" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E83">
-        <v>9.16</v>
+        <v>9.07</v>
       </c>
       <c r="F83" t="str">
-        <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="84">
@@ -2057,19 +2072,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B84">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C84" t="str">
-        <v>哇賽心理學</v>
+        <v>能量黑客</v>
       </c>
       <c r="D84" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E84">
-        <v>9.16</v>
+        <v>9.06</v>
       </c>
       <c r="F84" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
       </c>
     </row>
     <row r="85">
@@ -2077,19 +2092,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B85">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C85" t="str">
-        <v>郝聲音</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D85" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E85">
-        <v>9.09</v>
+        <v>9.04</v>
       </c>
       <c r="F85" t="str">
-        <v>[郝聲音：（下） 莊鈞涵（Car...] 節奏明快，主持人與來賓充滿朝氣，內容實用且具激勵性，適合通勤時提神醒腦。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目節奏明快，開頭活力十足，內容實用且具啟發性，適合通勤時提神醒腦與獲取新知。 | [郝聲音：成為人生更自由的「精銳...] 節奏明快，語調朝氣蓬勃，內容具啟發性，非常適合通勤時提神醒腦。</v>
+        <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
       </c>
     </row>
     <row r="86">
@@ -2097,19 +2112,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B86">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C86" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>閱讀聊樂KEY</v>
       </c>
       <c r="D86" t="str">
-        <v>丁菱娟</v>
+        <v>閱讀聊樂key</v>
       </c>
       <c r="E86">
-        <v>9.07</v>
+        <v>9.03</v>
       </c>
       <c r="F86" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
+        <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
       </c>
     </row>
     <row r="87">
@@ -2117,19 +2132,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B87">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C87" t="str">
-        <v>能量黑客</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D87" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E87">
-        <v>9.06</v>
+        <v>9.01</v>
       </c>
       <c r="F87" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
+        <v>[EP.322 流量破百萬卻賺不...] 節目節奏明快，內容資訊量高且具啟發性，主持人與來賓的清晰表達有助於通勤時提神醒腦，適合早晨收聽。 | [EP.318 行銷不是方法，是...] 節目節奏明快，內容資訊密度高，主持人與來賓的對談朝氣十足，具有通勤提神醒腦的效果。 | [EP.316 與其等流量，不如...] 節目節奏明快，主講人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="88">
@@ -2137,79 +2152,79 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B88">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C88" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D88" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E88">
-        <v>9.04</v>
+        <v>9.01</v>
       </c>
       <c r="F88" t="str">
-        <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
+        <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
+        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B89">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C89" t="str">
-        <v>閱讀聊樂KEY</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D89" t="str">
-        <v>閱讀聊樂key</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E89">
-        <v>9.03</v>
+        <v>8.72</v>
       </c>
       <c r="F89" t="str">
-        <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
+        <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
+        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B90">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C90" t="str">
-        <v>尼可這樣說</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D90" t="str">
-        <v>尼可這樣說</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E90">
-        <v>9.01</v>
+        <v>8.33</v>
       </c>
       <c r="F90" t="str">
-        <v>[EP.322 流量破百萬卻賺不...] 節目節奏明快，內容資訊量高且具啟發性，主持人與來賓的清晰表達有助於通勤時提神醒腦，適合早晨收聽。 | [EP.318 行銷不是方法，是...] 節目節奏明快，內容資訊密度高，主持人與來賓的對談朝氣十足，具有通勤提神醒腦的效果。 | [EP.316 與其等流量，不如...] 節目節奏明快，主講人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。</v>
+        <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
+        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B91">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C91" t="str">
-        <v>我的動齡限量版</v>
+        <v>五吉郎</v>
       </c>
       <c r="D91" t="str">
-        <v>我的動齡限量版</v>
+        <v>五吉郎</v>
       </c>
       <c r="E91">
-        <v>9.01</v>
+        <v>8.22</v>
       </c>
       <c r="F91" t="str">
-        <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
       </c>
     </row>
     <row r="92">
@@ -2217,19 +2232,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B92">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C92" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D92" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E92">
-        <v>8.72</v>
+        <v>8.21</v>
       </c>
       <c r="F92" t="str">
-        <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
       </c>
     </row>
     <row r="93">
@@ -2237,19 +2252,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B93">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C93" t="str">
-        <v>分手的99個理由</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D93" t="str">
-        <v>胡咪老師</v>
+        <v>梁哲維</v>
       </c>
       <c r="E93">
-        <v>8.33</v>
+        <v>8.16</v>
       </c>
       <c r="F93" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
+        <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
       </c>
     </row>
     <row r="94">
@@ -2257,19 +2272,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B94">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C94" t="str">
-        <v>五吉郎</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D94" t="str">
-        <v>五吉郎</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E94">
-        <v>8.22</v>
+        <v>8.14</v>
       </c>
       <c r="F94" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
       </c>
     </row>
     <row r="95">
@@ -2277,19 +2292,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B95">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C95" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D95" t="str">
-        <v>GK爸爸</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E95">
-        <v>8.21</v>
+        <v>8.1</v>
       </c>
       <c r="F95" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
+        <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
       </c>
     </row>
     <row r="96">
@@ -2297,19 +2312,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B96">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C96" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D96" t="str">
-        <v>梁哲維</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E96">
-        <v>8.16</v>
+        <v>8.07</v>
       </c>
       <c r="F96" t="str">
-        <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 對談風格輕鬆歡樂，主持人與來賓之間的幽默互動和生活化分享（如吃茶葉蛋、羊肉爐、生魚片）帶來解壓感，笑聲自然，營造出愉悅的氛圍。 | [莫菲穿搭27｜金曲幕後直擊！電...] 節目內容偏向專業分析與個人觀點分享，輕鬆歡樂的療癒感相對較低。 | [莫菲穿搭02｜2026流行色配...] 談話風格較為嚴肅認真，以知識分享為主，解壓療癒感普通，較少輕鬆歡樂的對話。</v>
       </c>
     </row>
     <row r="97">
@@ -2317,19 +2332,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B97">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C97" t="str">
-        <v>蘇心時光</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D97" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E97">
-        <v>8.14</v>
+        <v>8.07</v>
       </c>
       <c r="F97" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
       </c>
     </row>
     <row r="98">
@@ -2337,79 +2352,79 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B98">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C98" t="str">
-        <v>布姐的沙發</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D98" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>蕭邦</v>
       </c>
       <c r="E98">
-        <v>8.1</v>
+        <v>8.07</v>
       </c>
       <c r="F98" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 談話風格偏向認真探討，而非輕鬆歡樂的療癒感。 | [【蕭邦出任務】如何選擇適合自己...] 談話風格較為深入與嚴肅，著重於職涯挑戰與個人成長，因此日常廢話解壓感和療癒感相對較低。 | [幸福的人，通常「覺察力」都很強...] 談話風格真誠且具啟發性，能引導聽眾自我療癒與成長，但較少輕鬆歡樂的廢話解壓感。</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
+        <v>自我探索獎</v>
       </c>
       <c r="B99">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C99" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>五吉郎</v>
       </c>
       <c r="D99" t="str">
-        <v>莫菲穿搭</v>
+        <v>五吉郎</v>
       </c>
       <c r="E99">
-        <v>8.07</v>
+        <v>10</v>
       </c>
       <c r="F99" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 對談風格輕鬆歡樂，主持人與來賓之間的幽默互動和生活化分享（如吃茶葉蛋、羊肉爐、生魚片）帶來解壓感，笑聲自然，營造出愉悅的氛圍。 | [莫菲穿搭27｜金曲幕後直擊！電...] 節目內容偏向專業分析與個人觀點分享，輕鬆歡樂的療癒感相對較低。 | [莫菲穿搭02｜2026流行色配...] 談話風格較為嚴肅認真，以知識分享為主，解壓療癒感普通，較少輕鬆歡樂的對話。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 深度探討自由人生、自我成長、內在探索與心靈啟發，從個人經歷中提煉出普世價值，啟發性極強。 | [EP174｜越省反而越窮？別把...] 深度探討金錢觀、人生目的與自我成長，對聽眾的內在探索有很強的啟發。 | [EP164｜滑短影音是在浪費時...] 節目深度探討了閱讀如何影響個人成長、思維模式的轉變以及如何找回自我可能性，提供了豐富的內在探索與心靈啟發內容。</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
+        <v>自我探索獎</v>
       </c>
       <c r="B100">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C100" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D100" t="str">
-        <v>無所不試無樂不作</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E100">
-        <v>8.07</v>
+        <v>9.99</v>
       </c>
       <c r="F100" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
+        <v>自我探索獎</v>
       </c>
       <c r="B101">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C101" t="str">
-        <v>蕭邦相談室</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D101" t="str">
-        <v>蕭邦</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E101">
-        <v>8.07</v>
+        <v>9.98</v>
       </c>
       <c r="F101" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 談話風格偏向認真探討，而非輕鬆歡樂的療癒感。 | [【蕭邦出任務】如何選擇適合自己...] 談話風格較為深入與嚴肅，著重於職涯挑戰與個人成長，因此日常廢話解壓感和療癒感相對較低。 | [幸福的人，通常「覺察力」都很強...] 談話風格真誠且具啟發性，能引導聽眾自我療癒與成長，但較少輕鬆歡樂的廢話解壓感。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
       </c>
     </row>
     <row r="102">
@@ -2417,19 +2432,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B102">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C102" t="str">
-        <v>五吉郎</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D102" t="str">
-        <v>五吉郎</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E102">
-        <v>10</v>
+        <v>9.93</v>
       </c>
       <c r="F102" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 深度探討自由人生、自我成長、內在探索與心靈啟發，從個人經歷中提煉出普世價值，啟發性極強。 | [EP174｜越省反而越窮？別把...] 深度探討金錢觀、人生目的與自我成長，對聽眾的內在探索有很強的啟發。 | [EP164｜滑短影音是在浪費時...] 節目深度探討了閱讀如何影響個人成長、思維模式的轉變以及如何找回自我可能性，提供了豐富的內在探索與心靈啟發內容。</v>
+        <v>[EP470｜把人放在心上的共贏...] 節目深度探討了自我成長、內在價值觀與目的性創業，來賓對自信的定義也提供了深刻的心靈啟發。 | [EP433｜【中年轉型】從矽谷...] 深度探討個人職涯轉型、自我覺察與性格探索，提供豐富的心靈啟發與成長觀點，是本集的核心亮點。 | [EP466｜拒絕被朝九晚五綁架...] 本集節目核心圍繞著自我成長、內在探索與心靈啟發。來賓透過「百工計畫」的實踐，深入剖析了個人與社會的關係，以及如何找到內在平衡，啟發性極強。</v>
       </c>
     </row>
     <row r="103">
@@ -2437,19 +2452,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B103">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C103" t="str">
-        <v>哇賽心理學</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D103" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>蕭邦</v>
       </c>
       <c r="E103">
-        <v>9.99</v>
+        <v>9.9</v>
       </c>
       <c r="F103" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 深度探討自我成長、內在探索與心靈啟發，主持人分享個人轉變歷程，極具啟發性。 | [【蕭邦出任務】如何選擇適合自己...] 來賓的職涯轉型故事與主持人對自我價值的探討，提供了深刻的內在探索與心靈啟發，深度極高。 | [幸福的人，通常「覺察力」都很強...] 深度探討情緒的來源、自我批判的迴圈以及如何透過覺察進行自我調整，對內在探索與心靈啟發的深度極高。</v>
       </c>
     </row>
     <row r="104">
@@ -2457,19 +2472,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B104">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C104" t="str">
-        <v>蘇心時光</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D104" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>張忘形</v>
       </c>
       <c r="E104">
-        <v>9.98</v>
+        <v>9.86</v>
       </c>
       <c r="F104" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
+        <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
       </c>
     </row>
     <row r="105">
@@ -2477,19 +2492,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B105">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C105" t="str">
-        <v>布姐的沙發</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D105" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E105">
-        <v>9.93</v>
+        <v>9.83</v>
       </c>
       <c r="F105" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 節目深度探討了自我成長、內在價值觀與目的性創業，來賓對自信的定義也提供了深刻的心靈啟發。 | [EP433｜【中年轉型】從矽谷...] 深度探討個人職涯轉型、自我覺察與性格探索，提供豐富的心靈啟發與成長觀點，是本集的核心亮點。 | [EP466｜拒絕被朝九晚五綁架...] 本集節目核心圍繞著自我成長、內在探索與心靈啟發。來賓透過「百工計畫」的實踐，深入剖析了個人與社會的關係，以及如何找到內在平衡，啟發性極強。</v>
+        <v>[EP.617 《無限機器》讀後...] 節目深度探討了個人使命感、價值觀與對未來的思考，引導聽眾進行自我成長與內在探索���心靈啟發感極強。 | [EP.573 從 0 到 10...] 深度探討個人成長、心態轉變、面對困難的韌性，以及如何從內在尋找動力，心靈啟發感極強。 | [EP.607 《AI Firs...] 節目核心圍繞個人在AI時代的自我成長、能力提升與心態轉變，提供了深刻的內在探索與心靈啟發。</v>
       </c>
     </row>
     <row r="106">
@@ -2497,19 +2512,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B106">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C106" t="str">
-        <v>蕭邦相談室</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D106" t="str">
-        <v>蕭邦</v>
+        <v>梁哲維</v>
       </c>
       <c r="E106">
-        <v>9.9</v>
+        <v>9.82</v>
       </c>
       <c r="F106" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 深度探討自我成長、內在探索與心靈啟發，主持人分享個人轉變歷程，極具啟發性。 | [【蕭邦出任務】如何選擇適合自己...] 來賓的職涯轉型故事與主持人對自我價值的探討，提供了深刻的內在探索與心靈啟發，深度極高。 | [幸福的人，通常「覺察力」都很強...] 深度探討情緒的來源、自我批判的迴圈以及如何透過覺察進行自我調整，對內在探索與心靈啟發的深度極高。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目深度探討了創業者的初心、傳承的意義以及善意帶來的回饋，對聽眾的自我成長和內在探索有很強的啟發。 | [【EP302 把命盤變成行動藍...] 節目核心圍繞著個人命運、自我認知與未來規劃，深度啟發聽眾進行內在探索與自我成長，極具價值。 | [【EP312《超越我執的生活》...] 本集內容核心即為自我成長與內在探索，透過對「我執」的剖析和「臨在��的實踐，提供了深刻的心靈啟發，高度符合此獎項的評估維度。</v>
       </c>
     </row>
     <row r="107">
@@ -2517,19 +2532,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B107">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C107" t="str">
-        <v>人類行為研究社</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D107" t="str">
-        <v>張忘形</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E107">
-        <v>9.86</v>
+        <v>9.76</v>
       </c>
       <c r="F107" t="str">
-        <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 節目深度探討自我價值、原生家庭影響及個人成長，對聽眾的自我探索與心靈啟發有極大助益。 | [S0714-【關係修復室】5個...] 節目核心圍繞自我成長、內在探索與關係修復，提供了深刻的心靈啟發。 | [S0810-戀愛腦怎麼辦？太理...] 節目深度挖掘個人內在需求、童年經驗對關係模式的影響，並鼓勵聽眾向內探索，心靈啟發與自我成長的深度極高。</v>
       </c>
     </row>
     <row r="108">
@@ -2537,79 +2552,79 @@
         <v>自我探索獎</v>
       </c>
       <c r="B108">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C108" t="str">
-        <v>下一本讀什麼？</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D108" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E108">
-        <v>9.83</v>
+        <v>9.76</v>
       </c>
       <c r="F108" t="str">
-        <v>[EP.617 《無限機器》讀後...] 節目深度探討了個人使命感、價值觀與對未來的思考，引導聽眾進行自我成長與內在探索���心靈啟發感極強。 | [EP.573 從 0 到 10...] 深度探討個人成長、心態轉變、面對困難的韌性，以及如何從內在尋找動力，心靈啟發感極強。 | [EP.607 《AI Firs...] 節目核心圍繞個人在AI時代的自我成長、能力提升與心態轉變，提供了深刻的內在探索與心靈啟發。</v>
+        <v>[#801 市場震盪 17000...] 深度探討了投資中的心理層面、個人風險承受度與長期目標設定，對聽眾的自我成長與內在探索有很強的啟發性。 | [#809  買股票還在到處問明...] 節目不僅談投資，更強調學習、成長和建立系統思維，對自我探索和心靈啟發有深度，鼓勵聽眾提升自我。 | [#798 害怕投資賠錢？不用天...] 深度探討投資與個人生活目標的連結，鼓勵聽眾進行自我反思，建立符合自身價值觀的財務規劃，心靈啟發感極強。</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>自我探索獎</v>
+        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B109">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C109" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>說話人聲</v>
       </c>
       <c r="D109" t="str">
-        <v>梁哲維</v>
+        <v>聲音表達講師林依柔</v>
       </c>
       <c r="E109">
-        <v>9.82</v>
+        <v>10</v>
       </c>
       <c r="F109" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目深度探討了創業者的初心、傳承的意義以及善意帶來的回饋，對聽眾的自我成長和內在探索有很強的啟發。 | [【EP302 把命盤變成行動藍...] 節目核心圍繞著個人命運、自我認知與未來規劃，深度啟發聽眾進行內在探索與自我成長，極具價值。 | [【EP312《超越我執的生活》...] 本集內容核心即為自我成長與內在探索，透過對「我執」的剖析和「臨在��的實踐，提供了深刻的心靈啟發，高度符合此獎項的評估維度。</v>
+        <v>[EP.59｜【說話人聲-會客室...] 單集時長接近4小時，內容資訊密度極高，且能持續保持聽眾的專注與興趣，無明顯冷場，是優秀的長篇內容��</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>自我探索獎</v>
+        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B110">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C110" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>郝聲音</v>
       </c>
       <c r="D110" t="str">
-        <v>人生啊！小歐</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E110">
-        <v>9.76</v>
+        <v>9.59</v>
       </c>
       <c r="F110" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 節目深度探討自我價值、原生家庭影響及個人成長，對聽眾的自我探索與心靈啟發有極大助益。 | [S0714-【關係修復室】5個...] 節目核心圍繞自我成長、內在探索與關係修復，提供了深刻的心靈啟發。 | [S0810-戀愛腦怎麼辦？太理...] 節目深度挖掘個人內在需求、童年經驗對關係模式的影響，並鼓勵聽眾向內探索，心靈啟發與自我成長的深度極高。</v>
+        <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>自我探索獎</v>
+        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B111">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C111" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D111" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E111">
-        <v>9.76</v>
+        <v>9.49</v>
       </c>
       <c r="F111" t="str">
-        <v>[#801 市場震盪 17000...] 深度探討了投資中的心理層面、個人風險承受度與長期目標設定，對聽眾的自我成長與內在探索有很強的啟發性。 | [#809  買股票還在到處問明...] 節目不僅談投資，更強調學習、成長和建立系統思維，對自我探索和心靈啟發有深度，鼓勵聽眾提升自我。 | [#798 害怕投資賠錢？不用天...] 深度探討投資與個人生活目標的連結，鼓勵聽眾進行自我反思，建立符合自身價值觀的財務規劃，心靈啟發感極強。</v>
+        <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
       </c>
     </row>
     <row r="112">
@@ -2617,19 +2632,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B112">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C112" t="str">
-        <v>說話人聲</v>
+        <v>航海王的富人學</v>
       </c>
       <c r="D112" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>美股航海王</v>
       </c>
       <c r="E112">
-        <v>10</v>
+        <v>9.38</v>
       </c>
       <c r="F112" t="str">
-        <v>[EP.59｜【說話人聲-會客室...] 單集時長接近4小時，內容資訊密度極高，且能持續保持聽眾的專注與興趣，無明顯冷場，是優秀的長篇內容��</v>
+        <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
       </c>
     </row>
     <row r="113">
@@ -2637,19 +2652,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B113">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C113" t="str">
-        <v>郝聲音</v>
+        <v>FIRE 人生大學</v>
       </c>
       <c r="D113" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>Fire人生大學｜道哥</v>
       </c>
       <c r="E113">
-        <v>9.59</v>
+        <v>9.35</v>
       </c>
       <c r="F113" t="str">
-        <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
+        <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
       </c>
     </row>
     <row r="114">
@@ -2657,19 +2672,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B114">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C114" t="str">
-        <v>哇賽心理學</v>
+        <v>粉紅地獄辛辣麵</v>
       </c>
       <c r="D114" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>Vito大叔</v>
       </c>
       <c r="E114">
-        <v>9.49</v>
+        <v>8.9</v>
       </c>
       <c r="F114" t="str">
-        <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
+        <v>[S6EP30. 我到日本當漁夫...] 本集時長超過2小時，屬於長篇內容。節目在這麼長的時間內，資訊密度依然很高，對談流暢且引人入勝，沒有明顯的冷場，能讓聽眾持續投入。這展現了節目在長篇內容規劃與執行上的功力。</v>
       </c>
     </row>
     <row r="115">
@@ -2677,19 +2692,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B115">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C115" t="str">
-        <v>航海王的富人學</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D115" t="str">
-        <v>美股航海王</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E115">
-        <v>9.38</v>
+        <v>8.84</v>
       </c>
       <c r="F115" t="str">
-        <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
       </c>
     </row>
     <row r="116">
@@ -2697,19 +2712,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B116">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C116" t="str">
-        <v>FIRE 人生大學</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D116" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>梁哲維</v>
       </c>
       <c r="E116">
-        <v>9.35</v>
+        <v>8.82</v>
       </c>
       <c r="F116" t="str">
-        <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
+        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
       </c>
     </row>
     <row r="117">
@@ -2717,19 +2732,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B117">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C117" t="str">
-        <v>粉紅地獄辛辣麵</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D117" t="str">
-        <v>Vito大叔</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E117">
-        <v>8.9</v>
+        <v>8.51</v>
       </c>
       <c r="F117" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] 本集時長超過2小時，屬於長篇內容。節目在這麼長的時間內，資訊密度依然很高，對談流暢且引人入勝，沒有明顯的冷場，能讓聽眾持續投入。這展現了節目在長篇內容規劃與執行上的功力。</v>
+        <v>[EP.316 與其等流量，不如...] 單集時長約63分鐘，內容資訊密度高且全程保持引人入勝，無明顯冷場，符合長篇內容的評估標準。</v>
       </c>
     </row>
     <row r="118">
@@ -2737,79 +2752,79 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B118">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C118" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="D118" t="str">
-        <v>人生啊！小歐</v>
+        <v>Dr Selena</v>
       </c>
       <c r="E118">
-        <v>8.84</v>
+        <v>8.5</v>
       </c>
       <c r="F118" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
+        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
+        <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B119">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C119" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D119" t="str">
-        <v>梁哲維</v>
+        <v>蕭邦</v>
       </c>
       <c r="E119">
-        <v>8.82</v>
+        <v>9.74</v>
       </c>
       <c r="F119" t="str">
-        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
+        <v>[幸福的人，通常「覺察力」都很強...] 單集時長在10-15分鐘（11分48秒），內容精煉且傳播效率高，能在短時間內提供豐富的資訊與啟發。</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
+        <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B120">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C120" t="str">
-        <v>尼可這樣說</v>
+        <v>美業幹什麼</v>
       </c>
       <c r="D120" t="str">
-        <v>尼可這樣說</v>
+        <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="E120">
-        <v>8.51</v>
+        <v>9.57</v>
       </c>
       <c r="F120" t="str">
-        <v>[EP.316 與其等流量，不如...] 單集時長約63分鐘，內容資訊密度高且全程保持引人入勝，無明顯冷場，符合長篇內容的評估標準。</v>
+        <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
+        <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B121">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C121" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D121" t="str">
-        <v>Dr Selena</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E121">
-        <v>8.5</v>
+        <v>9.55</v>
       </c>
       <c r="F121" t="str">
-        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
+        <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
       </c>
     </row>
     <row r="122">
@@ -2817,19 +2832,19 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B122">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C122" t="str">
-        <v>蕭邦相談室</v>
+        <v>山姆書書</v>
       </c>
       <c r="D122" t="str">
-        <v>蕭邦</v>
+        <v>山姆書書</v>
       </c>
       <c r="E122">
-        <v>9.74</v>
+        <v>9.43</v>
       </c>
       <c r="F122" t="str">
-        <v>[幸福的人，通常「覺察力」都很強...] 單集時長在10-15分鐘（11分48秒），內容精煉且傳播效率高，能在短時間內提供豐富的資訊與啟發。</v>
+        <v>[EP134.真的找得到靈魂伴侶...] 單集時長約13分鐘，精煉且資訊密度高，在短時間內傳達了豐富的內容與思考，傳播效率極佳��</v>
       </c>
     </row>
     <row r="123">
@@ -2837,19 +2852,19 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B123">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C123" t="str">
-        <v>美業幹什麼</v>
+        <v>教出你的路</v>
       </c>
       <c r="D123" t="str">
-        <v>美業幹什麼｜蔡佩陵</v>
+        <v>治療師瑪奇</v>
       </c>
       <c r="E123">
-        <v>9.57</v>
+        <v>9.32</v>
       </c>
       <c r="F123" t="str">
-        <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
+        <v>[EP31 為了愛移民，她打造 ...] 單集時長約13分半，內容精煉且資訊密度高，傳播效率極佳，無冗餘。</v>
       </c>
     </row>
     <row r="124">
@@ -2857,147 +2872,159 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B124">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C124" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D124" t="str">
-        <v>GK爸爸</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E124">
-        <v>9.55</v>
+        <v>9.07</v>
       </c>
       <c r="F124" t="str">
-        <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
+        <v>[【大師專題】人在江湖，身不由己...] 單集時長約10分鐘，符合10-15分鐘的短篇內容範疇。內容精煉，資訊密度高，能在短時間內傳達深刻且完整的觀點，傳播效率極佳。</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B125">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C125" t="str">
-        <v>山姆書書</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D125" t="str">
-        <v>山姆書書</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E125">
-        <v>9.43</v>
+        <v>9.66</v>
       </c>
       <c r="F125" t="str">
-        <v>[EP134.真的找得到靈魂伴侶...] 單集時長約13分鐘，精煉且資訊密度高，在短時間內傳達了豐富的內容與思考，傳播效率極佳��</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B126">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C126" t="str">
-        <v>教出你的路</v>
+        <v>五吉郎</v>
       </c>
       <c r="D126" t="str">
-        <v>治療師瑪奇</v>
+        <v>五吉郎</v>
       </c>
       <c r="E126">
-        <v>9.32</v>
+        <v>9.55</v>
       </c>
       <c r="F126" t="str">
-        <v>[EP31 為了愛移民，她打造 ...] 單集時長約13分半，內容精煉且資訊密度高，傳播效率極佳，無冗餘。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B127">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C127" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D127" t="str">
-        <v>無所不試無樂不作</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E127">
-        <v>9.07</v>
+        <v>9.48</v>
       </c>
       <c r="F127" t="str">
-        <v>[【大師專題】人在江湖，身不由己...] 單集時長約10分鐘，符合10-15分鐘的短篇內容範疇。內容精煉，資訊密度高，能在短時間內傳達深刻且完整的觀點，傳播效率極佳。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B128">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C128" t="str">
-        <v>財富餐車不打烊</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D128" t="str">
-        <v>30節約男子</v>
+        <v>布姐陪你聰明工作創意生活</v>
+      </c>
+      <c r="E128">
+        <v>9.43</v>
       </c>
       <c r="F128" t="str">
-        <v>暫無該集數之評審打分。</v>
+        <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B129">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C129" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D129" t="str">
-        <v>丁菱娟</v>
+        <v>胡咪老師</v>
+      </c>
+      <c r="E129">
+        <v>9.43</v>
       </c>
       <c r="F129" t="str">
-        <v>暫無該集數之評審打分。</v>
+        <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B130">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C130" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D130" t="str">
-        <v>人生啊！小歐</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+      </c>
+      <c r="E130">
+        <v>9.39</v>
       </c>
       <c r="F130" t="str">
-        <v>暫無該集數之評審打分。</v>
+        <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B131">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C131" t="str">
-        <v>下半場人生陪談師</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D131" t="str">
-        <v>下半場人生事務有限公司</v>
+        <v>蕭邦</v>
+      </c>
+      <c r="E131">
+        <v>9.34</v>
       </c>
       <c r="F131" t="str">
-        <v>暫無該集數之評審打分。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
       </c>
     </row>
     <row r="132">
@@ -3005,19 +3032,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B132">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C132" t="str">
-        <v>哇賽心理學</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D132" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>梁哲維</v>
       </c>
       <c r="E132">
-        <v>9.66</v>
+        <v>9.32</v>
       </c>
       <c r="F132" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
+        <v>[【EP330 帶著善意行動，最...] 主持人與來賓的對談充滿情感溫度，真誠的交流讓聽眾感受到靈魂的陪伴，具有很強的黏著度。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的對談真誠且富有溫度，內容��人入勝，能有效提升聽眾的黏著度與持續收聽的意願。 | [【EP312《超越我執的生活》...] 主持人以真誠且富有洞察力的語氣分享，內容深度能引發聽眾共鳴與思考，建立起較強的黏著度與情感連結，讓人期待下一集。</v>
       </c>
     </row>
     <row r="133">
@@ -3025,19 +3052,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B133">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C133" t="str">
-        <v>五吉郎</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D133" t="str">
-        <v>五吉郎</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E133">
-        <v>9.55</v>
+        <v>9.26</v>
       </c>
       <c r="F133" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
+        <v>[#801 市場震盪 17000...] 主持人以真誠且具同理心的語氣與聽眾對話，建立深厚的連結，情感溫度高，能有效提升聽眾黏著度。 | [#809  買股票還在到處問明...] 主持人與來賓的對談真誠，內容實用且具啟發性，能有效吸引聽眾持續收聽，建立黏著度。 | [#798 害怕投資賠錢？不用天...] 主持人與來賓透過分享個人經驗和真誠的對談，與聽眾建立了深厚的情感連結，讓人期待下一集的內容。</v>
       </c>
     </row>
     <row r="134">
@@ -3045,159 +3072,159 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B134">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C134" t="str">
-        <v>蘇心時光</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D134" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E134">
-        <v>9.48</v>
+        <v>9.24</v>
       </c>
       <c r="F134" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 主持人與來賓的對談真誠且富有情感溫度，內容引��入勝，讓聽眾對節目產生高度黏著度，期待未來能聽到更多類似的深度分享，具有強烈的靈魂陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 主持人透過真誠的分享和專業的分析，與聽眾建立了良好的情感連結，具有較高的黏著度。 | [莫菲穿搭02｜2026流行色配...] 主持人以專業且親切的語氣分享實用知識，內容具備高度價值，能有效提升聽眾的黏著度與學習意願。</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B135">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C135" t="str">
-        <v>布姐的沙發</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D135" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E135">
-        <v>9.43</v>
+        <v>8.15</v>
       </c>
       <c r="F135" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
+        <v>AI 評審平均得分為 8.15 分，近半年累積 Apple Podcasts 評論數達 50 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B136">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C136" t="str">
-        <v>分手的99個理由</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="D136" t="str">
-        <v>胡咪老師</v>
+        <v>別人的工作最有趣｜Fiona</v>
       </c>
       <c r="E136">
-        <v>9.43</v>
+        <v>8.2</v>
       </c>
       <c r="F136" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
+        <v>AI 評審平均得分為 8.2 分，近半年累積 Apple Podcasts 評論數達 18 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B137">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C137" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>小思大維</v>
       </c>
       <c r="D137" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>小思大維｜雪柔</v>
       </c>
       <c r="E137">
-        <v>9.39</v>
+        <v>8.24</v>
       </c>
       <c r="F137" t="str">
-        <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
+        <v>AI 評審平均得分為 8.24 分，近半年累積 Apple Podcasts 評論數達 16 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B138">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C138" t="str">
-        <v>蕭邦相談室</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D138" t="str">
-        <v>蕭邦</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E138">
-        <v>9.34</v>
+        <v>8.29</v>
       </c>
       <c r="F138" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
+        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B139">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C139" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>山姆書書</v>
       </c>
       <c r="D139" t="str">
-        <v>梁哲維</v>
+        <v>山姆書書</v>
       </c>
       <c r="E139">
-        <v>9.32</v>
+        <v>8.19</v>
       </c>
       <c r="F139" t="str">
-        <v>[【EP330 帶著善意行動，最...] 主持人與來賓的對談充滿情感溫度，真誠的交流讓聽眾感受到靈魂的陪伴，具有很強的黏著度。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的對談真誠且富有溫度，內容��人入勝，能有效提升聽眾的黏著度與持續收聽的意願。 | [【EP312《超越我執的生活》...] 主持人以真誠且富有洞察力的語氣分享，內容深度能引發聽眾共鳴與思考，建立起較強的黏著度與情感連結，讓人期待下一集。</v>
+        <v>AI 評審平均得分為 8.19 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B140">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C140" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>航海王的富人學</v>
       </c>
       <c r="D140" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>美股航海王</v>
       </c>
       <c r="E140">
-        <v>9.26</v>
+        <v>8.15</v>
       </c>
       <c r="F140" t="str">
-        <v>[#801 市場震盪 17000...] 主持人以真誠且具同理心的語氣與聽眾對話，建立深厚的連結，情感溫度高，能有效提升聽眾黏著度。 | [#809  買股票還在到處問明...] 主持人與來賓的對談真誠，內容實用且具啟發性，能有效吸引聽眾持續收聽，建立黏著度。 | [#798 害怕投資賠錢？不用天...] 主持人與來賓透過分享個人經驗和真誠的對談，與聽眾建立了深厚的情感連結，讓人期待下一集的內容。</v>
+        <v>AI 評審平均得分為 8.15 分，近半年累積 Apple Podcasts 評論數達 13 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B141">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C141" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>FIRE 人生大學</v>
       </c>
       <c r="D141" t="str">
-        <v>莫菲穿搭</v>
+        <v>Fire人生大學｜道哥</v>
       </c>
       <c r="E141">
-        <v>9.24</v>
+        <v>8.17</v>
       </c>
       <c r="F141" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 主持人與來賓的對談真誠且富有情感溫度，內容引��入勝，讓聽眾對節目產生高度黏著度，期待未來能聽到更多類似的深度分享，具有強烈的靈魂陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 主持人透過真誠的分享和專業的分析，與聽眾建立了良好的情感連結，具有較高的黏著度。 | [莫菲穿搭02｜2026流行色配...] 主持人以專業且親切的語氣分享實用知識，內容具備高度價值，能有效提升聽眾的黏著度與學習意願。</v>
+        <v>AI 評審平均得分為 8.17 分，近半年累積 Apple Podcasts 評論數達 10 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="142">
@@ -3205,19 +3232,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B142">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C142" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D142" t="str">
-        <v>GK爸爸</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E142">
-        <v>8.15</v>
+        <v>8.29</v>
       </c>
       <c r="F142" t="str">
-        <v>AI 評審平均得分為 8.15 分，近半年累積 Apple Podcasts 評論數達 50 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 8 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="143">
@@ -3225,19 +3252,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B143">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C143" t="str">
-        <v>別人的工作最有趣</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D143" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E143">
-        <v>8.2</v>
+        <v>7.87</v>
       </c>
       <c r="F143" t="str">
-        <v>AI 評審平均得分為 8.2 分，近半年累積 Apple Podcasts 評論數達 18 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 7.87 分，近半年累積 Apple Podcasts 評論數達 11 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="144">
@@ -3245,27 +3272,27 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B144">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C144" t="str">
-        <v>小思大維</v>
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="D144" t="str">
-        <v>小思大維｜雪柔</v>
+        <v>Dr Selena</v>
       </c>
       <c r="E144">
-        <v>8.24</v>
+        <v>8.14</v>
       </c>
       <c r="F144" t="str">
-        <v>AI 評審平均得分為 8.24 分，近半年累積 Apple Podcasts 評論數達 16 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.14 分，近半年累積 Apple Podcasts 評論數達 7 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B145">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C145" t="str">
         <v>下一本讀什麼？</v>
@@ -3274,130 +3301,130 @@
         <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E145">
-        <v>8.29</v>
+        <v>44</v>
       </c>
       <c r="F145" t="str">
-        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #26.4 名。</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B146">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C146" t="str">
-        <v>山姆書書</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D146" t="str">
-        <v>山姆書書</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E146">
-        <v>8.19</v>
+        <v>44</v>
       </c>
       <c r="F146" t="str">
-        <v>AI 評審平均得分為 8.19 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #33.5 名。</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B147">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C147" t="str">
-        <v>航海王的富人學</v>
+        <v>郝聲音</v>
       </c>
       <c r="D147" t="str">
-        <v>美股航海王</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E147">
-        <v>8.15</v>
+        <v>44</v>
       </c>
       <c r="F147" t="str">
-        <v>AI 評審平均得分為 8.15 分，近半年累積 Apple Podcasts 評論數達 13 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #38.1 名。</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B148">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C148" t="str">
-        <v>FIRE 人生大學</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D148" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E148">
-        <v>8.17</v>
+        <v>44</v>
       </c>
       <c r="F148" t="str">
-        <v>AI 評審平均得分為 8.17 分，近半年累積 Apple Podcasts 評論數達 10 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #65 名。</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B149">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C149" t="str">
-        <v>哇賽心理學</v>
+        <v>文森說書</v>
       </c>
       <c r="D149" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>文森說書</v>
       </c>
       <c r="E149">
-        <v>8.29</v>
+        <v>36</v>
       </c>
       <c r="F149" t="str">
-        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 8 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 36 天，平均上榜排名為第 #64.6 名。</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B150">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C150" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="D150" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>別人的工作最有趣｜Fiona</v>
       </c>
       <c r="E150">
-        <v>7.87</v>
+        <v>7</v>
       </c>
       <c r="F150" t="str">
-        <v>AI 評審平均得分為 7.87 分，近半年累積 Apple Podcasts 評論數達 11 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B151">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C151" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>小思大維</v>
       </c>
       <c r="D151" t="str">
-        <v>Dr Selena</v>
+        <v>小思大維｜雪柔</v>
       </c>
       <c r="E151">
-        <v>8.14</v>
+        <v>4</v>
       </c>
       <c r="F151" t="str">
-        <v>AI 評審平均得分為 8.14 分，近半年累積 Apple Podcasts 評論數達 7 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
       </c>
     </row>
     <row r="152">
@@ -3405,159 +3432,159 @@
         <v>站著不走獎</v>
       </c>
       <c r="B152">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C152" t="str">
-        <v>下一本讀什麼？</v>
+        <v>佐依Zoey</v>
       </c>
       <c r="D152" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>佐依Zoey</v>
       </c>
       <c r="E152">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="F152" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #26.4 名。</v>
+        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B153">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C153" t="str">
-        <v>哇賽心理學</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D153" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E153">
-        <v>44</v>
+        <v>8.7</v>
       </c>
       <c r="F153" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #33.5 名。</v>
+        <v>平均評等 3.7 星，累計 50 則評論。綜合指標得分：8.7 / 10 分。</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B154">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C154" t="str">
-        <v>郝聲音</v>
+        <v>小思大維</v>
       </c>
       <c r="D154" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>小思大維｜雪柔</v>
       </c>
       <c r="E154">
-        <v>44</v>
+        <v>6.5</v>
       </c>
       <c r="F154" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #38.1 名。</v>
+        <v>平均評等 4.9 星，累計 16 則評論。綜合指標得分：6.5 / 10 分。</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B155">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C155" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D155" t="str">
-        <v>GK爸爸</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E155">
-        <v>44</v>
+        <v>6.2</v>
       </c>
       <c r="F155" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #65 名。</v>
+        <v>平均評等 4.8 星，累計 14 則評論。綜合指標得分：6.2 / 10 分。</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B156">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C156" t="str">
-        <v>文森說書</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D156" t="str">
-        <v>文森說書</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E156">
-        <v>36</v>
+        <v>6.1</v>
       </c>
       <c r="F156" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 36 天，平均上榜排名為第 #64.6 名。</v>
+        <v>平均評等 5 星，累計 11 則評論。綜合指標得分：6.1 / 10 分。</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B157">
+        <v>5</v>
+      </c>
+      <c r="C157" t="str">
+        <v>航海王的富人學</v>
+      </c>
+      <c r="D157" t="str">
+        <v>美股航海王</v>
+      </c>
+      <c r="E157">
         <v>6</v>
       </c>
-      <c r="C157" t="str">
-        <v>別人的工作最有趣</v>
-      </c>
-      <c r="D157" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
-      </c>
-      <c r="E157">
-        <v>7</v>
-      </c>
       <c r="F157" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
+        <v>平均評等 4.7 星，累計 13 則評論。綜合指標得分：6 / 10 分。</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B158">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C158" t="str">
-        <v>小思大維</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="D158" t="str">
-        <v>小思大維｜雪柔</v>
+        <v>別人的工作最有趣｜Fiona</v>
       </c>
       <c r="E158">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F158" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
+        <v>平均評等 4.2 星，累計 18 則評論。綜合指標得分：6 / 10 分。</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>站著不走獎</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B159">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C159" t="str">
-        <v>佐依Zoey</v>
+        <v>山姆書書</v>
       </c>
       <c r="D159" t="str">
-        <v>佐依Zoey</v>
+        <v>山姆書書</v>
       </c>
       <c r="E159">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F159" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
+        <v>平均評等 4.6 星，累計 14 則評論。綜合指標得分：6 / 10 分。</v>
       </c>
     </row>
     <row r="160">
@@ -3565,19 +3592,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B160">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C160" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>FIRE 人生大學</v>
       </c>
       <c r="D160" t="str">
-        <v>GK爸爸</v>
+        <v>Fire人生大學｜道哥</v>
       </c>
       <c r="E160">
-        <v>8.7</v>
+        <v>5.8</v>
       </c>
       <c r="F160" t="str">
-        <v>平均評等 3.7 星，累計 50 則評論。綜合指標得分：8.7 / 10 分。</v>
+        <v>平均評等 4.8 星，累計 10 則評論。綜合指標得分：5.8 / 10 分。</v>
       </c>
     </row>
     <row r="161">
@@ -3585,19 +3612,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B161">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C161" t="str">
-        <v>小思大維</v>
+        <v>文森說書</v>
       </c>
       <c r="D161" t="str">
-        <v>小思大維｜雪柔</v>
+        <v>文森說書</v>
       </c>
       <c r="E161">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="F161" t="str">
-        <v>平均評等 4.9 星，累計 16 則評論。綜合指標得分：6.5 / 10 分。</v>
+        <v>平均評等 4.8 星，累計 10 則評論。綜合指標得分：5.8 / 10 分。</v>
       </c>
     </row>
     <row r="162">
@@ -3605,27 +3632,27 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B162">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C162" t="str">
-        <v>下一本讀什麼？</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D162" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E162">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="F162" t="str">
-        <v>平均評等 4.8 星，累計 14 則評論。綜合指標得分：6.2 / 10 分。</v>
+        <v>平均評等 4.6 星，累計 8 則評論。綜合指標得分：5.4 / 10 分。</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B163">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C163" t="str">
         <v>不敗教主陳重銘</v>
@@ -3634,130 +3661,130 @@
         <v>不敗教主-陳重銘</v>
       </c>
       <c r="E163">
-        <v>6.1</v>
+        <v>0</v>
       </c>
       <c r="F163" t="str">
-        <v>平均評等 5 星，累計 11 則評論。綜合指標得分：6.1 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B164">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C164" t="str">
-        <v>航海王的富人學</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D164" t="str">
-        <v>美股航海王</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E164">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F164" t="str">
-        <v>平均評等 4.7 星，累計 13 則評論。綜合指標得分：6 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B165">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C165" t="str">
-        <v>別人的工作最有趣</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D165" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E165">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F165" t="str">
-        <v>平均評等 4.2 星，累計 18 則評論。綜合指標得分：6 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B166">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C166" t="str">
-        <v>山姆書書</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D166" t="str">
-        <v>山姆書書</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E166">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F166" t="str">
-        <v>平均評等 4.6 星，累計 14 則評論。綜合指標得分：6 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B167">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C167" t="str">
-        <v>FIRE 人生大學</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D167" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E167">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="F167" t="str">
-        <v>平均評等 4.8 星，累計 10 則評論。綜合指標得分：5.8 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B168">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C168" t="str">
-        <v>文森說書</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D168" t="str">
-        <v>文森說書</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E168">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="F168" t="str">
-        <v>平均評等 4.8 星，累計 10 則評論。綜合指標得分：5.8 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B169">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C169" t="str">
-        <v>哇賽心理學</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D169" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E169">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="F169" t="str">
-        <v>平均評等 4.6 星，累計 8 則評論。綜合指標得分：5.4 / 10 分。</v>
+        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
     <row r="170">
@@ -3765,13 +3792,13 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B170">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C170" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D170" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E170">
         <v>0</v>
@@ -3785,13 +3812,13 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B171">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C171" t="str">
-        <v>布姐的沙發</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D171" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>張忘形</v>
       </c>
       <c r="E171">
         <v>0</v>
@@ -3805,13 +3832,13 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B172">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C172" t="str">
-        <v>尼可這樣說</v>
+        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
       <c r="D172" t="str">
-        <v>尼可這樣說</v>
+        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E172">
         <v>0</v>
@@ -3820,149 +3847,9 @@
         <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B173">
-        <v>4</v>
-      </c>
-      <c r="C173" t="str">
-        <v>無所不試 無樂不作</v>
-      </c>
-      <c r="D173" t="str">
-        <v>無所不試無樂不作</v>
-      </c>
-      <c r="E173">
-        <v>0</v>
-      </c>
-      <c r="F173" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B174">
-        <v>5</v>
-      </c>
-      <c r="C174" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
-      </c>
-      <c r="D174" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
-      </c>
-      <c r="E174">
-        <v>0</v>
-      </c>
-      <c r="F174" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B175">
-        <v>6</v>
-      </c>
-      <c r="C175" t="str">
-        <v>丁菱娟的邊走邊想</v>
-      </c>
-      <c r="D175" t="str">
-        <v>丁菱娟</v>
-      </c>
-      <c r="E175">
-        <v>0</v>
-      </c>
-      <c r="F175" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B176">
-        <v>7</v>
-      </c>
-      <c r="C176" t="str">
-        <v>楊肉盧</v>
-      </c>
-      <c r="D176" t="str">
-        <v>楊月娥（楊肉爐）</v>
-      </c>
-      <c r="E176">
-        <v>0</v>
-      </c>
-      <c r="F176" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B177">
-        <v>8</v>
-      </c>
-      <c r="C177" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
-      </c>
-      <c r="D177" t="str">
-        <v>人生啊！小歐</v>
-      </c>
-      <c r="E177">
-        <v>0</v>
-      </c>
-      <c r="F177" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B178">
-        <v>9</v>
-      </c>
-      <c r="C178" t="str">
-        <v>人類行為研究社</v>
-      </c>
-      <c r="D178" t="str">
-        <v>張忘形</v>
-      </c>
-      <c r="E178">
-        <v>0</v>
-      </c>
-      <c r="F178" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B179">
-        <v>10</v>
-      </c>
-      <c r="C179" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
-      </c>
-      <c r="D179" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
-      </c>
-      <c r="E179">
-        <v>0</v>
-      </c>
-      <c r="F179" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F179"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F172"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Recalculate with complete dataset, tie-breakers, and Excel definitions
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="評選決審 Top 10" sheetId="1" r:id="rId1"/>
+    <sheet name="評選定義與細則" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -441,7 +442,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E2">
-        <v>9.55</v>
+        <v>9.4545</v>
       </c>
       <c r="F2" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [EP174｜越省反而越窮？別把...] 主持人開場鋪陳完整，話題引導流暢，結尾有總結，整體架構清晰。 | [EP164｜滑短影音是在浪費時...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。</v>
@@ -461,7 +462,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E3">
-        <v>9.49</v>
+        <v>9.4046</v>
       </c>
       <c r="F3" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [《財富自由心理學》：賺錢，只是...] 節目開場鋪陳完整，話題轉折自然流暢，主持人能有效引導對談並適時拉回核心，結尾亦有精要總結，架構清晰。 | [手總是停不下來？那是焦慮在尋找...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
@@ -475,16 +476,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D4" t="str">
-        <v>梁哲維</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E4">
-        <v>9.32</v>
+        <v>9.251</v>
       </c>
       <c r="F4" t="str">
-        <v>[【EP330 帶著善意行動，最...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [【EP302 把命盤變成行動藍...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。 | [【EP312《超越我執的生活》...] 主持人開場鋪陳清晰，能有效引導聽眾進入主題。內容邏輯性強，轉折自然，結尾亦有精要總結與行動呼籲，架構完整。</v>
+        <v>[EP289  七巨頭變七矮人！...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [EP275 股市變賭場？巴菲特...] 節目開場清晰，主題鋪陳有條理，各段落間的轉折流暢，結尾總結與行動呼籲明確，整體內容架構完整且邏輯性強。 | [EP251國防預算暴漲 5 成...] 主持人開場直接切入主題，中間分析市場數據和政策影響，邏輯清晰。雖然語速快，但內容結構完整。</v>
       </c>
     </row>
     <row r="5">
@@ -495,16 +496,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D5" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>梁哲維</v>
       </c>
       <c r="E5">
-        <v>9.26</v>
+        <v>9.25</v>
       </c>
       <c r="F5" t="str">
-        <v>[#801 市場震盪 17000...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [#809  買股票還在到處問明...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。 | [#798 害怕投資賠錢？不用天...] 主持人開場鋪陳完整，中途能流暢引導話題，從基礎概念到實務應用，再到心態調整，架構清晰，結尾亦有精要總結。</v>
+        <v>[【EP330 帶著善意行動，最...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [【EP302 把命盤變成行動藍...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。 | [【EP312《超越我執的生活》...] 主持人開場鋪陳清晰，能有效引導聽眾進入主題。內容邏輯性強，轉折自然，結尾亦有精要總結與行動呼籲，架構完整。</v>
       </c>
     </row>
     <row r="6">
@@ -515,16 +516,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D6" t="str">
-        <v>莫菲穿搭</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E6">
-        <v>9.24</v>
+        <v>9.25</v>
       </c>
       <c r="F6" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 節目開場鋪陳完整，主題明確。主持人能流暢引導話題，從個人經驗到宏觀趨勢，轉折自然，結尾亦有精要總結，架構清晰。 | [莫菲穿搭27｜金曲幕後直擊！電...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [莫菲穿搭02｜2026流行色配...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。</v>
+        <v>[#801 市場震盪 17000...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [#809  買股票還在到處問明...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。 | [#798 害怕投資賠錢？不用天...] 主持人開場鋪陳完整，中途能流暢引導話題，從基礎概念到實務應用，再到心態調整，架構清晰，結尾亦有精要總結。</v>
       </c>
     </row>
     <row r="7">
@@ -535,16 +536,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="str">
-        <v>蕭邦相談室</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D7" t="str">
-        <v>蕭邦</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E7">
-        <v>9.24</v>
+        <v>9.155</v>
       </c>
       <c r="F7" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [【蕭邦出任務】如何選擇適合自己...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [幸福的人，通常「覺察力」都很強...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
+        <v>[EP611 00998A(主動...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀分析到具體投資標的，結尾亦有精要總結，架構清晰。 | [EP628昇陽半導體(8028...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀產業趨勢到具體個股分析，結尾亦有精要總結，架構清晰。 | [EP621《富媽媽 窮媽媽》第...] 節目開場清晰，主體內容透過故事案例層層推進，邏輯嚴謹，結尾有明確的行動呼籲與總結，架構完整。</v>
       </c>
     </row>
     <row r="8">
@@ -561,7 +562,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E8">
-        <v>9.22</v>
+        <v>9.155</v>
       </c>
       <c r="F8" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人開場鋪陳清晰，中途提問引導流暢，能有效推進對話，結尾總結亦有深度，整體內��架構完整。 | [EP218：愛自己｜放下完美執...] 節目開場鋪陳流暢，透過個人經驗引入主題與來賓。中段內容圍繞人類圖的核心概念、案例分析與關係互動，轉折自然。結尾則聚焦於線上課程的推廣與總結，整體架構清晰，引導得宜。 | [EP219：【非典家庭CEO】...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。</v>
@@ -575,16 +576,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D9" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E9">
-        <v>9.21</v>
+        <v>9.15</v>
       </c>
       <c r="F9" t="str">
-        <v>[EP611 00998A(主動...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀分析到具體投資標的，結尾亦有精要總結，架構清晰。 | [EP628昇陽半導體(8028...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀產業趨勢到具體個股分析，結尾亦有精要總結，架構清晰。 | [EP621《富媽媽 窮媽媽》第...] 節目開場清晰，主體內容透過故事案例層層推進，邏輯嚴謹，結尾有明確的行動呼籲與總結，架構完整。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 節目開場鋪陳完整，主題明確。主持人能流暢引導話題，從個人經驗到宏觀趨勢，轉折自然，結尾亦有精要總結，架構清晰。 | [莫菲穿搭27｜金曲幕後直擊！電...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [莫菲穿搭02｜2026流行色配...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。</v>
       </c>
     </row>
     <row r="10">
@@ -595,16 +596,16 @@
         <v>9</v>
       </c>
       <c r="C10" t="str">
-        <v>下一本讀什麼？</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D10" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>蕭邦</v>
       </c>
       <c r="E10">
-        <v>9.16</v>
+        <v>9.15</v>
       </c>
       <c r="F10" t="str">
-        <v>[EP.617 《無限機器》讀後...] 主持人開場鋪陳完整，中途能流暢引導話題，透過六個重點清晰地呈現書中精華，結尾亦有精要總結，內容架構清晰。 | [EP.573 從 0 到 10...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。內容邏輯清晰，層次分明。 | [EP.607 《AI Firs...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [【蕭邦出任務】如何選擇適合自己...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [幸福的人，通常「覺察力」都很強...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
       </c>
     </row>
     <row r="11">
@@ -615,16 +616,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>宋家小館</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D11" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E11">
-        <v>9.15</v>
+        <v>9.1048</v>
       </c>
       <c r="F11" t="str">
-        <v>[EP162 | 從房地產到Ma...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [EP191 | 《我到日本當漁...] 主持人開場鋪陳完整，中途能流暢引導話題，透過提問深入挖掘來賓故事，結尾亦有精要總結，整體內容架構清晰。 | [EP182 | 聽見身體的聲音...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。來賓的專業知識分享也很有條理。</v>
+        <v>[EP.617 《無限機器》讀後...] 主持人開場鋪陳完整，中途能流暢引導話題，透過六個重點清晰地呈現書中精華，結尾亦有精要總結，內容架構清晰。 | [EP.573 從 0 到 10...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。內容邏輯清晰，層次分明。 | [EP.607 《AI Firs...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
       </c>
     </row>
     <row r="12">
@@ -641,7 +642,7 @@
         <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E12">
-        <v>9.31</v>
+        <v>9.1981</v>
       </c>
       <c r="F12" t="str">
         <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
@@ -661,7 +662,7 @@
         <v>胡咪老師</v>
       </c>
       <c r="E13">
-        <v>9.16</v>
+        <v>9.1966</v>
       </c>
       <c r="F13" t="str">
         <v>[S4.EP4｜性平教育20年，...] 兩位主持人互動自然，接話流暢，笑聲同步率高，展現良好默契。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人默契極佳，對話流暢自然，能互相接話並適時加入幽默感，共同營造出引人入勝的節目氛圍。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契，接話流暢，插話頻率適中，彼此的幽默感與共鳴笑聲自然，共同營造出輕鬆愉快的對話氛圍。</v>
@@ -681,7 +682,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E14">
-        <v>8.89</v>
+        <v>8.8099</v>
       </c>
       <c r="F14" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
@@ -701,7 +702,7 @@
         <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E15">
-        <v>8.89</v>
+        <v>8.7765</v>
       </c>
       <c r="F15" t="str">
         <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
@@ -715,16 +716,16 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <v>能量黑客</v>
+        <v>粉紅地獄辛辣麵</v>
       </c>
       <c r="D16" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>Vito大叔</v>
       </c>
       <c r="E16">
-        <v>8.73</v>
+        <v>8.7215</v>
       </c>
       <c r="F16" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人互動自然，接話流暢，彼此間的幽默感和笑聲也增加了節目的親和力。女主持人興奮時的插話，男主持人也能很好地承接。 | [別人眼中的高光時刻，卻是我最耗...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高��尤其在幽默解釋「麻場」和「鐵軌」時，默契十足。 | [別急著振作！高能量的人允許自己...] 雙主持人Hank與Vicky之間的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現了良好的默契與引導能力。</v>
+        <v>[S6EP30. 我到日本當漁夫...] Vito和品希作為雙人主持，展現了良好的默契。他們接話流暢，很少出現互相打斷的情況，品希的提問常帶有女性的細膩與同理心，Vito則負責更宏觀的引導與專業提問。兩人的笑聲自然，共同營造了輕鬆愉快的對談氛圍。 | [S6EP19. 沐樂MOReL...] Vito與品希之間展現了極佳的默契，對話流暢自然，常有幽默的插科打諢和同步的笑聲，互動感強烈。 | [S6EP4. 放飛。萬哩露｜村...] 雙主持與來賓互動自然，接話流暢，笑聲同步率高，尤其在幽默對話時默契十足，��節目增添了活力。</v>
       </c>
     </row>
     <row r="17">
@@ -735,16 +736,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="str">
-        <v>粉紅地獄辛辣麵</v>
+        <v>能量黑客</v>
       </c>
       <c r="D17" t="str">
-        <v>Vito大叔</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E17">
-        <v>8.73</v>
+        <v>8.6549</v>
       </c>
       <c r="F17" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] Vito和品希作為雙人主持，展現了良好的默契。他們接話流暢，很少出現互相打斷的情況，品希的提問常帶有女性的細膩與同理心，Vito則負責更宏觀的引導與專業提問。兩人的笑聲自然，共同營造了輕鬆愉快的對談氛圍。 | [S6EP19. 沐樂MOReL...] Vito與品希之間展現了極佳的默契，對話流暢自然，常有幽默的插科打諢和同步的笑聲，互動感強烈。 | [S6EP4. 放飛。萬哩露｜村...] 雙主持與來賓互動自然，接話流暢，笑聲同步率高，尤其在幽默對話時默契十足，��節目增添了活力。</v>
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人互動自然，接話流暢，彼此間的幽默感和笑聲也增加了節目的親和力。女主持人興奮時的插話，男主持人也能很好地承接。 | [別人眼中的高光時刻，卻是我最耗...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高��尤其在幽默解釋「麻場」和「鐵軌」時，默契十足。 | [別急著振作！高能量的人允許自己...] 雙主持人Hank與Vicky之間的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現了良好的默契與引導能力。</v>
       </c>
     </row>
     <row r="18">
@@ -761,7 +762,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E18">
-        <v>8.57</v>
+        <v>8.505</v>
       </c>
       <c r="F18" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 主持人與來賓之間的對話流暢自然，接話得體，沒有明顯的搶話或插話，展現了良好的互動默契。 | [【中年，正在試】把世界走成一本...] Norman和Summer的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現良好默契。</v>
@@ -781,7 +782,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E19">
-        <v>10</v>
+        <v>9.9545</v>
       </c>
       <c r="F19" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 選題新穎，結合個人IP變現與美業轉型，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [EP174｜越省反而越窮？別把...] 選題結合心理學與財富自由，觀點新穎且具深度，案例生動，內容含金量高。 | [EP164｜滑短影音是在浪費時...] 選題新穎且具深度，圍繞來賓新書的核心理念展開，提供了許多關於閱讀與自我成長的實用觀點與啟發，內容含金量極高。</v>
@@ -801,7 +802,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E20">
-        <v>9.99</v>
+        <v>9.9046</v>
       </c>
       <c r="F20" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 選題非常新穎且具時事性，從藥物機制到社會政策的討論深度極高，內容含金量豐富。 | [《財富自由心理學》：賺錢，只是...] 選題「財富自由心理學」新穎且具深度，透過個人故事與哲學思辨，將財富議題提升至心靈層次，內容含金量高，案例生動具啟發性。 | [手總是停不下來？那是焦慮在尋找...] 選題新穎且具深度，深入探討身體重複行為的心理學面向，案例生動且內容含金量極高。</v>
@@ -821,7 +822,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E21">
-        <v>9.82</v>
+        <v>9.75</v>
       </c>
       <c r="F21" t="str">
         <v>[【EP330 帶著善意行動，最...] 節目以一本關於「好感影響力」的書為引子，邀請書中提及的創業家來分享故事，選題獨特且具深度。來賓的70年滷味傳承與公益行動，提供了豐富的內容含金量和啟發性。 | [【EP302 把命盤變成行動藍...] 選題新穎，結合「九紫離火運」與AI、全球局勢、個人發展等多元面向，案例生動且內容含金量極高。 | [【EP312《超越我執的生活》...] 選題「超越我執」具備深度與啟發性，結合心理學與靈性成長，內容含金量高，案例（如內在聲音、吃飯專注）生動且具體，展現了優秀的單元企劃能力。</v>
@@ -841,7 +842,7 @@
         <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E22">
-        <v>9.76</v>
+        <v>9.75</v>
       </c>
       <c r="F22" t="str">
         <v>[#801 市場震盪 17000...] 選題緊扣時事（股市下跌），並結合個人財務規劃與情緒管理，案例生動且內容含金量極高。 | [#809  買股票還在到處問明...] 選題「獲利加速系統」具備高度實用性與深度，結合AI工具的應用，內容含金量極高，企劃新穎。 | [#798 害怕投資賠錢？不用天...] 選題新穎且具備深度，聚焦於媽媽族群的投資教育與心態建立，內容含金量高，並透過生動的比喻（如游泳、無印良品櫃子）提升理解度。</v>
@@ -855,16 +856,16 @@
         <v>5</v>
       </c>
       <c r="C23" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D23" t="str">
-        <v>莫菲穿搭</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E23">
-        <v>9.74</v>
+        <v>9.6796</v>
       </c>
       <c r="F23" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
+        <v>[EP289  七巨頭變七矮人！...] 選題新穎且具時效性，深入分析了科技巨頭的市場變化與供應鏈影響，內容含金量極高。 | [EP275 股市變賭場？巴菲特...] 選題緊扣時事熱點（巴菲特、AI、台股美股），內容深度足夠，結合了宏觀經濟分析、產業趨勢與個股案例，資訊含金量高，企劃具備高度專業性。 | [EP251國防預算暴漲 5 成...] 選題結合時事（軍工股、AI、經濟預測），數據分析詳盡，提供獨到見解，內容含金量高。</v>
       </c>
     </row>
     <row r="24">
@@ -875,16 +876,16 @@
         <v>6</v>
       </c>
       <c r="C24" t="str">
-        <v>蕭邦相談室</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D24" t="str">
-        <v>蕭邦</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E24">
-        <v>9.74</v>
+        <v>9.655</v>
       </c>
       <c r="F24" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
+        <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
       </c>
     </row>
     <row r="25">
@@ -895,16 +896,16 @@
         <v>7</v>
       </c>
       <c r="C25" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D25" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E25">
-        <v>9.72</v>
+        <v>9.6549</v>
       </c>
       <c r="F25" t="str">
-        <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
+        <v>[[EP0063] 50+Con...] 選題新穎，結合「第三人生大學」與「大嬸陪聊」概念，案例生動且含金量極高，具備深度思考與社會連結。 | [[EP0071] 50+Con...] 選題新穎且具深度，聚焦於二代接班與職涯轉型，來賓的個人案例生動且含金量極高，提供了獨特的視角和實用建議。 | [[EP0045] 50+Con...] 選題深入探討紫微斗數的「四化」與「殺破狼」命格，不僅新穎且具備高度的專業含金量。來賓的案例分享與對社會現象的連結，讓內容更具啟發性與實用價值。</v>
       </c>
     </row>
     <row r="26">
@@ -915,16 +916,16 @@
         <v>8</v>
       </c>
       <c r="C26" t="str">
-        <v>我的動齡限量版</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D26" t="str">
-        <v>我的動齡限量版</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E26">
-        <v>9.68</v>
+        <v>9.65</v>
       </c>
       <c r="F26" t="str">
-        <v>[[EP0063] 50+Con...] 選題新穎，結合「第三人生大學」與「大嬸陪聊」概念，案例生動且含金量極高，具備深度思考與社會連結。 | [[EP0071] 50+Con...] 選題新穎且具深度，聚焦於二代接班與職涯轉型，來賓的個人案例生動且含金量極高，提供了獨特的視角和實用建議。 | [[EP0045] 50+Con...] 選題深入探討紫微斗數的「四化」與「殺破狼」命格，不僅新穎且具備高度的專業含金量。來賓的案例分享與對社會現象的連結，讓內容更具啟發性與實用價值。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
       </c>
     </row>
     <row r="27">
@@ -935,16 +936,16 @@
         <v>9</v>
       </c>
       <c r="C27" t="str">
-        <v>下一本讀什麼？</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D27" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>蕭邦</v>
       </c>
       <c r="E27">
-        <v>9.66</v>
+        <v>9.65</v>
       </c>
       <c r="F27" t="str">
-        <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
       </c>
     </row>
     <row r="28">
@@ -955,16 +956,16 @@
         <v>10</v>
       </c>
       <c r="C28" t="str">
-        <v>宋家小館</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D28" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E28">
-        <v>9.65</v>
+        <v>9.6048</v>
       </c>
       <c r="F28" t="str">
-        <v>[EP162 | 從房地產到Ma...] 選題新穎，結合來賓的獨特職涯與創業經驗，案例生動且內容含金量極高，具備深度思考與利基選題。 | [EP191 | 《我到日本當漁...] 選題新穎且具備高度利基性，探討台灣人赴日擔任漁夫的獨特經歷，結合家族養殖業歷史，內容含金量高且引人入勝。 | [EP182 | 聽見身體的聲音...] 選題新穎且具深度，將頌缽音療的歷史、科學原理、身心影���及實際應用解釋得非常透徹，內容含金量高。</v>
+        <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
       </c>
     </row>
     <row r="29">
@@ -981,7 +982,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E29">
-        <v>9.55</v>
+        <v>9.4545</v>
       </c>
       <c r="F29" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 男主持人聲音清晰、有活力，中低音共鳴感佳，語速穩定度高，但口頭禪「就是」和「然後」出現頻率稍高。 | [EP174｜越省反而越窮？別把...] Andy的聲音溫暖清晰，語速穩定。好哥和蔡宇哲老師的聲音也很有特色，整體男聲表現優異。 | [EP164｜滑短影音是在浪費時...] 兩位男主持人的聲音皆具備良好的中低音共鳴。主主持人Andy口條流暢，語速穩定，但偶有口頭禪；來賓好哥的聲音則更為沉穩且富有磁性，整體播音表現優異。</v>
@@ -1001,7 +1002,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E30">
-        <v>9.49</v>
+        <v>9.4046</v>
       </c>
       <c r="F30" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 男來賓（蔡醫師）口條流暢，聲音專業且具說服力，解釋複雜概念清晰易懂，語速雖快但穩定。 | [《財富自由心理學》：賺錢，只是...] 兩位男主持人皆表現出色。主講人雨哲口條流暢，聲音清晰溫和，語速穩定。來賓好哥聲線低沉有磁性，論述力強。整體播音實力優異。</v>
@@ -1015,16 +1016,16 @@
         <v>3</v>
       </c>
       <c r="C31" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D31" t="str">
-        <v>梁哲維</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E31">
-        <v>9.32</v>
+        <v>9.313</v>
       </c>
       <c r="F31" t="str">
-        <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
+        <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
       </c>
     </row>
     <row r="32">
@@ -1035,16 +1036,16 @@
         <v>4</v>
       </c>
       <c r="C32" t="str">
-        <v>蕭邦相談室</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D32" t="str">
-        <v>蕭邦</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E32">
-        <v>9.24</v>
+        <v>9.2586</v>
       </c>
       <c r="F32" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
       </c>
     </row>
     <row r="33">
@@ -1055,16 +1056,16 @@
         <v>5</v>
       </c>
       <c r="C33" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D33" t="str">
-        <v>GK爸爸</v>
+        <v>梁哲維</v>
       </c>
       <c r="E33">
-        <v>9.21</v>
+        <v>9.25</v>
       </c>
       <c r="F33" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
+        <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
       </c>
     </row>
     <row r="34">
@@ -1075,16 +1076,16 @@
         <v>6</v>
       </c>
       <c r="C34" t="str">
-        <v>下一本讀什麼？</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D34" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>蕭邦</v>
       </c>
       <c r="E34">
-        <v>9.16</v>
+        <v>9.15</v>
       </c>
       <c r="F34" t="str">
-        <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
+        <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
       </c>
     </row>
     <row r="35">
@@ -1095,16 +1096,16 @@
         <v>7</v>
       </c>
       <c r="C35" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D35" t="str">
-        <v>人生啊！小歐</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E35">
-        <v>9.09</v>
+        <v>9.1048</v>
       </c>
       <c r="F35" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
+        <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
       </c>
     </row>
     <row r="36">
@@ -1121,7 +1122,7 @@
         <v>30節約男子</v>
       </c>
       <c r="E36">
-        <v>9.07</v>
+        <v>9</v>
       </c>
       <c r="F36" t="str">
         <v>[【EP39】矽谷阿雅｜貸款七百...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，但口頭禪「就是」和「然後」出現頻率稍高。 | [【EP51】胡咪＆Vito大叔...] Vito大叔的口條流暢，聲音低沉有磁性，語速穩定，能有效傳達情感。偶爾的口頭禪「就是」略多但不影響整體表現。 | [【EP36】明白｜父母雙亡，獨...] 男主持人聲音厚實有共鳴，語速雖快但咬字清晰，表達流暢。口頭禪「然後」、「就是」出現頻率稍高，但整體不影響專業度。</v>
@@ -1135,16 +1136,16 @@
         <v>9</v>
       </c>
       <c r="C37" t="str">
-        <v>夢想家說股事</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D37" t="str">
-        <v>美股夢想家</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E37">
-        <v>9.06</v>
+        <v>8.955</v>
       </c>
       <c r="F37" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
       </c>
     </row>
     <row r="38">
@@ -1161,7 +1162,7 @@
         <v>張忘形</v>
       </c>
       <c r="E38">
-        <v>9.03</v>
+        <v>8.955</v>
       </c>
       <c r="F38" t="str">
         <v>[EP61｜為什麼越努力經營，反...] 男主持人聲音清晰、能量高，中低音共鳴感良好，語速雖快但仍能保持清晰度。情緒感染力強，但口頭禪「就是」出現頻率稍高。 | [EP50｜看到什麼都東西都想拍...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰，情感表達豐富。但口頭禪「就是」和「然後」出現頻率稍高，略影響流暢度。 | [EP65｜ 對方因為小事就對你...] 男主持人聲音厚實有共鳴，語速偏快但清晰度高，情感表達豐富。然而，「就是」和「那」等口頭禪出現頻率較高，略影響流暢度。</v>
@@ -1181,7 +1182,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E39">
-        <v>9.43</v>
+        <v>9.3265</v>
       </c>
       <c r="F39" t="str">
         <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
@@ -1201,7 +1202,7 @@
         <v>莫菲穿搭</v>
       </c>
       <c r="E40">
-        <v>9.41</v>
+        <v>9.3049</v>
       </c>
       <c r="F40" t="str">
         <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
@@ -1215,16 +1216,16 @@
         <v>3</v>
       </c>
       <c r="C41" t="str">
-        <v>宋家小館</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D41" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E41">
-        <v>9.32</v>
+        <v>9.2715</v>
       </c>
       <c r="F41" t="str">
-        <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
       </c>
     </row>
     <row r="42">
@@ -1235,16 +1236,16 @@
         <v>4</v>
       </c>
       <c r="C42" t="str">
-        <v>說話人聲</v>
+        <v>宋家小館</v>
       </c>
       <c r="D42" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E42">
-        <v>9.31</v>
+        <v>9.2549</v>
       </c>
       <c r="F42" t="str">
-        <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
+        <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
       </c>
     </row>
     <row r="43">
@@ -1255,16 +1256,16 @@
         <v>5</v>
       </c>
       <c r="C43" t="str">
-        <v>蘇心時光</v>
+        <v>說話人聲</v>
       </c>
       <c r="D43" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>聲音表達講師林依柔</v>
       </c>
       <c r="E43">
-        <v>9.31</v>
+        <v>9.2549</v>
       </c>
       <c r="F43" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
+        <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
       </c>
     </row>
     <row r="44">
@@ -1281,7 +1282,7 @@
         <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E44">
-        <v>9.26</v>
+        <v>9.25</v>
       </c>
       <c r="F44" t="str">
         <v>[#801 市場震盪 17000...] 女主持人聲音清晰、溫暖且具共鳴，語速穩定舒適，情緒感染��佳，但偶有贅字。 | [#809  買股票還在到處問明...] Cindy2聲音圓潤清晰，語速適中，語調親和，具備溫馨陪伴感，引導能力強。 | [#798 害怕投資賠錢？不用天...] 兩位女主持人聲音清晰、語速快但穩定，高音域圓潤且具備溫馨陪伴感，無刺耳爆音。主講人Sandy的語速較快，但整體表現優異。</v>
@@ -1301,7 +1302,7 @@
         <v>丁菱娟</v>
       </c>
       <c r="E45">
-        <v>9.23</v>
+        <v>9.1599</v>
       </c>
       <c r="F45" t="str">
         <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
@@ -1321,7 +1322,7 @@
         <v>我的動齡限量版</v>
       </c>
       <c r="E46">
-        <v>9.18</v>
+        <v>9.1549</v>
       </c>
       <c r="F46" t="str">
         <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
@@ -1341,7 +1342,7 @@
         <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="E47">
-        <v>9.07</v>
+        <v>9.05</v>
       </c>
       <c r="F47" t="str">
         <v>[EP199-別再相信快速致富：...] 女主持人阿莉口條流暢，聲音清晰且富有感染力，語速雖快但穩定，高音域圓潤，具備溫馨陪伴感。 | [EP192-當貴人還沒出現時，...] 女主持人阿令的聲音明亮清晰，高音域圓潤且富有親和力，語速偏快但咬字清晰，情感表達真誠，具有良好的播音魅力。 | [EP210-會做不一定會贏｜表...] 女主持人阿林口條流暢，聲音清晰，語速穩定，高音域圓潤且具陪伴感，但偶有贅字。</v>
@@ -1361,7 +1362,7 @@
         <v>尼可這樣說</v>
       </c>
       <c r="E48">
-        <v>9.01</v>
+        <v>8.8846</v>
       </c>
       <c r="F48" t="str">
         <v>[EP.322 流量破百萬卻賺不...] 女主持人聲音清晰、溫暖且富有感染力，語速較快但口條流暢，能有效傳達資訊與情感。 | [EP.318 行銷不是方法，是...] 女主持人聲音清晰、溫暖，語速穩定舒適，高音域圓潤，具備溫馨陪伴感，播音實力優異。 | [EP.316 與其等流量，不如...] 主講人Nico聲音清晰、語速穩定且富有活力，高音域圓潤，雖有口頭禪但整體播音品質優良。</v>
@@ -1381,7 +1382,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E49">
-        <v>8.88</v>
+        <v>8.776</v>
       </c>
       <c r="F49" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 結尾有明確呼籲聽眾行動，力道足夠，能有效催化聽眾實踐。 | [EP174｜越省反而越窮？別把...] 結尾有明確的行動呼籲，鼓勵聽眾訂閱、留言、並嘗試微小行動，力道足夠。 | [EP164｜滑短影音是在浪費時...] 節目中多次提及來賓的新書，並在結尾有明確的行動呼籲，但力道尚可加強，未達到極強的催化效果。</v>
@@ -1395,16 +1396,16 @@
         <v>2</v>
       </c>
       <c r="C50" t="str">
-        <v>哇賽心理學</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D50" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E50">
-        <v>8.83</v>
+        <v>8.75</v>
       </c>
       <c r="F50" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
+        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
       </c>
     </row>
     <row r="51">
@@ -1415,16 +1416,16 @@
         <v>3</v>
       </c>
       <c r="C51" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D51" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E51">
-        <v>8.76</v>
+        <v>8.7261</v>
       </c>
       <c r="F51" t="str">
-        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
       </c>
     </row>
     <row r="52">
@@ -1441,7 +1442,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E52">
-        <v>8.72</v>
+        <v>8.655</v>
       </c>
       <c r="F52" t="str">
         <v>[EP225：【非典家庭CEO】...] 結尾有明確的行動呼籲，鼓勵聽眾點擊連結或撥打專線了解寄養家庭資訊，力道足夠且具體。 | [EP218：愛自己｜放下完美執...] 節目結尾的行動呼籲明確，針對線上課程提供了專屬優惠碼，具體且有吸引力，能有效促使聽眾採取行動。 | [EP219：【非典家庭CEO】...] 結尾有明確呼籲聽眾行動，力道足夠，鼓勵聽眾參與動物音樂會。</v>
@@ -1461,7 +1462,7 @@
         <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E53">
-        <v>8.66</v>
+        <v>8.6048</v>
       </c>
       <c r="F53" t="str">
         <v>[EP.617 《無限機器》讀後...] 結尾有明確呼籲聽眾訂閱電子報與節目，行動呼籲力道足夠且自然。 | [EP.573 從 0 到 10...] 結尾有明確呼籲聽眾填寫問卷和分享電子報，力道足夠且具體。 | [EP.607 《AI Firs...] 節目開頭與結尾都有明確且具說服力的行動呼籲，引導聽眾參與社群或閱讀書籍，催化力道足夠。</v>
@@ -1475,16 +1476,16 @@
         <v>6</v>
       </c>
       <c r="C54" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D54" t="str">
-        <v>梁哲維</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E54">
-        <v>8.66</v>
+        <v>8.6037</v>
       </c>
       <c r="F54" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
       </c>
     </row>
     <row r="55">
@@ -1495,16 +1496,16 @@
         <v>7</v>
       </c>
       <c r="C55" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D55" t="str">
-        <v>GK爸爸</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E55">
-        <v>8.55</v>
+        <v>8.5725</v>
       </c>
       <c r="F55" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
+        <v>[EP289  七巨頭變七矮人！...] 節目開頭和結尾都有明確且具吸引力的行動呼籲，鼓勵聽眾留言領取資訊或加入社群。 | [EP275 股市變賭場？巴菲特...] 節目結尾明確且多次呼籲聽眾加入社群、訂閱APP，並提供限時優惠，行動呼籲的強度與實踐催化力足夠。 | [EP251國防預算暴漲 5 成...] 節目結尾有推薦商品和下週節目預告，但行動呼籲的直接性與催化力中等。</v>
       </c>
     </row>
     <row r="56">
@@ -1515,16 +1516,16 @@
         <v>8</v>
       </c>
       <c r="C56" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D56" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>梁哲維</v>
       </c>
       <c r="E56">
-        <v>8.54</v>
+        <v>8.5715</v>
       </c>
       <c r="F56" t="str">
-        <v>[EP611 00998A(主動...] 結尾有明確呼籲聽眾查詢ETF資訊並諮詢營業員，行動呼籲清晰但力道中等。 | [EP628昇陽半導體(8028...] 結尾有明確呼籲聽眾參與其課程，行動呼籲力道足夠且資訊完整。 | [EP621《富媽媽 窮媽媽》第...] 結尾明確呼籲聽眾購買書籍以獲取更多資訊，並分享節目，行動呼籲清晰且具體。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
       </c>
     </row>
     <row r="57">
@@ -1535,16 +1536,16 @@
         <v>9</v>
       </c>
       <c r="C57" t="str">
-        <v>尼可這樣說</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D57" t="str">
-        <v>尼可這樣說</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E57">
-        <v>8.51</v>
+        <v>8.5535</v>
       </c>
       <c r="F57" t="str">
-        <v>[EP.322 流量破百萬卻賺不...] 節目中段與結尾皆有明確的行動呼籲，引導聽眾訂閱、諮詢或了解更多資訊，力道足夠且具體。 | [EP.318 行銷不是方法，是...] 在節目中段和結尾都有明確且具說服力的行動呼籲，力道足夠，能有效催化聽眾實踐。 | [EP.316 與其等流量，不如...] 結尾行動呼籲明確，針對線上課程提供折扣碼與期限，具備足夠的催化力。</v>
+        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
       </c>
     </row>
     <row r="58">
@@ -1555,16 +1556,16 @@
         <v>10</v>
       </c>
       <c r="C58" t="str">
-        <v>分手的99個理由</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D58" t="str">
-        <v>胡咪老師</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E58">
-        <v>8.49</v>
+        <v>8.4765</v>
       </c>
       <c r="F58" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
+        <v>[EP611 00998A(主動...] 結尾有明確呼籲聽眾查詢ETF資訊並諮詢營業員，行動呼籲清晰但力道中等。 | [EP628昇陽半導體(8028...] 結尾有明確呼籲聽眾參與其課程，行動呼籲力道足夠且資訊完整。 | [EP621《富媽媽 窮媽媽》第...] 結尾明確呼籲聽眾購買書籍以獲取更多資訊，並分享節目，行動呼籲清晰且具體。</v>
       </c>
     </row>
     <row r="59">
@@ -1581,7 +1582,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E59">
-        <v>9.22</v>
+        <v>9.155</v>
       </c>
       <c r="F59" t="str">
         <v>[EP225：【非典家庭CEO】...] 寄養家庭議題雖然非絕對冷門，但節目深入探討其背後的挑戰、家庭動員與個人成長，提供了獨特的視角和豐富的細節，論述完整且具深度。 | [EP218：愛自己｜放下完美執...] 人類圖本身即為利基市場，本集更深入探討流日、閘門與關係互動等細節，論述完整且具專業度，滿足了特定聽眾群的深度需求。 | [EP219：【非典家庭CEO】...] 雖然育兒是廣泛議題，但從專業音樂家角度切入，並結合獨特的動物音樂會推廣，使其具備高度利基市場價值。</v>
@@ -1601,7 +1602,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E60">
-        <v>9.16</v>
+        <v>9.0595</v>
       </c>
       <c r="F60" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
@@ -1621,7 +1622,7 @@
         <v>宋家小館｜Becky</v>
       </c>
       <c r="E61">
-        <v>8.99</v>
+        <v>8.9215</v>
       </c>
       <c r="F61" t="str">
         <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
@@ -1641,7 +1642,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E62">
-        <v>8.9</v>
+        <v>8.8148</v>
       </c>
       <c r="F62" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
@@ -1661,7 +1662,7 @@
         <v>蕭邦</v>
       </c>
       <c r="E63">
-        <v>8.74</v>
+        <v>8.6296</v>
       </c>
       <c r="F63" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
@@ -1675,16 +1676,16 @@
         <v>6</v>
       </c>
       <c r="C64" t="str">
-        <v>教出你的路</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D64" t="str">
-        <v>治療師瑪奇</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E64">
-        <v>8.66</v>
+        <v>8.6049</v>
       </c>
       <c r="F64" t="str">
-        <v>[EP47 有團隊的感覺如何？教...] 解剖學結合運動教學是一個相對利基的市場，主持人以獨特視角切入，論述完整且具深度，不易被取代。 | [EP31 為了愛移民，她打造 ...] 以植物性飲食為核心，並強調非卡路里導向的理念，在健康飲食領域中具備獨特的利基市場視角。 | [EP35 為什麼堅持開「解剖學...] 「應用解剖運動學」是一個相對專業且具利基性的市場，主持人對此議題的論述深入且完整，有效觸及目標受眾的需求。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
       </c>
     </row>
     <row r="65">
@@ -1701,7 +1702,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E65">
-        <v>8.66</v>
+        <v>8.5598</v>
       </c>
       <c r="F65" t="str">
         <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
@@ -1715,16 +1716,16 @@
         <v>8</v>
       </c>
       <c r="C66" t="str">
-        <v>蘇心時光</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D66" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E66">
-        <v>8.64</v>
+        <v>8.5331</v>
       </c>
       <c r="F66" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
+        <v>[S4.EP4｜性平教育20年，...] 議題探討深入，特別關注數位時代下的約會暴力、男性及LGBTQ+受害者的困境，具備高度利基市場的獨特性。 | [S4.EP8｜我不想再跟你生活...] 議題聚焦於離婚後的心理歷程與微小生活習慣的影響，雖非極度冷門，但論述角度獨特且完整。 | [S4.EP14｜有些人沒有成為...] 「比前任更難忘的非前任」這一議題雖然具有普世性，但節目從心理學、文學和個人經驗等多維度進行深入探討，使其在同類節目中具備獨特的利基市場論述。</v>
       </c>
     </row>
     <row r="67">
@@ -1735,16 +1736,16 @@
         <v>9</v>
       </c>
       <c r="C67" t="str">
-        <v>財富餐車不打烊</v>
+        <v>教出你的路</v>
       </c>
       <c r="D67" t="str">
-        <v>30節約男子</v>
+        <v>治療師瑪奇</v>
       </c>
       <c r="E67">
-        <v>8.57</v>
+        <v>8.5265</v>
       </c>
       <c r="F67" t="str">
-        <v>[【EP39】矽谷阿雅｜貸款七百...] AI驅動的男士時尚租賃服務是一個非常具體的利基市場，節目對其論述完整且深入。 | [【EP51】胡咪＆Vito大叔...] 理財主題雖廣泛，但結合來賓的「30節約男」個人故事和「斷捨離」等具體實踐，使其在同類節目中具有一定的獨特性。 | [【EP36】明白｜父母雙亡，獨...] 議題稀有度高，將「獨生女」概念延伸至人生獨自面對挑戰的普遍性，論述完整且具啟發性。</v>
+        <v>[EP47 有團隊的感覺如何？教...] 解剖學結合運動教學是一個相對利基的市場，主持人以獨特視角切入，論述完整且具深度，不易被取代。 | [EP31 為了愛移民，她打造 ...] 以植物性飲食為核心，並強調非卡路里導向的理念，在健康飲食領域中具備獨特的利基市場視角。 | [EP35 為什麼堅持開「解剖學...] 「應用解剖運動學」是一個相對專業且具利基性的市場，主持人對此議題的論述深入且完整，有效觸及目標受眾的需求。</v>
       </c>
     </row>
     <row r="68">
@@ -1761,7 +1762,7 @@
         <v>丁菱娟</v>
       </c>
       <c r="E68">
-        <v>8.57</v>
+        <v>8.505</v>
       </c>
       <c r="F68" t="str">
         <v>[ep21. 用台灣腦袋，看透全...] 議題聚焦台灣科技產業的供應鏈與產業分析，雖非極度冷門，但論述深度與專業性使其在利基市場中表現突出。 | [ep11. Z世代難搞嗎？用對...] Z世代議題雖非極度冷門，但節目從職場管理、品牌行銷等多維度深入剖析，並結合實務經驗，提供了獨特的觀點與論述，使其在同類議題中具備差異化。 | [ep23. 主動出擊的力量有多...] 議題雖非極度冷門，但以「搭訕」為切入點，並將其應用於廣泛的生活層面，論述獨特且完整。</v>
@@ -1781,7 +1782,7 @@
         <v>蘇絢慧分享空間</v>
       </c>
       <c r="E69">
-        <v>9.31</v>
+        <v>9.2715</v>
       </c>
       <c r="F69" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
@@ -1795,16 +1796,16 @@
         <v>2</v>
       </c>
       <c r="C70" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D70" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E70">
-        <v>9.06</v>
+        <v>9.0535</v>
       </c>
       <c r="F70" t="str">
-        <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
+        <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
       </c>
     </row>
     <row r="71">
@@ -1815,16 +1816,16 @@
         <v>3</v>
       </c>
       <c r="C71" t="str">
-        <v>宋家小館</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D71" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E71">
-        <v>8.99</v>
+        <v>8.9765</v>
       </c>
       <c r="F71" t="str">
-        <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
+        <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
       </c>
     </row>
     <row r="72">
@@ -1835,16 +1836,16 @@
         <v>4</v>
       </c>
       <c r="C72" t="str">
-        <v>分手的99個理由</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D72" t="str">
-        <v>胡咪老師</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E72">
-        <v>8.99</v>
+        <v>8.9252</v>
       </c>
       <c r="F72" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="73">
@@ -1855,16 +1856,16 @@
         <v>5</v>
       </c>
       <c r="C73" t="str">
-        <v>布姐的沙發</v>
+        <v>宋家小館</v>
       </c>
       <c r="D73" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E73">
-        <v>8.93</v>
+        <v>8.9022</v>
       </c>
       <c r="F73" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
+        <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
       </c>
     </row>
     <row r="74">
@@ -1875,16 +1876,16 @@
         <v>6</v>
       </c>
       <c r="C74" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D74" t="str">
-        <v>無所不試無樂不作</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E74">
-        <v>8.9</v>
+        <v>8.8265</v>
       </c>
       <c r="F74" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
+        <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
       </c>
     </row>
     <row r="75">
@@ -1895,16 +1896,16 @@
         <v>7</v>
       </c>
       <c r="C75" t="str">
-        <v>五吉郎</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D75" t="str">
-        <v>五吉郎</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E75">
-        <v>8.88</v>
+        <v>8.8265</v>
       </c>
       <c r="F75" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 整體語調平穩溫和，適合深夜靜聽，但部分討論較為熱情，略有起伏。 | [EP174｜越省反而越窮？別把...] 聲音平穩，語調溫和，適合深夜聆聽，無突兀尖銳音。 | [EP164｜滑短影音是在浪費時...] 節目氛圍沉穩且具思考性，兩位主持人的語調平穩溫和，適合聽眾在夜晚靜心聆聽與反思，無突兀尖銳音效。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="76">
@@ -1915,16 +1916,16 @@
         <v>8</v>
       </c>
       <c r="C76" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>下半場人生陪談師</v>
       </c>
       <c r="D76" t="str">
-        <v>GK爸爸</v>
+        <v>下半場人生事務有限公司</v>
       </c>
       <c r="E76">
-        <v>8.88</v>
+        <v>8.8098</v>
       </c>
       <c r="F76" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
+        <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="77">
@@ -1935,16 +1936,16 @@
         <v>9</v>
       </c>
       <c r="C77" t="str">
-        <v>下半場人生陪談師</v>
+        <v>五吉郎</v>
       </c>
       <c r="D77" t="str">
-        <v>下半場人生事務有限公司</v>
+        <v>五吉郎</v>
       </c>
       <c r="E77">
-        <v>8.86</v>
+        <v>8.776</v>
       </c>
       <c r="F77" t="str">
-        <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 整體語調平穩溫和，適合深夜靜聽，但部分討論較為熱情，略有起伏。 | [EP174｜越省反而越窮？別把...] 聲音平穩，語調溫和，適合深夜聆聽，無突兀尖銳音。 | [EP164｜滑短影音是在浪費時...] 節目氛圍沉穩且具思考性，兩位主持人的語調平穩溫和，適合聽眾在夜晚靜心聆聽與反思，無突兀尖銳音效。</v>
       </c>
     </row>
     <row r="78">
@@ -1961,7 +1962,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E78">
-        <v>8.82</v>
+        <v>8.75</v>
       </c>
       <c r="F78" t="str">
         <v>[【EP330 帶著善意行動，最...] 聲音平穩溫和，談話內容有深度，適合深夜靜聽與思考。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的語調溫和穩定，聲音品質優良，適合在深夜時段放鬆聆聽，具有陪伴治癒感。 | [【EP312《超越我執的生活》...] 主持人語調溫和穩定，聲音沉穩，內容具備深度思考，無突兀尖銳爆音，非常適合深夜聆聽，能帶來陪伴與沉靜感。</v>
@@ -1975,16 +1976,16 @@
         <v>1</v>
       </c>
       <c r="C79" t="str">
-        <v>五吉郎</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D79" t="str">
-        <v>五吉郎</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E79">
-        <v>9.22</v>
+        <v>9.251</v>
       </c>
       <c r="F79" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
+        <v>[EP289  七巨頭變七矮人！...] 節目節奏明快，主持人語調充滿朝氣，內容資訊量大，非常適合通勤時提神醒腦。 | [EP275 股市變賭場？巴菲特...] 節目節奏明快，主講人語調充滿活力且資訊量豐富，非常適合通勤或早晨時段收聽，有助於提神醒腦並快速掌握市場動態。 | [EP251國防預算暴漲 5 成...] 節奏明快，語調朝氣蓬勃，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="80">
@@ -1995,16 +1996,16 @@
         <v>2</v>
       </c>
       <c r="C80" t="str">
-        <v>下一本讀什麼？</v>
+        <v>五吉郎</v>
       </c>
       <c r="D80" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>五吉郎</v>
       </c>
       <c r="E80">
-        <v>9.16</v>
+        <v>9.1094</v>
       </c>
       <c r="F80" t="str">
-        <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
       </c>
     </row>
     <row r="81">
@@ -2015,16 +2016,16 @@
         <v>3</v>
       </c>
       <c r="C81" t="str">
-        <v>哇賽心理學</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D81" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E81">
-        <v>9.16</v>
+        <v>9.1048</v>
       </c>
       <c r="F81" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
+        <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="82">
@@ -2041,7 +2042,7 @@
         <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E82">
-        <v>9.09</v>
+        <v>9.0543</v>
       </c>
       <c r="F82" t="str">
         <v>[郝聲音：（下） 莊鈞涵（Car...] 節奏明快，主持人與來賓充滿朝氣，內容實用且具激勵性，適合通勤時提神醒腦。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目節奏明快，開頭活力十足，內容實用且具啟發性，適合通勤時提神醒腦與獲取新知。 | [郝聲音：成為人生更自由的「精銳...] 節奏明快，語調朝氣蓬勃，內容具啟發性，非常適合通勤時提神醒腦。</v>
@@ -2055,16 +2056,16 @@
         <v>5</v>
       </c>
       <c r="C83" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D83" t="str">
-        <v>丁菱娟</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E83">
-        <v>9.07</v>
+        <v>9.0477</v>
       </c>
       <c r="F83" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
       </c>
     </row>
     <row r="84">
@@ -2075,16 +2076,16 @@
         <v>6</v>
       </c>
       <c r="C84" t="str">
-        <v>能量黑客</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D84" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E84">
-        <v>9.06</v>
+        <v>9</v>
       </c>
       <c r="F84" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
+        <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="85">
@@ -2095,16 +2096,16 @@
         <v>7</v>
       </c>
       <c r="C85" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>能量黑客</v>
       </c>
       <c r="D85" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E85">
-        <v>9.04</v>
+        <v>9</v>
       </c>
       <c r="F85" t="str">
-        <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
       </c>
     </row>
     <row r="86">
@@ -2115,16 +2116,16 @@
         <v>8</v>
       </c>
       <c r="C86" t="str">
-        <v>閱讀聊樂KEY</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D86" t="str">
-        <v>閱讀聊樂key</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E86">
-        <v>9.03</v>
+        <v>8.9846</v>
       </c>
       <c r="F86" t="str">
-        <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="87">
@@ -2135,16 +2136,16 @@
         <v>9</v>
       </c>
       <c r="C87" t="str">
-        <v>尼可這樣說</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D87" t="str">
-        <v>尼可這樣說</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E87">
-        <v>9.01</v>
+        <v>8.9765</v>
       </c>
       <c r="F87" t="str">
-        <v>[EP.322 流量破百萬卻賺不...] 節目節奏明快，內容資訊量高且具啟發性，主持人與來賓的清晰表達有助於通勤時提神醒腦，適合早晨收聽。 | [EP.318 行銷不是方法，是...] 節目節奏明快，內容資訊密度高，主持人與來賓的對談朝氣十足，具有通勤提神醒腦的效果。 | [EP.316 與其等流量，不如...] 節目節奏明快，主講人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。</v>
+        <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
       </c>
     </row>
     <row r="88">
@@ -2155,16 +2156,16 @@
         <v>10</v>
       </c>
       <c r="C88" t="str">
-        <v>我的動齡限量版</v>
+        <v>閱讀聊樂KEY</v>
       </c>
       <c r="D88" t="str">
-        <v>我的動齡限量版</v>
+        <v>閱讀聊樂key</v>
       </c>
       <c r="E88">
-        <v>9.01</v>
+        <v>8.9715</v>
       </c>
       <c r="F88" t="str">
-        <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
+        <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
       </c>
     </row>
     <row r="89">
@@ -2181,7 +2182,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E89">
-        <v>8.72</v>
+        <v>8.6346</v>
       </c>
       <c r="F89" t="str">
         <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
@@ -2201,7 +2202,7 @@
         <v>胡咪老師</v>
       </c>
       <c r="E90">
-        <v>8.33</v>
+        <v>8.3557</v>
       </c>
       <c r="F90" t="str">
         <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
@@ -2215,16 +2216,16 @@
         <v>3</v>
       </c>
       <c r="C91" t="str">
-        <v>五吉郎</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D91" t="str">
-        <v>五吉郎</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E91">
-        <v>8.22</v>
+        <v>8.2468</v>
       </c>
       <c r="F91" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
       </c>
     </row>
     <row r="92">
@@ -2235,16 +2236,16 @@
         <v>4</v>
       </c>
       <c r="C92" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>五吉郎</v>
       </c>
       <c r="D92" t="str">
-        <v>GK爸爸</v>
+        <v>五吉郎</v>
       </c>
       <c r="E92">
-        <v>8.21</v>
+        <v>8.1094</v>
       </c>
       <c r="F92" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
       </c>
     </row>
     <row r="93">
@@ -2255,16 +2256,16 @@
         <v>5</v>
       </c>
       <c r="C93" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D93" t="str">
-        <v>梁哲維</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E93">
-        <v>8.16</v>
+        <v>8.0742</v>
       </c>
       <c r="F93" t="str">
-        <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
       </c>
     </row>
     <row r="94">
@@ -2275,16 +2276,16 @@
         <v>6</v>
       </c>
       <c r="C94" t="str">
-        <v>蘇心時光</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D94" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>梁哲維</v>
       </c>
       <c r="E94">
-        <v>8.14</v>
+        <v>8.0598</v>
       </c>
       <c r="F94" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
+        <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
       </c>
     </row>
     <row r="95">
@@ -2301,7 +2302,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E95">
-        <v>8.1</v>
+        <v>7.9846</v>
       </c>
       <c r="F95" t="str">
         <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
@@ -2315,16 +2316,16 @@
         <v>8</v>
       </c>
       <c r="C96" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D96" t="str">
-        <v>莫菲穿搭</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E96">
-        <v>8.07</v>
+        <v>7.9696</v>
       </c>
       <c r="F96" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 對談風格輕鬆歡樂，主持人與來賓之間的幽默互動和生活化分享（如吃茶葉蛋、羊肉爐、生魚片）帶來解壓感，笑聲自然，營造出愉悅的氛圍。 | [莫菲穿搭27｜金曲幕後直擊！電...] 節目內容偏向專業分析與個人觀點分享，輕鬆歡樂的療癒感相對較低。 | [莫菲穿搭02｜2026流行色配...] 談話風格較為嚴肅認真，以知識分享為主，解壓療癒感普通，較少輕鬆歡樂的對話。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
       </c>
     </row>
     <row r="97">
@@ -2335,16 +2336,16 @@
         <v>9</v>
       </c>
       <c r="C97" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D97" t="str">
-        <v>無所不試無樂不作</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E97">
-        <v>8.07</v>
+        <v>7.9598</v>
       </c>
       <c r="F97" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 對談風格輕鬆歡樂，主持人與來賓之間的幽默互動和生活化分享（如吃茶葉蛋、羊肉爐、生魚片）帶來解壓感，笑聲自然，營造出愉悅的氛圍。 | [莫菲穿搭27｜金曲幕後直擊！電...] 節目內容偏向專業分析與個人觀點分享，輕鬆歡樂的療癒感相對較低。 | [莫菲穿搭02｜2026流行色配...] 談話風格較為嚴肅認真，以知識分享為主，解壓療癒感普通，較少輕鬆歡樂的對話。</v>
       </c>
     </row>
     <row r="98">
@@ -2361,7 +2362,7 @@
         <v>蕭邦</v>
       </c>
       <c r="E98">
-        <v>8.07</v>
+        <v>7.9598</v>
       </c>
       <c r="F98" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 談話風格偏向認真探討，而非輕鬆歡樂的療癒感。 | [【蕭邦出任務】如何選擇適合自己...] 談話風格較為深入與嚴肅，著重於職涯挑戰與個人成長，因此日常廢話解壓感和療癒感相對較低。 | [幸福的人，通常「覺察力」都很強...] 談話風格真誠且具啟發性，能引導聽眾自我療癒與成長，但較少輕鬆歡樂的廢話解壓感。</v>
@@ -2381,7 +2382,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E99">
-        <v>10</v>
+        <v>9.9545</v>
       </c>
       <c r="F99" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 深度探討自由人生、自我成長、內在探索與心靈啟發，從個人經歷中提煉出普世價值，啟發性極強。 | [EP174｜越省反而越窮？別把...] 深度探討金錢觀、人生目的與自我成長，對聽眾的內在探索有很強的啟發。 | [EP164｜滑短影音是在浪費時...] 節目深度探討了閱讀如何影響個人成長、思維模式的轉變以及如何找回自我可能性，提供了豐富的內在探索與心靈啟發內容。</v>
@@ -2395,16 +2396,16 @@
         <v>2</v>
       </c>
       <c r="C100" t="str">
-        <v>哇賽心理學</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D100" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E100">
-        <v>9.99</v>
+        <v>9.95</v>
       </c>
       <c r="F100" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
       </c>
     </row>
     <row r="101">
@@ -2415,16 +2416,16 @@
         <v>3</v>
       </c>
       <c r="C101" t="str">
-        <v>蘇心時光</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D101" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E101">
-        <v>9.98</v>
+        <v>9.8842</v>
       </c>
       <c r="F101" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
       </c>
     </row>
     <row r="102">
@@ -2441,7 +2442,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E102">
-        <v>9.93</v>
+        <v>9.8265</v>
       </c>
       <c r="F102" t="str">
         <v>[EP470｜把人放在心上的共贏...] 節目深度探討了自我成長、內在價值觀與目的性創業，來賓對自信的定義也提供了深刻的心靈啟發。 | [EP433｜【中年轉型】從矽谷...] 深度探討個人職涯轉型、自我覺察與性格探索，提供豐富的心靈啟發與成長觀點，是本集的核心亮點。 | [EP466｜拒絕被朝九晚五綁架...] 本集節目核心圍繞著自我成長、內在探索與心靈啟發。來賓透過「百工計畫」的實踐，深入剖析了個人與社會的關係，以及如何找到內在平衡，啟發性極強。</v>
@@ -2461,7 +2462,7 @@
         <v>蕭邦</v>
       </c>
       <c r="E103">
-        <v>9.9</v>
+        <v>9.8049</v>
       </c>
       <c r="F103" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 深度探討自我成長、內在探索與心靈啟發，主持人分享個人轉變歷程，極具啟發性。 | [【蕭邦出任務】如何選擇適合自己...] 來賓的職涯轉型故事與主持人對自我價值的探討，提供了深刻的內在探索與心靈啟發，深度極高。 | [幸福的人，通常「覺察力」都很強...] 深度探討情緒的來源、自我批判的迴圈以及如何透過覺察進行自我調整，對內在探索與心靈啟發的深度極高。</v>
@@ -2481,7 +2482,7 @@
         <v>張忘形</v>
       </c>
       <c r="E104">
-        <v>9.86</v>
+        <v>9.7765</v>
       </c>
       <c r="F104" t="str">
         <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
@@ -2501,7 +2502,7 @@
         <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E105">
-        <v>9.83</v>
+        <v>9.7597</v>
       </c>
       <c r="F105" t="str">
         <v>[EP.617 《無限機器》讀後...] 節目深度探討了個人使命感、價值觀與對未來的思考，引導聽眾進行自我成長與內在探索���心靈啟發感極強。 | [EP.573 從 0 到 10...] 深度探討個人成長、心態轉變、面對困難的韌性，以及如何從內在尋找動力，心靈啟發感極強。 | [EP.607 《AI Firs...] 節目核心圍繞個人在AI時代的自我成長、能力提升與心態轉變，提供了深刻的內在探索與心靈啟發。</v>
@@ -2521,7 +2522,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E106">
-        <v>9.82</v>
+        <v>9.75</v>
       </c>
       <c r="F106" t="str">
         <v>[【EP330 帶著善意行動，最...] 節目深度探討了創業者的初心、傳承的意義以及善意帶來的回饋，對聽眾的自我成長和內在探索有很強的啟發。 | [【EP302 把命盤變成行動藍...] 節目核心圍繞著個人命運、自我認知與未來規劃，深度啟發聽眾進行內在探索與自我成長，極具價值。 | [【EP312《超越我執的生活》...] 本集內容核心即為自我成長與內在探索，透過對「我執」的剖析和「臨在��的實踐，提供了深刻的心靈啟發，高度符合此獎項的評估維度。</v>
@@ -2535,16 +2536,16 @@
         <v>9</v>
       </c>
       <c r="C107" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D107" t="str">
-        <v>人生啊！小歐</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E107">
-        <v>9.76</v>
+        <v>9.75</v>
       </c>
       <c r="F107" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 節目深度探討自我價值、原生家庭影響及個人成長，對聽眾的自我探索與心靈啟發有極大助益。 | [S0714-【關係修復室】5個...] 節目核心圍繞自我成長、內在探索與關係修復，提供了深刻的心靈啟發。 | [S0810-戀愛腦怎麼辦？太理...] 節目深度挖掘個人內在需求、童年經驗對關係模式的影響，並鼓勵聽眾向內探索，心靈啟發與自我成長的深度極高。</v>
+        <v>[#801 市場震盪 17000...] 深度探討了投資中的心理層面、個人風險承受度與長期目標設定，對聽眾的自我成長與內在探索有很強的啟發性。 | [#809  買股票還在到處問明...] 節目不僅談投資，更強調學習、成長和建立系統思維，對自我探索和心靈啟發有深度，鼓勵聽眾提升自我。 | [#798 害怕投資賠錢？不用天...] 深度探討投資與個人生活目標的連結，鼓勵聽眾進行自我反思，建立符合自身價值觀的財務規劃，心靈啟發感極強。</v>
       </c>
     </row>
     <row r="108">
@@ -2555,16 +2556,16 @@
         <v>10</v>
       </c>
       <c r="C108" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D108" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E108">
-        <v>9.76</v>
+        <v>9.655</v>
       </c>
       <c r="F108" t="str">
-        <v>[#801 市場震盪 17000...] 深度探討了投資中的心理層面、個人風險承受度與長期目標設定，對聽眾的自我成長與內在探索有很強的啟發性。 | [#809  買股票還在到處問明...] 節目不僅談投資，更強調學習、成長和建立系統思維，對自我探索和心靈啟發有深度，鼓勵聽眾提升自我。 | [#798 害怕投資賠錢？不用天...] 深度探討投資與個人生活目標的連結，鼓勵聽眾進行自我反思，建立符合自身價值觀的財務規劃，心靈啟發感極強。</v>
+        <v>[EP225：【非典家庭CEO】...] 節目深度探討了個人在面對生命挑戰時的內在轉變、成長與自我超越，特別是保會媽媽從「後悔」到「互相陪伴」的心路歷程，極具心靈啟發深度。 | [EP218：愛自己｜放下完美執...] 人類圖的核心價值即是自我探索與成長。本集透過解析個人特質、關係模式及流日影響，提供了豐富的工具與視角，深刻啟發聽眾認識自我、理解他人，並引導心靈成長。 | [EP219：【非典家庭CEO】...] 深度探討育兒過程中的自我成長、內在探索與心靈啟發，提供豐富的思考面向。</v>
       </c>
     </row>
     <row r="109">
@@ -2601,7 +2602,7 @@
         <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E110">
-        <v>9.59</v>
+        <v>9.5543</v>
       </c>
       <c r="F110" t="str">
         <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
@@ -2621,7 +2622,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E111">
-        <v>9.49</v>
+        <v>9.4046</v>
       </c>
       <c r="F111" t="str">
         <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
@@ -2641,7 +2642,7 @@
         <v>美股航海王</v>
       </c>
       <c r="E112">
-        <v>9.38</v>
+        <v>9.3547</v>
       </c>
       <c r="F112" t="str">
         <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
@@ -2661,7 +2662,7 @@
         <v>Fire人生大學｜道哥</v>
       </c>
       <c r="E113">
-        <v>9.35</v>
+        <v>9.3048</v>
       </c>
       <c r="F113" t="str">
         <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
@@ -2695,16 +2696,16 @@
         <v>7</v>
       </c>
       <c r="C115" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D115" t="str">
-        <v>人生啊！小歐</v>
+        <v>梁哲維</v>
       </c>
       <c r="E115">
-        <v>8.84</v>
+        <v>8.75</v>
       </c>
       <c r="F115" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
+        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
       </c>
     </row>
     <row r="116">
@@ -2715,16 +2716,16 @@
         <v>8</v>
       </c>
       <c r="C116" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D116" t="str">
-        <v>梁哲維</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E116">
-        <v>8.82</v>
+        <v>8.6925</v>
       </c>
       <c r="F116" t="str">
-        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
       </c>
     </row>
     <row r="117">
@@ -2735,16 +2736,16 @@
         <v>9</v>
       </c>
       <c r="C117" t="str">
-        <v>尼可這樣說</v>
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="D117" t="str">
-        <v>尼可這樣說</v>
+        <v>Dr Selena</v>
       </c>
       <c r="E117">
-        <v>8.51</v>
+        <v>8.5044</v>
       </c>
       <c r="F117" t="str">
-        <v>[EP.316 與其等流量，不如...] 單集時長約63分鐘，內容資訊密度高且全程保持引人入勝，無明顯冷場，符合長篇內容的評估標準。</v>
+        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
       </c>
     </row>
     <row r="118">
@@ -2755,16 +2756,16 @@
         <v>10</v>
       </c>
       <c r="C118" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>你也想紅嗎</v>
       </c>
       <c r="D118" t="str">
-        <v>Dr Selena</v>
+        <v>品牌女子A娜</v>
       </c>
       <c r="E118">
-        <v>8.5</v>
+        <v>8.45</v>
       </c>
       <c r="F118" t="str">
-        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
+        <v>[EP66｜你沒辦法用過去有限能...] 單集時長53分鐘，資訊密度高且內容豐富，無明顯冷場，符合長篇內容的評估標準。</v>
       </c>
     </row>
     <row r="119">
@@ -2781,7 +2782,7 @@
         <v>蕭邦</v>
       </c>
       <c r="E119">
-        <v>9.74</v>
+        <v>9.65</v>
       </c>
       <c r="F119" t="str">
         <v>[幸福的人，通常「覺察力」都很強...] 單集時長在10-15分鐘（11分48秒），內容精煉且傳播效率高，能在短時間內提供豐富的資訊與啟發。</v>
@@ -2795,16 +2796,16 @@
         <v>2</v>
       </c>
       <c r="C120" t="str">
-        <v>美業幹什麼</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D120" t="str">
-        <v>美業幹什麼｜蔡佩陵</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E120">
-        <v>9.57</v>
+        <v>9.6037</v>
       </c>
       <c r="F120" t="str">
-        <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
+        <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
       </c>
     </row>
     <row r="121">
@@ -2815,16 +2816,16 @@
         <v>3</v>
       </c>
       <c r="C121" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>美業幹什麼</v>
       </c>
       <c r="D121" t="str">
-        <v>GK爸爸</v>
+        <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="E121">
         <v>9.55</v>
       </c>
       <c r="F121" t="str">
-        <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
+        <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
       </c>
     </row>
     <row r="122">
@@ -2841,7 +2842,7 @@
         <v>山姆書書</v>
       </c>
       <c r="E122">
-        <v>9.43</v>
+        <v>9.3546</v>
       </c>
       <c r="F122" t="str">
         <v>[EP134.真的找得到靈魂伴侶...] 單集時長約13分鐘，精煉且資訊密度高，在短時間內傳達了豐富的內容與思考，傳播效率極佳��</v>
@@ -2861,7 +2862,7 @@
         <v>治療師瑪奇</v>
       </c>
       <c r="E123">
-        <v>9.32</v>
+        <v>9.205</v>
       </c>
       <c r="F123" t="str">
         <v>[EP31 為了愛移民，她打造 ...] 單集時長約13分半，內容精煉且資訊密度高，傳播效率極佳，無冗餘。</v>
@@ -2881,7 +2882,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E124">
-        <v>9.07</v>
+        <v>9.005</v>
       </c>
       <c r="F124" t="str">
         <v>[【大師專題】人在江湖，身不由己...] 單集時長約10分鐘，符合10-15分鐘的短篇內容範疇。內容精煉，資訊密度高，能在短時間內傳達深刻且完整的觀點，傳播效率極佳。</v>
@@ -2901,7 +2902,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E125">
-        <v>9.66</v>
+        <v>9.5595</v>
       </c>
       <c r="F125" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
@@ -2915,16 +2916,16 @@
         <v>2</v>
       </c>
       <c r="C126" t="str">
-        <v>五吉郎</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D126" t="str">
-        <v>五吉郎</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E126">
-        <v>9.55</v>
+        <v>9.4821</v>
       </c>
       <c r="F126" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
+        <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
       </c>
     </row>
     <row r="127">
@@ -2935,16 +2936,16 @@
         <v>3</v>
       </c>
       <c r="C127" t="str">
-        <v>蘇心時光</v>
+        <v>五吉郎</v>
       </c>
       <c r="D127" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>五吉郎</v>
       </c>
       <c r="E127">
-        <v>9.48</v>
+        <v>9.4545</v>
       </c>
       <c r="F127" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
       </c>
     </row>
     <row r="128">
@@ -2955,16 +2956,16 @@
         <v>4</v>
       </c>
       <c r="C128" t="str">
-        <v>布姐的沙發</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D128" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E128">
-        <v>9.43</v>
+        <v>9.45</v>
       </c>
       <c r="F128" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
       </c>
     </row>
     <row r="129">
@@ -2975,16 +2976,16 @@
         <v>5</v>
       </c>
       <c r="C129" t="str">
-        <v>分手的99個理由</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D129" t="str">
-        <v>胡咪老師</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E129">
-        <v>9.43</v>
+        <v>9.3265</v>
       </c>
       <c r="F129" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
+        <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
       </c>
     </row>
     <row r="130">
@@ -3001,7 +3002,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E130">
-        <v>9.39</v>
+        <v>9.3099</v>
       </c>
       <c r="F130" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
@@ -3015,16 +3016,16 @@
         <v>7</v>
       </c>
       <c r="C131" t="str">
-        <v>蕭邦相談室</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D131" t="str">
-        <v>蕭邦</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E131">
-        <v>9.34</v>
+        <v>9.2586</v>
       </c>
       <c r="F131" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人透過引人入勝的敘事和情感連結，成功建立與聽眾的深厚關係，讓人期待後續故事發展，黏著度高。 | [春暖花開小旅行...] 主持人透過生動的敘述與角色扮演，與聽眾建立起良好的情感連結，具有高度的黏著度與陪伴感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 故事引人入勝，結尾的懸念設計強烈，讓聽眾對後續發展充滿期待，黏著度高。</v>
       </c>
     </row>
     <row r="132">
@@ -3041,7 +3042,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E132">
-        <v>9.32</v>
+        <v>9.25</v>
       </c>
       <c r="F132" t="str">
         <v>[【EP330 帶著善意行動，最...] 主持人與來賓的對談充滿情感溫度，真誠的交流讓聽眾感受到靈魂的陪伴，具有很強的黏著度。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的對談真誠且富有溫度，內容��人入勝，能有效提升聽眾的黏著度與持續收聽的意願。 | [【EP312《超越我執的生活》...] 主持人以真誠且富有洞察力的語氣分享，內容深度能引發聽眾共鳴與思考，建立起較強的黏著度與情感連結，讓人期待下一集。</v>
@@ -3061,7 +3062,7 @@
         <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E133">
-        <v>9.26</v>
+        <v>9.25</v>
       </c>
       <c r="F133" t="str">
         <v>[#801 市場震盪 17000...] 主持人以真誠且具同理心的語氣與聽眾對話，建立深厚的連結，情感溫度高，能有效提升聽眾黏著度。 | [#809  買股票還在到處問明...] 主持人與來賓的對談真誠，內容實用且具啟發性，能有效吸引聽眾持續收聽，建立黏著度。 | [#798 害怕投資賠錢？不用天...] 主持人與來賓透過分享個人經驗和真誠的對談，與聽眾建立了深厚的情感連結，讓人期待下一集的內容。</v>
@@ -3075,16 +3076,16 @@
         <v>10</v>
       </c>
       <c r="C134" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D134" t="str">
-        <v>莫菲穿搭</v>
+        <v>蕭邦</v>
       </c>
       <c r="E134">
-        <v>9.24</v>
+        <v>9.2429</v>
       </c>
       <c r="F134" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 主持人與來賓的對談真誠且富有情感溫度，內容引��入勝，讓聽眾對節目產生高度黏著度，期待未來能聽到更多類似的深度分享，具有強烈的靈魂陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 主持人透過真誠的分享和專業的分析，與聽眾建立了良好的情感連結，具有較高的黏著度。 | [莫菲穿搭02｜2026流行色配...] 主持人以專業且親切的語氣分享實用知識，內容具備高度價值，能有效提升聽眾的黏著度與學習意願。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
       </c>
     </row>
     <row r="135">
@@ -3301,10 +3302,10 @@
         <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E145">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F145" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #26.4 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #26.3 名。</v>
       </c>
     </row>
     <row r="146">
@@ -3321,10 +3322,10 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E146">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F146" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #33.5 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #33.3 名。</v>
       </c>
     </row>
     <row r="147">
@@ -3341,10 +3342,10 @@
         <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E147">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F147" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #38.1 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #38.2 名。</v>
       </c>
     </row>
     <row r="148">
@@ -3361,10 +3362,10 @@
         <v>GK爸爸</v>
       </c>
       <c r="E148">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F148" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 44 天，平均上榜排名為第 #65 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #65.7 名。</v>
       </c>
     </row>
     <row r="149">
@@ -3381,10 +3382,10 @@
         <v>文森說書</v>
       </c>
       <c r="E149">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F149" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 36 天，平均上榜排名為第 #64.6 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 37 天，平均上榜排名為第 #64.3 名。</v>
       </c>
     </row>
     <row r="150">
@@ -3404,7 +3405,7 @@
         <v>7</v>
       </c>
       <c r="F150" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
       </c>
     </row>
     <row r="151">
@@ -3424,7 +3425,7 @@
         <v>4</v>
       </c>
       <c r="F151" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
       </c>
     </row>
     <row r="152">
@@ -3444,7 +3445,7 @@
         <v>2</v>
       </c>
       <c r="F152" t="str">
-        <v>於評選區間（統計 44 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
       </c>
     </row>
     <row r="153">
@@ -3852,4 +3853,229 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F172"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="150.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>大會獎項</v>
+      </c>
+      <c r="B1" t="str">
+        <v>評選定義與細則 (AI 評審指標)</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>1. 【最佳內容架構獎】 (Best Content Structure)</v>
+      </c>
+      <c r="B2" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本分析)
+*   **評估重點**：
+    *   **開場引導**：是否能在前 2 分鐘內迅速切入重點，點出本集核心與聽眾痛點？
+    *   **段落轉折**：各段落是否有清晰的邏輯架構與過渡，而非漫無目的的散漫聊天？
+    *   **結尾總結**：主持人是否在尾聲對內容進行精闢總結或提供重點整理？
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>2. 【最佳默契獎】 (Best Chemistry &amp; Interaction)</v>
+      </c>
+      <c r="B3" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文字互動) + ♊ 軌道 B (聲音物理)
+*   **評估重點**：
+    *   **第一輪文本 (軌道 A)**：雙人或多人的接話頻率與流暢度。搭檔是給予延伸觀點、幽默吐槽，還是僅生硬回答「對、嗯、沒錯」？
+    *   **第二輪聲音 (軌道 B)**：是否有共鳴笑聲同步率？是否常出現 1.5 秒以上的尷尬無聲空白？是否頻繁惡意搶話或打斷發言？
+*   **評分級距**：1.0 - 10.0 分（單人節目請填 null）</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>3. 【最神單元企劃獎】 (Best Episode Planning)</v>
+      </c>
+      <c r="B4" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本分析)
+*   **評估重點**：
+    *   **選題創意**：議題切入角度是否具備市場差異化或新穎包裝？
+    *   **實用價值與深度**：內容是否具備清晰的實操工具、生動案例，或能啟發深度思考？
+    *   **訪談深度**（若有來賓）：問題是否具備引導性，能激發來賓分享未曾公開的精彩內容？
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>4. 【最佳男播音員獎】 (Best Male Host / Voice)</v>
+      </c>
+      <c r="B5" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (口條表達) + ♊ 軌道 B (聲音特徵)
+*   **評估重點**：
+    *   **第一輪文本 (軌道 A)**：口語表達的流暢度與贅字率（呃、然後、那、就是 的出現頻率）。
+    *   **第二輪聲音 (軌道 B)**：語速是否穩定在 180-220 字/分鐘，音量平穩無爆音噴麥，具備中低音共鳴與情感渲染力。
+*   **評分級距**：1.0 - 10.0 分（若無男主持人請填 null）</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>5. 【最佳女播音員獎】 (Best Female Host / Voice)</v>
+      </c>
+      <c r="B6" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (口條表達) + ♊ 軌道 B (聲音特徵)
+*   **評估重點**：
+    *   **第一輪文本 (軌道 A)**：口語表達的流暢度與贅字率（呃、然後、那、就是 的出現頻率）。
+    *   **第二輪聲音 (軌道 B)**：語速是否穩定在 180-220 字/分鐘，音量平穩無爆音噴麥，高音域圓潤溫暖、親和力高。
+*   **評分級距**：1.0 - 10.0 分（若無女主持人請填 null）
+---
+## 🎧 第二類：【情境與行為影響力組－Podcast 氛圍獎】
+&gt; **評選焦點：** 節目產生的聽眾行為催化、陪伴感與情感共鳴。</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>6. 【聽完馬上獎 / 不然現在獎 / 動滋動滋獎 / 推坑王獎】 (Best Action &amp; CTA)</v>
+      </c>
+      <c r="B7" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本分析)
+*   **評估重點**：
+    *   **行動呼籲 (CTA) 強度**：引導訂閱社群、追蹤電子報、或購買商品的呼籲是否自然且有力？
+    *   **生活實踐催化力**：內容是否傳遞極強的驅動力，讓聽眾聽完後「想立刻付諸行動」（如立刻去整理房間、去運動或實踐某種方法）？
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>7. 【只有你在獎 / 稀有保護動物獎 / 原來可以這樣獎 / 化腐朽為神奇獎】 (Rare Blue Ocean Guardian)</v>
+      </c>
+      <c r="B8" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本分析)
+*   **評估重點**：
+    *   **議題稀有度**：探討的話飯是否為市場極罕見、冷門，或「只有你在講」的獨特小眾藍海議題？
+    *   **論述完整度**：即使是小眾題材，內容是否維持極高完整度、論述清晰，成功保護該領域的知識火苗？
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>8. 【深夜輕輕獎 / 暖心陪伴獎 / 獎悄悄話獎】 (Best Midnight Companion)</v>
+      </c>
+      <c r="B9" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (意向分析) + ♊ 軌道 B (語調分析)
+*   **評估重點**：
+    *   **第一輪文本 (軌道 A)**：對談語意是否具備強烈安慰、安撫、陪伴與真誠特質。
+    *   **第二輪聲音 (軌道 B)**：AI 偵測音訊是否平穩溫柔，無高音爆音或情緒劇烈波動，聽感極具催眠與治癒感。
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>9. 【天亮了還在獎 (Alex都上101了你還沒講完)】 (Best Long-form Masterpiece)</v>
+      </c>
+      <c r="B10" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本結構分析)
+*   **評估重點**：
+    *   **時長門檻**：單集音檔時長是否超過 60 分鐘。
+    *   **資訊密度與流暢度**：在漫長的時間中，節目是否能維持高密度的核心價值與知識含金量，且聊天流暢、毫無冷場拖沓？
+*   **評分級距**：1.0 - 10.0 分（時長小於 60 分鐘請填 null 或低分）</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>10. 【到底有沒有獎 / 泡麵沒熟獎】 (Best Short &amp; Concise Content)</v>
+      </c>
+      <c r="B11" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本結構分析)
+*   **評估重點**：
+    *   **時長限制**：單集時長是否控制在 10-15 分鐘內（黃金極短篇）。
+    *   **精煉傳播效率**：是否能在極短時間內精準切入重點、直擊痛點、給出清晰解法，資訊提煉效率極高？
+*   **評分級距**：1.0 - 10.0 分（時長大於 15 分鐘請填 null 或低分）</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>11. 【醒醒再獎 / 激勵人心 / 起床氣消散】 (Best Morning Energy booster)</v>
+      </c>
+      <c r="B12" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (意向分析) + ♊ 軌道 B (聲音能量)
+*   **評估重點**：
+    *   **第一輪文本 (軌道 A)**：主題是否積極、正向、激勵人心，充滿早晨活力。
+    *   **第二輪聲音 (軌道 B)**：音頻節奏明快、語調高昂有朝氣、語速中偏快，通勤聽了能讓人瞬間精神百倍。
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>12. 【年度療癒獎 / 療癒 / 歡樂 / 獎廢話金牌獎】 (Ultimate Healing &amp; Relaxation)</v>
+      </c>
+      <c r="B13" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (意向分析) + ♊ 軌道 B (聲音氛圍)
+*   **評估重點**：
+    *   **第一輪文本 (軌道 A)**：談話風格是否輕鬆、幽默、高情商日常廢話，不給聽眾任何燒腦壓力。
+    *   **第二輪聲音 (軌道 B)**：氣氛歡樂、笑聲自然，能徹底安撫浮躁、卸下防備、達到深度放鬆。
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>13. 【自我探索獎】 (Best Self-Exploration)</v>
+      </c>
+      <c r="B14" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本分析)
+*   **評估重點**：
+    *   **議題深度**：對談中是否深入探討自我成長、內在探索、自我追尋與生命課題。
+    *   **心靈啟發力**：引導聽眾深度反思與內省，鼓勵獨立思考與活出個人風采的啟發性。
+*   **評分級距**：1.0 - 10.0 分</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>14. 【請你繼續獎 / 年度大獎 (我要跟老師獎)】 (Audience Choice &amp; Longevity)</v>
+      </c>
+      <c r="B15" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **評估軌道**：🪶 軌道 A (文本情感) + 📊 軌道 C (聽眾依存度)
+*   **評估重點**：
+    *   結合聽眾真實留言的依賴度（軌道 C）與 AI 判定主持人對聽眾的黏著引導力（軌道 A）。專門獎勵「Podcast 界沒有你不行」的靈魂節目。
+*   **評分級距**：1.0 - 10.0 分
+---
+## 📊 第三類：【客觀數據與市場亮點組－資源與紀律獎】
+&gt; **評選焦點：** 基於事實數據與大數據備份判定，不涉及 AI 內容主觀打分。</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>15. 【欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分】 (Social Shareability Award)</v>
+      </c>
+      <c r="B16" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **判定依據**：📊 軌道 C (社群大數據) + 🪶 軌道 A (AI 綜合評選最高分)
+*   **判定標準**：根據 Facebook、Instagram 推廣貼文的自然留言、分享與轉發熱度評估，結合 AI 評比平均總分最高者。由 Meta.AI 輔助評選出社群影響力最高之作品。</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>16. 【站著不走獎】 (Chart Longevity Champion)</v>
+      </c>
+      <c r="B17" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **判定依據**：📊 軌道 C (榜單備份)
+*   **判定標準**：依據 `daily_top100_archive.csv` 歷史統計，計算節目在評選區間內，佔據 Apple Podcasts 百大排行榜的**總天數**與**在榜率**。</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>17. 【聽眾都要跟你獎】 (Public Interaction Master)</v>
+      </c>
+      <c r="B18" t="str" xml:space="preserve">
+        <v xml:space="preserve">*   **判定依據**：📊 軌道 C (公開評論)
+*   **判定標準**：依據 Apple Podcasts API 抓取的**聽眾真實評論留言總量**與**平均星等評分**（包含僅有星等評價 rating 但無文字留言者，進行大數據排行統計）。</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Resume full evaluation with curl-based downloads
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F172"/>
+  <dimension ref="A1:F174"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E2">
-        <v>9.4545</v>
+        <v>9.45</v>
       </c>
       <c r="F2" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [EP174｜越省反而越窮？別把...] 主持人開場鋪陳完整，話題引導流暢，結尾有總結，整體架構清晰。 | [EP164｜滑短影音是在浪費時...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。</v>
@@ -462,7 +462,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E3">
-        <v>9.4046</v>
+        <v>9.4</v>
       </c>
       <c r="F3" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [《財富自由心理學》：賺錢，只是...] 節目開場鋪陳完整，話題轉折自然流暢，主持人能有效引導對談並適時拉回核心，結尾亦有精要總結，架構清晰。 | [手總是停不下來？那是焦慮在尋找...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
@@ -482,7 +482,7 @@
         <v>美股夢想家</v>
       </c>
       <c r="E4">
-        <v>9.251</v>
+        <v>9.25</v>
       </c>
       <c r="F4" t="str">
         <v>[EP289  七巨頭變七矮人！...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [EP275 股市變賭場？巴菲特...] 節目開場清晰，主題鋪陳有條理，各段落間的轉折流暢，結尾總結與行動呼籲明確，整體內容架構完整且邏輯性強。 | [EP251國防預算暴漲 5 成...] 主持人開場直接切入主題，中間分析市場數據和政策影響，邏輯清晰。雖然語速快，但內容結構完整。</v>
@@ -542,7 +542,7 @@
         <v>不敗教主-陳重銘</v>
       </c>
       <c r="E7">
-        <v>9.155</v>
+        <v>9.15</v>
       </c>
       <c r="F7" t="str">
         <v>[EP611 00998A(主動...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀分析到具體投資標的，結尾亦有精要總結，架構清晰。 | [EP628昇陽半導體(8028...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀產業趨勢到具體個股分析，結尾亦有精要總結，架構清晰。 | [EP621《富媽媽 窮媽媽》第...] 節目開場清晰，主體內容透過故事案例層層推進，邏輯嚴謹，結尾有明確的行動呼籲與總結，架構完整。</v>
@@ -562,7 +562,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E8">
-        <v>9.155</v>
+        <v>9.15</v>
       </c>
       <c r="F8" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人開場鋪陳清晰，中途提問引導流暢，能有效推進對話，結尾總結亦有深度，整體內��架構完整。 | [EP218：愛自己｜放下完美執...] 節目開場鋪陳流暢，透過個人經驗引入主題與來賓。中段內容圍繞人類圖的核心概念、案例分析與關係互動，轉折自然。結尾則聚焦於線上課程的推廣與總結，整體架構清晰，引導得宜。 | [EP219：【非典家庭CEO】...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。</v>
@@ -622,7 +622,7 @@
         <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E11">
-        <v>9.1048</v>
+        <v>9.1</v>
       </c>
       <c r="F11" t="str">
         <v>[EP.617 《無限機器》讀後...] 主持人開場鋪陳完整，中途能流暢引導話題，透過六個重點清晰地呈現書中精華，結尾亦有精要總結，內容架構清晰。 | [EP.573 從 0 到 10...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。內容邏輯清晰，層次分明。 | [EP.607 《AI Firs...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
@@ -636,16 +636,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="str">
-        <v>楊肉盧</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D12" t="str">
-        <v>楊月娥（楊肉爐）</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E12">
-        <v>9.1981</v>
+        <v>9.1931</v>
       </c>
       <c r="F12" t="str">
-        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
+        <v>[S4.EP4｜性平教育20年，...] 兩位主持人互動自然，接話流暢，笑聲同步率高，展現良好默契。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人默契極佳，對話流暢自然，能互相接話並適時加入幽默感，共同營造出引人入勝的節目氛圍。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契，接話流暢，插話頻率適中，彼此的幽默感與共鳴笑聲自然，共同營造出輕鬆愉快的對話氛圍。</v>
       </c>
     </row>
     <row r="13">
@@ -656,16 +656,16 @@
         <v>2</v>
       </c>
       <c r="C13" t="str">
-        <v>分手的99個理由</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D13" t="str">
-        <v>胡咪老師</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E13">
-        <v>9.1966</v>
+        <v>9.1931</v>
       </c>
       <c r="F13" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 兩位主持人互動自然，接話流暢，笑聲同步率高，展現良好默契。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人默契極佳，對話流暢自然，能互相接話並適時加入幽默感，共同營造出引人入勝的節目氛圍。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契，接話流暢，插話頻率適中，彼此的幽默感與共鳴笑聲自然，共同營造出輕鬆愉快的對話氛圍。</v>
+        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
       </c>
     </row>
     <row r="14">
@@ -682,7 +682,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E14">
-        <v>8.8099</v>
+        <v>8.8049</v>
       </c>
       <c r="F14" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
@@ -702,7 +702,7 @@
         <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E15">
-        <v>8.7765</v>
+        <v>8.7715</v>
       </c>
       <c r="F15" t="str">
         <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
@@ -762,7 +762,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E18">
-        <v>8.505</v>
+        <v>8.5</v>
       </c>
       <c r="F18" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 主持人與來賓之間的對話流暢自然，接話得體，沒有明顯的搶話或插話，展現了良好的互動默契。 | [【中年，正在試】把世界走成一本...] Norman和Summer的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現良好默契。</v>
@@ -770,22 +770,22 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>最神單元企劃獎</v>
+        <v>最佳默契獎</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C19" t="str">
-        <v>五吉郎</v>
+        <v>任性歐逆機智生活</v>
       </c>
       <c r="D19" t="str">
-        <v>五吉郎</v>
+        <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="E19">
-        <v>9.9545</v>
+        <v>8.25</v>
       </c>
       <c r="F19" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 選題新穎，結合個人IP變現與美業轉型，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [EP174｜越省反而越窮？別把...] 選題結合心理學與財富自由，觀點新穎且具深度，案例生動，內容含金量高。 | [EP164｜滑短影音是在浪費時...] 選題新穎且具深度，圍繞來賓新書的核心理念展開，提供了許多關於閱讀與自我成長的實用觀點與啟發，內容含金量極高。</v>
+        <v>[跟長輩一樣就能學會AI？陶韻智...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高，但偶有輕微搶話情況，整體默契良好。</v>
       </c>
     </row>
     <row r="20">
@@ -793,19 +793,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="str">
-        <v>哇賽心理學</v>
+        <v>五吉郎</v>
       </c>
       <c r="D20" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>五吉郎</v>
       </c>
       <c r="E20">
-        <v>9.9046</v>
+        <v>9.95</v>
       </c>
       <c r="F20" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 選題非常新穎且具時事性，從藥物機制到社會政策的討論深度極高，內容含金量豐富。 | [《財富自由心理學》：賺錢，只是...] 選題「財富自由心理學」新穎且具深度，透過個人故事與哲學思辨，將財富議題提升至心靈層次，內容含金量高，案例生動具啟發性。 | [手總是停不下來？那是焦慮在尋找...] 選題新穎且具深度，深入探討身體重複行為的心理學面向，案例生動且內容含金量極高。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 選題新穎，結合個人IP變現與美業轉型，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [EP174｜越省反而越窮？別把...] 選題結合心理學與財富自由，觀點新穎且具深度，案例生動，內容含金量高。 | [EP164｜滑短影音是在浪費時...] 選題新穎且具深度，圍繞來賓新書的核心理念展開，提供了許多關於閱讀與自我成長的實用觀點與啟發，內容含金量極高。</v>
       </c>
     </row>
     <row r="21">
@@ -813,19 +813,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D21" t="str">
-        <v>梁哲維</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E21">
-        <v>9.75</v>
+        <v>9.9</v>
       </c>
       <c r="F21" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目以一本關於「好感影響力」的書為引子，邀請書中提及的創業家來分享故事，選題獨特且具深度。來賓的70年滷味傳承與公益行動，提供了豐富的內容含金量和啟發性。 | [【EP302 把命盤變成行動藍...] 選題新穎，結合「九紫離火運」與AI、全球局勢、個人發展等多元面向，案例生動且內容含金量極高。 | [【EP312《超越我執的生活》...] 選題「超越我執」具備深度與啟發性，結合心理學與靈性成長，內容含金量高，案例（如內在聲音、吃飯專注）生動且具體，展現了優秀的單元企劃能力。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 選題非常新穎且具時事性，從藥物機制到社會政策的討論深度極高，內容含金量豐富。 | [《財富自由心理學》：賺錢，只是...] 選題「財富自由心理學」新穎且具深度，透過個人故事與哲學思辨，將財富議題提升至心靈層次，內容含金量高，案例生動具啟發性。 | [手總是停不下來？那是焦慮在尋找...] 選題新穎且具深度，深入探討身體重複行為的心理學面向，案例生動且內容含金量極高。</v>
       </c>
     </row>
     <row r="22">
@@ -833,19 +833,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C22" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D22" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>梁哲維</v>
       </c>
       <c r="E22">
         <v>9.75</v>
       </c>
       <c r="F22" t="str">
-        <v>[#801 市場震盪 17000...] 選題緊扣時事（股市下跌），並結合個人財務規劃與情緒管理，案例生動且內容含金量極高。 | [#809  買股票還在到處問明...] 選題「獲利加速系統」具備高度實用性與深度，結合AI工具的應用，內容含金量極高，企劃新穎。 | [#798 害怕投資賠錢？不用天...] 選題新穎且具備深度，聚焦於媽媽族群的投資教育與心態建立，內容含金量高，並透過生動的比喻（如游泳、無印良品櫃子）提升理解度。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目以一本關於「好感影響力」的書為引子，邀請書中提及的創業家來分享故事，選題獨特且具深度。來賓的70年滷味傳承與公益行動，提供了豐富的內容含金量和啟發性。 | [【EP302 把命盤變成行動藍...] 選題新穎，結合「九紫離火運」與AI、全球局勢、個人發展等多元面向，案例生動且內容含金量極高。 | [【EP312《超越我執的生活》...] 選題「超越我執」具備深度與啟發性，結合心理學與靈性成長，內容含金量高，案例（如內在聲音、吃飯專注）生動且具體，展現了優秀的單元企劃能力。</v>
       </c>
     </row>
     <row r="23">
@@ -853,19 +853,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C23" t="str">
-        <v>夢想家說股事</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D23" t="str">
-        <v>美股夢想家</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E23">
-        <v>9.6796</v>
+        <v>9.75</v>
       </c>
       <c r="F23" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 選題新穎且具時效性，深入分析了科技巨頭的市場變化與供應鏈影響，內容含金量極高。 | [EP275 股市變賭場？巴菲特...] 選題緊扣時事熱點（巴菲特、AI、台股美股），內容深度足夠，結合了宏觀經濟分析、產業趨勢與個股案例，資訊含金量高，企劃具備高度專業性。 | [EP251國防預算暴漲 5 成...] 選題結合時事（軍工股、AI、經濟預測），數據分析詳盡，提供獨到見解，內容含金量高。</v>
+        <v>[#801 市場震盪 17000...] 選題緊扣時事（股市下跌），並結合個人財務規劃與情緒管理，案例生動且內容含金量極高。 | [#809  買股票還在到處問明...] 選題「獲利加速系統」具備高度實用性與深度，結合AI工具的應用，內容含金量極高，企劃新穎。 | [#798 害怕投資賠錢？不用天...] 選題新穎且具備深度，聚焦於媽媽族群的投資教育與心態建立，內容含金量高，並透過生動的比喻（如游泳、無印良品櫃子）提升理解度。</v>
       </c>
     </row>
     <row r="24">
@@ -873,19 +873,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C24" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D24" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E24">
-        <v>9.655</v>
+        <v>9.6786</v>
       </c>
       <c r="F24" t="str">
-        <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
+        <v>[EP289  七巨頭變七矮人！...] 選題新穎且具時效性，深入分析了科技巨頭的市場變化與供應鏈影響，內容含金量極高。 | [EP275 股市變賭場？巴菲特...] 選題緊扣時事熱點（巴菲特、AI、台股美股），內容深度足夠，結合了宏觀經濟分析、產業趨勢與個股案例，資訊含金量高，企劃具備高度專業性。 | [EP251國防預算暴漲 5 成...] 選題結合時事（軍工股、AI、經濟預測），數據分析詳盡，提供獨到見解，內容含金量高。</v>
       </c>
     </row>
     <row r="25">
@@ -893,7 +893,7 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C25" t="str">
         <v>我的動齡限量版</v>
@@ -913,19 +913,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C26" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D26" t="str">
-        <v>莫菲穿搭</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E26">
         <v>9.65</v>
       </c>
       <c r="F26" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
+        <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
       </c>
     </row>
     <row r="27">
@@ -933,19 +933,19 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" t="str">
-        <v>蕭邦相談室</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D27" t="str">
-        <v>蕭邦</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E27">
         <v>9.65</v>
       </c>
       <c r="F27" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
       </c>
     </row>
     <row r="28">
@@ -953,39 +953,39 @@
         <v>最神單元企劃獎</v>
       </c>
       <c r="B28">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C28" t="str">
-        <v>下一本讀什麼？</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D28" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>蕭邦</v>
       </c>
       <c r="E28">
-        <v>9.6048</v>
+        <v>9.65</v>
       </c>
       <c r="F28" t="str">
-        <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>最佳男播音員獎</v>
+        <v>最神單元企劃獎</v>
       </c>
       <c r="B29">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C29" t="str">
-        <v>五吉郎</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D29" t="str">
-        <v>五吉郎</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E29">
-        <v>9.4545</v>
+        <v>9.6</v>
       </c>
       <c r="F29" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 男主持人聲音清晰、有活力，中低音共鳴感佳，語速穩定度高，但口頭禪「就是」和「然後」出現頻率稍高。 | [EP174｜越省反而越窮？別把...] Andy的聲音溫暖清晰，語速穩定。好哥和蔡宇哲老師的聲音也很有特色，整體男聲表現優異。 | [EP164｜滑短影音是在浪費時...] 兩位男主持人的聲音皆具備良好的中低音共鳴。主主持人Andy口條流暢，語速穩定，但偶有口頭禪；來賓好哥的聲音則更為沉穩且富有磁性，整體播音表現優異。</v>
+        <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
       </c>
     </row>
     <row r="30">
@@ -993,19 +993,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" t="str">
-        <v>哇賽心理學</v>
+        <v>五吉郎</v>
       </c>
       <c r="D30" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>五吉郎</v>
       </c>
       <c r="E30">
-        <v>9.4046</v>
+        <v>9.45</v>
       </c>
       <c r="F30" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 男來賓（蔡醫師）口條流暢，聲音專業且具說服力，解釋複雜概念清晰易懂，語速雖快但穩定。 | [《財富自由心理學》：賺錢，只是...] 兩位男主持人皆表現出色。主講人雨哲口條流暢，聲音清晰溫和，語速穩定。來賓好哥聲線低沉有磁性，論述力強。整體播音實力優異。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 男主持人聲音清晰、有活力，中低音共鳴感佳，語速穩定度高，但口頭禪「就是」和「然後」出現頻率稍高。 | [EP174｜越省反而越窮？別把...] Andy的聲音溫暖清晰，語速穩定。好哥和蔡宇哲老師的聲音也很有特色，整體男聲表現優異。 | [EP164｜滑短影音是在浪費時...] 兩位男主持人的聲音皆具備良好的中低音共鳴。主主持人Andy口條流暢，語速穩定，但偶有口頭禪；來賓好哥的聲音則更為沉穩且富有磁性，整體播音表現優異。</v>
       </c>
     </row>
     <row r="31">
@@ -1013,19 +1013,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" t="str">
-        <v>夢想家說股事</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D31" t="str">
-        <v>美股夢想家</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E31">
-        <v>9.313</v>
+        <v>9.4</v>
       </c>
       <c r="F31" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 男來賓（蔡醫師）口條流暢，聲音專業且具說服力，解釋複雜概念清晰易懂，語速雖快但穩定。 | [《財富自由心理學》：賺錢，只是...] 兩位男主持人皆表現出色。主講人雨哲口條流暢，聲音清晰溫和，語速穩定。來賓好哥聲線低沉有磁性，論述力強。整體播音實力優異。</v>
       </c>
     </row>
     <row r="32">
@@ -1033,19 +1033,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C32" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D32" t="str">
-        <v>GK爸爸</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E32">
-        <v>9.2586</v>
+        <v>9.312</v>
       </c>
       <c r="F32" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
+        <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
       </c>
     </row>
     <row r="33">
@@ -1053,19 +1053,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C33" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D33" t="str">
-        <v>梁哲維</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E33">
-        <v>9.25</v>
+        <v>9.2549</v>
       </c>
       <c r="F33" t="str">
-        <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
       </c>
     </row>
     <row r="34">
@@ -1073,19 +1073,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C34" t="str">
-        <v>蕭邦相談室</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D34" t="str">
-        <v>蕭邦</v>
+        <v>梁哲維</v>
       </c>
       <c r="E34">
-        <v>9.15</v>
+        <v>9.25</v>
       </c>
       <c r="F34" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
+        <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
       </c>
     </row>
     <row r="35">
@@ -1093,19 +1093,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B35">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C35" t="str">
-        <v>下一本讀什麼？</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D35" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>蕭邦</v>
       </c>
       <c r="E35">
-        <v>9.1048</v>
+        <v>9.15</v>
       </c>
       <c r="F35" t="str">
-        <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
+        <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
       </c>
     </row>
     <row r="36">
@@ -1113,19 +1113,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C36" t="str">
-        <v>財富餐車不打烊</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D36" t="str">
-        <v>30節約男子</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E36">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="F36" t="str">
-        <v>[【EP39】矽谷阿雅｜貸款七百...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，但口頭禪「就是」和「然後」出現頻率稍高。 | [【EP51】胡咪＆Vito大叔...] Vito大叔的口條流暢，聲音低沉有磁性，語速穩定，能有效傳達情感。偶爾的口頭禪「就是」略多但不影響整體表現。 | [【EP36】明白｜父母雙亡，獨...] 男主持人聲音厚實有共鳴，語速雖快但咬字清晰，表達流暢。口頭禪「然後」、「就是」出現頻率稍高，但整體不影響專業度。</v>
+        <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
       </c>
     </row>
     <row r="37">
@@ -1133,19 +1133,19 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B37">
+        <v>8</v>
+      </c>
+      <c r="C37" t="str">
+        <v>財富餐車不打烊</v>
+      </c>
+      <c r="D37" t="str">
+        <v>30節約男子</v>
+      </c>
+      <c r="E37">
         <v>9</v>
       </c>
-      <c r="C37" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
-      </c>
-      <c r="D37" t="str">
-        <v>人生啊！小歐</v>
-      </c>
-      <c r="E37">
-        <v>8.955</v>
-      </c>
       <c r="F37" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
+        <v>[【EP39】矽谷阿雅｜貸款七百...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，但口頭禪「就是」和「然後」出現頻率稍高。 | [【EP51】胡咪＆Vito大叔...] Vito大叔的口條流暢，聲音低沉有磁性，語速穩定，能有效傳達情感。偶爾的口頭禪「就是」略多但不影響整體表現。 | [【EP36】明白｜父母雙亡，獨...] 男主持人聲音厚實有共鳴，語速雖快但咬字清晰，表達流暢。口頭禪「然後」、「就是」出現頻率稍高，但整體不影響專業度。</v>
       </c>
     </row>
     <row r="38">
@@ -1153,39 +1153,39 @@
         <v>最佳男播音員獎</v>
       </c>
       <c r="B38">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C38" t="str">
-        <v>人類行為研究社</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D38" t="str">
-        <v>張忘形</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E38">
-        <v>8.955</v>
+        <v>8.95</v>
       </c>
       <c r="F38" t="str">
-        <v>[EP61｜為什麼越努力經營，反...] 男主持人聲音清晰、能量高，中低音共鳴感良好，語速雖快但仍能保持清晰度。情緒感染力強，但口頭禪「就是」出現頻率稍高。 | [EP50｜看到什麼都東西都想拍...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰，情感表達豐富。但口頭禪「就是」和「然後」出現頻率稍高，略影響流暢度。 | [EP65｜ 對方因為小事就對你...] 男主持人聲音厚實有共鳴，語速偏快但清晰度高，情感表達豐富。然而，「就是」和「那」等口頭禪出現頻率較高，略影響流暢度。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>最佳女播音員獎</v>
+        <v>最佳男播音員獎</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C39" t="str">
-        <v>布姐的沙發</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D39" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>張忘形</v>
       </c>
       <c r="E39">
-        <v>9.3265</v>
+        <v>8.95</v>
       </c>
       <c r="F39" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
+        <v>[EP61｜為什麼越努力經營，反...] 男主持人聲音清晰、能量高，中低音共鳴感良好，語速雖快但仍能保持清晰度。情緒感染力強，但口頭禪「就是」出現頻率稍高。 | [EP50｜看到什麼都東西都想拍...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰，情感表達豐富。但口頭禪「就是」和「然後」出現頻率稍高，略影響流暢度。 | [EP65｜ 對方因為小事就對你...] 男主持人聲音厚實有共鳴，語速偏快但清晰度高，情感表達豐富。然而，「就是」和「那」等口頭禪出現頻率較高，略影響流暢度。</v>
       </c>
     </row>
     <row r="40">
@@ -1193,19 +1193,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D40" t="str">
-        <v>莫菲穿搭</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E40">
-        <v>9.3049</v>
+        <v>9.3215</v>
       </c>
       <c r="F40" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
+        <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
       </c>
     </row>
     <row r="41">
@@ -1213,19 +1213,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C41" t="str">
-        <v>蘇心時光</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D41" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E41">
-        <v>9.2715</v>
+        <v>9.3049</v>
       </c>
       <c r="F41" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
       </c>
     </row>
     <row r="42">
@@ -1233,19 +1233,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C42" t="str">
-        <v>宋家小館</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D42" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E42">
-        <v>9.2549</v>
+        <v>9.2715</v>
       </c>
       <c r="F42" t="str">
-        <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
       </c>
     </row>
     <row r="43">
@@ -1253,19 +1253,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B43">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C43" t="str">
-        <v>說話人聲</v>
+        <v>宋家小館</v>
       </c>
       <c r="D43" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E43">
         <v>9.2549</v>
       </c>
       <c r="F43" t="str">
-        <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
+        <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
       </c>
     </row>
     <row r="44">
@@ -1273,19 +1273,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B44">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C44" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>說話人聲</v>
       </c>
       <c r="D44" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>聲音表達講師林依柔</v>
       </c>
       <c r="E44">
-        <v>9.25</v>
+        <v>9.2549</v>
       </c>
       <c r="F44" t="str">
-        <v>[#801 市場震盪 17000...] 女主持人聲音清晰、溫暖且具共鳴，語速穩定舒適，情緒感染��佳，但偶有贅字。 | [#809  買股票還在到處問明...] Cindy2聲音圓潤清晰，語速適中，語調親和，具備溫馨陪伴感，引導能力強。 | [#798 害怕投資賠錢？不用天...] 兩位女主持人聲音清晰、語速快但穩定，高音域圓潤且具備溫馨陪伴感，無刺耳爆音。主講人Sandy的語速較快，但整體表現優異。</v>
+        <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
       </c>
     </row>
     <row r="45">
@@ -1293,19 +1293,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C45" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D45" t="str">
-        <v>丁菱娟</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E45">
-        <v>9.1599</v>
+        <v>9.25</v>
       </c>
       <c r="F45" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
+        <v>[#801 市場震盪 17000...] 女主持人聲音清晰、溫暖且具共鳴，語速穩定舒適，情緒感染��佳，但偶有贅字。 | [#809  買股票還在到處問明...] Cindy2聲音圓潤清晰，語速適中，語調親和，具備溫馨陪伴感，引導能力強。 | [#798 害怕投資賠錢？不用天...] 兩位女主持人聲音清晰、語速快但穩定，高音域圓潤且具備溫馨陪伴感，無刺耳爆音。主講人Sandy的語速較快，但整體表現優異。</v>
       </c>
     </row>
     <row r="46">
@@ -1313,19 +1313,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B46">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C46" t="str">
-        <v>我的動齡限量版</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D46" t="str">
-        <v>我的動齡限量版</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E46">
         <v>9.1549</v>
       </c>
       <c r="F46" t="str">
-        <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
       </c>
     </row>
     <row r="47">
@@ -1333,19 +1333,19 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B47">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C47" t="str">
-        <v>美業幹什麼</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D47" t="str">
-        <v>美業幹什麼｜蔡佩陵</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E47">
-        <v>9.05</v>
+        <v>9.1549</v>
       </c>
       <c r="F47" t="str">
-        <v>[EP199-別再相信快速致富：...] 女主持人阿莉口條流暢，聲音清晰且富有感染力，語速雖快但穩定，高音域圓潤，具備溫馨陪伴感。 | [EP192-當貴人還沒出現時，...] 女主持人阿令的聲音明亮清晰，高音域圓潤且富有親和力，語速偏快但咬字清晰，情感表達真誠，具有良好的播音魅力。 | [EP210-會做不一定會贏｜表...] 女主持人阿林口條流暢，聲音清晰，語速穩定，高音域圓潤且具陪伴感，但偶有贅字。</v>
+        <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
       </c>
     </row>
     <row r="48">
@@ -1353,39 +1353,39 @@
         <v>最佳女播音員獎</v>
       </c>
       <c r="B48">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C48" t="str">
-        <v>尼可這樣說</v>
+        <v>美業幹什麼</v>
       </c>
       <c r="D48" t="str">
-        <v>尼可這樣說</v>
+        <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="E48">
-        <v>8.8846</v>
+        <v>9.05</v>
       </c>
       <c r="F48" t="str">
-        <v>[EP.322 流量破百萬卻賺不...] 女主持人聲音清晰、溫暖且富有感染力，語速較快但口條流暢，能有效傳達資訊與情感。 | [EP.318 行銷不是方法，是...] 女主持人聲音清晰、溫暖，語速穩定舒適，高音域圓潤，具備溫馨陪伴感，播音實力優異。 | [EP.316 與其等流量，不如...] 主講人Nico聲音清晰、語速穩定且富有活力，高音域圓潤，雖有口頭禪但整體播音品質優良。</v>
+        <v>[EP199-別再相信快速致富：...] 女主持人阿莉口條流暢，聲音清晰且富有感染力，語速雖快但穩定，高音域圓潤，具備溫馨陪伴感。 | [EP192-當貴人還沒出現時，...] 女主持人阿令的聲音明亮清晰，高音域圓潤且富有親和力，語速偏快但咬字清晰，情感表達真誠，具有良好的播音魅力。 | [EP210-會做不一定會贏｜表...] 女主持人阿林口條流暢，聲音清晰，語速穩定，高音域圓潤且具陪伴感，但偶有贅字。</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
+        <v>最佳女播音員獎</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C49" t="str">
-        <v>五吉郎</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D49" t="str">
-        <v>五吉郎</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E49">
-        <v>8.776</v>
+        <v>8.8846</v>
       </c>
       <c r="F49" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 結尾有明確呼籲聽眾行動，力道足夠，能有效催化聽眾實踐。 | [EP174｜越省反而越窮？別把...] 結尾有明確的行動呼籲，鼓勵聽眾訂閱、留言、並嘗試微小行動，力道足夠。 | [EP164｜滑短影音是在浪費時...] 節目中多次提及來賓的新書，並在結尾有明確的行動呼籲，但力道尚可加強，未達到極強的催化效果。</v>
+        <v>[EP.322 流量破百萬卻賺不...] 女主持人聲音清晰、溫暖且富有感染力，語速較快但口條流暢，能有效傳達資訊與情感。 | [EP.318 行銷不是方法，是...] 女主持人聲音清晰、溫暖，語速穩定舒適，高音域圓潤，具備溫馨陪伴感，播音實力優異。 | [EP.316 與其等流量，不如...] 主講人Nico聲音清晰、語速穩定且富有活力，高音域圓潤，雖有口頭禪但整體播音品質優良。</v>
       </c>
     </row>
     <row r="50">
@@ -1393,19 +1393,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>五吉郎</v>
       </c>
       <c r="D50" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>五吉郎</v>
       </c>
       <c r="E50">
-        <v>8.75</v>
+        <v>8.7715</v>
       </c>
       <c r="F50" t="str">
-        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 結尾有明確呼籲聽眾行動，力道足夠，能有效催化聽眾實踐。 | [EP174｜越省反而越窮？別把...] 結尾有明確的行動呼籲，鼓勵聽眾訂閱、留言、並嘗試微小行動，力道足夠。 | [EP164｜滑短影音是在浪費時...] 節目中多次提及來賓的新書，並在結尾有明確的行動呼籲，但力道尚可加強，未達到極強的催化效果。</v>
       </c>
     </row>
     <row r="51">
@@ -1413,19 +1413,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C51" t="str">
-        <v>哇賽心理學</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D51" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E51">
-        <v>8.7261</v>
+        <v>8.75</v>
       </c>
       <c r="F51" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
+        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
       </c>
     </row>
     <row r="52">
@@ -1433,19 +1433,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B52">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C52" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D52" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E52">
-        <v>8.655</v>
+        <v>8.7215</v>
       </c>
       <c r="F52" t="str">
-        <v>[EP225：【非典家庭CEO】...] 結尾有明確的行動呼籲，鼓勵聽眾點擊連結或撥打專線了解寄養家庭資訊，力道足夠且具體。 | [EP218：愛自己｜放下完美執...] 節目結尾的行動呼籲明確，針對線上課程提供了專屬優惠碼，具體且有吸引力，能有效促使聽眾採取行動。 | [EP219：【非典家庭CEO】...] 結尾有明確呼籲聽眾行動，力道足夠，鼓勵聽眾參與動物音樂會。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
       </c>
     </row>
     <row r="53">
@@ -1453,19 +1453,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C53" t="str">
-        <v>下一本讀什麼？</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D53" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E53">
-        <v>8.6048</v>
+        <v>8.65</v>
       </c>
       <c r="F53" t="str">
-        <v>[EP.617 《無限機器》讀後...] 結尾有明確呼籲聽眾訂閱電子報與節目，行動呼籲力道足夠且自然。 | [EP.573 從 0 到 10...] 結尾有明確呼籲聽眾填寫問卷和分享電子報，力道足夠且具體。 | [EP.607 《AI Firs...] 節目開頭與結尾都有明確且具說服力的行動呼籲，引導聽眾參與社群或閱讀書籍，催化力道足夠。</v>
+        <v>[EP225：【非典家庭CEO】...] 結尾有明確的行動呼籲，鼓勵聽眾點擊連結或撥打專線了解寄養家庭資訊，力道足夠且具體。 | [EP218：愛自己｜放下完美執...] 節目結尾的行動呼籲明確，針對線上課程提供了專屬優惠碼，具體且有吸引力，能有效促使聽眾採取行動。 | [EP219：【非典家庭CEO】...] 結尾有明確呼籲聽眾行動，力道足夠，鼓勵聽眾參與動物音樂會。</v>
       </c>
     </row>
     <row r="54">
@@ -1473,19 +1473,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C54" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D54" t="str">
-        <v>GK爸爸</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E54">
-        <v>8.6037</v>
+        <v>8.6</v>
       </c>
       <c r="F54" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
+        <v>[EP.617 《無限機器》讀後...] 結尾有明確呼籲聽眾訂閱電子報與節目，行動呼籲力道足夠且自然。 | [EP.573 從 0 到 10...] 結尾有明確呼籲聽眾填寫問卷和分享電子報，力道足夠且具體。 | [EP.607 《AI Firs...] 節目開頭與結尾都有明確且具說服力的行動呼籲，引導聽眾參與社群或閱讀書籍，催化力道足夠。</v>
       </c>
     </row>
     <row r="55">
@@ -1493,19 +1493,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B55">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C55" t="str">
-        <v>夢想家說股事</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D55" t="str">
-        <v>美股夢想家</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E55">
-        <v>8.5725</v>
+        <v>8.6</v>
       </c>
       <c r="F55" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 節目開頭和結尾都有明確且具吸引力的行動呼籲，鼓勵聽眾留言領取資訊或加入社群。 | [EP275 股市變賭場？巴菲特...] 節目結尾明確且多次呼籲聽眾加入社群、訂閱APP，並提供限時優惠，行動呼籲的強度與實踐催化力足夠。 | [EP251國防預算暴漲 5 成...] 節目結尾有推薦商品和下週節目預告，但行動呼籲的直接性與催化力中等。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
       </c>
     </row>
     <row r="56">
@@ -1513,19 +1513,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B56">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C56" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D56" t="str">
-        <v>梁哲維</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E56">
         <v>8.5715</v>
       </c>
       <c r="F56" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
+        <v>[EP289  七巨頭變七矮人！...] 節目開頭和結尾都有明確且具吸引力的行動呼籲，鼓勵聽眾留言領取資訊或加入社群。 | [EP275 股市變賭場？巴菲特...] 節目結尾明確且多次呼籲聽眾加入社群、訂閱APP，並提供限時優惠，行動呼籲的強度與實踐催化力足夠。 | [EP251國防預算暴漲 5 成...] 節目結尾有推薦商品和下週節目預告，但行動呼籲的直接性與催化力中等。</v>
       </c>
     </row>
     <row r="57">
@@ -1533,19 +1533,19 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B57">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C57" t="str">
-        <v>分手的99個理由</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D57" t="str">
-        <v>胡咪老師</v>
+        <v>梁哲維</v>
       </c>
       <c r="E57">
-        <v>8.5535</v>
+        <v>8.5715</v>
       </c>
       <c r="F57" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
       </c>
     </row>
     <row r="58">
@@ -1553,39 +1553,39 @@
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B58">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C58" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D58" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E58">
-        <v>8.4765</v>
+        <v>8.55</v>
       </c>
       <c r="F58" t="str">
-        <v>[EP611 00998A(主動...] 結尾有明確呼籲聽眾查詢ETF資訊並諮詢營業員，行動呼籲清晰但力道中等。 | [EP628昇陽半導體(8028...] 結尾有明確呼籲聽眾參與其課程，行動呼籲力道足夠且資訊完整。 | [EP621《富媽媽 窮媽媽》第...] 結尾明確呼籲聽眾購買書籍以獲取更多資訊，並分享節目，行動呼籲清晰且具體。</v>
+        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
+        <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
       <c r="B59">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C59" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D59" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E59">
-        <v>9.155</v>
+        <v>8.4715</v>
       </c>
       <c r="F59" t="str">
-        <v>[EP225：【非典家庭CEO】...] 寄養家庭議題雖然非絕對冷門，但節目深入探討其背後的挑戰、家庭動員與個人成長，提供了獨特的視角和豐富的細節，論述完整且具深度。 | [EP218：愛自己｜放下完美執...] 人類圖本身即為利基市場，本集更深入探討流日、閘門與關係互動等細節，論述完整且具專業度，滿足了特定聽眾群的深度需求。 | [EP219：【非典家庭CEO】...] 雖然育兒是廣泛議題，但從專業音樂家角度切入，並結合獨特的動物音樂會推廣，使其具備高度利基市場價值。</v>
+        <v>[EP611 00998A(主動...] 結尾有明確呼籲聽眾查詢ETF資訊並諮詢營業員，行動呼籲清晰但力道中等。 | [EP628昇陽半導體(8028...] 結尾有明確呼籲聽眾參與其課程，行動呼籲力道足夠且資訊完整。 | [EP621《富媽媽 窮媽媽》第...] 結尾明確呼籲聽眾購買書籍以獲取更多資訊，並分享節目，行動呼籲清晰且具體。</v>
       </c>
     </row>
     <row r="60">
@@ -1593,19 +1593,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" t="str">
-        <v>哇賽心理學</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D60" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E60">
-        <v>9.0595</v>
+        <v>9.15</v>
       </c>
       <c r="F60" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
+        <v>[EP225：【非典家庭CEO】...] 寄養家庭議題雖然非絕對冷門，但節目深入探討其背後的挑戰、家庭動員與個人成長，提供了獨特的視角和豐富的細節，論述完整且具深度。 | [EP218：愛自己｜放下完美執...] 人類圖本身即為利基市場，本集更深入探討流日、閘門與關係互動等細節，論述完整且具專業度，滿足了特定聽眾群的深度需求。 | [EP219：【非典家庭CEO】...] 雖然育兒是廣泛議題，但從專業音樂家角度切入，並結合獨特的動物音樂會推廣，使其具備高度利基市場價值。</v>
       </c>
     </row>
     <row r="61">
@@ -1613,19 +1613,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B61">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C61" t="str">
-        <v>宋家小館</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D61" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E61">
-        <v>8.9215</v>
+        <v>9.0549</v>
       </c>
       <c r="F61" t="str">
-        <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
       </c>
     </row>
     <row r="62">
@@ -1633,19 +1633,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B62">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C62" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>宋家小館</v>
       </c>
       <c r="D62" t="str">
-        <v>無所不試無樂不作</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E62">
-        <v>8.8148</v>
+        <v>8.9215</v>
       </c>
       <c r="F62" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
+        <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
       </c>
     </row>
     <row r="63">
@@ -1653,19 +1653,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C63" t="str">
-        <v>蕭邦相談室</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D63" t="str">
-        <v>蕭邦</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E63">
-        <v>8.6296</v>
+        <v>8.8098</v>
       </c>
       <c r="F63" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
       </c>
     </row>
     <row r="64">
@@ -1673,19 +1673,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B64">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C64" t="str">
-        <v>蘇心時光</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D64" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>蕭邦</v>
       </c>
       <c r="E64">
-        <v>8.6049</v>
+        <v>8.6296</v>
       </c>
       <c r="F64" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
       </c>
     </row>
     <row r="65">
@@ -1693,19 +1693,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B65">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C65" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D65" t="str">
-        <v>梁哲維</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E65">
-        <v>8.5598</v>
+        <v>8.6049</v>
       </c>
       <c r="F65" t="str">
-        <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
       </c>
     </row>
     <row r="66">
@@ -1713,19 +1713,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B66">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C66" t="str">
-        <v>分手的99個理由</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D66" t="str">
-        <v>胡咪老師</v>
+        <v>梁哲維</v>
       </c>
       <c r="E66">
-        <v>8.5331</v>
+        <v>8.5598</v>
       </c>
       <c r="F66" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 議題探討深入，特別關注數位時代下的約會暴力、男性及LGBTQ+受害者的困境，具備高度利基市場的獨特性。 | [S4.EP8｜我不想再跟你生活...] 議題聚焦於離婚後的心理歷程與微小生活習慣的影響，雖非極度冷門，但論述角度獨特且完整。 | [S4.EP14｜有些人沒有成為...] 「比前任更難忘的非前任」這一議題雖然具有普世性，但節目從心理學、文學和個人經驗等多維度進行深入探討，使其在同類節目中具備獨特的利基市場論述。</v>
+        <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
       </c>
     </row>
     <row r="67">
@@ -1733,19 +1733,19 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B67">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C67" t="str">
-        <v>教出你的路</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D67" t="str">
-        <v>治療師瑪奇</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E67">
-        <v>8.5265</v>
+        <v>8.5296</v>
       </c>
       <c r="F67" t="str">
-        <v>[EP47 有團隊的感覺如何？教...] 解剖學結合運動教學是一個相對利基的市場，主持人以獨特視角切入，論述完整且具深度，不易被取代。 | [EP31 為了愛移民，她打造 ...] 以植物性飲食為核心，並強調非卡路里導向的理念，在健康飲食領域中具備獨特的利基市場視角。 | [EP35 為什麼堅持開「解剖學...] 「應用解剖運動學」是一個相對專業且具利基性的市場，主持人對此議題的論述深入且完整，有效觸及目標受眾的需求。</v>
+        <v>[S4.EP4｜性平教育20年，...] 議題探討深入，特別關注數位時代下的約會暴力、男性及LGBTQ+受害者的困境，具備高度利基市場的獨特性。 | [S4.EP8｜我不想再跟你生活...] 議題聚焦於離婚後的心理歷程與微小生活習慣的影響，雖非極度冷門，但論述角度獨特且完整。 | [S4.EP14｜有些人沒有成為...] 「比前任更難忘的非前任」這一議題雖然具有普世性，但節目從心理學、文學和個人經驗等多維度進行深入探討，使其在同類節目中具備獨特的利基市場論述。</v>
       </c>
     </row>
     <row r="68">
@@ -1753,39 +1753,39 @@
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B68">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C68" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>教出你的路</v>
       </c>
       <c r="D68" t="str">
-        <v>丁菱娟</v>
+        <v>治療師瑪奇</v>
       </c>
       <c r="E68">
-        <v>8.505</v>
+        <v>8.5215</v>
       </c>
       <c r="F68" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 議題聚焦台灣科技產業的供應鏈與產業分析，雖非極度冷門，但論述深度與專業性使其在利基市場中表現突出。 | [ep11. Z世代難搞嗎？用對...] Z世代議題雖非極度冷門，但節目從職場管理、品牌行銷等多維度深入剖析，並結合實務經驗，提供了獨特的觀點與論述，使其在同類議題中具備差異化。 | [ep23. 主動出擊的力量有多...] 議題雖非極度冷門，但以「搭訕」為切入點，並將其應用於廣泛的生活層面，論述獨特且完整。</v>
+        <v>[EP47 有團隊的感覺如何？教...] 解剖學結合運動教學是一個相對利基的市場，主持人以獨特視角切入，論述完整且具深度，不易被取代。 | [EP31 為了愛移民，她打造 ...] 以植物性飲食為核心，並強調非卡路里導向的理念，在健康飲食領域中具備獨特的利基市場視角。 | [EP35 為什麼堅持開「解剖學...] 「應用解剖運動學」是一個相對專業且具利基性的市場，主持人對此議題的論述深入且完整，有效觸及目標受眾的需求。</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
+        <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
       <c r="B69">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C69" t="str">
-        <v>蘇心時光</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D69" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E69">
-        <v>9.2715</v>
+        <v>8.5</v>
       </c>
       <c r="F69" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 議題聚焦台灣科技產業的供應鏈與產業分析，雖非極度冷門，但論述深度與專業性使其在利基市場中表現突出。 | [ep11. Z世代難搞嗎？用對...] Z世代議題雖非極度冷門，但節目從職場管理、品牌行銷等多維度深入剖析，並結合實務經驗，提供了獨特的觀點與論述，使其在同類議題中具備差異化。 | [ep23. 主動出擊的力量有多...] 議題雖非極度冷門，但以「搭訕」為切入點，並將其應用於廣泛的生活層面，論述獨特且完整。</v>
       </c>
     </row>
     <row r="70">
@@ -1793,19 +1793,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70" t="str">
-        <v>分手的99個理由</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D70" t="str">
-        <v>胡咪老師</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E70">
-        <v>9.0535</v>
+        <v>9.2715</v>
       </c>
       <c r="F70" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
       </c>
     </row>
     <row r="71">
@@ -1813,19 +1813,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D71" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E71">
-        <v>8.9765</v>
+        <v>9.05</v>
       </c>
       <c r="F71" t="str">
-        <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
+        <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
       </c>
     </row>
     <row r="72">
@@ -1833,19 +1833,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C72" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D72" t="str">
-        <v>GK爸爸</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E72">
-        <v>8.9252</v>
+        <v>8.9715</v>
       </c>
       <c r="F72" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
+        <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
       </c>
     </row>
     <row r="73">
@@ -1853,19 +1853,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B73">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C73" t="str">
-        <v>宋家小館</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D73" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E73">
-        <v>8.9022</v>
+        <v>8.9215</v>
       </c>
       <c r="F73" t="str">
-        <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="74">
@@ -1873,19 +1873,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B74">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C74" t="str">
-        <v>布姐的沙發</v>
+        <v>宋家小館</v>
       </c>
       <c r="D74" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E74">
-        <v>8.8265</v>
+        <v>8.9022</v>
       </c>
       <c r="F74" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
+        <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
       </c>
     </row>
     <row r="75">
@@ -1893,19 +1893,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C75" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D75" t="str">
-        <v>無所不試無樂不作</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E75">
-        <v>8.8265</v>
+        <v>8.8215</v>
       </c>
       <c r="F75" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
+        <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
       </c>
     </row>
     <row r="76">
@@ -1913,19 +1913,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B76">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C76" t="str">
-        <v>下半場人生陪談師</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D76" t="str">
-        <v>下半場人生事務有限公司</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E76">
-        <v>8.8098</v>
+        <v>8.8215</v>
       </c>
       <c r="F76" t="str">
-        <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="77">
@@ -1933,19 +1933,19 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B77">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C77" t="str">
-        <v>五吉郎</v>
+        <v>下半場人生陪談師</v>
       </c>
       <c r="D77" t="str">
-        <v>五吉郎</v>
+        <v>下半場人生事務有限公司</v>
       </c>
       <c r="E77">
-        <v>8.776</v>
+        <v>8.8098</v>
       </c>
       <c r="F77" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 整體語調平穩溫和，適合深夜靜聽，但部分討論較為熱情，略有起伏。 | [EP174｜越省反而越窮？別把...] 聲音平穩，語調溫和，適合深夜聆聽，無突兀尖銳音。 | [EP164｜滑短影音是在浪費時...] 節目氛圍沉穩且具思考性，兩位主持人的語調平穩溫和，適合聽眾在夜晚靜心聆聽與反思，無突兀尖銳音效。</v>
+        <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
       </c>
     </row>
     <row r="78">
@@ -1953,39 +1953,39 @@
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B78">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C78" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>五吉郎</v>
       </c>
       <c r="D78" t="str">
-        <v>梁哲維</v>
+        <v>五吉郎</v>
       </c>
       <c r="E78">
-        <v>8.75</v>
+        <v>8.7715</v>
       </c>
       <c r="F78" t="str">
-        <v>[【EP330 帶著善意行動，最...] 聲音平穩溫和，談話內容有深度，適合深夜靜聽與思考。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的語調溫和穩定，聲音品質優良，適合在深夜時段放鬆聆聽，具有陪伴治癒感。 | [【EP312《超越我執的生活》...] 主持人語調溫和穩定，聲音沉穩，內容具備深度思考，無突兀尖銳爆音，非常適合深夜聆聽，能帶來陪伴與沉靜感。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 整體語調平穩溫和，適合深夜靜聽，但部分討論較為熱情，略有起伏。 | [EP174｜越省反而越窮？別把...] 聲音平穩，語調溫和，適合深夜聆聽，無突兀尖銳音。 | [EP164｜滑短影音是在浪費時...] 節目氛圍沉穩且具思考性，兩位主持人的語調平穩溫和，適合聽眾在夜晚靜心聆聽與反思，無突兀尖銳音效。</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
+        <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
       <c r="B79">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C79" t="str">
-        <v>夢想家說股事</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D79" t="str">
-        <v>美股夢想家</v>
+        <v>梁哲維</v>
       </c>
       <c r="E79">
-        <v>9.251</v>
+        <v>8.75</v>
       </c>
       <c r="F79" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 節目節奏明快，主持人語調充滿朝氣，內容資訊量大，非常適合通勤時提神醒腦。 | [EP275 股市變賭場？巴菲特...] 節目節奏明快，主講人語調充滿活力且資訊量豐富，非常適合通勤或早晨時段收聽，有助於提神醒腦並快速掌握市場動態。 | [EP251國防預算暴漲 5 成...] 節奏明快，語調朝氣蓬勃，資訊密度高，非常適合通勤時提神醒腦。</v>
+        <v>[【EP330 帶著善意行動，最...] 聲音平穩溫和，談話內容有深度，適合深夜靜聽與思考。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的語調溫和穩定，聲音品質優良，適合在深夜時段放鬆聆聽，具有陪伴治癒感。 | [【EP312《超越我執的生活》...] 主持人語調溫和穩定，聲音沉穩，內容具備深度思考，無突兀尖銳爆音，非常適合深夜聆聽，能帶來陪伴與沉靜感。</v>
       </c>
     </row>
     <row r="80">
@@ -1993,19 +1993,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B80">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C80" t="str">
-        <v>五吉郎</v>
+        <v>夢想家說股事</v>
       </c>
       <c r="D80" t="str">
-        <v>五吉郎</v>
+        <v>美股夢想家</v>
       </c>
       <c r="E80">
-        <v>9.1094</v>
+        <v>9.25</v>
       </c>
       <c r="F80" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
+        <v>[EP289  七巨頭變七矮人！...] 節目節奏明快，主持人語調充滿朝氣，內容資訊量大，非常適合通勤時提神醒腦。 | [EP275 股市變賭場？巴菲特...] 節目節奏明快，主講人語調充滿活力且資訊量豐富，非常適合通勤或早晨時段收聽，有助於提神醒腦並快速掌握市場動態。 | [EP251國防預算暴漲 5 成...] 節奏明快，語調朝氣蓬勃，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="81">
@@ -2013,19 +2013,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B81">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C81" t="str">
-        <v>下一本讀什麼？</v>
+        <v>五吉郎</v>
       </c>
       <c r="D81" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>五吉郎</v>
       </c>
       <c r="E81">
-        <v>9.1048</v>
+        <v>9.1049</v>
       </c>
       <c r="F81" t="str">
-        <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
       </c>
     </row>
     <row r="82">
@@ -2033,19 +2033,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B82">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C82" t="str">
-        <v>郝聲音</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D82" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E82">
-        <v>9.0543</v>
+        <v>9.1</v>
       </c>
       <c r="F82" t="str">
-        <v>[郝聲音：（下） 莊鈞涵（Car...] 節奏明快，主持人與來賓充滿朝氣，內容實用且具激勵性，適合通勤時提神醒腦。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目節奏明快，開頭活力十足，內容實用且具啟發性，適合通勤時提神醒腦與獲取新知。 | [郝聲音：成為人生更自由的「精銳...] 節奏明快，語調朝氣蓬勃，內容具啟發性，非常適合通勤時提神醒腦。</v>
+        <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="83">
@@ -2053,19 +2053,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B83">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C83" t="str">
-        <v>哇賽心理學</v>
+        <v>郝聲音</v>
       </c>
       <c r="D83" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E83">
-        <v>9.0477</v>
+        <v>9.05</v>
       </c>
       <c r="F83" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
+        <v>[郝聲音：（下） 莊鈞涵（Car...] 節奏明快，主持人與來賓充滿朝氣，內容實用且具激勵性，適合通勤時提神醒腦。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目節奏明快，開頭活力十足，內容實用且具啟發性，適合通勤時提神醒腦與獲取新知。 | [郝聲音：成為人生更自由的「精銳...] 節奏明快，語調朝氣蓬勃，內容具啟發性，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="84">
@@ -2073,19 +2073,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B84">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C84" t="str">
-        <v>我的動齡限量版</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D84" t="str">
-        <v>我的動齡限量版</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E84">
-        <v>9</v>
+        <v>9.0431</v>
       </c>
       <c r="F84" t="str">
-        <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
       </c>
     </row>
     <row r="85">
@@ -2093,19 +2093,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B85">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C85" t="str">
-        <v>能量黑客</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D85" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E85">
         <v>9</v>
       </c>
       <c r="F85" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
+        <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="86">
@@ -2113,19 +2113,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B86">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C86" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>能量黑客</v>
       </c>
       <c r="D86" t="str">
-        <v>丁菱娟</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E86">
-        <v>8.9846</v>
+        <v>9</v>
       </c>
       <c r="F86" t="str">
-        <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
       </c>
     </row>
     <row r="87">
@@ -2133,19 +2133,19 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B87">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C87" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>丁菱娟的邊走邊想</v>
       </c>
       <c r="D87" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>丁菱娟</v>
       </c>
       <c r="E87">
-        <v>8.9765</v>
+        <v>8.9796</v>
       </c>
       <c r="F87" t="str">
-        <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
+        <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
       </c>
     </row>
     <row r="88">
@@ -2153,39 +2153,39 @@
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B88">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C88" t="str">
-        <v>閱讀聊樂KEY</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D88" t="str">
-        <v>閱讀聊樂key</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E88">
         <v>8.9715</v>
       </c>
       <c r="F88" t="str">
-        <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
+        <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
+        <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
       <c r="B89">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C89" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>閱讀聊樂KEY</v>
       </c>
       <c r="D89" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>閱讀聊樂key</v>
       </c>
       <c r="E89">
-        <v>8.6346</v>
+        <v>8.9715</v>
       </c>
       <c r="F89" t="str">
-        <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
+        <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
       </c>
     </row>
     <row r="90">
@@ -2193,19 +2193,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C90" t="str">
-        <v>分手的99個理由</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D90" t="str">
-        <v>胡咪老師</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E90">
-        <v>8.3557</v>
+        <v>8.6296</v>
       </c>
       <c r="F90" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
+        <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
       </c>
     </row>
     <row r="91">
@@ -2213,19 +2213,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B91">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C91" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D91" t="str">
-        <v>GK爸爸</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E91">
-        <v>8.2468</v>
+        <v>8.3522</v>
       </c>
       <c r="F91" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
+        <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
       </c>
     </row>
     <row r="92">
@@ -2233,19 +2233,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B92">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C92" t="str">
-        <v>五吉郎</v>
+        <v>聰明生活投資學</v>
       </c>
       <c r="D92" t="str">
-        <v>五吉郎</v>
+        <v>聰明主婦的生活投資學</v>
       </c>
       <c r="E92">
-        <v>8.1094</v>
+        <v>8.3375</v>
       </c>
       <c r="F92" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
+        <v>[EP84. 愛與勇氣，威宇老師...] 節目對談真誠，來賓分享的生命故事具有療癒力量，主持人也展現了同理心，能帶來情感上的釋放。 | [EP 91. 越放鬆、越豐盛！...] 節目探討自我接納、放下恐懼與信任等主題，對話真誠且富有啟發性，能帶來心靈上的慰藉與療癒感。</v>
       </c>
     </row>
     <row r="93">
@@ -2253,19 +2253,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B93">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C93" t="str">
-        <v>蘇心時光</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D93" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E93">
-        <v>8.0742</v>
+        <v>8.2431</v>
       </c>
       <c r="F93" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
       </c>
     </row>
     <row r="94">
@@ -2273,19 +2273,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B94">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C94" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>五吉郎</v>
       </c>
       <c r="D94" t="str">
-        <v>梁哲維</v>
+        <v>五吉郎</v>
       </c>
       <c r="E94">
-        <v>8.0598</v>
+        <v>8.1049</v>
       </c>
       <c r="F94" t="str">
-        <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
       </c>
     </row>
     <row r="95">
@@ -2293,19 +2293,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B95">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C95" t="str">
-        <v>布姐的沙發</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D95" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E95">
-        <v>7.9846</v>
+        <v>8.0742</v>
       </c>
       <c r="F95" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
       </c>
     </row>
     <row r="96">
@@ -2313,19 +2313,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B96">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C96" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D96" t="str">
-        <v>無所不試無樂不作</v>
+        <v>梁哲維</v>
       </c>
       <c r="E96">
-        <v>7.9696</v>
+        <v>8.0598</v>
       </c>
       <c r="F96" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
+        <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
       </c>
     </row>
     <row r="97">
@@ -2333,19 +2333,19 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B97">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C97" t="str">
-        <v>【莫轉台】-試穿新人生</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D97" t="str">
-        <v>莫菲穿搭</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E97">
-        <v>7.9598</v>
+        <v>7.9796</v>
       </c>
       <c r="F97" t="str">
-        <v>[莫菲穿搭20｜球具只是通行證？...] 對談風格輕鬆歡樂，主持人與來賓之間的幽默互動和生活化分享（如吃茶葉蛋、羊肉爐、生魚片）帶來解壓感，笑聲自然，營造出愉悅的氛圍。 | [莫菲穿搭27｜金曲幕後直擊！電...] 節目內容偏向專業分析與個人觀點分享，輕鬆歡樂的療癒感相對較低。 | [莫菲穿搭02｜2026流行色配...] 談話風格較為嚴肅認真，以知識分享為主，解壓療癒感普通，較少輕鬆歡樂的對話。</v>
+        <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
       </c>
     </row>
     <row r="98">
@@ -2353,39 +2353,39 @@
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B98">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C98" t="str">
-        <v>蕭邦相談室</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D98" t="str">
-        <v>蕭邦</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E98">
-        <v>7.9598</v>
+        <v>7.9646</v>
       </c>
       <c r="F98" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 談話風格偏向認真探討，而非輕鬆歡樂的療癒感。 | [【蕭邦出任務】如何選擇適合自己...] 談話風格較為深入與嚴肅，著重於職涯挑戰與個人成長，因此日常廢話解壓感和療癒感相對較低。 | [幸福的人，通常「覺察力」都很強...] 談話風格真誠且具啟發性，能引導聽眾自我療癒與成長，但較少輕鬆歡樂的廢話解壓感。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>自我探索獎</v>
+        <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
       <c r="B99">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C99" t="str">
-        <v>五吉郎</v>
+        <v>【莫轉台】-試穿新人生</v>
       </c>
       <c r="D99" t="str">
-        <v>五吉郎</v>
+        <v>莫菲穿搭</v>
       </c>
       <c r="E99">
-        <v>9.9545</v>
+        <v>7.9598</v>
       </c>
       <c r="F99" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 深度探討自由人生、自我成長、內在探索與心靈啟發，從個人經歷中提煉出普世價值，啟發性極強。 | [EP174｜越省反而越窮？別把...] 深度探討金錢觀、人生目的與自我成長，對聽眾的內在探索有很強的啟發。 | [EP164｜滑短影音是在浪費時...] 節目深度探討了閱讀如何影響個人成長、思維模式的轉變以及如何找回自我可能性，提供了豐富的內在探索與心靈啟發內容。</v>
+        <v>[莫菲穿搭20｜球具只是通行證？...] 對談風格輕鬆歡樂，主持人與來賓之間的幽默互動和生活化分享（如吃茶葉蛋、羊肉爐、生魚片）帶來解壓感，笑聲自然，營造出愉悅的氛圍。 | [莫菲穿搭27｜金曲幕後直擊！電...] 節目內容偏向專業分析與個人觀點分享，輕鬆歡樂的療癒感相對較低。 | [莫菲穿搭02｜2026流行色配...] 談話風格較為嚴肅認真，以知識分享為主，解壓療癒感普通，較少輕鬆歡樂的對話。</v>
       </c>
     </row>
     <row r="100">
@@ -2393,19 +2393,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B100">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C100" t="str">
-        <v>蘇心時光</v>
+        <v>五吉郎</v>
       </c>
       <c r="D100" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>五吉郎</v>
       </c>
       <c r="E100">
         <v>9.95</v>
       </c>
       <c r="F100" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 深度探討自由人生、自我成長、內在探索與心靈啟發，從個人經歷中提煉出普世價值，啟發性極強。 | [EP174｜越省反而越窮？別把...] 深度探討金錢觀、人生目的與自我成長，對聽眾的內在探索有很強的啟發。 | [EP164｜滑短影音是在浪費時...] 節目深度探討了閱讀如何影響個人成長、思維模式的轉變以及如何找回自我可能性，提供了豐富的內在探索與心靈啟發內容。</v>
       </c>
     </row>
     <row r="101">
@@ -2413,19 +2413,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B101">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C101" t="str">
-        <v>哇賽心理學</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D101" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E101">
-        <v>9.8842</v>
+        <v>9.95</v>
       </c>
       <c r="F101" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
       </c>
     </row>
     <row r="102">
@@ -2433,19 +2433,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B102">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C102" t="str">
-        <v>布姐的沙發</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D102" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E102">
-        <v>9.8265</v>
+        <v>9.8796</v>
       </c>
       <c r="F102" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 節目深度探討了自我成長、內在價值觀與目的性創業，來賓對自信的定義也提供了深刻的心靈啟發。 | [EP433｜【中年轉型】從矽谷...] 深度探討個人職涯轉型、自我覺察與性格探索，提供豐富的心靈啟發與成長觀點，是本集的核心亮點。 | [EP466｜拒絕被朝九晚五綁架...] 本集節目核心圍繞著自我成長、內在探索與心靈啟發。來賓透過「百工計畫」的實踐，深入剖析了個人與社會的關係，以及如何找到內在平衡，啟發性極強。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
       </c>
     </row>
     <row r="103">
@@ -2453,19 +2453,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B103">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C103" t="str">
-        <v>蕭邦相談室</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D103" t="str">
-        <v>蕭邦</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E103">
-        <v>9.8049</v>
+        <v>9.8215</v>
       </c>
       <c r="F103" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 深度探討自我成長、內在探索與心靈啟發，主持人分享個人轉變歷程，極具啟發性。 | [【蕭邦出任務】如何選擇適合自己...] 來賓的職涯轉型故事與主持人對自我價值的探討，提供了深刻的內在探索與心靈啟發，深度極高。 | [幸福的人，通常「覺察力」都很強...] 深度探討情緒的來源、自我批判的迴圈以及如何透過覺察進行自我調整，對內在探索與心靈啟發的深度極高。</v>
+        <v>[EP470｜把人放在心上的共贏...] 節目深度探討了自我成長、內在價值觀與目的性創業，來賓對自信的定義也提供了深刻的心靈啟發。 | [EP433｜【中年轉型】從矽谷...] 深度探討個人職涯轉型、自我覺察與性格探索，提供豐富的心靈啟發與成長觀點，是本集的核心亮點。 | [EP466｜拒絕被朝九晚五綁架...] 本集節目核心圍繞著自我成長、內在探索與心靈啟發。來賓透過「百工計畫」的實踐，深入剖析了個人與社會的關係，以及如何找到內在平衡，啟發性極強。</v>
       </c>
     </row>
     <row r="104">
@@ -2473,19 +2473,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B104">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C104" t="str">
-        <v>人類行為研究社</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D104" t="str">
-        <v>張忘形</v>
+        <v>蕭邦</v>
       </c>
       <c r="E104">
-        <v>9.7765</v>
+        <v>9.8049</v>
       </c>
       <c r="F104" t="str">
-        <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 深度探討自我成長、內在探索與心靈啟發，主持人分享個人轉變歷程，極具啟發性。 | [【蕭邦出任務】如何選擇適合自己...] 來賓的職涯轉型故事與主持人對自我價值的探討，提供了深刻的內在探索與心靈啟發，深度極高。 | [幸福的人，通常「覺察力」都很強...] 深度探討情緒的來源、自我批判的迴圈以及如何透過覺察進行自我調整，對內在探索與心靈啟發的深度極高。</v>
       </c>
     </row>
     <row r="105">
@@ -2493,19 +2493,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B105">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C105" t="str">
-        <v>下一本讀什麼？</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D105" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>張忘形</v>
       </c>
       <c r="E105">
-        <v>9.7597</v>
+        <v>9.7715</v>
       </c>
       <c r="F105" t="str">
-        <v>[EP.617 《無限機器》讀後...] 節目深度探討了個人使命感、價值觀與對未來的思考，引導聽眾進行自我成長與內在探索���心靈啟發感極強。 | [EP.573 從 0 到 10...] 深度探討個人成長、心態轉變、面對困難的韌性，以及如何從內在尋找動力，心靈啟發感極強。 | [EP.607 《AI Firs...] 節目核心圍繞個人在AI時代的自我成長、能力提升與心態轉變，提供了深刻的內在探索與心靈啟發。</v>
+        <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
       </c>
     </row>
     <row r="106">
@@ -2513,19 +2513,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B106">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C106" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D106" t="str">
-        <v>梁哲維</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E106">
-        <v>9.75</v>
+        <v>9.7549</v>
       </c>
       <c r="F106" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目深度探討了創業者的初心、傳承的意義以及善意帶來的回饋，對聽眾的自我成長和內在探索有很強的啟發。 | [【EP302 把命盤變成行動藍...] 節目核心圍繞著個人命運、自我認知與未來規劃，深度啟發聽眾進行內在探索與自我成長，極具價值。 | [【EP312《超越我執的生活》...] 本集內容核心即為自我成長與內在探索，透過對「我執」的剖析和「臨在��的實踐，提供了深刻的心靈啟發，高度符合此獎項的評估維度。</v>
+        <v>[EP.617 《無限機器》讀後...] 節目深度探討了個人使命感、價值觀與對未來的思考，引導聽眾進行自我成長與內在探索���心靈啟發感極強。 | [EP.573 從 0 到 10...] 深度探討個人成長、心態轉變、面對困難的韌性，以及如何從內在尋找動力，心靈啟發感極強。 | [EP.607 《AI Firs...] 節目核心圍繞個人在AI時代的自我成長、能力提升與心態轉變，提供了深刻的內在探索與心靈啟發。</v>
       </c>
     </row>
     <row r="107">
@@ -2533,19 +2533,19 @@
         <v>自我探索獎</v>
       </c>
       <c r="B107">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C107" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D107" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>梁哲維</v>
       </c>
       <c r="E107">
         <v>9.75</v>
       </c>
       <c r="F107" t="str">
-        <v>[#801 市場震盪 17000...] 深度探討了投資中的心理層面、個人風險承受度與長期目標設定，對聽眾的自我成長與內在探索有很強的啟發性。 | [#809  買股票還在到處問明...] 節目不僅談投資，更強調學習、成長和建立系統思維，對自我探索和心靈啟發有深度，鼓勵聽眾提升自我。 | [#798 害怕投資賠錢？不用天...] 深度探討投資與個人生活目標的連結，鼓勵聽眾進行自我反思，建立符合自身價值觀的財務規劃，心靈啟發感極強。</v>
+        <v>[【EP330 帶著善意行動，最...] 節目深度探討了創業者的初心、傳承的意義以及善意帶來的回饋，對聽眾的自我成長和內在探索有很強的啟發。 | [【EP302 把命盤變成行動藍...] 節目核心圍繞著個人命運、自我認知與未來規劃，深度啟發聽眾進行內在探索與自我成長，極具價值。 | [【EP312《超越我執的生活》...] 本集內容核心即為自我成長與內在探索，透過對「我執」的剖析和「臨在��的實踐，提供了深刻的心靈啟發，高度符合此獎項的評估維度。</v>
       </c>
     </row>
     <row r="108">
@@ -2553,39 +2553,39 @@
         <v>自我探索獎</v>
       </c>
       <c r="B108">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C108" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D108" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E108">
-        <v>9.655</v>
+        <v>9.75</v>
       </c>
       <c r="F108" t="str">
-        <v>[EP225：【非典家庭CEO】...] 節目深度探討了個人在面對生命挑戰時的內在轉變、成長與自我超越，特別是保會媽媽從「後悔」到「互相陪伴」的心路歷程，極具心靈啟發深度。 | [EP218：愛自己｜放下完美執...] 人類圖的核心價值即是自我探索與成長。本集透過解析個人特質、關係模式及流日影響，提供了豐富的工具與視角，深刻啟發聽眾認識自我、理解他人，並引導心靈成長。 | [EP219：【非典家庭CEO】...] 深度探討育兒過程中的自我成長、內在探索與心靈啟發，提供豐富的思考面向。</v>
+        <v>[#801 市場震盪 17000...] 深度探討了投資中的心理層面、個人風險承受度與長期目標設定，對聽眾的自我成長與內在探索有很強的啟發性。 | [#809  買股票還在到處問明...] 節目不僅談投資，更強調學習、成長和建立系統思維，對自我探索和心靈啟發有深度，鼓勵聽眾提升自我。 | [#798 害怕投資賠錢？不用天...] 深度探討投資與個人生活目標的連結，鼓勵聽眾進行自我反思，建立符合自身價值觀的財務規劃，心靈啟發感極強。</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
+        <v>自我探索獎</v>
       </c>
       <c r="B109">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C109" t="str">
-        <v>說話人聲</v>
+        <v>下半場人生陪談師</v>
       </c>
       <c r="D109" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>下半場人生事務有限公司</v>
       </c>
       <c r="E109">
-        <v>10</v>
+        <v>9.6549</v>
       </c>
       <c r="F109" t="str">
-        <v>[EP.59｜【說話人聲-會客室...] 單集時長接近4小時，內容資訊密度極高，且能持續保持聽眾的專注與興趣，無明顯冷場，是優秀的長篇內容��</v>
+        <v>[44-解開品牌人生的迷思，從認...] 節目核心圍繞自我成長、內在探索與心靈啟發，深度探討個人價值觀與人生方向，啟發性極強。 | [57-慢活的幸福人生 – 台灣...] 節目深度探討了個人成長、內在探索與心靈啟發，鼓勵聽眾透過慢活理念重新認識自我與世界，具備極高的自我探索價值。 | [59-人生下半場，人際好感怎麽...] 節目核心主題圍繞自我成長、內在探索與心靈啟發，深度極高，能有效引導聽眾反思自身。</v>
       </c>
     </row>
     <row r="110">
@@ -2593,19 +2593,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B110">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C110" t="str">
-        <v>郝聲音</v>
+        <v>說話人聲</v>
       </c>
       <c r="D110" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>聲音表達講師林依柔</v>
       </c>
       <c r="E110">
-        <v>9.5543</v>
+        <v>10</v>
       </c>
       <c r="F110" t="str">
-        <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
+        <v>[EP.59｜【說話人聲-會客室...] 單集時長接近4小時，內容資訊密度極高，且能持續保持聽眾的專注與興趣，無明顯冷場，是優秀的長篇內容��</v>
       </c>
     </row>
     <row r="111">
@@ -2613,19 +2613,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B111">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C111" t="str">
-        <v>哇賽心理學</v>
+        <v>郝聲音</v>
       </c>
       <c r="D111" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E111">
-        <v>9.4046</v>
+        <v>9.55</v>
       </c>
       <c r="F111" t="str">
-        <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
+        <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
       </c>
     </row>
     <row r="112">
@@ -2633,19 +2633,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B112">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C112" t="str">
-        <v>航海王的富人學</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D112" t="str">
-        <v>美股航海王</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E112">
-        <v>9.3547</v>
+        <v>9.4</v>
       </c>
       <c r="F112" t="str">
-        <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
+        <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
       </c>
     </row>
     <row r="113">
@@ -2653,19 +2653,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B113">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C113" t="str">
-        <v>FIRE 人生大學</v>
+        <v>航海王的富人學</v>
       </c>
       <c r="D113" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>美股航海王</v>
       </c>
       <c r="E113">
-        <v>9.3048</v>
+        <v>9.35</v>
       </c>
       <c r="F113" t="str">
-        <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
+        <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
       </c>
     </row>
     <row r="114">
@@ -2673,19 +2673,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B114">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C114" t="str">
-        <v>粉紅地獄辛辣麵</v>
+        <v>FIRE 人生大學</v>
       </c>
       <c r="D114" t="str">
-        <v>Vito大叔</v>
+        <v>Fire人生大學｜道哥</v>
       </c>
       <c r="E114">
-        <v>8.9</v>
+        <v>9.3</v>
       </c>
       <c r="F114" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] 本集時長超過2小時，屬於長篇內容。節目在這麼長的時間內，資訊密度依然很高，對談流暢且引人入勝，沒有明顯的冷場，能讓聽眾持續投入。這展現了節目在長篇內容規劃與執行上的功力。</v>
+        <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
       </c>
     </row>
     <row r="115">
@@ -2693,19 +2693,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B115">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C115" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>粉紅地獄辛辣麵</v>
       </c>
       <c r="D115" t="str">
-        <v>梁哲維</v>
+        <v>Vito大叔</v>
       </c>
       <c r="E115">
-        <v>8.75</v>
+        <v>8.9</v>
       </c>
       <c r="F115" t="str">
-        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
+        <v>[S6EP30. 我到日本當漁夫...] 本集時長超過2小時，屬於長篇內容。節目在這麼長的時間內，資訊密度依然很高，對談流暢且引人入勝，沒有明顯的冷場，能讓聽眾持續投入。這展現了節目在長篇內容規劃與執行上的功力。</v>
       </c>
     </row>
     <row r="116">
@@ -2713,19 +2713,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B116">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C116" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D116" t="str">
-        <v>人生啊！小歐</v>
+        <v>梁哲維</v>
       </c>
       <c r="E116">
-        <v>8.6925</v>
+        <v>8.75</v>
       </c>
       <c r="F116" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
+        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
       </c>
     </row>
     <row r="117">
@@ -2733,19 +2733,19 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B117">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C117" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D117" t="str">
-        <v>Dr Selena</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E117">
-        <v>8.5044</v>
+        <v>8.6875</v>
       </c>
       <c r="F117" t="str">
-        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
+        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
       </c>
     </row>
     <row r="118">
@@ -2753,39 +2753,39 @@
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B118">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C118" t="str">
-        <v>你也想紅嗎</v>
+        <v>小資變有錢｜Dr.Selena生活理財王</v>
       </c>
       <c r="D118" t="str">
-        <v>品牌女子A娜</v>
+        <v>Dr Selena</v>
       </c>
       <c r="E118">
-        <v>8.45</v>
+        <v>8.5</v>
       </c>
       <c r="F118" t="str">
-        <v>[EP66｜你沒辦法用過去有限能...] 單集時長53分鐘，資訊密度高且內容豐富，無明顯冷場，符合長篇內容的評估標準。</v>
+        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>到底有沒有獎 (泡麵沒熟獎)</v>
+        <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
       <c r="B119">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C119" t="str">
-        <v>蕭邦相談室</v>
+        <v>你也想紅嗎</v>
       </c>
       <c r="D119" t="str">
-        <v>蕭邦</v>
+        <v>品牌女子A娜</v>
       </c>
       <c r="E119">
-        <v>9.65</v>
+        <v>8.45</v>
       </c>
       <c r="F119" t="str">
-        <v>[幸福的人，通常「覺察力」都很強...] 單集時長在10-15分鐘（11分48秒），內容精煉且傳播效率高，能在短時間內提供豐富的資訊與啟發。</v>
+        <v>[EP66｜你沒辦法用過去有限能...] 單集時長53分鐘，資訊密度高且內容豐富，無明顯冷場，符合長篇內容的評估標準。</v>
       </c>
     </row>
     <row r="120">
@@ -2793,19 +2793,19 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B120">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C120" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D120" t="str">
-        <v>GK爸爸</v>
+        <v>蕭邦</v>
       </c>
       <c r="E120">
-        <v>9.6037</v>
+        <v>9.65</v>
       </c>
       <c r="F120" t="str">
-        <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
+        <v>[幸福的人，通常「覺察力」都很強...] 單集時長在10-15分鐘（11分48秒），內容精煉且傳播效率高，能在短時間內提供豐富的資訊與啟發。</v>
       </c>
     </row>
     <row r="121">
@@ -2813,19 +2813,19 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B121">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C121" t="str">
-        <v>美業幹什麼</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D121" t="str">
-        <v>美業幹什麼｜蔡佩陵</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E121">
-        <v>9.55</v>
+        <v>9.6</v>
       </c>
       <c r="F121" t="str">
-        <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
+        <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
       </c>
     </row>
     <row r="122">
@@ -2833,19 +2833,19 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B122">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C122" t="str">
-        <v>山姆書書</v>
+        <v>美業幹什麼</v>
       </c>
       <c r="D122" t="str">
-        <v>山姆書書</v>
+        <v>美業幹什麼｜蔡佩陵</v>
       </c>
       <c r="E122">
-        <v>9.3546</v>
+        <v>9.55</v>
       </c>
       <c r="F122" t="str">
-        <v>[EP134.真的找得到靈魂伴侶...] 單集時長約13分鐘，精煉且資訊密度高，在短時間內傳達了豐富的內容與思考，傳播效率極佳��</v>
+        <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
       </c>
     </row>
     <row r="123">
@@ -2853,19 +2853,19 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B123">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C123" t="str">
-        <v>教出你的路</v>
+        <v>山姆書書</v>
       </c>
       <c r="D123" t="str">
-        <v>治療師瑪奇</v>
+        <v>山姆書書</v>
       </c>
       <c r="E123">
-        <v>9.205</v>
+        <v>9.35</v>
       </c>
       <c r="F123" t="str">
-        <v>[EP31 為了愛移民，她打造 ...] 單集時長約13分半，內容精煉且資訊密度高，傳播效率極佳，無冗餘。</v>
+        <v>[EP134.真的找得到靈魂伴侶...] 單集時長約13分鐘，精煉且資訊密度高，在短時間內傳達了豐富的內容與思考，傳播效率極佳��</v>
       </c>
     </row>
     <row r="124">
@@ -2873,39 +2873,39 @@
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B124">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C124" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>教出你的路</v>
       </c>
       <c r="D124" t="str">
-        <v>無所不試無樂不作</v>
+        <v>治療師瑪奇</v>
       </c>
       <c r="E124">
-        <v>9.005</v>
+        <v>9.2</v>
       </c>
       <c r="F124" t="str">
-        <v>[【大師專題】人在江湖，身不由己...] 單集時長約10分鐘，符合10-15分鐘的短篇內容範疇。內容精煉，資訊密度高，能在短時間內傳達深刻且完整的觀點，傳播效率極佳。</v>
+        <v>[EP31 為了愛移民，她打造 ...] 單集時長約13分半，內容精煉且資訊密度高，傳播效率極佳，無冗餘。</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
+        <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
       <c r="B125">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C125" t="str">
-        <v>哇賽心理學</v>
+        <v>無所不試 無樂不作</v>
       </c>
       <c r="D125" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>無所不試無樂不作</v>
       </c>
       <c r="E125">
-        <v>9.5595</v>
+        <v>9</v>
       </c>
       <c r="F125" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
+        <v>[【大師專題】人在江湖，身不由己...] 單集時長約10分鐘，符合10-15分鐘的短篇內容範疇。內容精煉，資訊密度高，能在短時間內傳達深刻且完整的觀點，傳播效率極佳。</v>
       </c>
     </row>
     <row r="126">
@@ -2913,19 +2913,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B126">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C126" t="str">
-        <v>分手的99個理由</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D126" t="str">
-        <v>胡咪老師</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E126">
-        <v>9.4821</v>
+        <v>9.5549</v>
       </c>
       <c r="F126" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
+        <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
       </c>
     </row>
     <row r="127">
@@ -2933,19 +2933,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B127">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C127" t="str">
-        <v>五吉郎</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D127" t="str">
-        <v>五吉郎</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E127">
-        <v>9.4545</v>
+        <v>9.4786</v>
       </c>
       <c r="F127" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
+        <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
       </c>
     </row>
     <row r="128">
@@ -2953,19 +2953,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B128">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C128" t="str">
-        <v>蘇心時光</v>
+        <v>五吉郎</v>
       </c>
       <c r="D128" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>五吉郎</v>
       </c>
       <c r="E128">
         <v>9.45</v>
       </c>
       <c r="F128" t="str">
-        <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
+        <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
       </c>
     </row>
     <row r="129">
@@ -2973,19 +2973,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B129">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C129" t="str">
-        <v>布姐的沙發</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D129" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E129">
-        <v>9.3265</v>
+        <v>9.45</v>
       </c>
       <c r="F129" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
+        <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
       </c>
     </row>
     <row r="130">
@@ -2993,19 +2993,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B130">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C130" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D130" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E130">
-        <v>9.3099</v>
+        <v>9.3215</v>
       </c>
       <c r="F130" t="str">
-        <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
+        <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
       </c>
     </row>
     <row r="131">
@@ -3013,19 +3013,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B131">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C131" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D131" t="str">
-        <v>GK爸爸</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E131">
-        <v>9.2586</v>
+        <v>9.3049</v>
       </c>
       <c r="F131" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人透過引人入勝的敘事和情感連結，成功建立與聽眾的深厚關係，讓人期待後續故事發展，黏著度高。 | [春暖花開小旅行...] 主持人透過生動的敘述與角色扮演，與聽眾建立起良好的情感連結，具有高度的黏著度與陪伴感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 故事引人入勝，結尾的懸念設計強烈，讓聽眾對後續發展充滿期待，黏著度高。</v>
+        <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
       </c>
     </row>
     <row r="132">
@@ -3033,19 +3033,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B132">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C132" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D132" t="str">
-        <v>梁哲維</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E132">
-        <v>9.25</v>
+        <v>9.2549</v>
       </c>
       <c r="F132" t="str">
-        <v>[【EP330 帶著善意行動，最...] 主持人與來賓的對談充滿情感溫度，真誠的交流讓聽眾感受到靈魂的陪伴，具有很強的黏著度。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的對談真誠且富有溫度，內容��人入勝，能有效提升聽眾的黏著度與持續收聽的意願。 | [【EP312《超越我執的生活》...] 主持人以真誠且富有洞察力的語氣分享，內容深度能引發聽眾共鳴與思考，建立起較強的黏著度與情感連結，讓人期待下一集。</v>
+        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人透過引人入勝的敘事和情感連結，成功建立與聽眾的深厚關係，讓人期待後續故事發展，黏著度高。 | [春暖花開小旅行...] 主持人透過生動的敘述與角色扮演，與聽眾建立起良好的情感連結，具有高度的黏著度與陪伴感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 故事引人入勝，結尾的懸念設計強烈，讓聽眾對後續發展充滿期待，黏著度高。</v>
       </c>
     </row>
     <row r="133">
@@ -3053,19 +3053,19 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B133">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C133" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D133" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>梁哲維</v>
       </c>
       <c r="E133">
         <v>9.25</v>
       </c>
       <c r="F133" t="str">
-        <v>[#801 市場震盪 17000...] 主持人以真誠且具同理心的語氣與聽眾對話，建立深厚的連結，情感溫度高，能有效提升聽眾黏著度。 | [#809  買股票還在到處問明...] 主持人與來賓的對談真誠，內容實用且具啟發性，能有效吸引聽眾持續收聽，建立黏著度。 | [#798 害怕投資賠錢？不用天...] 主持人與來賓透過分享個人經驗和真誠的對談，與聽眾建立了深厚的情感連結，讓人期待下一集的內容。</v>
+        <v>[【EP330 帶著善意行動，最...] 主持人與來賓的對談充滿情感溫度，真誠的交流讓聽眾感受到靈魂的陪伴，具有很強的黏著度。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的對談真誠且富有溫度，內容��人入勝，能有效提升聽眾的黏著度與持續收聽的意願。 | [【EP312《超越我執的生活》...] 主持人以真誠且富有洞察力的語氣分享，內容深度能引發聽眾共鳴與思考，建立起較強的黏著度與情感連結，讓人期待下一集。</v>
       </c>
     </row>
     <row r="134">
@@ -3073,39 +3073,39 @@
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B134">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C134" t="str">
-        <v>蕭邦相談室</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D134" t="str">
-        <v>蕭邦</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E134">
-        <v>9.2429</v>
+        <v>9.25</v>
       </c>
       <c r="F134" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
+        <v>[#801 市場震盪 17000...] 主持人以真誠且具同理心的語氣與聽眾對話，建立深厚的連結，情感溫度高，能有效提升聽眾黏著度。 | [#809  買股票還在到處問明...] 主持人與來賓的對談真誠，內容實用且具啟發性，能有效吸引聽眾持續收聽，建立黏著度。 | [#798 害怕投資賠錢？不用天...] 主持人與來賓透過分享個人經驗和真誠的對談，與聽眾建立了深厚的情感連結，讓人期待下一集的內容。</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
       <c r="B135">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C135" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D135" t="str">
-        <v>GK爸爸</v>
+        <v>蕭邦</v>
       </c>
       <c r="E135">
-        <v>8.15</v>
+        <v>9.2429</v>
       </c>
       <c r="F135" t="str">
-        <v>AI 評審平均得分為 8.15 分，近半年累積 Apple Podcasts 評論數達 50 則，社群擴散影響力極佳。</v>
+        <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
       </c>
     </row>
     <row r="136">
@@ -3113,19 +3113,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B136">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C136" t="str">
-        <v>別人的工作最有趣</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D136" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E136">
-        <v>8.2</v>
+        <v>8.45</v>
       </c>
       <c r="F136" t="str">
-        <v>AI 評審平均得分為 8.2 分，近半年累積 Apple Podcasts 評論數達 18 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.45 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="137">
@@ -3133,19 +3133,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B137">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C137" t="str">
-        <v>小思大維</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D137" t="str">
-        <v>小思大維｜雪柔</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E137">
-        <v>8.24</v>
+        <v>8.44</v>
       </c>
       <c r="F137" t="str">
-        <v>AI 評審平均得分為 8.24 分，近半年累積 Apple Podcasts 評論數達 16 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="138">
@@ -3153,19 +3153,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B138">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C138" t="str">
-        <v>下一本讀什麼？</v>
+        <v>聰明生活投資學</v>
       </c>
       <c r="D138" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>聰明主婦的生活投資學</v>
       </c>
       <c r="E138">
-        <v>8.29</v>
+        <v>8.4</v>
       </c>
       <c r="F138" t="str">
-        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.4 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="139">
@@ -3173,19 +3173,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B139">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C139" t="str">
-        <v>山姆書書</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D139" t="str">
-        <v>山姆書書</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E139">
-        <v>8.19</v>
+        <v>8.18</v>
       </c>
       <c r="F139" t="str">
-        <v>AI 評審平均得分為 8.19 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.18 分，近半年累積 Apple Podcasts 評論數達 2 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="140">
@@ -3193,19 +3193,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B140">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C140" t="str">
-        <v>航海王的富人學</v>
+        <v>蘇心時光</v>
       </c>
       <c r="D140" t="str">
-        <v>美股航海王</v>
+        <v>蘇絢慧分享空間</v>
       </c>
       <c r="E140">
-        <v>8.15</v>
+        <v>8.33</v>
       </c>
       <c r="F140" t="str">
-        <v>AI 評審平均得分為 8.15 分，近半年累積 Apple Podcasts 評論數達 13 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.33 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="141">
@@ -3213,19 +3213,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B141">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C141" t="str">
-        <v>FIRE 人生大學</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="D141" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>我的動齡限量版</v>
       </c>
       <c r="E141">
-        <v>8.17</v>
+        <v>8.32</v>
       </c>
       <c r="F141" t="str">
-        <v>AI 評審平均得分為 8.17 分，近半年累積 Apple Podcasts 評論數達 10 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.32 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="142">
@@ -3233,7 +3233,7 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B142">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C142" t="str">
         <v>哇賽心理學</v>
@@ -3245,7 +3245,7 @@
         <v>8.29</v>
       </c>
       <c r="F142" t="str">
-        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 8 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="143">
@@ -3253,19 +3253,19 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B143">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C143" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D143" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E143">
-        <v>7.87</v>
+        <v>8.29</v>
       </c>
       <c r="F143" t="str">
-        <v>AI 評審平均得分為 7.87 分，近半年累積 Apple Podcasts 評論數達 11 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="144">
@@ -3273,39 +3273,39 @@
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B144">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C144" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D144" t="str">
-        <v>Dr Selena</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E144">
-        <v>8.14</v>
+        <v>8.29</v>
       </c>
       <c r="F144" t="str">
-        <v>AI 評審平均得分為 8.14 分，近半年累積 Apple Podcasts 評論數達 7 則，社群擴散影響力極佳。</v>
+        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B145">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C145" t="str">
-        <v>下一本讀什麼？</v>
+        <v>宋家小館</v>
       </c>
       <c r="D145" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E145">
-        <v>45</v>
+        <v>8.29</v>
       </c>
       <c r="F145" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #26.3 名。</v>
+        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
     </row>
     <row r="146">
@@ -3313,19 +3313,19 @@
         <v>站著不走獎</v>
       </c>
       <c r="B146">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C146" t="str">
-        <v>哇賽心理學</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D146" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E146">
         <v>45</v>
       </c>
       <c r="F146" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #33.3 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #26.3 名。</v>
       </c>
     </row>
     <row r="147">
@@ -3333,19 +3333,19 @@
         <v>站著不走獎</v>
       </c>
       <c r="B147">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C147" t="str">
-        <v>郝聲音</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D147" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E147">
         <v>45</v>
       </c>
       <c r="F147" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #38.2 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #33.3 名。</v>
       </c>
     </row>
     <row r="148">
@@ -3353,19 +3353,19 @@
         <v>站著不走獎</v>
       </c>
       <c r="B148">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C148" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>郝聲音</v>
       </c>
       <c r="D148" t="str">
-        <v>GK爸爸</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E148">
         <v>45</v>
       </c>
       <c r="F148" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #65.7 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #38.2 名。</v>
       </c>
     </row>
     <row r="149">
@@ -3373,19 +3373,19 @@
         <v>站著不走獎</v>
       </c>
       <c r="B149">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C149" t="str">
-        <v>文森說書</v>
+        <v>GK爸爸原創故事繪本</v>
       </c>
       <c r="D149" t="str">
-        <v>文森說書</v>
+        <v>GK爸爸</v>
       </c>
       <c r="E149">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F149" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 37 天，平均上榜排名為第 #64.3 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #65.7 名。</v>
       </c>
     </row>
     <row r="150">
@@ -3393,19 +3393,19 @@
         <v>站著不走獎</v>
       </c>
       <c r="B150">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C150" t="str">
-        <v>別人的工作最有趣</v>
+        <v>文森說書</v>
       </c>
       <c r="D150" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
+        <v>文森說書</v>
       </c>
       <c r="E150">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="F150" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 37 天，平均上榜排名為第 #64.3 名。</v>
       </c>
     </row>
     <row r="151">
@@ -3413,19 +3413,19 @@
         <v>站著不走獎</v>
       </c>
       <c r="B151">
+        <v>6</v>
+      </c>
+      <c r="C151" t="str">
+        <v>別人的工作最有趣</v>
+      </c>
+      <c r="D151" t="str">
+        <v>別人的工作最有趣｜Fiona</v>
+      </c>
+      <c r="E151">
         <v>7</v>
       </c>
-      <c r="C151" t="str">
-        <v>小思大維</v>
-      </c>
-      <c r="D151" t="str">
-        <v>小思大維｜雪柔</v>
-      </c>
-      <c r="E151">
-        <v>4</v>
-      </c>
       <c r="F151" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
       </c>
     </row>
     <row r="152">
@@ -3433,59 +3433,59 @@
         <v>站著不走獎</v>
       </c>
       <c r="B152">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C152" t="str">
-        <v>佐依Zoey</v>
+        <v>鄧惠文</v>
       </c>
       <c r="D152" t="str">
-        <v>佐依Zoey</v>
+        <v>鄧惠文</v>
       </c>
       <c r="E152">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F152" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B153">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C153" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>小思大維</v>
       </c>
       <c r="D153" t="str">
-        <v>GK爸爸</v>
+        <v>小思大維｜雪柔</v>
       </c>
       <c r="E153">
-        <v>8.7</v>
+        <v>4</v>
       </c>
       <c r="F153" t="str">
-        <v>平均評等 3.7 星，累計 50 則評論。綜合指標得分：8.7 / 10 分。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B154">
+        <v>9</v>
+      </c>
+      <c r="C154" t="str">
+        <v>佐依Zoey</v>
+      </c>
+      <c r="D154" t="str">
+        <v>佐依Zoey</v>
+      </c>
+      <c r="E154">
         <v>2</v>
       </c>
-      <c r="C154" t="str">
-        <v>小思大維</v>
-      </c>
-      <c r="D154" t="str">
-        <v>小思大維｜雪柔</v>
-      </c>
-      <c r="E154">
-        <v>6.5</v>
-      </c>
       <c r="F154" t="str">
-        <v>平均評等 4.9 星，累計 16 則評論。綜合指標得分：6.5 / 10 分。</v>
+        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
       </c>
     </row>
     <row r="155">
@@ -3493,19 +3493,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B155">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C155" t="str">
-        <v>下一本讀什麼？</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D155" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E155">
-        <v>6.2</v>
+        <v>5.2</v>
       </c>
       <c r="F155" t="str">
-        <v>平均評等 4.8 星，累計 14 則評論。綜合指標得分：6.2 / 10 分。</v>
+        <v>平均評等 5 星，累計 2 則評論。綜合指標得分：5.2 / 10 分。</v>
       </c>
     </row>
     <row r="156">
@@ -3513,19 +3513,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B156">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C156" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>迷途艾比</v>
       </c>
       <c r="D156" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>迷途艾比</v>
       </c>
       <c r="E156">
-        <v>6.1</v>
+        <v>0</v>
       </c>
       <c r="F156" t="str">
-        <v>平均評等 5 星，累計 11 則評論。綜合指標得分：6.1 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="157">
@@ -3533,19 +3533,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B157">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C157" t="str">
-        <v>航海王的富人學</v>
+        <v>山姆書書</v>
       </c>
       <c r="D157" t="str">
-        <v>美股航海王</v>
+        <v>山姆書書</v>
       </c>
       <c r="E157">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F157" t="str">
-        <v>平均評等 4.7 星，累計 13 則評論。綜合指標得分：6 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="158">
@@ -3553,19 +3553,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B158">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C158" t="str">
-        <v>別人的工作最有趣</v>
+        <v>宋家小館</v>
       </c>
       <c r="D158" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E158">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F158" t="str">
-        <v>平均評等 4.2 星，累計 18 則評論。綜合指標得分：6 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="159">
@@ -3573,19 +3573,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B159">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C159" t="str">
-        <v>山姆書書</v>
+        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
       <c r="D159" t="str">
-        <v>山姆書書</v>
+        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E159">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F159" t="str">
-        <v>平均評等 4.6 星，累計 14 則評論。綜合指標得分：6 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="160">
@@ -3593,19 +3593,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B160">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C160" t="str">
-        <v>FIRE 人生大學</v>
+        <v>任性歐逆機智生活</v>
       </c>
       <c r="D160" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="E160">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="F160" t="str">
-        <v>平均評等 4.8 星，累計 10 則評論。綜合指標得分：5.8 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="161">
@@ -3613,19 +3613,19 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B161">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C161" t="str">
-        <v>文森說書</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D161" t="str">
-        <v>文森說書</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E161">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="F161" t="str">
-        <v>平均評等 4.8 星，累計 10 則評論。綜合指標得分：5.8 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="162">
@@ -3633,59 +3633,59 @@
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B162">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C162" t="str">
-        <v>哇賽心理學</v>
+        <v>爛泥Jill式優雅</v>
       </c>
       <c r="D162" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>爛泥媽媽的重生日記（Jill)</v>
       </c>
       <c r="E162">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="F162" t="str">
-        <v>平均評等 4.6 星，累計 8 則評論。綜合指標得分：5.4 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B163">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C163" t="str">
-        <v>不敗教主陳重銘</v>
+        <v>人生啊｜陪你一起看懂人生</v>
       </c>
       <c r="D163" t="str">
-        <v>不敗教主-陳重銘</v>
+        <v>人生啊！小歐</v>
       </c>
       <c r="E163">
         <v>0</v>
       </c>
       <c r="F163" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B164">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C164" t="str">
-        <v>布姐的沙發</v>
+        <v>下半場人生陪談師</v>
       </c>
       <c r="D164" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>下半場人生事務有限公司</v>
       </c>
       <c r="E164">
         <v>0</v>
       </c>
       <c r="F164" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="165">
@@ -3693,7 +3693,7 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B165">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C165" t="str">
         <v>尼可這樣說</v>
@@ -3713,19 +3713,19 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B166">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C166" t="str">
-        <v>無所不試 無樂不作</v>
+        <v>迷途艾比</v>
       </c>
       <c r="D166" t="str">
-        <v>無所不試無樂不作</v>
+        <v>迷途艾比</v>
       </c>
       <c r="E166">
         <v>0</v>
       </c>
       <c r="F166" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="167">
@@ -3733,19 +3733,19 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B167">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C167" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>山姆書書</v>
       </c>
       <c r="D167" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>山姆書書</v>
       </c>
       <c r="E167">
         <v>0</v>
       </c>
       <c r="F167" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="168">
@@ -3753,19 +3753,19 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B168">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C168" t="str">
-        <v>丁菱娟的邊走邊想</v>
+        <v>宋家小館</v>
       </c>
       <c r="D168" t="str">
-        <v>丁菱娟</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E168">
         <v>0</v>
       </c>
       <c r="F168" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="169">
@@ -3773,19 +3773,19 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B169">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C169" t="str">
-        <v>楊肉盧</v>
+        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
       <c r="D169" t="str">
-        <v>楊月娥（楊肉爐）</v>
+        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E169">
         <v>0</v>
       </c>
       <c r="F169" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="170">
@@ -3793,19 +3793,19 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B170">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C170" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>任性歐逆機智生活</v>
       </c>
       <c r="D170" t="str">
-        <v>人生啊！小歐</v>
+        <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="E170">
         <v>0</v>
       </c>
       <c r="F170" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="171">
@@ -3813,19 +3813,19 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B171">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C171" t="str">
-        <v>人類行為研究社</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D171" t="str">
-        <v>張忘形</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E171">
         <v>0</v>
       </c>
       <c r="F171" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
     <row r="172">
@@ -3833,24 +3833,64 @@
         <v>聽眾都要跟你獎 (近半年有評論數)</v>
       </c>
       <c r="B172">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C172" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
+        <v>爛泥Jill式優雅</v>
       </c>
       <c r="D172" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
+        <v>爛泥媽媽的重生日記（Jill)</v>
       </c>
       <c r="E172">
         <v>0</v>
       </c>
       <c r="F172" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
+      </c>
+      <c r="B173">
+        <v>9</v>
+      </c>
+      <c r="C173" t="str">
+        <v>人生啊｜陪你一起看懂人生</v>
+      </c>
+      <c r="D173" t="str">
+        <v>人生啊！小歐</v>
+      </c>
+      <c r="E173">
+        <v>0</v>
+      </c>
+      <c r="F173" t="str">
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>聽眾都要跟你獎 (近半年有評論數)</v>
+      </c>
+      <c r="B174">
+        <v>10</v>
+      </c>
+      <c r="C174" t="str">
+        <v>下半場人生陪談師</v>
+      </c>
+      <c r="D174" t="str">
+        <v>下半場人生事務有限公司</v>
+      </c>
+      <c r="E174">
+        <v>0</v>
+      </c>
+      <c r="F174" t="str">
+        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F174"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update UI: Remove Demo badge and highlight Top 10 section
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -398,14 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F176"/>
+  <dimension ref="A1:G158"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="100.83203125" customWidth="1"/>
+    <col min="6" max="6" width="80.83203125" customWidth="1"/>
+    <col min="7" max="7" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -427,8 +428,11 @@
       <c r="F1" t="str">
         <v>評選理由 (Reason)</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="G1" t="str">
+        <v>最推薦聆聽片段 (Recommended Segment)</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -447,8 +451,14 @@
       <c r="F2" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [EP174｜越省反而越窮？別把...] 主持人開場鋪陳完整，話題引導流暢，結尾有總結，整體架構清晰。 | [EP164｜滑短影音是在浪費時...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 學習動機的深度剖析】
+時間: 11:48 - 12:34
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 在此片段中，主持人Andy精準地總結了來賓先前關於學習樂趣與被迫學習痛苦的觀點，並提出關於內在動機的深刻見解（「當你今天帶著問題去找答案，回來學習的時候，那個動力跟你讓自己去學會的那個底層是完全不一樣的」）。來賓的即時認同與補充，展現了兩人良好的默契與對話流暢度。這段對話不僅提升了內容深度，也突顯了主持人卓越的引導與控場能力，非常適合評選「最佳內容架構獎」與「最佳默契獎」。</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -467,8 +477,14 @@
       <c r="F3" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [《財富自由心理學》：賺錢，只是...] 節目開場鋪陳完整，話題轉折自然流暢，主持人能有效引導對談並適時拉回核心，結尾亦有精要總結，架構清晰。 | [手總是停不下來？那是焦慮在尋找...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 探討藥物對情緒的影響】
+時間: 00:50:00 - 00:53:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 主持人敏銳地提出聽眾可能關心的藥物對情緒的影響，並分享身邊案例，引導來賓從生理角度（如低血糖）解釋可能的原因。這展現了主持人對聽眾需求的洞察力，以及引導對話深入探討的控場能力，互動自然流暢。</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -487,8 +503,14 @@
       <c r="F4" t="str">
         <v>[EP289  七巨頭變七矮人！...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [EP275 股市變賭場？巴菲特...] 節目開場清晰，主題鋪陳有條理，各段落間的轉折流暢，結尾總結與行動呼籲明確，整體內容架構完整且邏輯性強。 | [EP251國防預算暴漲 5 成...] 主持人開場直接切入主題，中間分析市場數據和政策影響，邏輯清晰。雖然語速快，但內容結構完整。</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 七巨頭表現分化與市場資金輪動分析】
+時間: 04:08 - 04:25
+單集: EP251國防預算暴漲 5 成！必看這五檔股票！跟者川普賺一波？
+理由: 主持人在此段落清晰地分析了去年美股七巨頭中，僅有兩家跑贏大盤的現象，並解釋了資金輪動的快速性。他以數據為基礎，流暢地從個股表現過渡到整體市場的資金流向，展現了其在複雜資訊中提煉重點、引導聽眾理解市場變化的控場能力。語速雖快，但邏輯清晰，能有效傳達訊息。</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -507,8 +529,14 @@
       <c r="F5" t="str">
         <v>[【EP330 帶著善意行動，最...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [【EP302 把命盤變成行動藍...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。 | [【EP312《超越我執的生活》...] 主持人開場鋪陳清晰，能有效引導聽眾進入主題。內容邏輯性強，轉折自然，結尾亦有精要總結與行動呼籲，架構完整。</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 主持人提問創業挑戰，來賓真誠分享掙扎】
+時間: 10:13 - 12:12
+單集: 【EP330 帶著善意行動，最能累積長期信任資本《好感影響力》ft. Hey yo雞腳創辦人 惠蓮＆又又】
+理由: 主持人提出了一個非常關鍵且深入的問題：「有沒有想過放棄？」這直接觸及了創業過程中的真實挑戰。惠蓮的回答誠實地表達了「還是不要這麼麻煩」的掙扎，以及後續在如何呈現公益活動時遇到的困境，展現了人性的真實面。主持人透過這個問題，成功引導來賓分享了更深層次的思考和情感，顯示了其引導對話和挖掘深度的能力。</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -527,8 +555,14 @@
       <c r="F6" t="str">
         <v>[#801 市場震盪 17000...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [#809  買股票還在到處問明...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。 | [#798 害怕投資賠錢？不用天...] 主持人開場鋪陳完整，中途能流暢引導話題，從基礎概念到實務應用，再到心態調整，架構清晰，結尾亦有精要總結。</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 投資前的家庭財務規劃與長期策略】
+時間: 10:14 - 12:19
+單集: #801 市場震盪 17000 點，費半重挫、台股回檔，你該急著逃，還是重新檢查資產配置？給剛進場投資人的一堂情緒與現金流課
+理由: 在此片段中，主持人巧妙地引導聽眾進行投資前的家庭財務規劃，包括評估收入、支出、債務和緊急預備金。她強調建立堅實「安全網」的重要性，以避免在市場波動時做出情緒化決策。主持人隨後流暢地轉向投資進場策略，提倡紀律性的「分批進場」而非盲目「接刀子」。她清晰地區分了短期與長期投資心態，展現了卓越的內容架構能力，並能以引人入勝的方式闡述複雜的金融概念，對於單人主持而言，控場表現極佳。</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
       <c r="A7" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -547,8 +581,14 @@
       <c r="F7" t="str">
         <v>[EP611 00998A(主動...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀分析到具體投資標的，結尾亦有精要總結，架構清晰。 | [EP628昇陽半導體(8028...] 主持人開場鋪陳完整，中途能流暢引導話題，從宏觀產業趨勢到具體個股分析，結尾亦有精要總結，架構清晰。 | [EP621《富媽媽 窮媽媽》第...] 節目開場清晰，主體內容透過故事案例層層推進，邏輯嚴謹，結尾有明確的行動呼籲與總結，架構完整。</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 金融業併購趨勢與個人資產配置的連結】
+時間: 03:02 - 04:00
+單集: EP611 00998A(主動復華金融股息)鎖定歐洲大型金融股，優缺點在哪裡呢？
+理由: 主持人在此段落流暢地從金融業的併購趨勢，過渡到個人資產配置的理念，巧妙地將宏觀經濟現象與微觀投資策略結合。他透過清晰的邏輯推演和適時的提問（如「是不是？」），引導聽眾思考，展現了單人主持下對內容的精準控場能力，確保話題聚焦且具連貫性。這段展現了主持人如何有效引導聽眾思考，而非僅單向輸出資訊，符合【最佳內容架構獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
       <c r="A8" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -567,8 +607,14 @@
       <c r="F8" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人開場鋪陳清晰，中途提問引導流暢，能有效推進對話，結尾總結亦有深度，整體內��架構完整。 | [EP218：愛自己｜放下完美執...] 節目開場鋪陳流暢，透過個人經驗引入主題與來賓。中段內容圍繞人類圖的核心概念、案例分析與關係互動，轉折自然。結尾則聚焦於線上課程的推廣與總結，整體架構清晰，引導得宜。 | [EP219：【非典家庭CEO】...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。</v>
       </c>
-    </row>
-    <row r="9">
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 伴侶關係中的人類圖互動與建議】
+時間: 24:44 - 28:07
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段充分展現了主持人與來賓之間流暢且自然的互動。Cherry分享了她與顯示生產者丈夫在專案啟動上的困擾，小可也補充了她丈夫的不同情況，來賓Anka則巧妙地將話題拉回人類圖的「閘門」概念，並解析了兩位主持人伴侶的月亮閘門（Gate 1的創意與Gate 42的完成使命感）。Anka不僅精準點出特質，更提供了投射者（主持人）如何與顯示者（伴侶）有效溝通的實用建議（透過提問而非指令）。整個過程充滿了自然的對話、共鳴與實用性，完美體現了「最佳默契獎」與「最佳內容架構獎」的評估標準。</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
       <c r="A9" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -587,8 +633,14 @@
       <c r="F9" t="str">
         <v>[莫菲穿搭20｜球具只是通行證？...] 節目開場鋪陳完整，主題明確。主持人能流暢引導話題，從個人經驗到宏觀趨勢，轉折自然，結尾亦有精要總結，架構清晰。 | [莫菲穿搭27｜金曲幕後直擊！電...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [莫菲穿搭02｜2026流行色配...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。</v>
       </c>
-    </row>
-    <row r="10">
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 進香路上的幽默互動與生活百態】
+時間: 07:25 - 09:05
+單集: 莫菲穿搭20｜球具只是通行證？Leo揭秘老闆們：白天捐救護車，晚上忙什麼？（下）
+理由: 此片段展現了主持人與來賓之間自然且幽默的互動。女主持人以輕鬆的語氣提問關於進香穿搭的細節，並透過自身參與的趣事（如幫忙吃茶葉蛋）與來賓的生動描述（如吃到羊肉爐、看到超大盤生魚片）產生共鳴。兩人的對話充滿生活感，笑聲自然，即使話題偶爾跳脫，也能在輕鬆的氛圍中順暢地拉回核心，展現了極佳的控場能力和雙向互動的默契，讓聽眾彷彿置身其中，感受到進香路���的溫暖與人情味。</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -607,8 +659,14 @@
       <c r="F10" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，內容架構清晰。 | [【蕭邦出任務】如何選擇適合自己...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體架構清晰。 | [幸福的人，通常「覺察力」都很強...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 揭露行銷產業的真實面貌】
+時間: 22:09 - 23:58
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 在此片段中，來賓Katie深入解釋了行銷產業並非表面光鮮亮麗，而是需要無數次的數據研究、假設、驗證、失敗與優化。主持人小幫在此段展現了良好的互動與控場能力，透過適時的「沒錯，沒錯」等回應，不僅表達了對來賓觀點的認同，也引導聽眾更深入理解行銷工作的本質。這種互動方式讓對話保持流暢，並有效強化了內容的深度與可信度，避免了話題的偏離，展現了【最佳內容��構獎】與【最佳默契獎】所需的主持功力。</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
       <c r="A11" t="str">
         <v>最佳內容架構獎</v>
       </c>
@@ -627,8 +685,14 @@
       <c r="F11" t="str">
         <v>[EP.617 《無限機器》讀後...] 主持人開場鋪陳完整，中途能流暢引導話題，透過六個重點清晰地呈現書中精華，結尾亦有精要總結，內容架構清晰。 | [EP.573 從 0 到 10...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結。內容邏輯清晰，層次分明。 | [EP.607 《AI Firs...] 主持人開場鋪陳完整，中途能流暢引導話題，結尾亦有精要總結，整體內容架構清晰。</v>
       </c>
-    </row>
-    <row r="12">
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 獨自奮鬥的血淚與找到同路人的感動】
+時間: 01:44:00 - 01:45:30
+單集: EP.573 從 0 到 10 萬訂閱：我經營免費電子報六年的三個體悟
+理由: 主持人分享了在建構電子報系統時，面對技術挑戰和中文資源匱乏的孤獨感。他生動描述了當時的掙扎，以及後來意外發現有其他創作者（如YouTuber張修修）也採用相同複雜架構時的「血淚」與感動。這段內容展現了主持人真誠且富有感染力的敘事能力，他透過分享個人脆弱面，成功拉近與聽眾的距離，並營造出強烈的共鳴感，雖然是單人主持，但其情感表達與故事鋪陳極具吸引力。</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
       <c r="A12" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -636,19 +700,25 @@
         <v>1</v>
       </c>
       <c r="C12" t="str">
-        <v>分手的99個理由</v>
+        <v>能量黑客</v>
       </c>
       <c r="D12" t="str">
-        <v>胡咪老師</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E12">
-        <v>9.1931</v>
+        <v>10</v>
       </c>
       <c r="F12" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 兩位主持人互動自然，接話流暢，笑聲同步率高，展現良好默契。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人默契極佳，對話流暢自然，能互相接話並適時加入幽默感，共同營造出引人入勝的節目氛圍。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契，接話流暢，插話頻率適中，彼此的幽默感與共鳴笑聲自然，共同營造出輕鬆愉快的對話氛圍。</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人展現了極高的默契與自然流暢的對話。他們頻繁地接話、補充彼此的觀點，並透過提問與分享個人經驗（如Vicky的跑步經歷、Hank的決策原則）來深化討論。彼此間的幽默感與支持性互動，不僅讓對話充滿活力，也成功營造出輕鬆愉快的氛圍，使聽眾能更投入地聆聽，並感受到主持人之間真誠的連結。 | [別人眼中的高光時刻，卻是我最耗...] 兩位主持人展現了極佳的默契與引導能力。他們不僅能精準地提問，更透過自身的經驗分享（如Hank的「相見恨晚」），與來賓建立深厚的連結，讓來賓願意敞開心扉分享最私密的經歷。Vicky的歸納與提問也讓對話更具深度與流暢性，整體氣氛溫暖且具感染力。 | [別急著振作！高能量的人允許自己...] 兩位主持人展現了極佳的默契與引導能力。他們的問題深入且具啟發性，能有效引導來賓分享更深層的經驗與見解。Vicky的提問與生活化比喻，常能精準捕捉聽眾的疑問並讓氣氛更活潑；Hank則以其專業背景提出關鍵問題，並在適時處給予來賓肯定與支持。兩人互動流暢自然，彼此的補充與呼應讓對話內容更豐富，也讓來賓感到被理解與尊重，進而更願意敞開心扉，使節目氛圍充滿正向能量與深度。</v>
+      </c>
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 跑步發現新世界】
+時間: 12:14 - 13:22
+單集: 新年特輯—火馬年續航攻略：吃睡練＋情緒＋決策＋意義感｜能量黑客S3EP11
+理由: 女主持人在此段分享了她因跑步而意外發現河堤美景的個人經歷，生動的敘述方式（「我一走過去的時候，噔噔！」）引人入勝。男主持人則以積極的傾聽和簡短的肯定（「我知道，我知道，你們那裡我常跑，我知道」）來支持對話，沒有打斷女主持人的故事流暢性，展現了雙人主持間自然且流暢的互動默契。此片段完美體現了主持人如何透過個人故事來豐富內容，並維持良好的對話節奏，符合【最佳內容��構獎】與【最佳默契獎】的評選標準。</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
       <c r="A13" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -656,19 +726,25 @@
         <v>2</v>
       </c>
       <c r="C13" t="str">
-        <v>楊肉盧</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D13" t="str">
-        <v>楊月娥（楊肉爐）</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E13">
-        <v>9.1931</v>
+        <v>10</v>
       </c>
       <c r="F13" t="str">
-        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>[S4.EP4｜性平教育20年，...] 兩位主持人展現了極佳的默契與流暢的互動。女主持人提供詳盡的資訊與引導，男主持人則以貼近聽眾的反應、提問及個人經驗（如對長輩世代的觀察）來回應，不僅讓對話更具深度與廣度，也有效活絡了節目氣氛。男主持人的情感反應（如「太可怕了啦」、「我聽到這邊好難過喔」）更增添了節目的真實感與共鳴，使聽眾能更投入地聆聽這個嚴肅的議題。 | [S4.EP8｜我不想再跟你生活...] 胡咪與畢頭大叔展現了極高的默契與互動性。胡咪老師在朗讀書摘時情感豐沛，畢頭大叔則能即時給予真誠且具個人色彩的回應，無論是幽默的自嘲（如「我這個書名就讓我心碎了」）或是深刻的共鳴（如「你不要再說了啦，我聽到這邊我突然好難過」），都讓對話充滿層次感。兩人能自然地接話、延伸話題，並透過彼此的視角（男性與女性）豐富了討論的廣度與深度，使節目氣氛溫暖而引人入勝，讓聽眾彷彿也參與其中，共同感受情感的流動。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現��極佳的默契與自然互動，對話流暢且充滿趣味。他們能巧妙地接話、補充彼此觀點，並透過幽默感與個人經驗分享，讓嚴肅的自我探索主題變得輕鬆且引人入勝。這種互動氛圍不僅鼓勵彼此更深入地表達，也讓聽眾感到被邀請參與其中，極具渲染力。</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">【幽默互動：性愛暗號與身心益處大揭密】
+時間: 15:33 - 24:47
+單集: S3.EP81｜越做越愛的關係續命術
+理由: 主持人討論如何用「小暗號」來表達性需求，Humi舉例「歡樂的世界」等幽默對話，展現了良好的互動與趣味性。接著，他們詳細列舉了性愛對免疫系統、心血管、睡眠、大腦、皮膚、骨骼等多方面的生理益處，內容豐富且具說服力，Vito最後的「做愛治百病」總結更是畫龍點睛。</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
       <c r="A14" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -676,19 +752,25 @@
         <v>3</v>
       </c>
       <c r="C14" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>粉紅地獄辛辣麵</v>
       </c>
       <c r="D14" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>Vito大叔</v>
       </c>
       <c r="E14">
-        <v>8.8049</v>
+        <v>9.9</v>
       </c>
       <c r="F14" t="str">
-        <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>[S6EP30. 我到日本當漁夫...] Vito 大叔與品希的搭檔默契極佳，兩位主持人一搭一唱，提問精準且富有層次，能有效引導來賓 Taku 深入分享其經歷與感受。他們不僅展現出對來賓故事的濃厚興趣，更透過適時的驚嘆、幽默的互動與同理心的回應，營造出輕鬆愉悅且充滿支持的對話氛圍，讓 Taku 能夠暢所欲言，使節目內容更加豐富動人。兩人的互動也讓聽眾彷彿置身其中，共同感受故事的起伏。 | [S6EP19. 沐樂MOReL...] 楊梅老師與V-Tou大叔展現了極佳的默契與互動。兩人之間的幽默感與互相吐槽（如楊梅老師調侃V-Tou交到女友就忘記她，或V-Tou分享處理體味的「年代金曲」）為節目營造了輕鬆愉快的氛圍。他們的問題引導性強，能讓來賓范范自在地分享專業知識、個人經歷，甚至是一些敏感話題（如如何委婉告知客戶有體味）。兩位主持人不僅讓來賓暢所欲言，也透過自身的參與和反應，讓整個對話充滿活力與趣味，使聽眾能更投入地聆聽。 | [S6EP4. 放飛。萬哩露｜村...] B頭大叔和品希與來賓凱莉哥的互動非常流暢且充滿默契。他們不僅提出深入的問題，也適時分享個人經驗，讓凱莉哥更願意敞開心扉。品希分享兒子在校園的經歷，與凱莉哥的「放手」哲學形成對比，豐富了討論的層次。主持人之間的幽默感和相互支持也讓節目氣氛輕鬆愉快，引導來賓和彼此更深入地交流。</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">【音樂在日常中的療癒力與幽默互動】
+時間: 1:40:00 - 1:42:00
+單集: S6EP24. 五感研究苑｜顏爾呈：用音頻啟動修復！找回內在節奏與平靜
+理由: 男性主持人分享他載女兒上學時，透過聆聽大自然音樂來放鬆身心的個人經驗，展現音樂療癒在日常生活中潛移默化的影響力。女兒對「漏水」的幽默反應，也為節目增添了輕鬆有趣的互動，讓聽眾感受到音樂療癒的實用性與生活化。</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
       <c r="A15" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -696,19 +778,25 @@
         <v>4</v>
       </c>
       <c r="C15" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
+        <v>楊肉盧</v>
       </c>
       <c r="D15" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
+        <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E15">
-        <v>8.7715</v>
+        <v>9.1931</v>
       </c>
       <c r="F15" t="str">
-        <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
+      </c>
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 魅力源於自身擁有的深刻洞察】
+時間: 02:40:00 - 02:43:00
+單集: EP128｜【母女鍋】魅力是可以學習的
+理由: 楊月娥在此段精闢地闡述了「你如果沒有，你看 不見」的深刻觀點，挑戰了聽眾對魅力的傳統認知。她以自信且具說服力的語氣，引導聽眾反思自身價值，展現了其作為主持人的深度思考能力和引導聽眾進行自我探索的功力。小真在旁適時的簡短回應，也顯示了兩人對話的流暢與默契。</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
       <c r="A16" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -716,19 +804,25 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <v>粉紅地獄辛辣麵</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D16" t="str">
-        <v>Vito大叔</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E16">
-        <v>8.7215</v>
+        <v>8.8049</v>
       </c>
       <c r="F16" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] Vito和品希作為雙人主持，展現了良好的默契。他們接話流暢，很少出現互相打斷的情況，品希的提問常帶有女性的細膩與同理心，Vito則負責更宏觀的引導與專業提問。兩人的笑聲自然，共同營造了輕鬆愉快的對談氛圍。 | [S6EP19. 沐樂MOReL...] Vito與品希之間展現了極佳的默契，對話流暢自然，常有幽默的插科打諢和同步的笑聲，互動感強烈。 | [S6EP4. 放飛。萬哩露｜村...] 雙主持與來賓互動自然，接話流暢，笑聲同步率高，尤其在幽默對話時默契十足，��節目增添了活力。</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
+      </c>
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 伴侶關係中的人類圖互動與建議】
+時間: 24:44 - 28:07
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段充分展現了主持人與來賓之間流暢且自然的互動。Cherry分享了她與顯示生產者丈夫在專案啟動上的困擾，小可也補充了她丈夫的不同情況，來賓Anka則巧妙地將話題拉回人類圖的「閘門」概念，並解析了兩位主持人伴侶的月亮閘門（Gate 1的創意與Gate 42的完成使命感）。Anka不僅精準點出特質，更提供了投射者（主持人）如何與顯示者（伴侶）有效溝通的實用建議（透過提問而非指令）。整個過程充滿了自然的對話、共鳴與實用性，完美體現了「最佳默契獎」與「最佳內容架構獎」的評估標準。</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
       <c r="A17" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -736,19 +830,25 @@
         <v>6</v>
       </c>
       <c r="C17" t="str">
-        <v>能量黑客</v>
+        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
       <c r="D17" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E17">
-        <v>8.6549</v>
+        <v>8.7715</v>
       </c>
       <c r="F17" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人互動自然，接話流暢，彼此間的幽默感和笑聲也增加了節目的親和力。女主持人興奮時的插話，男主持人也能很好地承接。 | [別人眼中的高光時刻，卻是我最耗...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高��尤其在幽默解釋「麻場」和「鐵軌」時，默契十足。 | [別急著振作！高能量的人允許自己...] 雙主持人Hank與Vicky之間的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現了良好的默契與引導能力。</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 針對學員需求的引導與溝通】
+時間: 05:48 - 07:16
+單集: EP36｜30歲以後的身體，需要的不是更努力，而是更有覺察 ft. Eva
+理由: 此片段主持人與來賓討論了學員最常許的願望和遇到的身體問題，以及教練如何應對。來賓詳細說明了她會如何評估學員的身體狀況（功能性評估）和目標，並強調了動作品質的重要性。主持人適時地提出問題，例如「什麼是功能性評估？」，幫助聽眾理解專業術語，並以自身經驗（「我們就是兩個想要增肌減脂的小白」）拉近與來賓的距離，展現了流暢的互動和控場能���，符合【最佳內容架構獎】與【最佳默契獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
       <c r="A18" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -767,8 +867,14 @@
       <c r="F18" t="str">
         <v>[跟長輩一樣就能學會AI？陶韻智...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高，但偶有輕微搶話情況，整體默契良好。 | [再不用證明自己給誰看 feat...] 雙主持人與來賓之間的互動自然，接話流暢，笑聲具感染力，展現了良好的默契，即使有插話也多能順暢銜接。 | [好像很爽，我們也去當個旅遊作家...] 兩位主持人與來賓之間的對話流暢自然，接話和反應迅速，共同營造了輕鬆愉快的氛圍，默契良好。</v>
       </c>
-    </row>
-    <row r="19">
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 突破慣性：從個人到企業的AI應用】
+時間: 05:21 - 06:15
+單集: 跟長輩一樣就能學會AI？陶韻智老師的反慣性AI學《 AI First 自我升級革命》
+理由: Mandy 提出「最難改的慣性」這個核心問題，引導老師分享了人類基因中根深蒂固的「從眾」與「不改變」的慣性。老師以生動的例子（如不被老虎吃掉的走路方式）解釋了這些慣性如何影響我們對新事物的接受度。這段對話展現了主持人提問的精準度，能夠引導來賓深入淺出地闡述複雜概念，同時保持了對話的流暢與互動性，為聽眾提供了極具啟發性的思考。</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
       <c r="A19" t="str">
         <v>最佳默契獎</v>
       </c>
@@ -787,8 +893,14 @@
       <c r="F19" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 主持人與來賓之間的對話流暢自然，接話得體，沒有明顯的搶話或插話，展現了良好的互動默契。 | [【中年，正在試】把世界走成一本...] Norman和Summer的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現良好默契。</v>
       </c>
-    </row>
-    <row r="20">
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 團隊年輕化背後的共同理念】
+時間: 01:47:00 - 01:53:00
+單集: 從流浪到回家：浪人食堂的溫柔守護與陪伴 ft.蔡明潔店長
+理由: Norman在此段提出關於團隊成員普遍年輕化的觀察，並引導明潔深入解釋這背後共同的理念。Norman的提問精準且開放，讓明潔能充分表達團隊「善待人」的核心價值。這展現了主持人良好的控場能力，能將對話引導至更深層次的討論，同時保持流暢自然的互動，符合「最佳內容架構獎」與「最佳默契獎」的評估標準。</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
       <c r="A20" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -807,8 +919,14 @@
       <c r="F20" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 選題新穎，結合個人IP變現與美業轉型，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [EP174｜越省反而越窮？別把...] 選題結合心理學與財富自由，觀點新穎且具深度，案例生動，內容含金量高。 | [EP164｜滑短影音是在浪費時...] 選題新穎且具深度，圍繞來賓新書的核心理念展開，提供了許多關於閱讀與自我成長的實用觀點與啟發，內容含金量極高。</v>
       </c>
-    </row>
-    <row r="21">
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 來賓電商逆襲的核心思考】
+時間: 04:43 - 06:56
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 此片段詳細闡述了來賓從代理產品轉向自創品牌的「悲慘故事」，揭示了市場亂象（經銷商跳過代理、價格戰）如何迫使她做出戰略轉變。內容充滿創業洞察，展現了對市場動態和個人價值的深刻理解。主持人Andy的問題引導來賓揭示了其核心動機，使這段敘述極具啟發性，非常適合評選「最神單元企劃」與「自我探索獎」。</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
       <c r="A21" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -827,8 +945,14 @@
       <c r="F21" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 選題非常新穎且具時事性，從藥物機制到社會政策的討論深度極高，內容含金量豐富。 | [《財富自由心理學》：賺錢，只是...] 選題「財富自由心理學」新穎且具深度，透過個人故事與哲學思辨，將財富議題提升至心靈層次，內容含金量高，案例生動具啟發性。 | [手總是停不下來？那是焦慮在尋找...] 選題新穎且具深度，深入探討身體重複行為的心理學面向，案例生動且內容含金量極高。</v>
       </c>
-    </row>
-    <row r="22">
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 美國健康政策與生活型態結合】
+時間: 01:50:00 - 01:53:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段來賓深入探討美國最新的健康政策，如何將藥物治療與生活型態調整結合，並提出「Balance」計畫。這不僅展現了選題的深度與前瞻性，也提供了超越單純藥物討論的宏觀視角，極具單元企劃與啟發價值。</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
       <c r="A22" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -847,8 +971,14 @@
       <c r="F22" t="str">
         <v>[【EP330 帶著善意行動，最...] 節目以一本關於「好感影響力」的書為引子，邀請書中提及的創業家來分享故事，選題獨特且具深度。來賓的70年滷味傳承與公益行動，提供了豐富的內容含金量和啟發性。 | [【EP302 把命盤變成行動藍...] 選題新穎，結合「九紫離火運」與AI、全球局勢、個人發展等多元面向，案例生動且內容含金量極高。 | [【EP312《超越我執的生活》...] 選題「超越我執」具備深度與啟發性，結合心理學與靈性成長，內容含金量高，案例（如內在聲音、吃飯專注）生動且具體，展現了優秀的單元企劃能力。</v>
       </c>
-    </row>
-    <row r="23">
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">【「主角模式」核心概念闡述】
+時間: 00:00 - 00:49
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
       <c r="A23" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -867,8 +997,14 @@
       <c r="F23" t="str">
         <v>[#801 市場震盪 17000...] 選題緊扣時事（股市下跌），並結合個人財務規劃與情緒管理，案例生動且內容含金量極高。 | [#809  買股票還在到處問明...] 選題「獲利加速系統」具備高度實用性與深度，結合AI工具的應用，內容含金量極高，企劃新穎。 | [#798 害怕投資賠錢？不用天...] 選題新穎且具備深度，聚焦於媽媽族群的投資教育與心態建立，內容含金量高，並透過生動的比喻（如游泳、無印良品櫃子）提升理解度。</v>
       </c>
-    </row>
-    <row r="24">
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 股市下跌時的情緒管理與長期投資心法】
+時間: 03:07 - 04:38
+單集: #801 市場震盪 17000 點，費半重挫、台股回檔，你該急著逃，還是重新檢查資產配置？給剛進場投資人的一堂情緒與現金流課
+理由: 此片段全面探討了市場下跌時投資者的情緒管理。主持人深入分析了新進投資者常見的後悔與恐懼心理，強調市場的不可預測性，並引導聽眾思考投資標的的基本面價值與長期成長潛力。她透過對比長期持有者與近期進場者的經驗，提供了在市場波動中保持信念、避免恐慌性賣出的寶貴見解，對於自我探索與建立穩健的投資心態極具啟發價值。</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
       <c r="A24" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -887,8 +1023,14 @@
       <c r="F24" t="str">
         <v>[EP289  七巨頭變七矮人！...] 選題新穎且具時效性，深入分析了科技巨頭的市場變化與供應鏈影響，內容含金量極高。 | [EP275 股市變賭場？巴菲特...] 選題緊扣時事熱點（巴菲特、AI、台股美股），內容深度足夠，結合了宏觀經濟分析、產業趨勢與個股案例，資訊含金量高，企劃具備高度專業性。 | [EP251國防預算暴漲 5 成...] 選題結合時事（軍工股、AI、經濟預測），數據分析詳盡，提供獨到見解，內容含金量高。</v>
       </c>
-    </row>
-    <row r="25">
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 川普對軍工股的政策轉變與市場影響】
+時間: 00:28 - 00:59
+單集: EP251國防預算暴漲 5 成！必看這五檔股票！跟者川普賺一波？
+理由: 主持人詳細解釋了川普對軍工股的看法，以及為何傳統軍工巨頭表現不佳，而無人機等輕巧裝備概念股崛起。這段內容不僅提供了市場分析的深度，也揭示了政策與產業趨勢的關聯性，展現了節目在選題和內容深度上的企劃能力。</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
       <c r="A25" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -907,8 +1049,14 @@
       <c r="F25" t="str">
         <v>[[EP0063] 50+Con...] 選題新穎，結合「第三人生大學」與「大嬸陪聊」概念，案例生動且含金量極高，具備深度思考與社會連結。 | [[EP0071] 50+Con...] 選題新穎且具深度，聚焦於二代接班與職涯轉型，來賓的個人案例生動且含金量極高，提供了獨特的視角和實用建議。 | [[EP0045] 50+Con...] 選題深入探討紫微斗數的「四化」與「殺破狼」命格，不僅新穎且具備高度的專業含金量。來賓的案例分享與對社會現象的連結，讓內容更具啟發性與實用價值。</v>
       </c>
-    </row>
-    <row r="26">
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 「大嬸陪聊」的社會價值與個人連結】
+時間: 02:44 - 03:49
+單集: [EP0063] 50+Connie大嬸 x 大嬸陪聊的第一個攤位：法律系系主任如何在實踐 68 週年校慶中替我打開校園之門 (上)
+理由: 此片段主持人Connie深入闡述「大嬸陪聊」這個概念如何回應「孤獨經濟」的社會現象，提供陪伴與解惑的價值。她將此概念與自身年齡（奔六）和人生經驗連結，創造出「Auntie Connie」的個人品牌，展現了深刻的自我探索與獨特的利基選題。內容不僅具備社會觀察的深度，也充滿個人實踐的啟發性，極具單元企劃的巧思與含金量。</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
       <c r="A26" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -927,8 +1075,14 @@
       <c r="F26" t="str">
         <v>[EP225：【非典家庭CEO】...] 選題「寄養家庭」本身就具備高度社會意義與情感深度，且從「金牌CEO」的角度切入，結合個人生命故事，內容含金量極高，案例生動且具啟發性。 | [EP218：愛自己｜放下完美執...] 選題新穎且具深度，將人類圖的流日、閘門、關係互動等複雜概念，透過具體案例和個人經驗分享，變得易於理解且富有啟發性。線上課程的設計也很有創意，結合實時運勢更新，含金量高。 | [EP219：【非典家庭CEO】...] 選題新穎，結合音樂家爸爸的育兒經驗，案例生動且內容含金量極高。</v>
       </c>
-    </row>
-    <row r="27">
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 人類圖個案解析：情緒出口與能量管理】
+時間: 15:43 - 19:09
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段來賓Anka分享了兩個具體的個案：一個是情緒中心空白、能量中心多且定義的孩童（有ADHD傾向），另一個是薦骨中心空白的投射者成人。Anka透過人類圖的視角，深入解析了他們行為背後的原因（如情緒不穩定、過度承擔），並提供了實用的建議（如增加活動、心理諮商、學習能量管理）。這些案例不僅具體生動，也展現了人類圖在理解個人特質和提供解決方案上的深度與實用價值，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
       <c r="A27" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -947,8 +1101,14 @@
       <c r="F27" t="str">
         <v>[莫菲穿搭20｜球具只是通行證？...] 選題新穎且具深度，將傳統媽祖進香活動與時尚、科技、宗教經濟等現代議題結合，案例生動具體（如三邊媽祖換裝、GPS App、AI互動），內容含金量極高，提供獨特視角。 | [莫菲穿搭27｜金曲幕後直擊！電...] 選題新穎，結合個人形象顧問的專業視角，對金曲獎紅毯造型進行深度分析，案例生動且含金量極高。 | [莫菲穿搭02｜2026流行色配...] 選題新穎，結合2026流行色與個人品牌變現，案例生動且含金量極高，具備深度與實用性。</v>
       </c>
-    </row>
-    <row r="28">
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 媽祖的時尚與宗教經濟學】
+時間: 09:44 - 11:13
+單集: 莫菲穿搭20｜球具只是通行證？Leo揭秘老闆們：白天捐救護車，晚上忙什麼？（下）
+理由: 此片段深入探討了白沙屯媽祖進香活動如何與時尚、商業經濟結合，從媽祖帽的設計、每年更換服飾，到星宇航空的聯名合作，展現了宗教文化在現代社會的創新與演變。男主持人提供了豐富的案例和獨到見解，將傳統信仰與潮流趨勢巧妙連結，女主持人則以好奇的提問引導，讓聽眾對「宗教經濟」這一新興概念有更深刻的理解，極具內容含金量與企劃深度。</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
       <c r="A28" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -967,8 +1127,14 @@
       <c r="F28" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 選題新穎，結合個人財務困境、家族背景、玄學與心智成長，案例生動且含金量極高，具備深度思考。 | [【蕭邦出任務】如何選擇適合自己...] 選題新穎，結合個人職涯轉型與自我探索，案例生動且內容含金量極高，具備深度思考與利基選題的特點。 | [幸福的人，通常「覺察力」都很強...] 選題「覺察」新穎且具深度，結合個人經驗與心理學概念，案例生動且含金量極高，對聽眾有實質啟發。</v>
       </c>
-    </row>
-    <row r="29">
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 從車禍到職涯轉型的自我探索】
+時間: 06:55 - 08:41
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
       <c r="A29" t="str">
         <v>最神單元企劃獎</v>
       </c>
@@ -987,8 +1153,14 @@
       <c r="F29" t="str">
         <v>[EP.617 《無限機器》讀後...] 選題新穎且具深度，探討AI創始人的核心動機與哲學思考，案例生動且含金量極高，引人深思。 | [EP.573 從 0 到 10...] 選題新穎，結合個人IP變現與電子報經營，案例生動且含金量極高，提供了獨特的視角和實用建議。 | [EP.607 《AI Firs...] 選題緊扣AI時代的個人與職場轉型，新穎且具備深度，來賓的經驗分享與書籍內容提供了豐富的乾貨與實用建議。</v>
       </c>
-    </row>
-    <row r="30">
+      <c r="G29" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 為什麼要做電子報？從原子習慣作者學到的啟發】
+時間: 03:52 - 05:20
+單集: EP.573 從 0 到 10 萬訂閱：我經營免費電子報六年的三個體悟
+理由: 主持人深入探討了在社群媒體發達的時代，為何仍要經營電子報的策略性思考。他以《原子習慣》作者James Clear為例，說明了電子報作為一個「不會被演算法影響」的溝通渠道，以及其在建立長期信任關係上的獨特價值。這段內容不僅提供了實用的商業洞察，也展現了選題的深度與啟發性，非常符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
       <c r="A30" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1007,8 +1179,14 @@
       <c r="F30" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 男主持人聲音清晰、有活力，中低音共鳴感佳，語速穩定度高，但口頭禪「就是」和「然後」出現頻率稍高。 | [EP174｜越省反而越窮？別把...] Andy的聲音溫暖清晰，語速穩定。好哥和蔡宇哲老師的聲音也很有特色，整體男聲表現優異。 | [EP164｜滑短影音是在浪費時...] 兩位男主持人的聲音皆具備良好的中低音共鳴。主主持人Andy口條流暢，語速穩定，但偶有口頭禪；來賓好哥的聲音則更為沉穩且富有磁性，整體播音表現優異。</v>
       </c>
-    </row>
-    <row r="31">
+      <c r="G30" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人���線特質] 節目收尾的啟發與展望】
+時間: 41:25 - 42:14
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 這段是主持人Andy的獨白，他以清晰、有力的聲線總結了本集的核心啟發，特別是關於美業從技術導向轉向思維導向的趨勢。他的語速控制得宜（約240-250字/分），發音清晰，情感真誠，沒有任何刺耳或爆音現象。這段發言展現了主持人作為「最佳男播音員」的專業素養與魅力，同時也為節目畫下了一個充滿啟發性的句點。</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
       <c r="A31" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1027,8 +1205,14 @@
       <c r="F31" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 男來賓（蔡醫師）口條流暢，聲音專業且具說服力，解釋複雜概念清晰易懂，語速雖快但穩定。 | [《財富自由心理學》：賺錢，只是...] 兩位男主持人皆表現出色。主講人雨哲口條流暢，聲音清晰溫和，語速穩定。來賓好哥聲線低沉有磁性，論述力強。整體播音實力優異。</v>
       </c>
-    </row>
-    <row r="32">
+      <c r="G31" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 節目系列介紹】
+時間: 00:13:00 - 00:16:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段主持人以清晰、快速且充滿活力的語調介紹節目系列與訪談內容，發音精準，語速雖快但內容傳達效率高，展現了其作為播音員的專業素質與魅力，為節目奠定積極的基調。</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
       <c r="A32" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1047,8 +1231,14 @@
       <c r="F32" t="str">
         <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
       </c>
-    </row>
-    <row r="33">
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 開場問候與節目主題介紹】
+時間: 00:05 - 00:15
+單集: EP251國防預算暴漲 5 成！必看這五檔股票！跟者川普賺一波？
+理由: 主持人以充滿活力和清晰的語調開場，語速雖快但發音字字分明，沒有含糊不清之處。他的聲音具有良好的中低音共鳴，給人一種專業且自信的印象，能迅速抓住聽眾的注意力，為���目定下積極的基調。</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
       <c r="A33" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1067,8 +1257,14 @@
       <c r="F33" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
       </c>
-    </row>
-    <row r="34">
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[聲線特質] 外星人對媽媽超能力的解釋】
+時間: 18:29 - 19:31
+單集: 原創歌曲〈愛喲愛你喲〉+ 我的媽媽被外星人抓走了
+理由: 在此片段中，主持人以略帶趣味的外星人聲線，清晰且富有感染力地闡述了媽媽們的「超能力」。語速保持在舒適的範圍內（約200-210字/分），發音字正腔圓，情感真摯，成功傳達了對媽媽的讚頌。整個過程無��何刺耳或爆音，展現了主持人優異的播音實力與情感渲染力。</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
       <c r="A34" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1087,8 +1283,14 @@
       <c r="F34" t="str">
         <v>[【EP330 帶著善意行動，最...] 男主持人聲音厚實有共鳴，語速穩定，發音清晰。雖然口頭禪「就是」和「那」出現頻率稍高，但整體表現專業且具親和力。 | [【EP302 把命盤變成行動藍...] 男主持人澤維的口條流暢，聲音清晰且富有中低音共鳴，語速穩定舒適，但口頭禪「那」和「我覺得」出現頻率稍高。 | [【EP312《超越我執的生活》...] 男主持人聲音厚實有共鳴，語速穩定且發音清晰。雖然口頭禪「那」、「就是」、「其實」出現頻率稍高，但整體口條流暢，情感渲染力佳。</v>
       </c>
-    </row>
-    <row r="35">
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">【被低估的領導力特質：樂觀、謙虛與公正】
+時間: 06:46 - 10:14
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人分享書中提及三個常被低估的領導力特質：樂觀（非盲目，而是看見可能）、謙虛（開放的態度）和公正。這部分內容提供了實用的領導力洞見，聲音共鳴極佳，傳達出強烈的說服力與專業感。</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
       <c r="A35" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1107,8 +1309,14 @@
       <c r="F35" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，情感表達豐富。但「對」和「然後」等口頭禪頻率稍高。</v>
       </c>
-    </row>
-    <row r="36">
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">【人生不能等，陪伴最珍貴】
+時間: 05:39 - 07:21
+單集: 人生最難的不是賺錢，而是______
+理由: 主持人分享翻看父母老照片的個人感觸，深刻體悟到時間的流逝與陪伴的重要性。這段情感真摯、語氣充滿感染力，是整集的情感高潮，提醒聽眾珍惜當下。</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
       <c r="A36" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1127,8 +1335,14 @@
       <c r="F36" t="str">
         <v>[EP.617 《無限機器》讀後...] 男主持人聲音厚實有共鳴，語速雖快但清晰穩定，口條��暢。儘管口頭禪「那」和「就是」偶爾出現，但整體表現仍屬優秀。 | [EP.573 從 0 到 10...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，情感表達真誠。口頭禪「然後」、「就是」頻率稍高，但整體不影響聆聽體驗。 | [EP.607 《AI Firs...] 主持人瓦基的口條流暢，聲音清晰且富有共鳴，語速穩定。雖然偶有「那」、「就是」等口頭禪，但不影響整體聽感���</v>
       </c>
-    </row>
-    <row r="37">
+      <c r="G36" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖且具啟發性的總結與鼓勵】
+時間: 03:56:00 - 03:59:00
+單集: EP.573 從 0 到 10 萬訂閱：我經營免費電子報六年的三個體悟
+理由: 在這段總結中，主持人以穩定且富有溫度的語調，分享了他對「真實比完美重要」的深刻體悟。他的發音清晰，語速保持在舒適的範圍內，沒有任何刺耳的爆音或噴麥。他透過真誠的聲音表情，傳達出對聽眾的理解與鼓勵，展現了極佳的情緒感染力與陪伴感，非常適合【最佳男播音員獎】與【深夜輕輕獎】的評估。</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
       <c r="A37" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1147,8 +1361,14 @@
       <c r="F37" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 男主持人聲音清晰、語速穩定，中低音共鳴感強，具有良好的渲染力。口頭禪「就是」和「然後」的頻率略高，但整體不影響流暢度。 | [我們可能會成為最殘忍的一代｜《...] 男主持��聲音共鳴感強，中低音厚實，語速穩定且清晰，情感渲染力佳，能有效傳達複雜的內容。雖然偶有口頭禪，但不影響整體專業度。</v>
       </c>
-    </row>
-    <row r="38">
+      <c r="G37" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 空虛感與幻想自傷的闡述】
+時間: 01:57:00 - 01:58:50
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 在此片段中，主持人以沉穩且富有同理心的語氣���闡述了「空虛感」極端化後，人們可能透過幻想自傷來尋求存在感或感受。儘管主題沉重，他仍保持了清晰的發音和適中的語速，聲音的溫暖共鳴感有效緩和了內容的衝擊性，展現了出色的播音實力與情緒感染力，非常適合「最佳男播音員獎」與「深夜輕輕獎」的評估。</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
       <c r="A38" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1167,8 +1387,14 @@
       <c r="F38" t="str">
         <v>[【EP39】矽谷阿雅｜貸款七百...] 男主持人聲音厚實有共鳴，語速適中，發音清晰，但口頭禪「就是」和「然後」出現頻率稍高。 | [【EP51】胡咪＆Vito大叔...] Vito大叔的口條流暢，聲音低沉有磁性，語速穩定，能有效傳達情感。偶爾的口頭禪「就是」略多但不影響整體表現。 | [【EP36】明白｜父母雙亡，獨...] 男主持人聲音厚實有共鳴，語速雖快但咬字清晰，表達流暢。口頭禪「然後」、「就是」出現頻率稍高，但整體不影響專業度。</v>
       </c>
-    </row>
-    <row r="39">
+      <c r="G38" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 主持人開場的專業聲線】
+時間: 00:08 - 00:12
+單集: 【EP39】矽谷阿雅｜貸款七百萬去美國留學值得嗎？成立 AI 公司幫男生選衣服？
+理由: 男主持人的開場白清晰、語調穩定且富有吸引力。他的聲音展現了良好的中低音共鳴和專業質感。語速適中，沒有明顯的噴麥或爆音���聲音缺陷，聽感舒適，充分展現了其播音實力。</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
       <c r="A39" t="str">
         <v>最佳男播音員獎</v>
       </c>
@@ -1187,8 +1413,14 @@
       <c r="F39" t="str">
         <v>[S0807-翻臉反擊、討好退讓...] 男主持人聲音厚實有共鳴，語速穩定且清晰。但口頭禪「然後」、「就是」出現頻率稍高。 | [S0714-【關係修復室】5個...] 男主持人聲音厚實有共鳴，語速雖快但清晰度高，��備專業播音員特質。口頭禪「就是」稍多，但整體不影響聽感。 | [S0810-戀愛腦怎麼辦？太理...] 男主持人聲音沉穩有磁性，語速穩定，發音清晰。但在對話中，「就是」與「然後」等口頭禪使用頻率稍高。</v>
       </c>
-    </row>
-    <row r="40">
+      <c r="G39" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖且具啟發性的結尾】
+時間: 52:00 - 53:23
+單集: S0807-翻臉反擊、討好退讓之外的第三條路，有彈性的邊界感 ft Ginn
+理由: 在節目結尾，男主持人以清晰、溫暖且富有磁性的聲音進行總結。語速適中（約180-190字/分），讓聽眾能輕鬆吸收最終的訊息。發音清晰，沒有任何聲音缺陷。情感傳達上充滿鼓勵與支持，完美契合了「請你繼續獎」的評估維度，為節目畫下了一個令人感到安心的句點。</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
       <c r="A40" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1207,8 +1439,14 @@
       <c r="F40" t="str">
         <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
       </c>
-    </row>
-    <row r="41">
+      <c r="G40" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 節目結尾的溫馨總結與行動呼籲】
+時間: 01:53:50 - 01:56:30
+單集: EP470｜把人放在心上的共贏哲學！因為利他而打造瑜珈生態圈 feat. ASify 創辦人 Alice
+理由: 在節目的收尾階段，主持人不姐獨自發言，總結了本集對話的精華，特別是來賓對於「自信女性」的定義。她的語速在此段保持在約204字/分，語調溫和而穩定，發音清晰，沒有任何刺耳的爆音或噴麥。她以真誠的語氣分享個人共鳴，並自然地引導聽眾參與團購及分享節目，展現了其聲音的播音實力與魅力，以及強烈的深夜安撫陪伴感，符合【最佳女播音員獎】與【深夜輕輕獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
       <c r="A41" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1227,8 +1465,14 @@
       <c r="F41" t="str">
         <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
       </c>
-    </row>
-    <row r="42">
+      <c r="G41" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖收尾與真誠感謝】
+時間: 16:15 - 16:44
+單集: 莫菲穿搭20｜球具只是通行證？Leo揭秘老闆們：白天捐救護車，晚上忙什麼？（下）
+理由: 此片段為女主持人的節目收尾，她的聲音特質在此展露無遺。語速舒適（約200字/分），發音清晰，語調溫柔且穩定，沒有任何刺耳或突兀的爆音。她以真誠的語氣感謝來賓的分享，並向聽眾傳達了溫馨的告別，展現了強烈的情緒感染力與深夜安撫陪伴感，讓聽眾在節目結束後仍能感受到一份暖意與連結，非常符合「最佳女播音員獎」與「深夜輕輕獎」的評選維度。</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
       <c r="A42" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1247,8 +1491,14 @@
       <c r="F42" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
       </c>
-    </row>
-    <row r="43">
+      <c r="G42" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫柔引導的內在療癒】
+時間: 22:33 - 25:00
+單集: EP30｜愛自己，為什麼這麼難？
+理由: 此片段為一段引導式的內在療癒練習，完美展現了主講人獨特的聲線魅力。她的語速明顯放緩（約180-190字/分），語調極其溫和、穩定且富有磁性，營造出極具安撫與陪伴感的氛圍。發音清晰，沒有任何刺耳或突兀的爆音，讓聽眾能完全放鬆並專注於內在感受。這種聲音特質對於需要心靈慰藉的聽眾而言，具有強烈的治癒效果，是「深夜輕輕獎」的絕佳範例。</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
       <c r="A43" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1267,8 +1517,14 @@
       <c r="F43" t="str">
         <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
       </c>
-    </row>
-    <row r="44">
+      <c r="G43" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 主持人開場與節目介紹】
+時間: 00:08 - 00:54
+單集: EP162 | 從房地產到MarTech：愛酷智能創辦人Jason的創業心法與人脈哲學
+理由: 主持人Becky���節目開場時，以清晰、溫暖且富有親和力的語調介紹了節目與來賓，並分享了宋家小館的創立緣由。她的語速穩定，發音清晰，聲音共鳴感佳，展現了良好的播音實力與溫馨陪伴感，且無刺耳爆音。儘管此片段長度未達建議的1.5分鐘，但已是本集最長的主持人單獨發言區間，足以展現其聲線特質。</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
       <c r="A44" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1287,8 +1543,14 @@
       <c r="F44" t="str">
         <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
       </c>
-    </row>
-    <row r="45">
+      <c r="G44" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 主持人伊柔的開場白與聲音特質】
+時間: 01:01 - 01:14
+單集: EP.61｜【說話人聲-會客室】別再逼自己當「完美父母」！挑剔孩子其實是在懲罰不完美的你
+理由: 此片段是主持人伊柔的開場白，完美展現了她獨特的聲線魅力。她的聲音清晰、明亮且充滿活力，語速雖快但咬字精準，沒有任何刺耳的音頻。她的語調充滿自信與熱情，同時又帶有溫馨的陪伴感，讓聽眾在節目一開始就能感受到被歡迎與被理解。這段開場白不僅有效傳達了節目的核心理念，也充分體現了她作為女播音員在聲音特質上的優勢，非常符合「溫馨陪伴感」的評估維度。</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
       <c r="A45" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1307,8 +1569,14 @@
       <c r="F45" t="str">
         <v>[#801 市場震盪 17000...] 女主持人聲音清晰、溫暖且具共鳴，語速穩定舒適，情緒感染��佳，但偶有贅字。 | [#809  買股票還在到處問明...] Cindy2聲音圓潤清晰，語速適中，語調親和，具備溫馨陪伴感，引導能力強。 | [#798 害怕投資賠錢？不用天...] 兩位女主持人聲音清晰、語速快但穩定，高音域圓潤且具備溫馨陪伴感，無刺耳爆音。主講人Sandy的語速較快，但整體表現優異。</v>
       </c>
-    </row>
-    <row r="46">
+      <c r="G45" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲���特質] 股市新手的心情與市場的不可預測性】
+時間: 01:47 - 03:38
+單集: #801 市場震盪 17000 點，費半重挫、台股回檔，你該急著逃，還是重新檢查資產配置？給剛進場投資人的一堂情緒與現金流課
+理由: 在這段較長的片段中，主持人溫和地談論了大量新進投資者湧入市場，以及他們在市場修正時所經歷的情緒波動。她的聲音始終清晰、沉穩且富有同理心，尤其在安撫聽眾「不要擔心」並理解他們的焦慮時，語氣更顯真誠。語速穩定舒適，讓聽眾能輕鬆理解內容，沒有任何刺耳的音調或錄音缺陷。她的表達傳達出強烈的溫暖陪伴感和信任感，充分展現了「最佳女播音員獎」的實力，並營造出適合「深夜輕輕獎」的氛圍。</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
       <c r="A46" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1327,8 +1595,14 @@
       <c r="F46" t="str">
         <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
       </c>
-    </row>
-    <row r="47">
+      <c r="G46" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖總結與「教學相長」的理念】
+時間: 26:21 - 26:59
+單集: ep11. Z世代難搞嗎？用對方法其實很好懂！ft.張裕昌 奧美公關董事總經理
+理由: 在節目尾聲，女主持人丁菱娟獨自總結，語速約295字/分，清晰且舒適。她的聲線溫暖而富有感染力，語調真誠，強調主管應以開放心態與Z世代溝通，提供舞台並從中學習，達到「教學相長」。這段發言展現了她作為主持人的專業播音實力，語氣充滿鼓勵與陪伴感，無任何刺耳或爆音，非常符合【最佳女播音員獎】與【深夜輕輕獎】的評選標準。</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
       <c r="A47" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1347,8 +1621,14 @@
       <c r="F47" t="str">
         <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
       </c>
-    </row>
-    <row r="48">
+      <c r="G47" t="str" xml:space="preserve">
+        <v xml:space="preserve">【男性溝通的獨特方式：肩並肩的陪伴】
+時間: 07:51 - 08:48
+單集: [EP0054] 50+Connie大嬸 x 中年低谷的轉身練習：Vito 大叔教你從失業到重啟人生 (下)
+理由: 這段深入剖析了男性在社交中偏好「肩並肩」而非「面對面」的溝通模式，透過共同勞動自然地建立連結與情感交流，解釋了「男士工棚」成功的心理基礎，極具洞察力。</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
       <c r="A48" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1367,8 +1647,14 @@
       <c r="F48" t="str">
         <v>[#95 ▍ 冷戰半年怎麼破冰？...] 女主持人聲音清晰、語速穩定且富有能量，高音域圓潤，雖語速較快但仍具陪伴感，發音無刺耳感。 | [#99 ▍別讓金錢焦慮，成了教...] 女主持人紫琳口條流暢，聲音清晰溫暖，語速穩定且富有親和力，高音域圓潤，給人溫馨陪伴感。 | [#93 ▍自學，不是逃避的出口...] 女主持人紫菱的口條流暢，聲音清晰溫暖，語速穩定且富有情感，高音域圓潤無刺耳感，具備極佳的陪伴與治癒特質。</v>
       </c>
-    </row>
-    <row r="49">
+      <c r="G48" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖而有力的結語與下集預告】
+時間: 19:00 - 20:30
+單集: #95 ▍ 冷戰半年怎麼破冰？「撩夫神技」大公開- 神老師愛的秘訣 - 愛你現在的樣子 -上集
+理由: 此片段為主持人獨自發言的結尾與下集預告。主持人���速雖快但發音清晰，聲音充滿活力與親和力，展現了其作為女播音員的專業素養。她的語調溫暖而富有感染力，能夠有效傳達節目的核心價值，並成功激發聽眾對下一集的期待。整個過程無任何刺耳或突兀的爆音，聲音共鳴感佳，展現了優異的播音實力。</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
       <c r="A49" t="str">
         <v>最佳女播音員獎</v>
       </c>
@@ -1387,8 +1673,14 @@
       <c r="F49" t="str">
         <v>[#336 #Zoey｜你覺得自...] 女主持人聲音清晰、語速穩定，高音域圓潤且富有陪伴感��口條流暢，整體播音實力優異。 | [#我，是誰？S2E2｜為什麼越...] 主持人Zoe的口條流暢，聲音清晰且語速穩定，高音域圓潤且富有陪伴感，情緒感染力佳。 | [#我，是誰？S2E3｜過度依賴...] 主持人Zoe的語速穩定，發音清晰，語調溫和，預期能給予聽眾溫馨的陪伴感，且在引導對話時展現專業度。</v>
       </c>
-    </row>
-    <row r="50">
+      <c r="G49" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖且清晰的開場】
+時間: 00:00:00 - 00:03:00
+單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
+理由: 這個開場片段完美展現了主講人卓越的播音實力與魅力。她的發音清晰，語速約在 180-190 字/分之間，非常舒適。聲音溫暖且富有情感，帶有強烈的深夜安撫陪伴感，沒有任何刺耳或爆音。她以真誠的語氣歡迎聽眾，立即建立起親和力，非常符合「最佳女播音員獎」與「深夜輕輕獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
       <c r="A50" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1402,13 +1694,19 @@
         <v>五吉郎</v>
       </c>
       <c r="E50">
-        <v>8.7715</v>
+        <v>9.45</v>
       </c>
       <c r="F50" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 結尾有明確呼籲聽眾行動，力道足夠，能有效催化聽眾實踐。 | [EP174｜越省反而越窮？別把...] 結尾有明確的行動呼籲，鼓勵聽眾訂閱、留言、並嘗試微小行動，力道足夠。 | [EP164｜滑短影音是在浪費時...] 節目中多次提及來賓的新書，並在結尾有明確的行動呼籲，但力道尚可加強，未達到極強的催化效果。</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>[EP133｜顛覆你對美容業的想...] 主持人與來賓在節目中明確推廣了「養膚管理」的理念、來賓的相關課程以及她自己的 Podcast 節目。來賓詳細分享了她從排斥美容到成為專業養膚師的轉變，以及她獨特的教學方法（如彩虹筆記法），這些內容極具說服力，讓人對她的專業知識和服務產生高度興趣。主持人也適時提及來賓的節目，整體而言，聽眾聽完會很想進一步了解並可能購買相關課程或服務。 | [EP174｜越省反而越窮？別把...] 節目中多次且自然地提及兩位來賓的著作《財富自由心理學》和《花錢有道》，並將書中的核心概念融入對談，讓聽眾在理解內容的同時，也對書籍產生高度興趣。尤其在結尾處，主持人與來賓分享了具體的「寫下五件成果」的行動，並強調這與書中理念的連結，有效激發了聽眾購買書籍以深入學習的意願。雖然沒有直接的「立即購買」指令，但其潛移默化的推坑效果非常顯著。 | [EP164｜滑短影音是在浪費時...] 節目中對好哥新書《好會讀書》的推廣非常到位且貫穿始終。主持人與來賓不斷引用書中核心理念，並提供具體實用的閱讀技巧（如快速瀏覽四步驟、兩分鐘閱讀法），將閱讀重新定義為「一場關於自由的修煉」，有效解決聽眾對閱讀的痛點。透過個人故事和生活化比喻（如榴槤、漫畫），讓書中概念更具吸引力與說服力，讓人聽完會產生強烈的購買慾望，想深入了解如何將這些理念應用於自身。</v>
+      </c>
+      <c r="G50" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 來賓電商逆襲的核心思考】
+時間: 04:43 - 06:56
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 此片段詳細闡述了來賓從代理產品轉向自創品牌的「悲慘故事」，揭示了市場亂象（經銷商跳過代理、價格戰）如何迫使她做出戰略轉變。內容充滿創業洞察，展現了對市場動態和個人價值的深刻理解。主持人Andy的問題引導來賓揭示了其核心動機，使這段敘述極具啟發性，非常適合評選「最神單元企劃」與「自我探索獎」。</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
       <c r="A51" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1416,19 +1714,25 @@
         <v>2</v>
       </c>
       <c r="C51" t="str">
-        <v>精算媽咪的家計簿</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D51" t="str">
-        <v>精算媽咪的家計簿｜珊迪兔</v>
+        <v>梁哲維</v>
       </c>
       <c r="E51">
-        <v>8.75</v>
+        <v>9.25</v>
       </c>
       <c r="F51" t="str">
-        <v>[#801 市場震盪 17000...] 結尾有明確的行動呼籲，引導聽眾加入社群或參與課程，力道足夠且具體。 | [#809  買股票還在到處問明...] 結尾有明確的課程優惠與開戶行動呼籲，力道足夠且具體，能有效促使聽眾行動。 | [#798 害怕投資賠錢？不用天...] 結尾有明確呼籲聽眾行動，推廣課程並提供折扣碼，力道足夠且資訊完整。</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>[【EP330 帶著善意行動，最...] 主持人與來賓在節目中詳細介紹了「黑右雞腳」這項具體商品，從其70年的歷史、製作理念、到如何透過線上平台與宅配服務讓全台聽眾都能品嚐。來賓們生動描述了商品的特色、包裝方式及食用情境（如露營、爬山），並分享了許多與顧客互動的溫馨故事，這些都大大提升了商品的吸引力。主持人也明確表示會將購買連結放在資訊欄，整體勸敗說服力極強，讓人聽完產生立即購買的衝動。 | [【EP302 把命盤變成行動藍...] 主持人澤維與來賓葛道老師在節目中多次且明確地推廣葛道老師的命理諮詢服務與課程。葛道老師詳細介紹了其60頁PPT的全面分析、多種命理工具的整合運用，以及線上線下服務的便利性，展現了專業度與價值。澤維則以自身體驗強力背書，強調服務的「物超所值」與「充滿希望」，並承諾提供預約資訊，極具說服力，讓人聽完有強烈的預約衝動。 | [【EP312《超越我執的生活》...] 主持人以深入淺出的方式，詳細闡述了書籍《超越我執的生活》的核心概念，並強調其對個人成長、情緒管理及人際關係的益處。雖然沒有直接的購買指令或連結，但透過對書中理念的強力推廣，成功地激發了聽眾對該書內容的興趣與求知慾，讓人產生想進一步閱讀該書以實踐這些理念的衝動，間接達到推坑效果。</v>
+      </c>
+      <c r="G51" t="str" xml:space="preserve">
+        <v xml:space="preserve">【「主角模式」核心概念闡述】
+時間: 00:00 - 00:49
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
+      </c>
+    </row>
+    <row r="52" xml:space="preserve">
       <c r="A52" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1436,19 +1740,25 @@
         <v>3</v>
       </c>
       <c r="C52" t="str">
-        <v>哇賽心理學</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D52" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>精算媽咪的家計簿｜珊迪兔</v>
       </c>
       <c r="E52">
-        <v>8.7215</v>
+        <v>9.25</v>
       </c>
       <c r="F52" t="str">
-        <v>[[深度]瘦瘦針是神藥？醫師教你...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動和提供回饋，具備一定的催化力。 | [《財富自由心理學》：賺錢，只是...] 節目結尾明確呼籲聽眾購買書籍與參與實體活動，行動呼籲清晰且具催化力。 | [手總是停不下來？那是焦慮在尋找...] 結尾有明確的行動呼籲，鼓勵聽眾在社群平台互動，但催化力道尚有提升空間。</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>[#801 市場震盪 17000...] 主持人明確推廣一堂價值不菲的「老屋改造」直播課程，並提供其學員免費參與的專屬福利。她清楚說明了如何成為學員以獲得此福利，並設定了明確的截止日期，有效激發了聽眾對課程的興趣和參與的緊迫感。雖然需要先成為學員，但其推坑的說服力與具體性仍屬上乘。 | [#809  買股票還在到處問明...] 主持人對於阮慕驊老師的「獲利加速系統」課程推廣非常具體且有說服力。節目中詳細介紹了課程內容、提供的工具（AI模組、專屬網站），並強調了其解決聽眾痛點（選股、風險管理、資產配置）的能力。透過實際案例（如嘉碧琪股票）和情感連結（為家庭財務規劃），加上限時優惠與折扣碼，成功營造出購買的急迫感與價值感，讓人聽完有強烈的購買衝動。 | [#798 害怕投資賠錢？不用天...] 節目中兩位主持人明確且詳細地介紹了「聰明主婦」的投資課程，從課程內容、學習目標到實際操作的細節，都進行了深入的說明。特別是提供了折扣碼，直接且有效地鼓勵聽眾報名，勸敗說服力十足，讓人聽完對課程產生高度興趣。</v>
+      </c>
+      <c r="G52" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 股市下跌時的情緒管理與長期投資心法】
+時間: 03:07 - 04:38
+單集: #801 市場震盪 17000 點，費半重挫、台股回檔，你該急著逃，還是重新檢查資產配置？給剛進場投資人的一堂情緒與現金流課
+理由: 此片段全面探討了市場下跌時投資者的情緒管理。主持人深入分析了新進投資者常見的後悔與恐懼心理，強調市場的不可預測性，並引導聽眾思考投資標的的基本面價值與長期成長潛力。她透過對比長期持有者與近期進場者的經驗，提供了在市場波動中保持信念、避免恐慌性賣出的寶貴見解，對於自我探索與建立穩健的投資心態極具啟發價值。</v>
+      </c>
+    </row>
+    <row r="53" xml:space="preserve">
       <c r="A53" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1456,19 +1766,25 @@
         <v>4</v>
       </c>
       <c r="C53" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>不敗教主陳重銘</v>
       </c>
       <c r="D53" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>不敗教主-陳重銘</v>
       </c>
       <c r="E53">
-        <v>8.65</v>
+        <v>9.15</v>
       </c>
       <c r="F53" t="str">
-        <v>[EP225：【非典家庭CEO】...] 結尾有明確的行動呼籲，鼓勵聽眾點擊連結或撥打專線了解寄養家庭資訊，力道足夠且具體。 | [EP218：愛自己｜放下完美執...] 節目結尾的行動呼籲明確，針對線上課程提供了專屬優惠碼，具體且有吸引力，能有效促使聽眾採取行動。 | [EP219：【非典家庭CEO】...] 結尾有明確呼籲聽眾行動，力道足夠，鼓勵聽眾參與動物音樂會。</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>[EP611 00998A(主動...] 主持人針對特定金融商品（00988A ETF）進行了極為詳細且具說服力的推廣。他不僅清楚闡述了該ETF的投資標的、稅務優勢、分散風險的特性，更提供了申購的具體時間與方式，並預先回應了潛在的疑慮（如管理費），有效激發聽眾的購買意願。其勸敗說服力極強，讓人聽完後會產生想進一步了解或購買的衝動。 | [EP628昇陽半導體(8028...] 主持人詳細說明了其付費課程的內容（遺產稅節稅、開設投資公司），明確指出課程能解決聽眾的痛點，並強調了「加量不加價」和「免費補課」的優惠，最後以「優惠即將結束」製造購買的急迫性，整體推銷具體且說服力強。 | [EP621《富媽媽 窮媽媽》第...] 主持人陳老師在節目中多次明確推銷其著作《富媽媽窮媽媽》，並強調購買書籍不僅能獲得寶貴的理財知識，更能支持他將版稅捐贈公益。他透過生動的案例（小明與小華的故事）具體說明書中「財富分身」的核心概念，並強調提早開始的重要性，有效激發聽眾對該書內容的好奇與購買慾望。他還提及書本價格便宜，進一步降低購買門檻，勸敗說服力極強。</v>
+      </c>
+      <c r="G53" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 金融股的多元獲利模式與經濟成長關聯】
+時間: 00:53 - 02:21
+單集: EP611 00998A(主動復華金融股息)鎖定歐洲大型金融股，優缺點在哪裡呢？
+理由: 此片段主持人深入剖析金融股的多元獲利模式，從經濟成長對銀行業務的帶動（交易量、市值擴大、房貸餘額）、到信用卡刷卡手續費、ETF經理費及保險業務等，全面且有條理地闡述金融業的穩健獲利基礎。內容含金量高，展現了對金融市場的深刻理解與精準的選題企劃能力，對於評選【最神單元企劃】與【自我探索獎】極具參考價值。</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
       <c r="A54" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1476,19 +1792,25 @@
         <v>5</v>
       </c>
       <c r="C54" t="str">
-        <v>下一本讀什麼？</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D54" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>蕭邦</v>
       </c>
       <c r="E54">
-        <v>8.6</v>
+        <v>9.15</v>
       </c>
       <c r="F54" t="str">
-        <v>[EP.617 《無限機器》讀後...] 結尾有明確呼籲聽眾訂閱電子報與節目，行動呼籲力道足夠且自然。 | [EP.573 從 0 到 10...] 結尾有明確呼籲聽眾填寫問卷和分享電子報，力道足夠且具體。 | [EP.607 《AI Firs...] 節目開頭與結尾都有明確且具說服力的行動呼籲，引導聽眾參與社群或閱讀書籍，催化力道足夠。</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>[【蕭邦出任務】負債 900 多...] 主持人Aaron透過自身與他人的親身經歷，詳細描述了某個「神奇的課程」如何幫助他們從負債累累走向財務自由，甚至累積了八位數的存款。他分享的具體數字和轉變過程極具說服力，讓人聽完後對該課程產生強烈的好奇心與購買衝動，儘管課程名稱未直接提及，但其推坑效果顯著。 | [幸福的人，通常「覺察力」都很強...] 主持人透過自身經歷，強烈且具說服力地闡述了「心理諮商」與「覺察」對個人成長與情緒管理的重要性。雖然沒有直接推銷特定商品或服務，但其真誠的分享與轉變，讓人聽完後會產生強烈的衝動，想去探索或投資相關的自我成長服務或課程，以達到類似的自我提升效果。這種間接但有效的勸敗力道，足以給予高分。</v>
+      </c>
+      <c r="G54" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 從車禍到職涯轉型的自我探索】
+時間: 06:55 - 08:41
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
       <c r="A55" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1496,19 +1818,25 @@
         <v>6</v>
       </c>
       <c r="C55" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D55" t="str">
-        <v>GK爸爸</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E55">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="F55" t="str">
-        <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 開頭與結尾的行動呼籲明確，引導聽眾分享歌曲並加入VIP社團，具備一定的催化力。 | [春暖花開小旅行...] 開場有明確的訂閱、關注與五星評價呼籲，力道足夠且位置恰當。 | [【QQ偵探：鳳梨酥失竊案 上集...] 結尾有明確的行動呼籲，引導聽眾期待下一集，催化力足夠。</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>[EP.617 《無限機器》讀後...] 主持人明確提及自身線上課程「AI 瓦基第二大腦」的銷售佳績（三天突破兩千人），並引導聽眾前往資訊欄了解更多課程內容。這種以成功案例為基礎的推廣方式，有效激發了聽眾的好奇心與購買意願，勸敗說服力強勁。 | [EP.607 《AI Firs...] 主持人瓦基在節目開頭明確且具體地推廣其付費線上社群「獨家攻略」，包含招募時間、名額限制及社群特色，並引導聽眾至資訊欄了解詳情，勸敗說服力強。節目中也多次提及來賓Sting的新書《AI First 自我升級革命》，並由來賓親自鼓勵聽眾購買，整體推坑力道十足。</v>
+      </c>
+      <c r="G55" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 為什麼要做電子報？從原子習慣作者學到的啟發】
+時間: 03:52 - 05:20
+單集: EP.573 從 0 到 10 萬訂閱：我經營免費電子報六年的三個體悟
+理由: 主持人深入探討了在社群媒體發達的時代，為何仍要經營電子報的策略性思考。他以《原子習慣》作者James Clear為例，說明了電子報作為一個「不會被演算法影響」的溝通渠道，以及其在建立長期信任關係上的獨特價值。這段內容不僅提供了實用的商業洞察，也展現了選題的深度與啟發性，非常符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="56" xml:space="preserve">
       <c r="A56" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1516,19 +1844,25 @@
         <v>7</v>
       </c>
       <c r="C56" t="str">
-        <v>文森說書</v>
+        <v>宋家小館</v>
       </c>
       <c r="D56" t="str">
-        <v>文森說書</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E56">
-        <v>8.5875</v>
+        <v>9.1</v>
       </c>
       <c r="F56" t="str">
-        <v>[這一集我準備了兩個月，但是太值...] 節目結尾有明確且具說服力的行動呼籲，鼓勵聽眾購買書籍並使用優惠連結，具有一定的實踐催化力。 | [我們可能會成為最殘忍的一代｜《...] 結尾的行動呼籲非常具體且真誠，主持人分享個人實踐，有效激勵聽眾思考並採取行動，催化力強。</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>[EP162 | 從房地產到Ma...] 節目中來賓詳細闡述了企業導入 AI 的痛點與解決方案，並明確指出其公司「愛酷智能」的價值在於協助企業定義問題並提供系統、AI 與服務。雖然沒有直接的「購買」呼籲，但整個討論過程極具說服力，讓人深刻理解導入 AI 的必要性以及尋求專業協助的重要性，有效推廣了其付費服務的價值。 | [EP191 | 《我到日本當漁...] 主持人明確地推廣了來賓的著作《我到日本當漁夫》，節目內容圍繞著書籍主題，透過深入訪談來賓在日本當漁夫的獨特經歷、挑戰與心路歷程，成功地激發聽眾對這本書的好奇心與購買慾。主持人對書籍內容的提問，以及來賓的分享，都讓這本書的吸引力大大提升，屬於非常具體的商品推廣。 | [EP182 | 聽見身體的聲音...] 主持人與來賓的互動，成功地將頌缽音療的課程與服務推廣給聽眾。主持人分享了自己親身體驗後的放鬆與入睡經驗，極具說服力。來賓詳細解釋了頌缽對腦波、情緒、身體疼痛及脈輪的益處，並提供了具體的課程資訊與聯絡方式。節目結尾的現場頌缽示範，更是直接讓聽眾感受其效果，大大提升了購買或體驗的衝動。</v>
+      </c>
+      <c r="G56" t="str" xml:space="preserve">
+        <v xml:space="preserve">【闆娘Becky的轉運概念】
+時間: 00:53 - 01:41
+單集: EP174 | 打造福氣好運的三部曲
+理由: 主持人以親切的語氣開場，透過洗床單的日常小事引導出「轉運」的核心概念，迅速拉近與聽眾的距離，引人入勝。</v>
+      </c>
+    </row>
+    <row r="57" xml:space="preserve">
       <c r="A57" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1536,19 +1870,25 @@
         <v>8</v>
       </c>
       <c r="C57" t="str">
-        <v>夢想家說股事</v>
+        <v>郝聲音</v>
       </c>
       <c r="D57" t="str">
-        <v>美股夢想家</v>
+        <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E57">
-        <v>8.5715</v>
+        <v>9.05</v>
       </c>
       <c r="F57" t="str">
-        <v>[EP289  七巨頭變七矮人！...] 節目開頭和結尾都有明確且具吸引力的行動呼籲，鼓勵聽眾留言領取資訊或加入社群。 | [EP275 股市變賭場？巴菲特...] 節目結尾明確且多次呼籲聽眾加入社群、訂閱APP，並提供限時優惠，行動呼籲的強度與實踐催化力足夠。 | [EP251國防預算暴漲 5 成...] 節目結尾有推薦商品和下週節目預告，但行動呼籲的直接性與催化力中等。</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>[郝聲音：（下） 莊鈞涵（Car...] 本集節目圍繞著一本名為《專攻20% 各科高分破解法》的書籍展開，主持人與兩位作者（來賓）深入探討書中的學習方法與理念。節目中不斷強調書中觀念如何解決學習痛點，並透過實際案例（如羅漢腳、論語解讀）證明其有效性。雖然沒有直接的「立即購買」呼籲，但整個節目內容都在強力推銷這本書所提供的解決方案，讓聽眾感受到其價值並產生購買的衝動。結尾再次提及書名，強化了推坑效果。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目中明確提及並詳細闡述了多種具體的付費服務與產品，包括企業導讀（B2B）、線上課程與「閱讀人生大學」（B2C），以及與政府單位的合作案（B2G）。主持人也主動引導來賓分享「變現」的策略，來賓的說明清晰且具體，展現了這些服務的實際可行性。雖然沒有直接的「立即購買」呼籲，但其說服力在於將這些服務呈現為價值交換的自然延伸，讓人聽完對「閱讀人」所提供的服務產生高度興趣與信任感。 | [郝聲音：成為人生更自由的「精銳...] 本集節目從頭到尾都圍繞著「精銳IP 旗艦變現流」這堂課程的核心概念、價值主張、課程內容與目標受眾進行深入探討。主持人與來賓不斷強調課程能幫助聽眾解決流量迷思、成本過高、定位不清等痛點，並提供具體的解決方案，如「活得下、活得久、活得好」的理念、建立信任資產、運用AI自動化、以及共學社群的陪伴。課程的推銷非常自然地融入在對話中，而非生硬的廣告，讓人聽完後對課程產生強烈的好奇心與購買衝動。雖然沒有直接的購買連結或促銷語句，但其內容的說服力已達到極高水準。</v>
+      </c>
+      <c r="G57" t="str" xml:space="preserve">
+        <v xml:space="preserve">【Threads平台「內容為王」的獨特魅力】
+時間: 05:13 - 06:02
+單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
+理由: 來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
       <c r="A58" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1556,19 +1896,25 @@
         <v>9</v>
       </c>
       <c r="C58" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D58" t="str">
-        <v>梁哲維</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E58">
-        <v>8.5715</v>
+        <v>9</v>
       </c>
       <c r="F58" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目結尾��確提供了來賓滷味店的線上購買方式，並承諾將連結放在資訊欄，行動呼籲清晰且實用。 | [【EP302 把命盤變成行動藍...] 結尾有明確的行動呼籲，引導聽眾尋找來賓的服務，但力道可再加強。 | [【EP312《超越我執的生活》...] 結尾明確呼籲聽眾實踐「覺察」與「臨在」，並推薦書籍，行動呼籲清晰且與內容緊密結合，具備一定的實踐催化力。</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>[EP470｜把人放在心上的共贏...] 主持人與來賓在節目中對「S-Fai」品牌及其瑜伽服飾產品進行了深入且富有情感的介紹。主持人親身穿著產品並分享了極具說服力的個人體驗，詳細描述了布料的舒適度、設計理念，以及產品如何與自我探索、自在生活等哲學概念連結。來賓也清晰闡述了品牌的核心價值與公益行動，進一步提升了品牌的吸引力。節目尾聲，主持人明確提及與S-Fai合作的團購連結，並鼓勵聽眾前往實體店面體驗，這些具體的行動呼籲，加上前面建立的情感連結與產品說服力，讓人產生強烈的購買慾望。 | [EP433｜【中年轉型】從矽谷...] 主持人與來賓的對談，巧妙地將來賓的專業知識與其著作（如節目開頭提及的《半熟人格》）融入其中。雖然沒有直接的「購買」呼籲，但整集節目透過來賓的親身經歷與對MBTI的深入解析，強力說服聽眾理解自我性格對於人生轉型的重要性。主持人結尾的總結，更將MBTI的應用價值具體化，讓聽眾產生強烈的動機去探索相關知識，進而可能尋求來賓的書籍或服務，屬於高說服力的間接推坑。 | [EP466｜拒絕被朝九晚五綁架...] 節目開頭的廣告明確推廣「股票王 Michael 洪老師」的付費訂閱方案，詳細說明了課程內容與效益，如掌握市場知識、超盤技巧、每日盤中資訊等，直接且具說服力地鼓勵聽眾付費訂閱以達成財富自由，符合推坑具體付費服務的標準。</v>
+      </c>
+      <c r="G58" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] Alice的公益理念與實踐】
+時間: 04:39 - 06:29
+單集: EP470｜把人放在心上的共贏哲學！因為利他而打造瑜珈生態圈 feat. ASify 創辦人 Alice
+理由: 此片段深入探討了來賓Alice從2023年起與罕見疾病基金會合作，提供瑜伽療癒課程及贊助瑜伽墊的公益行動。主持人提問其動機，Alice分享她認為企業家應承擔社會責任，並強調她希望透過實際參與而非僅是捐款來幫助病友與家屬，讓他們感受到社會的接納與支持。這段對話展現了深刻的企業社會責任觀點與個人價值觀的結合，極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="59" xml:space="preserve">
       <c r="A59" t="str">
         <v>聽完馬上獎 (不然現在獎/推坑王獎)</v>
       </c>
@@ -1576,19 +1922,25 @@
         <v>10</v>
       </c>
       <c r="C59" t="str">
-        <v>分手的99個理由</v>
+        <v>能量黑客</v>
       </c>
       <c r="D59" t="str">
-        <v>胡咪老師</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E59">
-        <v>8.55</v>
+        <v>9</v>
       </c>
       <c r="F59" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 結尾的行動呼籲明確且具體，鼓勵聽眾尋求協助，催化力道足夠。 | [S4.EP8｜我不想再跟你生活...] 節目開頭與結尾的行動呼籲明確，鼓勵聽眾訂閱、留言並購買推薦書籍，具備一定的催化力。 | [S4.EP14｜有些人沒有成為...] 節目結尾提供了多種行動呼籲，包括訂閱、留言互動、支持節目等，明確且具備一定的催化力，鼓勵聽眾參與。</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 節目主軸圍繞著「能量黑客」的「精力管理」概念，主持人透過提供具體且實用的建議（如運動、睡眠、情緒管理、決策方法），有效地建立其專業形象與品牌價值。雖然節目中未直接推銷特定付費商品或課程，但其內容的說服力與實用性，足以激發聽眾對其品牌理念產生高度認同，進而產生進一步探索或購買相關服務的潛在衝動。 | [別人眼中的高光時刻，卻是我最耗...] 主持人與來賓皆分享了透過付費課程（如NLP、自我探索、情緒排解、Tony Robbins的啟發）來解決個人困境的經驗。雖然沒有直接推銷特定商品，但其真誠的分享與課程帶來的顯著轉變，極具說服力，讓人聽完會產生強烈想去探索類似課程或服務的衝動。 | [別急著振作！高能量的人允許自己...] 節目內容本身即是來賓與主持人專業知識的展現，雖然沒有直接的「購買」呼籲，但來賓被介紹為「高能量溝通作者」與「講師」，其分享的實用技巧與心法，會讓聽眾產生強烈的好奇心與信任感，進而主動搜尋其相關書籍、課程或服務，達到間接且高效的推坑效果。</v>
+      </c>
+      <c r="G59" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 健康壽命的「1」與「0」】
+時間: 02:25 - 03:09
+單集: 新年特輯—火馬年續航攻略：吃睡練＋情緒＋決策＋意義感｜能量黑客S3EP11
+理由: 此片段男主持人清晰闡述了健康是所有財富與快樂的基礎（「1」與「0」的比喻），並強調運動與睡眠對於延長健康壽命的重要性。女主持人適時的幽默插話（「睡眠綁著運動，你知道很多不運動的人等一下會來那個K你」）展現了雙人主持的良好默契與節目趣味性，同時也強化了內容的實用性與啟發性，非常符合【最神單元企劃】與【自我探索獎】的評選維度。</v>
+      </c>
+    </row>
+    <row r="60" xml:space="preserve">
       <c r="A60" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1607,8 +1959,14 @@
       <c r="F60" t="str">
         <v>[EP225：【非典家庭CEO】...] 寄養家庭議題雖然非絕對冷門，但節目深入探討其背後的挑戰、家庭動員與個人成長，提供了獨特的視角和豐富的細節，論述完整且具深度。 | [EP218：愛自己｜放下完美執...] 人類圖本身即為利基市場，本集更深入探討流日、閘門與關係互動等細節，論述完整且具專業度，滿足了特定聽眾群的深度需求。 | [EP219：【非典家庭CEO】...] 雖然育兒是廣泛議題，但從專業音樂家角度切入，並結合獨特的動物音樂會推廣，使其具備高度利基市場價值。</v>
       </c>
-    </row>
-    <row r="61">
+      <c r="G60" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 人類圖個案解析：情緒出口與能量管理】
+時間: 15:43 - 19:09
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段來賓Anka分享了兩個具體的個案：一個是情緒中心空白、能量中心多且定義的孩童（有ADHD傾向），另一個是薦骨中心空白的投射者成人。Anka透過人類圖的視角，深入解析了他們行為背後的原因（如情緒不穩定、過度承擔），並提供了實用的建議（如增加活動、心理諮商、學習能量管理）。這些案例不僅具體生動，也展現了人類圖在理解個人特質和提供解決方案上的深度與實用價值，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="61" xml:space="preserve">
       <c r="A61" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1627,8 +1985,14 @@
       <c r="F61" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
       </c>
-    </row>
-    <row r="62">
+      <c r="G61" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 美國健康政策與生活型態結合】
+時間: 01:50:00 - 01:53:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段來賓深入探討美國最新的健康政策，如何將藥物治療與生活型態調整結合，並提出「Balance」計畫。這不僅展現了選題的深度與前瞻性，也提供了超越單純藥物討論的宏觀視角，極具單元企劃與啟發價值。</v>
+      </c>
+    </row>
+    <row r="62" xml:space="preserve">
       <c r="A62" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1647,8 +2011,14 @@
       <c r="F62" t="str">
         <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
       </c>
-    </row>
-    <row r="63">
+      <c r="G62" t="str" xml:space="preserve">
+        <v xml:space="preserve">【闆娘Becky的轉運概念】
+時間: 00:53 - 01:41
+單集: EP174 | 打造福氣好運的三部曲
+理由: 主持人以親切的語氣開場，透過洗床單的日常小事引導出「轉運」的核心概念，迅速拉近與聽眾的距離，引人入勝。</v>
+      </c>
+    </row>
+    <row r="63" xml:space="preserve">
       <c r="A63" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1667,8 +2037,14 @@
       <c r="F63" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
       </c>
-    </row>
-    <row r="64">
+      <c r="G63" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 疫情下「受助者變助人者」的深刻轉變】
+時間: 01:05:55 - 01:09:00
+單集: 從流浪到回家：浪人食堂的溫柔守護與陪伴 ft.蔡明潔店長
+理由: 明潔在此段闡述了浪人食堂在疫情期間，如何從單純的提供餐食，轉變為讓受助者也能參與助人，進而產生強烈的成就感和歸屬感。這個核心理念不僅獨特，更深入探討了人性的光輝與潛能，極具啟發性，完美符合「最神單元企劃」和「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="64" xml:space="preserve">
       <c r="A64" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1687,8 +2063,14 @@
       <c r="F64" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
       </c>
-    </row>
-    <row r="65">
+      <c r="G64" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 從車禍到職涯轉型的自我探索】
+時間: 06:55 - 08:41
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="65" xml:space="preserve">
       <c r="A65" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1707,8 +2089,14 @@
       <c r="F65" t="str">
         <v>[跟長輩一樣就能學會AI？陶韻智...] 議題具前瞻性與專業性，對特定受眾（如AI使用者、職場工作者）有高度吸引力，論述完整。 | [再不用證明自己給誰看 feat...] 節目聚焦於女性理財與自我成長，並結合家族企業轉型等議題，在特定受眾群體中具有較高的議題稀有度與論述完整度。 | [好像很爽，我們也去當個旅遊作家...] 節目聚焦於旅遊作家的職業生涯，是一個相對利基且被深入探討的市場，論述完整。</v>
       </c>
-    </row>
-    <row r="66">
+      <c r="G65" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] AI First 的核心挑戰與人類慣性】
+時間: 02:20 - 03:30
+單集: 跟長輩一樣就能學會AI？陶韻智老師的反慣性AI學《 AI First 自我升級革命》
+理由: 老師深入剖析了「AI First」概念的核心挑戰，解釋了人類為何難以直接信任AI，而是傾向於尋求專家或傳統知識來源。他從人類的慣性思維（如過去50年的學習模式）出發，闡述了AI作為新型知識工作者的獨特地位，以及在資訊交錯的時代，人們難以判斷AI權威性的困境。這段內容不僅提供了深刻的觀點，也為後續的討論奠定了堅實的理論基礎，展現了單元企劃的深度與啟發性。</v>
+      </c>
+    </row>
+    <row r="66" xml:space="preserve">
       <c r="A66" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1727,8 +2115,14 @@
       <c r="F66" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
       </c>
-    </row>
-    <row r="67">
+      <c r="G66" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 母愛對自我認同與愛的影響】
+時間: 01:26 - 02:02
+單集: EP30｜愛自己，為什麼這麼難？
+理由: 此片段深入探討了母親的愛（或缺乏）如何深刻影響一個人對自我價值的認同以及未來建立關係的能力。主講人清晰闡述了童年時期未能獲得真實的愛、連結與安全感，可能導致成年後難以愛自己和他人。這種從早期經驗追溯心理根源的內容，展現了節目在單元企劃上的深度與啟發性，對於自我探索具有極高的含金量。</v>
+      </c>
+    </row>
+    <row r="67" xml:space="preserve">
       <c r="A67" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1747,8 +2141,14 @@
       <c r="F67" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 「童年情感忽視」是一個相對小眾但極具深度的心理學議題，主持人對此議題的論述完整且具啟發性，符合利基市場的評估。 | [我們可能會成為最殘忍的一代｜《...] 「道德雄心」的議題雖然不完全是冷門，但主持人以獨特的角度和豐富的案例進行深入論述，使其在同類議題中脫穎而出，具備利基市場的完整度。</v>
       </c>
-    </row>
-    <row r="68">
+      <c r="G67" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
+時間: 01:03 - 03:05
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="68" xml:space="preserve">
       <c r="A68" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1767,8 +2167,14 @@
       <c r="F68" t="str">
         <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
       </c>
-    </row>
-    <row r="69">
+      <c r="G68" t="str" xml:space="preserve">
+        <v xml:space="preserve">【「主角模式」核心概念闡述】
+時間: 00:00 - 00:49
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
+      </c>
+    </row>
+    <row r="69" xml:space="preserve">
       <c r="A69" t="str">
         <v>只有你在獎 (稀有保護動物/化腐朽為神奇)</v>
       </c>
@@ -1787,8 +2193,14 @@
       <c r="F69" t="str">
         <v>[S4.EP4｜性平教育20年，...] 議題探討深入，特別關注數位時代下的約會暴力、男性及LGBTQ+受害者的困境，具備高度利基市場的獨特性。 | [S4.EP8｜我不想再跟你生活...] 議題聚焦於離婚後的心理歷程與微小生活習慣的影響，雖非極度冷門，但論述角度獨特且完整。 | [S4.EP14｜有些人沒有成為...] 「比前任更難忘的非前任」這一議題雖然具有普世性，但節目從心理學、文學和個人經驗等多維度進行深入探討，使其在同類節目中具備獨特的利基市場論述。</v>
       </c>
-    </row>
-    <row r="70">
+      <c r="G69" t="str" xml:space="preserve">
+        <v xml:space="preserve">【好哥新書與「四一讀書會」概念破題】
+時間: 01:08 - 01:51
+單集: S4.EP11｜不要再逼自己讀完整本書了！真正有用的是這一件事 feat.《郝會讀書》郝旭烈（郝哥）
+理由: 此片段迅速引入來賓好哥的新書《好會讀書》，並清晰闡述其核心概念「四一讀書會」。好哥以生動的語氣解釋了如何透過這種獨特方法輕鬆閱讀，有效吸引聽眾對節目主題產生興趣，是個引人入勝的開場。</v>
+      </c>
+    </row>
+    <row r="70" xml:space="preserve">
       <c r="A70" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1807,8 +2219,14 @@
       <c r="F70" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
       </c>
-    </row>
-    <row r="71">
+      <c r="G70" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫柔引導的內在療癒】
+時間: 22:33 - 25:00
+單集: EP30｜愛自己，為什麼這麼難？
+理由: 此片段為一段引導式的內在療癒練習，完美展現了主講人獨特的聲線魅力。她的語速明顯放緩（約180-190字/分），語調極其溫和、穩定且富有磁性，營造出極具安撫與陪伴感的氛圍。發音清晰，沒有任何刺耳或突兀的爆音，讓聽眾能完全放鬆並專注於內在感受。這種聲音特質對於需要心靈慰藉的聽眾而言，具有強烈的治癒效果，是「深夜輕輕獎」的絕佳範例。</v>
+      </c>
+    </row>
+    <row r="71" xml:space="preserve">
       <c r="A71" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1827,8 +2245,14 @@
       <c r="F71" t="str">
         <v>[S4.EP4｜性平教育20年，...] 語調溫柔穩定，內容雖嚴肅但傳達方式具同理心，適合深夜聆聽，提供陪伴治癒感。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人語調溫和穩定，對談充滿同理心，能營造出深夜陪伴與治癒的氛圍，無突兀尖銳音。 | [S4.EP14｜有些人沒有成為...] 兩位主持人的語調溫和穩定，對話內容引人��思，沒有突兀或尖銳的聲音，非常適合在深夜時分靜心聆聽，提供陪伴與治癒感。</v>
       </c>
-    </row>
-    <row r="72">
+      <c r="G71" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 女主持人清晰闡述暴力類型】
+時間: 00:03:34 - 00:03:50
+單集: S4.EP4｜性平教育20年，為什麼我們還是無法好好談戀愛？
+理由: 在此片段中，女主持人（胡咪）以清晰、有條理的語速，詳細闡述了肢體、精神和性三種約會暴力類型。她的發音精準，語調平穩且富有感染力，沒有任何爆音或刺耳的音頻，展現了優異的播音實力。這種專業且溫和的表達方式，讓聽眾在接收嚴肅資訊時感到舒適，非常符合「最佳女播音員獎」和「深夜輕輕獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="72" xml:space="preserve">
       <c r="A72" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1847,8 +2271,14 @@
       <c r="F72" t="str">
         <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
       </c>
-    </row>
-    <row r="73">
+      <c r="G72" t="str" xml:space="preserve">
+        <v xml:space="preserve">【溫暖的總結：無條件的接納與陪伴】
+時間: 28:48 - 29:45
+單集: EP225：【非典家庭CEO】打開家門讓愛住進來：24年守護26位寄養童，修補生命的補位馬拉松ft. 寶惠媽媽
+理由: 這段是主持人小可的結尾總結，她的聲音特質在此展現得淋漓盡致。語速穩定在約 190-200 字/分，發音清晰，語調溫柔且充滿情感。她用「笑笑的」、「溫和慈祥」、「溫暖」等詞彙形容保會媽媽，同時自己的聲音也散發出類似的特質，營造出極具陪伴感的氛圍。整個段落沒有任何刺耳的爆音或雜音，聲音共鳴圓潤，情感感染力強，完美符合「深夜輕輕獎」的評選標準，展現了卓越的播音實力與魅力。</v>
+      </c>
+    </row>
+    <row r="73" xml:space="preserve">
       <c r="A73" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1867,8 +2297,14 @@
       <c r="F73" t="str">
         <v>[#336 #Zoey｜你覺得自...] 主講人語調溫柔穩定，內容引人深思，無突兀尖銳爆音，非常適合深夜聆聽，提供治癒與陪伴感。 | [#我，是誰？S2E2｜為什麼越...] 主持人語調溫柔穩定，內容引人深思，無突兀尖銳音頻，非常適合深夜靜心聆聽，營造出治癒的陪伴感。 | [#我，是誰？S2E3｜過度依賴...] 節目主題深度且具反思性，主持人語調溫和穩定，預期能營造出適合深夜聆聽的平靜氛圍，無突兀尖銳音效。</v>
       </c>
-    </row>
-    <row r="74">
+      <c r="G73" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖且清晰的開場】
+時間: 00:00:00 - 00:03:00
+單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
+理由: 這個開場片段完美展現了主講人卓越的播音實力與魅力。她的發音清晰，語速約在 180-190 字/分之間，非常舒適。聲音溫暖且富有情感，帶有強烈的深夜安撫陪伴感，沒有任何刺耳或爆音。她以真誠的語氣歡迎聽眾，立即建立起親和力，非常符合「最佳女播音員獎」與「深夜輕輕獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="74" xml:space="preserve">
       <c r="A74" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1887,8 +2323,14 @@
       <c r="F74" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
       </c>
-    </row>
-    <row r="75">
+      <c r="G74" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[聲線特質] 外星人對媽媽超能力的解釋】
+時間: 18:29 - 19:31
+單集: 原創歌曲〈愛喲愛你喲〉+ 我的媽媽被外星人抓走了
+理由: 在此片段中，主持人以略帶趣味的外星人聲線，清晰且富有感染力地闡述了媽媽們的「超能力」。語速保持在舒適的範圍內（約200-210字/分），發音字正腔圓，情感真摯，成功傳達了對媽媽的讚頌。整個過程無��何刺耳或爆音，展現了主持人優異的播音實力與情感渲染力。</v>
+      </c>
+    </row>
+    <row r="75" xml:space="preserve">
       <c r="A75" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1907,8 +2349,14 @@
       <c r="F75" t="str">
         <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
       </c>
-    </row>
-    <row r="76">
+      <c r="G75" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 主持人開場與節目介紹】
+時間: 00:08 - 00:54
+單集: EP162 | 從房地產到MarTech：愛酷智能創辦人Jason的創業心法與人脈哲學
+理由: 主持人Becky���節目開場時，以清晰、溫暖且富有親和力的語調介紹了節目與來賓，並分享了宋家小館的創立緣由。她的語速穩定，發音清晰，聲音共鳴感佳，展現了良好的播音實力與溫馨陪伴感，且無刺耳爆音。儘管此片段長度未達建議的1.5分鐘，但已是本集最長的主持人單獨發言區間，足以展現其聲線特質。</v>
+      </c>
+    </row>
+    <row r="76" xml:space="preserve">
       <c r="A76" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1927,8 +2375,14 @@
       <c r="F76" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 主持人語調溫和穩定，聲音富有磁性，內容雖有深度但表達方式不具侵略性，非常適合深夜聆聽，具有陪伴治癒感。 | [我們可能會成為最殘忍的一代｜《...] 主持人語調溫和穩定，內容引人深思，沒有突兀的尖銳爆音，非常適合深夜聆聽，具有陪伴治癒感。</v>
       </c>
-    </row>
-    <row r="77">
+      <c r="G76" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 空虛感與幻想自傷的闡述】
+時間: 01:57:00 - 01:58:50
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 在此片段中，主持人以沉穩且富有同理心的語氣���闡述了「空虛感」極端化後，人們可能透過幻想自傷來尋求存在感或感受。儘管主題沉重，他仍保持了清晰的發音和適中的語速，聲音的溫暖共鳴感有效緩和了內容的衝擊性，展現了出色的播音實力與情緒感染力，非常適合「最佳男播音員獎」與「深夜輕輕獎」的評估。</v>
+      </c>
+    </row>
+    <row r="77" xml:space="preserve">
       <c r="A77" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1947,8 +2401,14 @@
       <c r="F77" t="str">
         <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
       </c>
-    </row>
-    <row r="78">
+      <c r="G77" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 節目結尾的溫馨總結與行動呼籲】
+時間: 01:53:50 - 01:56:30
+單集: EP470｜把人放在心上的共贏哲學！因為利他而打造瑜珈生態圈 feat. ASify 創辦人 Alice
+理由: 在節目的收尾階段，主持人不姐獨自發言，總結了本集對話的精華，特別是來賓對於「自信女性」的定義。她的語速在此段保持在約204字/分，語調溫和而穩定，發音清晰，沒有任何刺耳的爆音或噴麥。她以真誠的語氣分享個人共鳴，並自然地引導聽眾參與團購及分享節目，展現了其聲音的播音實力與魅力，以及強烈的深夜安撫陪伴感，符合【最佳女播音員獎】與【深夜輕輕獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="78" xml:space="preserve">
       <c r="A78" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1967,8 +2427,14 @@
       <c r="F78" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
       </c>
-    </row>
-    <row r="79">
+      <c r="G78" t="str" xml:space="preserve">
+        <v xml:space="preserve">【珍惜當下：愛與陪伴的真諦】
+時間: 12:41 - 13:09
+單集: 【悅讀專題】即使你忘了全世界，我依然記得愛你：《謝謝你留下來陪我》最動人的陪伴課
+理由: 主持人在結尾處總結了節目主旨，提醒聽眾珍惜眼前人，不要把愛和陪伴留到最後。他強調生命中最珍貴的不是擁有多少，而是在有限的時間裡真心愛過、陪��過、也被愛過。這段話語氣溫暖而富有哲理，聲音共鳴極佳，給予聽眾深刻的啟發與情感上的慰藉，是整集節目中最具力量和溫馨陪伴感的結語。</v>
+      </c>
+    </row>
+    <row r="79" xml:space="preserve">
       <c r="A79" t="str">
         <v>深夜輕輕獎 (暖心陪伴/悄悄話)</v>
       </c>
@@ -1987,8 +2453,14 @@
       <c r="F79" t="str">
         <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
       </c>
-    </row>
-    <row r="80">
+      <c r="G79" t="str" xml:space="preserve">
+        <v xml:space="preserve">【節目開場與溫馨陪伴】
+時間: 00:04 - 00:17
+單集: 42-結伴一起玩，樂享人生下半場（下）
+理由: 主持人以溫暖的語調清晰介紹節目宗旨，搭配柔和的背景音樂，營造出親切且具陪伴感的開場氛圍，迅速吸引聽眾進入節目主題。</v>
+      </c>
+    </row>
+    <row r="80" xml:space="preserve">
       <c r="A80" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2007,8 +2479,14 @@
       <c r="F80" t="str">
         <v>[EP289  七巨頭變七矮人！...] 節目節奏明快，主持人語調充滿朝氣，內容資訊量大，非常適合通勤時提神醒腦。 | [EP275 股市變賭場？巴菲特...] 節目節奏明快，主講人語調充滿活力且資訊量豐富，非常適合通勤或早晨時段收聽，有助於提神醒腦並快速掌握市場動態。 | [EP251國防預算暴漲 5 成...] 節奏明快，語調朝氣蓬勃，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
-    </row>
-    <row r="81">
+      <c r="G80" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 開場問候與節目主題介紹】
+時間: 00:05 - 00:15
+單集: EP251國防預算暴漲 5 成！必看這五檔股票！跟者川普賺一波？
+理由: 主持人以充滿活力和清晰的語調開場，語速雖快但發音字字分明，沒有含糊不清之處。他的聲音具有良好的中低音共鳴，給人一種專業且自信的印象，能迅速抓住聽眾的注意力，為���目定下積極的基調。</v>
+      </c>
+    </row>
+    <row r="81" xml:space="preserve">
       <c r="A81" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2027,8 +2505,14 @@
       <c r="F81" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
       </c>
-    </row>
-    <row r="82">
+      <c r="G81" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人���線特質] 節目收尾的啟發與展望】
+時間: 41:25 - 42:14
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 這段是主持人Andy的獨白，他以清晰、有力的聲線總結了本集的核心啟發，特別是關於美業從技術導向轉向思維導向的趨勢。他的語速控制得宜（約240-250字/分），發音清晰，情感真誠，沒有任何刺耳或爆音現象。這段發言展現了主持人作為「最佳男播音員」的專業素養與魅力，同時也為節目畫下了一個充滿啟發性的句點。</v>
+      </c>
+    </row>
+    <row r="82" xml:space="preserve">
       <c r="A82" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2047,8 +2531,14 @@
       <c r="F82" t="str">
         <v>[EP.617 《無限機器》讀後...] 節目節奏明快，開頭活力十足，內容資訊量高且引人入勝，具有提神醒腦的效果，適合通勤時收聽。 | [EP.573 從 0 到 10...] 節奏明快，開頭活力十足，內容具啟發性，有助於通勤時提神醒腦。 | [EP.607 《AI Firs...] 節目節奏明快，主持人開場充滿活力，內容資訊量高，有助於通勤時提神醒腦。</v>
       </c>
-    </row>
-    <row r="83">
+      <c r="G82" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖且具啟發性的總結與鼓勵】
+時間: 03:56:00 - 03:59:00
+單集: EP.573 從 0 到 10 萬訂閱：我經營免費電子報六年的三個體悟
+理由: 在這段總結中，主持人以穩定且富有溫度的語調，分享了他對「真實比完美重要」的深刻體悟。他的發音清晰，語速保持在舒適的範圍內，沒有任何刺耳的爆音或噴麥。他透過真誠的聲音表情，傳達出對聽眾的理解與鼓勵，展現了極佳的情緒感染力與陪伴感，非常適合【最佳男播音員獎】與【深夜輕輕獎】的評估。</v>
+      </c>
+    </row>
+    <row r="83" xml:space="preserve">
       <c r="A83" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2067,8 +2557,14 @@
       <c r="F83" t="str">
         <v>[郝聲音：（下） 莊鈞涵（Car...] 節奏明快，主持人與來賓充滿朝氣，內容實用且具激勵性，適合通勤時提神醒腦。 | [郝聲音：（下）「閱讀人」鄭俊德...] 節目節奏明快，開頭活力十足，內容實用且具啟發性，適合通勤時提神醒腦與獲取新知。 | [郝聲音：成為人生更自由的「精銳...] 節奏明快，語調朝氣蓬勃，內容具啟發性，非常適合通勤時提神醒腦。</v>
       </c>
-    </row>
-    <row r="84">
+      <c r="G83" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 好哥解讀《論語》與《詩經》的感悟】
+時間: 05:05 - 07:04
+單集: 郝聲音：（下） 莊鈞涵（Carol學姊）, 郭芃廷 「專攻20%，各科高分破解法」：進公立、上國立！國英數、自然與社會科，從放棄到高分的逆襲攻略，會考、學測、分科測驗都適用
+理由: 此片段由好哥主述，他分享了自己對《論語》中「詩無邪」的全新理解���透過解釋典故和文字背後的深層含義，展現了其卓越的播音實力。好哥的語速約在 250-270 字/分，清晰且富有感染力，中低音共鳴飽滿，情感真摯。他將複雜的文言文概念，以生動的故事和個人感悟娓娓道來，讓聽眾能清晰理解並產生共鳴，展現了極佳的聲音魅力與情緒渲染力。</v>
+      </c>
+    </row>
+    <row r="84" xml:space="preserve">
       <c r="A84" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2087,8 +2583,14 @@
       <c r="F84" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
       </c>
-    </row>
-    <row r="85">
+      <c r="G84" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 節目系列介紹】
+時間: 00:13:00 - 00:16:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段主持人以清晰、快速且充滿活力的語調介紹節目系列與訪談內容，發音精準，語速雖快但內容傳達效率高，展現了其作為播音員的專業素質與魅力，為節目奠定積極的基調。</v>
+      </c>
+    </row>
+    <row r="85" xml:space="preserve">
       <c r="A85" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2107,8 +2609,14 @@
       <c r="F85" t="str">
         <v>[[EP0063] 50+Con...] 主持人Connie的開場充滿活力，節奏明快，內容引人入勝，適合通勤時提神醒腦。 | [[EP0071] 50+Con...] 節目開場充滿活力，對話節奏明快，內容具啟發性，適合通勤時提神醒腦。 | [[EP0045] 50+Con...] 節目節奏明快，主持人與來賓的語氣都充滿活力，資訊密度高，非常適合通勤時提神醒腦。</v>
       </c>
-    </row>
-    <row r="86">
+      <c r="G85" t="str" xml:space="preserve">
+        <v xml:space="preserve">【男性溝通的獨特方式：肩並肩的陪伴】
+時間: 07:51 - 08:48
+單集: [EP0054] 50+Connie大嬸 x 中年低谷的轉身練習：Vito 大叔教你從失業到重啟人生 (下)
+理由: 這段深入剖析了男性在社交中偏好「肩並肩」而非「面對面」的溝通模式，透過共同勞動自然地建立連結與情感交流，解釋了「男士工棚」成功的心理基礎，極具洞察力。</v>
+      </c>
+    </row>
+    <row r="86" xml:space="preserve">
       <c r="A86" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2127,8 +2635,14 @@
       <c r="F86" t="str">
         <v>[新年特輯—火馬年續航攻略：吃睡...] 節目節奏明快，內容充滿實用建議和正能量，��常適合在通勤或早晨時段收聽，有助於提神醒腦並激發行動力。 | [別人眼中的高光時刻，卻是我最耗...] 節目節奏明快，主持人與來賓的對談充滿活力，內容積極向上，能夠在通勤或早晨時段提供提神醒腦的效果。 | [別急著振作！高能量的人允許自己...] 節奏明快，主持人與來賓的對談充滿活力，內容具啟發性，適合通勤時提神醒腦，能有效激發聽眾的思考。</v>
       </c>
-    </row>
-    <row r="87">
+      <c r="G86" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 建立決策軍師團】
+時間: 16:44 - 18:01
+單集: 新年特輯—火馬年續航攻略：吃睡練＋情緒＋決策＋意義感｜能量黑客S3EP11
+理由: 此片段由男主持人主講，他以穩定的語速（約250-260字/分）和清晰的發音，詳細解釋了如何建立「軍師團」來協助決策。他的聲音低沉且富有磁性，共鳴感極佳，傳達出專業與可靠的形象。整個過程沒有出現刺耳的爆音或噴麥，語調沉穩而具說服力，展現了其優異的播音實力與魅力，非常適合評選【最佳男播音員獎】。</v>
+      </c>
+    </row>
+    <row r="87" xml:space="preserve">
       <c r="A87" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2147,8 +2661,14 @@
       <c r="F87" t="str">
         <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
       </c>
-    </row>
-    <row r="88">
+      <c r="G87" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖總結與「教學相長」的理念】
+時間: 26:21 - 26:59
+單集: ep11. Z世代難搞嗎？用對方法其實很好懂！ft.張裕昌 奧美公關董事總經理
+理由: 在節目尾聲，女主持人丁菱娟獨自總結，語速約295字/分，清晰且舒適。她的聲線溫暖而富有感染力，語調真誠，強調主管應以開放心態與Z世代溝通，提供舞台並從中學習，達到「教學相長」。這段發言展現了她作為主持人的專業播音實力，語氣充滿鼓勵與陪伴感，無任何刺耳或爆音，非常符合【最佳女播音員獎】與【深夜輕輕獎】的評選標準。</v>
+      </c>
+    </row>
+    <row r="88" xml:space="preserve">
       <c r="A88" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2167,8 +2687,14 @@
       <c r="F88" t="str">
         <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
       </c>
-    </row>
-    <row r="89">
+      <c r="G88" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 開場介紹與主題引導】
+時間: 00:04 - 00:33
+單集: EP611 00998A(主動復華金融股息)鎖定歐洲大型金融股，優缺點在哪裡呢？
+理由: 此開場���段完美展現了主持人穩健且富有中低音共鳴的聲線特質。語速約為 205 字/分，清晰度極高，發音字正腔圓，沒有任何刺耳的爆音或噴麥現象。其語調平穩而專業，帶有適度的親和力，能迅速吸引聽眾注意力並建立信任感，為整個節目的資訊傳遞奠定良好基礎。這段是評選【最佳男播音員獎】的絕佳範例。</v>
+      </c>
+    </row>
+    <row r="89" xml:space="preserve">
       <c r="A89" t="str">
         <v>醒醒再獎 (激勵人心/起床氣消散)</v>
       </c>
@@ -2187,8 +2713,14 @@
       <c r="F89" t="str">
         <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
       </c>
-    </row>
-    <row r="90">
+      <c r="G89" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[聲線特質] 主持人小翔的節目收尾與聽眾互動】
+時間: 03:20:00 - 03:22:00
+單集: EP202 提升「語言含金量」，讓你每句話都帶有價值：商業自我介紹的5個關鍵｜竺宥璋《說到賣得動》
+理由: 在這段節目收尾中，主持人小翔的聲音特質展現得淋漓盡致。他的語速保持在舒適的範圍內（約200-210字/分），發音清晰且富有朝氣，沒有任何刺耳的爆音或噴麥。他以親切且具感染力的語氣，總結了本集內容，並明確地引導聽眾進行互動（留言分享學習心得），展現了良好的播音實力與對聽眾的黏著度。他的聲線明亮且穩定，能夠有效傳達節目的活力與專業性，非常適合「醒醒再獎」的評估維度，同時也符合「最佳男播音員獎」的標準。</v>
+      </c>
+    </row>
+    <row r="90" xml:space="preserve">
       <c r="A90" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2207,8 +2739,14 @@
       <c r="F90" t="str">
         <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
       </c>
-    </row>
-    <row r="91">
+      <c r="G90" t="str" xml:space="preserve">
+        <v xml:space="preserve">【溫暖的總結：無條件的接納與陪伴】
+時間: 28:48 - 29:45
+單集: EP225：【非典家庭CEO】打開家門讓愛住進來：24年守護26位寄養童，修補生命的補位馬拉松ft. 寶惠媽媽
+理由: 這段是主持人小可的結尾總結，她的聲音特質在此展現得淋漓盡致。語速穩定在約 190-200 字/分，發音清晰，語調溫柔且充滿情感。她用「笑笑的」、「溫和慈祥」、「溫暖」等詞彙形容保會媽媽，同時自己的聲音也散發出類似的特質，營造出極具陪伴感的氛圍。整個段落沒有任何刺耳的爆音或雜音，聲音共鳴圓潤，情感感染力強，完美符合「深夜輕輕獎」的評選標準，展現了卓越的播音實力與魅力。</v>
+      </c>
+    </row>
+    <row r="91" xml:space="preserve">
       <c r="A91" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2227,8 +2765,14 @@
       <c r="F91" t="str">
         <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
       </c>
-    </row>
-    <row r="92">
+      <c r="G91" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 女主持人清晰闡述暴力類型】
+時間: 00:03:34 - 00:03:50
+單集: S4.EP4｜性平教育20年，為什麼我們還是無法好好談戀愛？
+理由: 在此片段中，女主持人（胡咪）以清晰、有條理的語速，詳細闡述了肢體、精神和性三種約會暴力類型。她的發音精準，語調平穩且富有感染力，沒有任何爆音或刺耳的音頻，展現了優異的播音實力。這種專業且溫和的表達方式，讓聽眾在接收嚴肅資訊時感到舒適，非常符合「最佳女播音員獎」和「深夜輕輕獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="92" xml:space="preserve">
       <c r="A92" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2247,8 +2791,14 @@
       <c r="F92" t="str">
         <v>[#336 #Zoey｜你覺得自...] 節目內容雖具啟發性，但風格較為嚴肅與哲學，而非輕鬆歡樂的日常廢話，因此解壓療癒感相對較低。 | [#我，是誰？S2E2｜為什麼越...] 內容深度探討內在，能帶來心靈上的療癒，但談話風格較為嚴肅，非輕鬆歡樂的解壓類型。 | [#我，是誰？S2E3｜過度依賴...] 節目聚焦於自我成長、內在探索與接納，透過深度對話引導聽眾反思，具有強烈的療��與啟發感，有助於聽眾釋放壓力。</v>
       </c>
-    </row>
-    <row r="93">
+      <c r="G92" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖且清晰的開場】
+時間: 00:00:00 - 00:03:00
+單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
+理由: 這個開場片段完美展現了主講人卓越的播音實力與魅力。她的發音清晰，語速約在 180-190 字/分之間，非常舒適。聲音溫暖且富有情感，帶有強烈的深夜安撫陪伴感，沒有任何刺耳或爆音。她以真誠的語氣歡迎聽眾，立即建立起親和力，非常符合「最佳女播音員獎」與「深夜輕輕獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="93" xml:space="preserve">
       <c r="A93" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2267,8 +2817,14 @@
       <c r="F93" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
       </c>
-    </row>
-    <row r="94">
+      <c r="G93" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[聲線特質] 外星人對媽媽超能力的解釋】
+時間: 18:29 - 19:31
+單集: 原創歌曲〈愛喲愛你喲〉+ 我的媽媽被外星人抓走了
+理由: 在此片段中，主持人以略帶趣味的外星人聲線，清晰且富有感染力地闡述了媽媽們的「超能力」。語速保持在舒適的範圍內（約200-210字/分），發音字正腔圓，情感真摯，成功傳達了對媽媽的讚頌。整個過程無��何刺耳或爆音，展現了主持人優異的播音實力與情感渲染力。</v>
+      </c>
+    </row>
+    <row r="94" xml:space="preserve">
       <c r="A94" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2287,8 +2843,14 @@
       <c r="F94" t="str">
         <v>[#95 ▍ 冷戰半年怎麼破冰？...] 談話風格輕鬆且帶有幽默感，內容提供解決方案，能為聽眾帶來正向的解壓與療癒感受。 | [#99 ▍別讓金錢焦慮，成了教...] 談話風格真誠且富有同理心，透過分享個人經驗與心理學知識，能為聽眾帶來理解與療癒感。 | [#93 ▍自學，不是逃避的出口...] 透過真誠的對話與分享，提供情感上的支持與理解，有助於聽眾釋放壓力，但談話風格較為認真，非純粹輕鬆歡樂。</v>
       </c>
-    </row>
-    <row r="95">
+      <c r="G94" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫暖而有力的結語與下集預告】
+時間: 19:00 - 20:30
+單集: #95 ▍ 冷戰半年怎麼破冰？「撩夫神技」大公開- 神老師愛的秘訣 - 愛你現在的樣子 -上集
+理由: 此片段為主持人獨自發言的結尾與下集預告。主持人���速雖快但發音清晰，聲音充滿活力與親和力，展現了其作為女播音員的專業素養。她的語調溫暖而富有感染力，能夠有效傳達節目的核心價值，並成功激發聽眾對下一集的期待。整個過程無任何刺耳或突兀的爆音，聲音共鳴感佳，展現了優異的播音實力。</v>
+      </c>
+    </row>
+    <row r="95" xml:space="preserve">
       <c r="A95" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2307,8 +2869,14 @@
       <c r="F95" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
       </c>
-    </row>
-    <row r="96">
+      <c r="G95" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人���線特質] 節目收尾的啟發與展望】
+時間: 41:25 - 42:14
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 這段是主持人Andy的獨白，他以清晰、有力的聲線總結了本集的核心啟發，特別是關於美業從技術導向轉向思維導向的趨勢。他的語速控制得宜（約240-250字/分），發音清晰，情感真誠，沒有任何刺耳或爆音現象。這段發言展現了主持人作為「最佳男播音員」的專業素養與魅力，同時也為節目畫下了一個充滿啟發性的句點。</v>
+      </c>
+    </row>
+    <row r="96" xml:space="preserve">
       <c r="A96" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2327,8 +2895,14 @@
       <c r="F96" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
       </c>
-    </row>
-    <row r="97">
+      <c r="G96" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 溫柔引導的內在療癒】
+時間: 22:33 - 25:00
+單集: EP30｜愛自己，為什麼這麼難？
+理由: 此片段為一段引導式的內在療癒練習，完美展現了主講人獨特的聲線魅力。她的語速明顯放緩（約180-190字/分），語調極其溫和、穩定且富有磁性，營造出極具安撫與陪伴感的氛圍。發音清晰，沒有任何刺耳或突兀的爆音，讓聽眾能完全放鬆並專注於內在感受。這種聲音特質對於需要心靈慰藉的聽眾而言，具有強烈的治癒效果，是「深夜輕輕獎」的絕佳範例。</v>
+      </c>
+    </row>
+    <row r="97" xml:space="preserve">
       <c r="A97" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2347,8 +2921,14 @@
       <c r="F97" t="str">
         <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
       </c>
-    </row>
-    <row r="98">
+      <c r="G97" t="str" xml:space="preserve">
+        <v xml:space="preserve">【被低估的領導力特質：樂觀、謙虛與公正】
+時間: 06:46 - 10:14
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人分享書中提及三個常被低估的領導力特質：樂觀（非盲目，而是看見可能）、謙虛（開放的態度）和公正。這部分內容提供了實用的領導力洞見，聲音共鳴極佳，傳達出強烈的說服力與專業感。</v>
+      </c>
+    </row>
+    <row r="98" xml:space="preserve">
       <c r="A98" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2367,8 +2947,14 @@
       <c r="F98" t="str">
         <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
       </c>
-    </row>
-    <row r="99">
+      <c r="G98" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持人聲線特質] 節目結尾的溫馨總結與行動呼籲】
+時間: 01:53:50 - 01:56:30
+單集: EP470｜把人放在心上的共贏哲學！因為利他而打造瑜珈生態圈 feat. ASify 創辦人 Alice
+理由: 在節目的收尾階段，主持人不姐獨自發言，總結了本集對話的精華，特別是來賓對於「自信女性」的定義。她的語速在此段保持在約204字/分，語調溫和而穩定，發音清晰，沒有任何刺耳的爆音或噴麥。她以真誠的語氣分享個人共鳴，並自然地引導聽眾參與團購及分享節目，展現了其聲音的播音實力與魅力，以及強烈的深夜安撫陪伴感，符合【最佳女播音員獎】與【深夜輕輕獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="99" xml:space="preserve">
       <c r="A99" t="str">
         <v>年度療癒獎 (療癒/歡樂/獎廢話金牌)</v>
       </c>
@@ -2387,8 +2973,14 @@
       <c r="F99" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
       </c>
-    </row>
-    <row r="100">
+      <c r="G99" t="str" xml:space="preserve">
+        <v xml:space="preserve">【珍惜當下：愛與陪伴的真諦】
+時間: 12:41 - 13:09
+單集: 【悅讀專題】即使你忘了全世界，我依然記得愛你：《謝謝你留下來陪我》最動人的陪伴課
+理由: 主持人在結尾處總結了節目主旨，提醒聽眾珍惜眼前人，不要把愛和陪伴留到最後。他強調生命中最珍貴的不是擁有多少，而是在有限的時間裡真心愛過、陪��過、也被愛過。這段話語氣溫暖而富有哲理，聲音共鳴極佳，給予聽眾深刻的啟發與情感上的慰藉，是整集節目中最具力量和溫馨陪伴感的結語。</v>
+      </c>
+    </row>
+    <row r="100" xml:space="preserve">
       <c r="A100" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2405,10 +2997,16 @@
         <v>9.95</v>
       </c>
       <c r="F100" t="str">
-        <v>[EP133｜顛覆你對美容業的想...] 深度探討自由人生、自我成長、內在探索與心靈啟發，從個人經歷中提煉出普世價值，啟發性極強。 | [EP174｜越省反而越窮？別把...] 深度探討金錢觀、人生目的與自我成長，對聽眾的內在探索有很強的啟發。 | [EP164｜滑短影音是在浪費時...] 節目深度探討了閱讀如何影響個人成長、思維模式的轉變以及如何找回自我可能性，提供了豐富的內在探索與心靈啟發內容。</v>
-      </c>
-    </row>
-    <row r="101">
+        <v>[EP133｜顛覆你對美容業的想...] 節目開頭的介紹就明確指出這是關於「自我成長、人生經驗對談和內化學習輸出」的節目，完全符合自我探索的主軸。來賓分享了她從不愛讀書、排斥美容，到���為解決自身問題而熱愛學習、投身美容產業的歷程，這本身就是一個深刻的自我探索故事。節目中也探討了學習的動機、面對困難的態度、以及如何從不同階段的經驗中成長，這些都鼓勵聽眾向內覺察，思考自己的生命歷程與價值觀。 | [EP174｜越省反而越窮？別把...] 節目的核心主軸圍繞著「財富自由」的深層意義，超越了單純的金錢累積，轉向對個人價值觀、人生目標、幸福感和自我實現的探索。透過對金錢底層邏輯的討論、馬斯洛需求層次理論的翻轉（帆船模型），以及如何透過「花錢」來投資自我、創造正向循環，都旨在引導聽眾向內覺察，重新定義自己的「富有」與「自由」。節目內容鼓勵聽眾思考「我真正想要的是什麼」，而非盲目追求社會定義的成功，這與自我探索的宗旨高度契合。 | [EP164｜滑短影音是在浪費時...] 節目主軸明確聚焦於「自我成長、人生經驗對談和內化學習輸出」，與自我探索的核心精神高度契合。主持人與來賓不斷引導聽眾將所學知識與個人經驗連結，強調閱讀不僅是獲取資訊，更是為了產生內在動力、提升自我覺察、並活出更舒適、包容與正向的人生。節目中分享的許多故事，都旨在啟發聽眾向內觀照，重新定義自己的可能性，並鼓勵將生活中的每一天都視為一本值得閱讀的書，從中學習與成長。</v>
+      </c>
+      <c r="G100" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 來賓電商逆襲的核心思考】
+時間: 04:43 - 06:56
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 此片段詳細闡述了來賓從代理產品轉向自創品牌的「悲慘故事」，揭示了市場亂象（經銷商跳過代理、價格戰）如何迫使她做出戰略轉變。內容充滿創業洞察，展現了對市場動態和個人價值的深刻理解。主持人Andy的問題引導來賓揭示了其核心動機，使這段敘述極具啟發性，非常適合評選「最神單元企劃」與「自我探索獎」。</v>
+      </c>
+    </row>
+    <row r="101" xml:space="preserve">
       <c r="A101" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2427,8 +3025,14 @@
       <c r="F101" t="str">
         <v>[#336 #Zoey｜你覺得自...] 節目核心即為自我成長與內在探索，透過對自由、痛苦與無常的深刻剖析，提供了極強的心靈啟發深度。 | [#我，是誰？S2E2｜為什麼越...] 節目核心即為自我成長與內在探索，本集更是深入剖析了個人與情緒的關係，提供了深刻的心靈啟發，表現極為出色。 | [#我，是誰？S2E3｜過度依賴...] 本集節目核心即為自我探索，從「我是誰」出發，深入探討生命意義、內在批判者、以及如何與內在建立友善關係，提供了極高的心靈啟發與成長深度。</v>
       </c>
-    </row>
-    <row r="102">
+      <c r="G101" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 探討「一切皆無常」的第一個智慧】
+時間: 01:36:00 - 01:39:00
+單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
+理由: 此片段主講人深入闡述了她領悟到的第一個智慧：「一切皆無常」。她清晰地解釋了這個概念，並指出人們對無常的抗拒是痛苦的根源。這展現了節目在內容企劃上的深度與利基選題的獨特性，引導聽眾進行深刻的自我反思，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="102" xml:space="preserve">
       <c r="A102" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2447,8 +3051,14 @@
       <c r="F102" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 節目核心即為自我探索，深度剖析了愛自己的內在機制、童年影響與關係模式，提供了豐富的心靈啟發與成長路徑，是此獎項的強勁競爭者。 | [EP21｜為什麼總是替傷害你的...] 本集內容高度聚焦於自我成長、內在探索和心靈啟發，引導聽眾反思自身行為模式，深度極高。 | [EP28｜走進孩子的情緒小劇場...] 節目深度探討自我成長、內在探索與心靈啟發，來賓的個人歷程極具啟發性，符合「自我探索獎」的核心精神。</v>
       </c>
-    </row>
-    <row r="103">
+      <c r="G102" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 母愛對自我認同與愛的影響】
+時間: 01:26 - 02:02
+單集: EP30｜愛自己，為什麼這麼難？
+理由: 此片段深入探討了母親的愛（或缺乏）如何深刻影響一個人對自我價值的認同以及未來建立關係的能力。主講人清晰闡述了童年時期未能獲得真實的愛、連結與安全感，可能導致成年後難以愛自己和他人。這種從早期經驗追溯心理根源的內容，展現了節目在單元企劃上的深度與啟發性，對於自我探索具有極高的含金量。</v>
+      </c>
+    </row>
+    <row r="103" xml:space="preserve">
       <c r="A103" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2467,8 +3077,14 @@
       <c r="F103" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
       </c>
-    </row>
-    <row r="104">
+      <c r="G103" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 美國健康政策與生活型態結合】
+時間: 01:50:00 - 01:53:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段來賓深入探討美國最新的健康政策，如何將藥物治療與生活型態調整結合，並提出「Balance」計畫。這不僅展現了選題的深度與前瞻性，也提供了超越單純藥物討論的宏觀視角，極具單元企劃與啟發價值。</v>
+      </c>
+    </row>
+    <row r="104" xml:space="preserve">
       <c r="A104" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2487,8 +3103,14 @@
       <c r="F104" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 節目核心圍繞自我成長、內在探索與心靈啟發，主持人透過個人經驗與書中理論的結合，提供了極高的自我探索價值。 | [我們可能會成為最殘忍的一代｜《...] 節目核心即是引導聽眾進行自我反思與內在探索，透過多個案例挑戰聽眾的道德觀與行動力，心靈啟發深度極高。</v>
       </c>
-    </row>
-    <row r="105">
+      <c r="G104" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
+時間: 01:03 - 03:05
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="105" xml:space="preserve">
       <c r="A105" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2496,19 +3118,25 @@
         <v>6</v>
       </c>
       <c r="C105" t="str">
-        <v>布姐的沙發</v>
+        <v>人類行為研究社</v>
       </c>
       <c r="D105" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
+        <v>張忘形</v>
       </c>
       <c r="E105">
-        <v>9.8215</v>
+        <v>9.7715</v>
       </c>
       <c r="F105" t="str">
-        <v>[EP470｜把人放在心上的共贏...] 節目深度探討了自我成長、內在價值觀與目的性創業，來賓對自信的定義也提供了深刻的心靈啟發。 | [EP433｜【中年轉型】從矽谷...] 深度探討個人職涯轉型、自我覺察與性格探索，提供豐富的心靈啟發與成長觀點，是本集的核心亮點。 | [EP466｜拒絕被朝九晚五綁架...] 本集節目核心圍繞著自我成長、內在探索與心靈啟發。來賓透過「百工計畫」的實踐，深入剖析了個人與社會的關係，以及如何找到內在平衡，啟發性極強。</v>
-      </c>
-    </row>
-    <row r="106">
+        <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
+      </c>
+      <c r="G105" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 「好感影響力」的核心理念與長久之道】
+時間: 04:11 - 05:44
+單集: EP61｜為什麼越努力經營，反而覺得越內耗？也許你要先給自己『好感』 ft. 梁哲維老師
+理由: 來賓深入闡述「好感影響力」的底層邏輯，強調影響力不僅是說話，更關乎信任與理解的累積。他提出「如何做得久」是關鍵，並將其連結到「好的感覺」，這是一個獨特且具啟發性的觀點，展現了單元企劃的深度與含金量。</v>
+      </c>
+    </row>
+    <row r="106" xml:space="preserve">
       <c r="A106" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2516,19 +3144,25 @@
         <v>7</v>
       </c>
       <c r="C106" t="str">
-        <v>蕭邦相談室</v>
+        <v>OHMYBOOK｜哲維說書</v>
       </c>
       <c r="D106" t="str">
-        <v>蕭邦</v>
+        <v>梁哲維</v>
       </c>
       <c r="E106">
-        <v>9.8049</v>
+        <v>9.75</v>
       </c>
       <c r="F106" t="str">
-        <v>[【蕭邦出任務】負債 900 多...] 深度探討自我成長、內在探索與心靈啟發，主持人分享個人轉變歷程，極具啟發性。 | [【蕭邦出任務】如何選擇適合自己...] 來賓的職涯轉型故事與主持人對自我價值的探討，提供了深刻的內在探索與心靈啟發，深度極高。 | [幸福的人，通常「覺察力」都很強...] 深度探討情緒的來源、自我批判的迴圈以及如何透過覺察進行自我調整，對內在探索與心靈啟發的深度極高。</v>
-      </c>
-    </row>
-    <row r="107">
+        <v>[【EP330 帶著善意行動，最...] 節目主軸圍繞著「黑右雞腳」兩位主理人傳承家業、創業發展的歷程，深入探討了她們的「起心動念」、面對挑戰時的摸索與成長，��及透過美食傳遞幸福與善意的核心價值。她們分享了從迷茫到堅定信念的內在轉變，以及在與顧客互動中獲得的成就感與自我肯定。這不僅是一個創業故事，更是一個關於尋找生命意義、實踐利他精神的自我探索旅程，對於聽眾在個人價值觀與人生方向的覺察上，具有高度啟發性。 | [【EP302 把命盤變成行動藍...] 節目主軸明確圍繞「命理」如何幫助聽眾進行自我探索與覺察。主持人開宗明義地指出節目旨在幫助聽眾「了解命理是怎麼一回事」及「更了解自己」。來賓葛道老師也強調「��命不是算命運，而是運命」，鼓勵聽眾透過了解命盤來「運」自己的命，發揮天賦，順流而上。節目中提及的八字、紫微、占星、人類圖等工具，皆指向幫助個人認識自我、找到存在價值與意義，核心價值與自我探索高度契合。 | [【EP312《超越我執的生活》...] 節目主軸明確聚焦於「超越我執」、內在覺察、臨在練習以及區分自我與思緒等概念，這些都是自我探索與向內覺察的核心議題。主持人透過書籍內容的分享，引導聽眾反思自身的執念與情緒來源，並提供具體���練習方法，旨在幫助聽眾達到靈性成長與自我覺醒，完全符合自我探索獎的評選標準。</v>
+      </c>
+      <c r="G106" t="str" xml:space="preserve">
+        <v xml:space="preserve">【「主角模式」核心概念闡述】
+時間: 00:00 - 00:49
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
+      </c>
+    </row>
+    <row r="107" xml:space="preserve">
       <c r="A107" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2536,19 +3170,25 @@
         <v>8</v>
       </c>
       <c r="C107" t="str">
-        <v>人類行為研究社</v>
+        <v>下半場人生陪談師</v>
       </c>
       <c r="D107" t="str">
-        <v>張忘形</v>
+        <v>下半場人生事務有限公司</v>
       </c>
       <c r="E107">
-        <v>9.7715</v>
+        <v>9.6549</v>
       </c>
       <c r="F107" t="str">
-        <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
-      </c>
-    </row>
-    <row r="108">
+        <v>[44-解開品牌人生的迷思，從認...] 節目核心圍繞自我成長、內在探索與心靈啟發，深度探討個人價值觀與人生方向，啟發性極強。 | [57-慢活的幸福人生 – 台灣...] 節目深度探討了個人成長、內在探索與心靈啟發，鼓勵聽眾透過慢活理念重新認識自我與世界，具備極高的自我探索價值。 | [59-人生下半場，人際好感怎麽...] 節目核心主題圍繞自我成長、內在探索與心靈啟發，深度極高，能有效引導聽眾反思自身。</v>
+      </c>
+      <c r="G107" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 個人品牌的核心：認識自己與真實渴望】
+時間: 01:35 - 03:22
+單集: 44-解開品牌人生的迷思，從認識自己開始——品牌顧問黃馨儀 Cynthia 專訪（下）
+理由: 此片段中，來賓黃星頤深入闡述其著作《活成一道光，打造個人品牌的偉大航道》的核心理念。她強調個人品牌建立的基石是「認識自己」，理解內心真正的渴望，而非盲從社會期待。這段內容不僅提供了建立個人品牌的深度思考框架，更觸及了自我價值觀與人生方向的探索，極具啟發性與含金量，非常適合評選「最神單元企劃」與「自我探索獎」。</v>
+      </c>
+    </row>
+    <row r="108" xml:space="preserve">
       <c r="A108" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2556,19 +3196,25 @@
         <v>9</v>
       </c>
       <c r="C108" t="str">
-        <v>下一本讀什麼？</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D108" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E108">
-        <v>9.7549</v>
+        <v>9.65</v>
       </c>
       <c r="F108" t="str">
-        <v>[EP.617 《無限機器》讀後...] 節目深度探討了個人使命感、價值觀與對未來的思考，引導聽眾進行自我成長與內在探索���心靈啟發感極強。 | [EP.573 從 0 到 10...] 深度探討個人成長、心態轉變、面對困難的韌性，以及如何從內在尋找動力，心靈啟發感極強。 | [EP.607 《AI Firs...] 節目核心圍繞個人在AI時代的自我成長、能力提升與心態轉變，提供了深刻的內在探索與心靈啟發。</v>
-      </c>
-    </row>
-    <row r="109">
+        <v>[EP225：【非典家庭CEO】...] 節目深度探討了個人在面對生命挑戰時的內在轉變、成長與自我超越，特別是保會媽媽從「後悔」到「互相陪伴」的心路歷程，極具心靈啟發深度。 | [EP218：愛自己｜放下完美執...] 人類圖的核心價值即是自我探索與成長。本集透過解析個人特質、關係模式及流日影響，提供了豐富的工具與視角，深刻啟發聽眾認識自我、理解他人，並引導心靈成長。 | [EP219：【非典家庭CEO】...] 深度探討育兒過程中的自我成長、內在探索與心靈啟發，提供豐富的思考面向。</v>
+      </c>
+      <c r="G108" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 人類圖個案解析：情緒出口與能量管理】
+時間: 15:43 - 19:09
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段來賓Anka分享了兩個具體的個案：一個是情緒中心空白、能量中心多且定義的孩童（有ADHD傾向），另一個是薦骨中心空白的投射者成人。Anka透過人類圖的視角，深入解析了他們行為背後的原因（如情緒不穩定、過度承擔），並提供了實用的建議（如增加活動、心理諮商、學習能量管理）。這些案例不僅具體生動，也展現了人類圖在理解個人特質和提供解決方案上的深度與實用價值，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="109" xml:space="preserve">
       <c r="A109" t="str">
         <v>自我探索獎</v>
       </c>
@@ -2576,19 +3222,25 @@
         <v>10</v>
       </c>
       <c r="C109" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D109" t="str">
-        <v>梁哲維</v>
+        <v>蕭邦</v>
       </c>
       <c r="E109">
-        <v>9.75</v>
+        <v>9.65</v>
       </c>
       <c r="F109" t="str">
-        <v>[【EP330 帶著善意行動，最...] 節目深度探討了創業者的初心、傳承的意義以及善意帶來的回饋，對聽眾的自我成長和內在探索有很強的啟發。 | [【EP302 把命盤變成行動藍...] 節目核心圍繞著個人命運、自我認知與未來規劃，深度啟發聽眾進行內在探索與自我成長，極具價值。 | [【EP312《超越我執的生活》...] 本集內容核心即為自我成長與內在探索，透過對「我執」的剖析和「臨在��的實踐，提供了深刻的心靈啟發，高度符合此獎項的評估維度。</v>
-      </c>
-    </row>
-    <row r="110">
+        <v>[【蕭邦出任務】負債 900 多...] 節目主軸圍繞著Aaron從負債低谷到成功的心路歷程，深入探討了其成長背景、家庭對話如何塑造他的價值觀，以及他對「成功」的定義如何導致迷失。節目中大量篇幅用於探討「心智」、「潛意識」、「陰陽」與「冰山下的世界」等概念，並強調了自我覺察與內在轉變的重要性，完全符合自我探索獎的核心精神。 | [【蕭邦出任務】如何選擇適合自己...] 節目主軸圍繞著來賓 Katie 的職涯與人生轉折，從最初因家人建議選擇化工系，到後來發現不喜歡工程師工作，經歷車禍後被迫停下腳步，進而開始思考自己真正想做的事情。整個過程充滿了自我覺察、探索與成長，包括如何面對不喜歡的工作、如何找到自己的熱情、如��從迷茫中找到方向，以及如何堅持下去。來賓的分享非常真誠且具啟發性，主持人也引導得很好，讓聽眾能從中獲得許多自我探索的啟發。 | [幸福的人，通常「覺察力」都很強...] 本集節目主軸完全聚焦於「覺察」與「自我探索」。主持人從自身經驗出發，深入淺出地解釋了覺察的意義、如何透過覺察認識情緒、以及覺察在個人成長中的重要性。節目內容提供了具體的練習方法，並���討了覺察過程中可能遇到的挑戰與心態調整，旨在引導聽眾向內觀看、理解自我。其核心價值與節目主軸皆與自我探索高度契合，是此獎項的優秀範例。</v>
+      </c>
+      <c r="G109" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 從車禍到職涯轉型的自我探索】
+時間: 06:55 - 08:41
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="110" xml:space="preserve">
       <c r="A110" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2607,8 +3259,14 @@
       <c r="F110" t="str">
         <v>[EP.59｜【說話人聲-會客室...] 單集時長接近4小時，內容資訊密度極高，且能持續保持聽眾的專注與興趣，無明顯冷場，是優秀的長篇內容��</v>
       </c>
-    </row>
-    <row r="111">
+      <c r="G110" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] AI時代的親子連結與新書的附加價值】
+時間: 03:53 - 05:13
+單集: EP.61｜【說話人聲-會客室】別再逼自己當「完美父母」！挑剔孩子其實是在懲罰不完美的你
+理由: 此片段來賓紫菱深入探討在AI時代和疫情後，親子連結的重要性，並介紹她的新書如何回應這一需求。主持人伊柔精準提問關於新書的「附加價值」，引導紫菱分享她如何透過免費社群、直播課等方式，提供讀者超越書籍本身的持續支持與互動。這不僅展現了節目選題的深度與前瞻性，也突顯了來賓在內容企劃上的創新思維和對讀者的真誠承諾，極具啟發性。</v>
+      </c>
+    </row>
+    <row r="111" xml:space="preserve">
       <c r="A111" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2627,8 +3285,14 @@
       <c r="F111" t="str">
         <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
       </c>
-    </row>
-    <row r="112">
+      <c r="G111" t="str" xml:space="preserve">
+        <v xml:space="preserve">【Threads平台「內容為王」的獨特魅力】
+時間: 05:13 - 06:02
+單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
+理由: 來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
+      </c>
+    </row>
+    <row r="112" xml:space="preserve">
       <c r="A112" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2647,8 +3311,14 @@
       <c r="F112" t="str">
         <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
       </c>
-    </row>
-    <row r="113">
+      <c r="G112" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 美國健康政策與生活型態結合】
+時間: 01:50:00 - 01:53:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段來賓深入探討美國最新的健康政策，如何將藥物治療與生活型態調整結合，並提出「Balance」計畫。這不僅展現了選題的深度與前瞻性，也提供了超越單純藥物討論的宏觀視角，極具單元企劃與啟發價值。</v>
+      </c>
+    </row>
+    <row r="113" xml:space="preserve">
       <c r="A113" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2667,8 +3337,14 @@
       <c r="F113" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 單集時長超過60分鐘（約65分鐘），內容資訊密度高，主持人能持續輸出有價值的觀點和案例，全程無冷場��符合長篇內容的評估標準。 | [我們可能會成為最殘忍的一代｜《...] 單集時長超過60分鐘，且內容資訊密度極高，從頭到尾無冷場，引人入勝，非常符合長篇內容的評估標準。</v>
       </c>
-    </row>
-    <row r="114">
+      <c r="G113" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
+時間: 01:03 - 03:05
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="114" xml:space="preserve">
       <c r="A114" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2687,8 +3363,14 @@
       <c r="F114" t="str">
         <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
       </c>
-    </row>
-    <row r="115">
+      <c r="G114" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 專家與旁觀者的風險認知差異】
+時間: 04:48 - 06:00
+單集: 富人學🔆第一百零五堂｜『風險風險』
+理由: 主持人深入探討了攀岩者Alex對風險的專業評估與旁觀者因不了解而產生的恐懼，並將此觀點延伸至投資與人生決策。他強調了「被理解過的風險」與「被想像出來的風險」的區別，內容具備深度思考與啟發性，選題獨特且能引發聽眾共鳴，展現了節目在內容企劃上的高度與深度。</v>
+      </c>
+    </row>
+    <row r="115" xml:space="preserve">
       <c r="A115" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2707,8 +3389,14 @@
       <c r="F115" t="str">
         <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
       </c>
-    </row>
-    <row r="116">
+      <c r="G115" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 財富自由的定義：能力減去慾望】
+時間: 1:11:15 - 1:14:15
+單集: #71｜ 不為想像的明天而犧牲今天，就是退休｜《財富自由心理學》ft. 郝旭烈(郝哥) — 上
+理由: 此片段由來賓好哥深入闡述「財富自由」的獨特定義，提出「自由 = 能力 - 慾望」的核心公式，並延伸至「兩種宗教不能信：比較與計較」的深刻觀點。內容極具啟發性與深度，將財富自由從單純的金錢累積提升到心靈層面的選擇權，為聽眾提供了全新的思考框架，完全符合最神單元企劃與自我探索獎的評估維度。</v>
+      </c>
+    </row>
+    <row r="116" xml:space="preserve">
       <c r="A116" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2727,8 +3415,14 @@
       <c r="F116" t="str">
         <v>[S6EP30. 我到日本當漁夫...] 本集時長超過2小時，屬於長篇內容。節目在這麼長的時間內，資訊密度依然很高，對談流暢且引人入勝，沒有明顯的冷場，能讓聽眾持續投入。這展現了節目在長篇內容規劃與執行上的功力。</v>
       </c>
-    </row>
-    <row r="117">
+      <c r="G116" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 父母不讓繼承家業的獨特智慧與來賓的創業思維】
+時間: 01:49 - 03:40
+單集: S6EP30. 我到日本當漁夫｜Taku：叛逆的漁四代，在魚市場中的海鮮文化觀察！
+理由: 此片段來賓Taku分享了他父母不希望他繼承傳統養殖業，反而鼓勵他讀大學、追求更高發展的獨特觀點。這顛覆了許多人對家族事業繼承的傳統認知，展現了父母的遠見與智慧。Vito和品希對此表現出極大的驚訝與認同，並適時提問，引導Taku進一步闡述他如何從中找到自己的定位，並希望在產業鏈的更上游（繁殖業）發展。這段對話不僅內容新穎，也充滿了深度思考與自我探索的價值，非常符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="117" xml:space="preserve">
       <c r="A117" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2747,8 +3441,14 @@
       <c r="F117" t="str">
         <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
       </c>
-    </row>
-    <row r="118">
+      <c r="G117" t="str" xml:space="preserve">
+        <v xml:space="preserve">【「主角模式」核心概念闡述】
+時間: 00:00 - 00:49
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
+      </c>
+    </row>
+    <row r="118" xml:space="preserve">
       <c r="A118" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2767,8 +3467,14 @@
       <c r="F118" t="str">
         <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
       </c>
-    </row>
-    <row r="119">
+      <c r="G118" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 原則與習慣的邊界感】
+時間: 07:39 - 09:39
+單集: S0807-翻臉反擊、討好退讓之外的第三條路，有彈性的邊界感 ft Ginn
+理由: 此片段深入探討了「有彈性的邊界感」的核心概念，區分了「原則」與「習慣」的不同。主持人解釋了人們常將習慣誤認為原則，導致邊界僵化，難以協商。來賓的補充和例子（如送禮）進一步闡明了這一觀點，提供了獨到且具深度的內容洞察，極具啟發性。</v>
+      </c>
+    </row>
+    <row r="119" xml:space="preserve">
       <c r="A119" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -2787,8 +3493,14 @@
       <c r="F119" t="str">
         <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
       </c>
-    </row>
-    <row r="120">
+      <c r="G119" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 劇場的獨特性與文化價值】
+時間: 06:17 - 08:11
+單集: 遇見大來賓：專訪金鐘影后王琄：『人間條件8：凡人哥』~這齣戲，會讓你重新看見自己!
+理由: 來賓王娟深入闡述劇場作為「手工藝」的獨特性，強調其無法被AI取代的價值，並對比台灣與國際劇場的發展現況，探討語言障礙及文化融入的重要性。此段內容不僅具備深度思考，也為聽眾提供了對藝術形式的全新視角，極具「最神單元企劃」與「自我探索獎」的評估價值。</v>
+      </c>
+    </row>
+    <row r="120" xml:space="preserve">
       <c r="A120" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2807,8 +3519,14 @@
       <c r="F120" t="str">
         <v>[幸福的人，通常「覺察力」都很強...] 單集時長在10-15分鐘（11分48秒），內容精煉且傳播效率高，能在短時間內提供豐富的資訊與啟發。</v>
       </c>
-    </row>
-    <row r="121">
+      <c r="G120" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 從車禍到職涯轉型的自我探索】
+時間: 06:55 - 08:41
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="121" xml:space="preserve">
       <c r="A121" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2827,8 +3545,14 @@
       <c r="F121" t="str">
         <v>[春暖花開小旅行...] 單集時長約14分鐘，符合10-15分鐘的短篇內容標準，故事完整且傳播效率高。</v>
       </c>
-    </row>
-    <row r="122">
+      <c r="G121" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 節目主題與歌曲創作理念】
+時間: 00:00 - 00:26
+單集: 原創歌曲〈愛喲愛你喲〉+ 我的媽媽被外星人抓走了
+理由: 此片段清晰地介紹了本集節目的核心主題（對媽媽的愛），以及原創歌曲的創作背景（融入小朋友的投稿聲音）。主持人以真誠的語氣闡述了將愛擴展到所有關心之人的理念，展現了單元企劃的深度與溫馨，為整集奠定了情感基調，極具啟發價值。</v>
+      </c>
+    </row>
+    <row r="122" xml:space="preserve">
       <c r="A122" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2847,8 +3571,14 @@
       <c r="F122" t="str">
         <v>[EP199-別再相信快速致富：...] 單集時長約13分鐘，符合10-15分鐘的短篇內容標準，且內容精煉、資訊密度高，傳播效率極佳。</v>
       </c>
-    </row>
-    <row r="123">
+      <c r="G122" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 快速致富的迷思與創業的真實成本】
+時間: 00:08 - 02:22
+單集: EP199-別再相信快速致富：美業創業的現實與逆思維
+理由: 此片段從主持人提出「快速致富」的社會現象，引導來賓分享其創業初期對快速回本的期待與實際遇到的困難。來賓Louis老師具體闡述了地點、人流、高階客戶的重要性，以及開店所需的裝潢、器材、廣告等隱藏成本，揭示了創業的複雜性。主持人阿莉的提問與補充，讓內容更具深度與實用性，對於想在美業創業的聽眾而言，提供了寶貴的「乾貨」與深度思考，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="123" xml:space="preserve">
       <c r="A123" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2867,8 +3597,14 @@
       <c r="F123" t="str">
         <v>[EP134.真的找得到靈魂伴侶...] 單集時長約13分鐘，精煉且資訊密度高，在短時間內傳達了豐富的內容與思考，傳播效率極佳��</v>
       </c>
-    </row>
-    <row r="124">
+      <c r="G123" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 探索工作觀與人生觀，���計你的生命藍圖】
+時間: 03:30 - 05:10
+單集: EP131.「做自己的生命設計師」－打造全新生命藍圖
+理由: 主持人清晰地介紹了「工作觀」與「人生觀」這兩個核心概念，並引導聽眾思考其定義與重要性。他透過提問「工作是為了什麼？」、「什麼樣的人生才算美好？」等問題，鼓勵聽眾進行深度自我探索，找出個人價值觀與生命目標。這段內容不僅提供了實用的自我分析框架，也展現了節目在引導聽眾自我成長方面的深度與企劃力。</v>
+      </c>
+    </row>
+    <row r="124" xml:space="preserve">
       <c r="A124" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2887,8 +3623,14 @@
       <c r="F124" t="str">
         <v>[EP31 為了愛移民，她打造 ...] 單集時長約13分半，內容精煉且資訊密度高，傳播效率極佳，無冗餘。</v>
       </c>
-    </row>
-    <row r="125">
+      <c r="G124" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] Power 10：衝刺與平衡的智慧】
+時間: 02:49 - 04:26
+單集: EP47 有團隊的感覺如何？教解剖、教實體課與第一次當老闆日記
+理由: 主持人詳細解釋了「Power 10」這個源自划船比賽的概念，並巧妙地將其應用於生活與創作的節奏管理。她不僅清晰闡述了其定義與操作方式，更深入探討了如何在特定時刻全力衝刺，並在衝刺後獲得顯著進步。這個片段展現了節目選題的新穎性與內容的深度，將一個運動術語轉化為具啟發性的生活哲學，極具單元企劃價值。</v>
+      </c>
+    </row>
+    <row r="125" xml:space="preserve">
       <c r="A125" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2907,8 +3649,14 @@
       <c r="F125" t="str">
         <v>[【大師專題】人在江湖，身不由己...] 單集時長約10分鐘，符合10-15分鐘的短篇內容範疇。內容精煉，資訊密度高，能在短時間內傳達深刻且完整的觀點，傳播效率極佳。</v>
       </c>
-    </row>
-    <row r="126">
+      <c r="G125" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 疫情下「受助者變助人者」的深刻轉變】
+時間: 01:05:55 - 01:09:00
+單集: 從流浪到回家：浪人食堂的溫柔守護與陪伴 ft.蔡明潔店長
+理由: 明潔在此段闡述了浪人食堂在疫情期間，如何從單純的提供餐食，轉變為讓受助者也能參與助人，進而產生強烈的成就感和歸屬感。這個核心理念不僅獨特，更深入探討了人性的光輝與潛能，極具啟發性，完美符合「最神單元企劃」和「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="126" xml:space="preserve">
       <c r="A126" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2927,8 +3675,14 @@
       <c r="F126" t="str">
         <v>[EP351：AI的盡頭是電力！...] 單集時長約15分鐘，內容精煉且資訊密度高，傳播效率極佳，符合短篇內容的評估標準。</v>
       </c>
-    </row>
-    <row r="127">
+      <c r="G126" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] AI賦能個人，實現不可能的商業模式】
+時間: 06:00 - 07:30
+單集: EP346：一人公司時代來了？AI代理人如何重寫工作與商業規則 ft. 前Line台灣總經理陶韻智
+理由: 此片段來賓陶韻智分享他如何利用AI工具，從原本不擅長的領域（如寫程式）跨足到開發出媲美數十億美元公司的產品（如Kahoot和Gama），並成功推向全球市場。他強調AI讓他突破慣性思考，將產出提升十倍，甚至能處理管理、行銷、策略等過去認為自己無法做的事情。這段內容極具啟發性，展現了AI在個人創業和自我賦能上的巨大潛力，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="127" xml:space="preserve">
       <c r="A127" t="str">
         <v>到底有沒有獎 (泡麵沒熟獎)</v>
       </c>
@@ -2947,8 +3701,14 @@
       <c r="F127" t="str">
         <v>[EP19｜30歲後因為愛上這件...] 單集時長約10分鐘，符合短篇內容的定義。節目內容精煉，資訊密度高，在有限時間內傳達了豐富的觀點與啟發，傳播效率高。</v>
       </c>
-    </row>
-    <row r="128">
+      <c r="G127" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 女主持人超前部署的年終規劃】
+時間: 01:40 - 02:02
+單集: EP8｜領到年終去做這件事，居然能讓資產倍增！
+理由: 女主持人分享她如何提前規劃年終獎金，甚至細緻到2026年的紅包預算，並將資金分配到儲蓄戶頭。這段展現了她對金錢規劃的深度思考與實用方法，為聽眾提供了具體的理財啟發，符合『最神單元企劃』與『自我探索獎』的評估維度。</v>
+      </c>
+    </row>
+    <row r="128" xml:space="preserve">
       <c r="A128" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -2967,8 +3727,14 @@
       <c r="F128" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
       </c>
-    </row>
-    <row r="129">
+      <c r="G128" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 美國健康政策與生活型態結合】
+時間: 01:50:00 - 01:53:00
+單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
+理由: 此片段來賓深入探討美國最新的健康政策，如何將藥物治療與生活型態調整結合，並提出「Balance」計畫。這不僅展現了選題的深度與前瞻性，也提供了超越單純藥物討論的宏觀視角，極具單元企劃與啟發價值。</v>
+      </c>
+    </row>
+    <row r="129" xml:space="preserve">
       <c r="A129" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -2987,8 +3753,14 @@
       <c r="F129" t="str">
         <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
       </c>
-    </row>
-    <row r="130">
+      <c r="G129" t="str" xml:space="preserve">
+        <v xml:space="preserve">【好哥新書與「四一讀書會」概念破題】
+時間: 01:08 - 01:51
+單集: S4.EP11｜不要再逼自己讀完整本書了！真正有用的是這一件事 feat.《郝會讀書》郝旭烈（郝哥）
+理由: 此片段迅速引入來賓好哥的新書《好會讀書》，並清晰闡述其核心概念「四一讀書會」。好哥以生動的語氣解釋了如何透過這種獨特方法輕鬆閱讀，有效吸引聽眾對節目主題產生興趣，是個引人入勝的開場。</v>
+      </c>
+    </row>
+    <row r="130" xml:space="preserve">
       <c r="A130" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3007,8 +3779,14 @@
       <c r="F130" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 主持人與聽眾連結深厚，對談真誠有溫度，能給予聽眾靈魂陪伴感。 | [EP174｜越省反而越窮？別把...] 主持人與來賓的對談真誠且具啟發性，容易讓聽眾產生連結與黏著度。 | [EP164｜滑短影音是在浪費時...] 主持人與來賓的對談真誠且富有啟發性，內容引人入勝，讓聽眾對節目產生高度黏著度，期待繼續收聽。</v>
       </c>
-    </row>
-    <row r="131">
+      <c r="G130" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 來賓電商逆襲的核心思考】
+時間: 04:43 - 06:56
+單集: EP133｜顛覆你對美容業的想像！她用做企業的腦袋，重新定義「養膚管理」（Feat. 尖時養膚管理創辦人 劉欣玲·玲玲）
+理由: 此片段詳細闡述了來賓從代理產品轉向自創品牌的「悲慘故事」，揭示了市場亂象（經銷商跳過代理、價格戰）如何迫使她做出戰略轉變。內容充滿創業洞察，展現了對市場動態和個人價值的深刻理解。主持人Andy的問題引導來賓揭示了其核心動機，使這段敘述極具啟發性，非常適合評選「最神單元企劃」與「自我探索獎」。</v>
+      </c>
+    </row>
+    <row r="131" xml:space="preserve">
       <c r="A131" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3027,8 +3805,14 @@
       <c r="F131" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 主講人透過真誠且富有同理心的對談，與聽眾建立深厚的情感連結，其溫暖的陪伴感與對內在議題的深入探討，極具聽眾黏著度。 | [EP21｜為什麼總是替傷害你的...] 主講人透過真誠且富有洞察力的對談，與聽眾建立了深厚的情感連結，具有很高的黏著度和靈魂陪伴感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的對談情感真摯，內容引人入勝，能有效建立聽眾的黏著度與情感連結，讓人期待下一集。</v>
       </c>
-    </row>
-    <row r="132">
+      <c r="G131" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 母愛對自我認同與愛的影響】
+時間: 01:26 - 02:02
+單集: EP30｜愛自己，為什麼這麼難？
+理由: 此片段深入探討了母親的愛（或缺乏）如何深刻影響一個人對自我價值的認同以及未來建立關係的能力。主講人清晰闡述了童年時期未能獲得真實的愛、連結與安全感，可能導致成年後難以愛自己和他人。這種從早期經驗追溯心理根源的內容，展現了節目在單元企劃上的深度與啟發性，對於自我探索具有極高的含金量。</v>
+      </c>
+    </row>
+    <row r="132" xml:space="preserve">
       <c r="A132" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3047,8 +3831,14 @@
       <c r="F132" t="str">
         <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
       </c>
-    </row>
-    <row r="133">
+      <c r="G132" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] Alice的公益理念與實踐】
+時間: 04:39 - 06:29
+單集: EP470｜把人放在心上的共贏哲學！因為利他而打造瑜珈生態圈 feat. ASify 創辦人 Alice
+理由: 此片段深入探討了來賓Alice從2023年起與罕見疾病基金會合作，提供瑜伽療癒課程及贊助瑜伽墊的公益行動。主持人提問其動機，Alice分享她認為企業家應承擔社會責任，並強調她希望透過實際參與而非僅是捐款來幫助病友與家屬，讓他們感受到社會的接納與支持。這段對話展現了深刻的企業社會責任觀點與個人價值觀的結合，極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="133" xml:space="preserve">
       <c r="A133" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3067,8 +3857,14 @@
       <c r="F133" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
       </c>
-    </row>
-    <row r="134">
+      <c r="G133" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 人類圖個案解析：情緒出口與能量管理】
+時間: 15:43 - 19:09
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段來賓Anka分享了兩個具體的個案：一個是情緒中心空白、能量中心多且定義的孩童（有ADHD傾向），另一個是薦骨中心空白的投射者成人。Anka透過人類圖的視角，深入解析了他們行為背後的原因（如情緒不穩定、過度承擔），並提供了實用的建議（如增加活動、心理諮商、學習能量管理）。這些案例不僅具體生動，也展現了人類圖在理解個人特質和提供解決方案上的深度與實用價值，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="134" xml:space="preserve">
       <c r="A134" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3087,8 +3883,14 @@
       <c r="F134" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人透過引人入勝的敘事和情感連結，成功建立與聽眾的深厚關係，讓人期待後續故事發展，黏著度高。 | [春暖花開小旅行...] 主持人透過生動的敘述與角色扮演，與聽眾建立起良好的情感連結，具有高度的黏著度與陪伴感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 故事引人入勝，結尾的懸念設計強烈，讓聽眾對後續發展充滿期待，黏著度高。</v>
       </c>
-    </row>
-    <row r="135">
+      <c r="G134" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 節目主題與歌曲創作理念】
+時間: 00:00 - 00:26
+單集: 原創歌曲〈愛喲愛你喲〉+ 我的媽媽被外星人抓走了
+理由: 此片段清晰地介紹了本集節目的核心主題（對媽媽的愛），以及原創歌曲的創作背景（融入小朋友的投稿聲音）。主持人以真誠的語氣闡述了將愛擴展到所有關心之人的理念，展現了單元企劃的深度與溫馨，為整集奠定了情感基調，極具啟發價值。</v>
+      </c>
+    </row>
+    <row r="135" xml:space="preserve">
       <c r="A135" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3107,8 +3909,14 @@
       <c r="F135" t="str">
         <v>[【EP330 帶著善意行動，最...] 主持人與來賓的對談充滿情感溫度，真誠的交流讓聽眾感受到靈魂的陪伴，具有很強的黏著度。 | [【EP302 把命盤變成行動藍...] 主持人與來賓的對談真誠且富有溫度，內容��人入勝，能有效提升聽眾的黏著度與持續收聽的意願。 | [【EP312《超越我執的生活》...] 主持人以真誠且富有洞察力的語氣分享，內容深度能引發聽眾共鳴與思考，建立起較強的黏著度與情感連結，讓人期待下一集。</v>
       </c>
-    </row>
-    <row r="136">
+      <c r="G135" t="str" xml:space="preserve">
+        <v xml:space="preserve">【「主角模式」核心概念闡述】
+時間: 00:00 - 00:49
+單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
+理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
+      </c>
+    </row>
+    <row r="136" xml:space="preserve">
       <c r="A136" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3127,8 +3935,14 @@
       <c r="F136" t="str">
         <v>[#801 市場震盪 17000...] 主持人以真誠且具同理心的語氣與聽眾對話，建立深厚的連結，情感溫度高，能有效提升聽眾黏著度。 | [#809  買股票還在到處問明...] 主持人與來賓的對談真誠，內容實用且具啟發性，能有效吸引聽眾持續收聽，建立黏著度。 | [#798 害怕投資賠錢？不用天...] 主持人與來賓透過分享個人經驗和真誠的對談，與聽眾建立了深厚的情感連結，讓人期待下一集的內容。</v>
       </c>
-    </row>
-    <row r="137">
+      <c r="G136" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 股市下跌時的情緒管理與長期投資心法】
+時間: 03:07 - 04:38
+單集: #801 市場震盪 17000 點，費半重挫、台股回檔，你該急著逃，還是重新檢查資產配置？給剛進場投資人的一堂情緒與現金流課
+理由: 此片段全面探討了市場下跌時投資者的情緒管理。主持人深入分析了新進投資者常見的後悔與恐懼心理，強調市場的不可預測性，並引導聽眾思考投資標的的基本面價值與長期成長潛力。她透過對比長期持有者與近期進場者的經驗，提供了在市場波動中保持信念、避免恐慌性賣出的寶貴見解，對於自我探索與建立穩健的投資心態極具啟發價值。</v>
+      </c>
+    </row>
+    <row r="137" xml:space="preserve">
       <c r="A137" t="str">
         <v>請你繼續獎 (年度大獎/我要跟老師獎)</v>
       </c>
@@ -3147,8 +3961,14 @@
       <c r="F137" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
       </c>
-    </row>
-    <row r="138">
+      <c r="G137" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 從車禍到職涯轉型的自我探索】
+時間: 06:55 - 08:41
+單集: 【蕭邦出任務】如何選擇適合自己的工作 / 30 歲轉職會太晚嗎 / 職涯迷茫 feat. 網路行銷平台主管 Katy
+理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
+      </c>
+    </row>
+    <row r="138" xml:space="preserve">
       <c r="A138" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3156,19 +3976,25 @@
         <v>1</v>
       </c>
       <c r="C138" t="str">
-        <v>文森說書</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D138" t="str">
-        <v>文森說書</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E138">
-        <v>8.45</v>
+        <v>8.52</v>
       </c>
       <c r="F138" t="str">
-        <v>AI 評審平均得分為 8.45 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="139">
+        <v>AI 評審平均得分為 8.52 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G138" t="str" xml:space="preserve">
+        <v xml:space="preserve">【破題精采開場：從軍人到作家，刪不掉的生命故事】
+時間: 00:00 - 02:24
+單集: S3.EP92｜刪掉容易，忘掉很難：從軍人到寫故事的人 feat. 林思齊
+理由: 節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
+      </c>
+    </row>
+    <row r="139" xml:space="preserve">
       <c r="A139" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3176,19 +4002,25 @@
         <v>2</v>
       </c>
       <c r="C139" t="str">
-        <v>分手的99個理由</v>
+        <v>宋家小館</v>
       </c>
       <c r="D139" t="str">
-        <v>胡咪老師</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E139">
-        <v>8.45</v>
+        <v>8.47</v>
       </c>
       <c r="F139" t="str">
-        <v>AI 評審平均得分為 8.45 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="140">
+        <v>AI 評審平均得分為 8.47 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G139" t="str" xml:space="preserve">
+        <v xml:space="preserve">【闆娘Becky的轉運概念】
+時間: 00:53 - 01:41
+單集: EP174 | 打造福氣好運的三部曲
+理由: 主持人以親切的語氣開場，透過洗床單的日常小事引導出「轉運」的核心概念，迅速拉近與聽眾的距離，引人入勝。</v>
+      </c>
+    </row>
+    <row r="140" xml:space="preserve">
       <c r="A140" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3196,19 +4028,25 @@
         <v>3</v>
       </c>
       <c r="C140" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>文森說書</v>
       </c>
       <c r="D140" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>文森說書</v>
       </c>
       <c r="E140">
-        <v>8.44</v>
+        <v>8.45</v>
       </c>
       <c r="F140" t="str">
-        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="141">
+        <v>AI 評審平均得分為 8.45 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G140" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
+時間: 01:03 - 03:05
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="141" xml:space="preserve">
       <c r="A141" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3216,19 +4054,25 @@
         <v>4</v>
       </c>
       <c r="C141" t="str">
-        <v>尼可這樣說</v>
+        <v>布姐的沙發</v>
       </c>
       <c r="D141" t="str">
-        <v>尼可這樣說</v>
+        <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E141">
-        <v>8.18</v>
+        <v>8.44</v>
       </c>
       <c r="F141" t="str">
-        <v>AI 評審平均得分為 8.18 分，近半年累積 Apple Podcasts 評論數達 2 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="142">
+        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G141" t="str" xml:space="preserve">
+        <v xml:space="preserve">【浴室驚魂記：選擇的開端】
+時間: 00:00 - 00:57
+單集: EP455｜困難抉擇的關鍵心法：如何做出不後悔的選擇
+理由: 節目開場以一個生動且帶有戲劇性的個人故事破題，講述孩子對洗澡的恐懼以及主持人自身的無力感，迅速抓住聽眾注意力。這段不僅展現了主講人的敘事能力，也為後續關於人生選擇的討論奠定了情感基礎，語速與語氣的掌握恰到好處。</v>
+      </c>
+    </row>
+    <row r="142" xml:space="preserve">
       <c r="A142" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3236,19 +4080,25 @@
         <v>5</v>
       </c>
       <c r="C142" t="str">
-        <v>琄蜜莉的異想世界</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D142" t="str">
-        <v>王琄</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E142">
-        <v>8.37</v>
+        <v>8.44</v>
       </c>
       <c r="F142" t="str">
-        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="143">
+        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G142" t="str" xml:space="preserve">
+        <v xml:space="preserve">【同理心與育兒修羅場的開場】
+時間: 00:04 - 00:29
+單集: EP222：【非典家庭CEO】卸下心理師光環後的肉搏與自白：從母親節的失落，看職場父母如何在瑣碎生活中拼湊「夠好的自己」ft. 曾心怡心理師
+理由: 節目開場以平靜的語氣定義「同理心」，隨後立即切換至孩子們的吵鬧聲和母親崩潰的獨白，形成強烈對比。這種戲劇性的轉折，生動地呈現了育兒的真實挑戰，迅速抓住聽眾的注意力，並為節目主題做了精彩的破題。</v>
+      </c>
+    </row>
+    <row r="143" xml:space="preserve">
       <c r="A143" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3256,19 +4106,25 @@
         <v>6</v>
       </c>
       <c r="C143" t="str">
-        <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
+        <v>能量黑客</v>
       </c>
       <c r="D143" t="str">
-        <v>孫子玲</v>
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
       </c>
       <c r="E143">
-        <v>8.37</v>
+        <v>8.43</v>
       </c>
       <c r="F143" t="str">
-        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="144">
+        <v>AI 評審平均得分為 8.43 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G143" t="str" xml:space="preserve">
+        <v xml:space="preserve">【能量駭客的開場白與節目宗旨】
+時間: 00:00 - 00:30
+單集: 內耗怎麼停？先抽離，再復盤：把情緒變成行動｜能量黑客S2EP9
+理由: 這段是節目的標準開場，由兩位主持人輪流介紹節目理念。Hank大叔以「在忙碌生活中，有餘力去做快樂的事，並在重要時刻拿出最好的狀態」點出節目核心，Betty則補充「能量不只是體力，還包含專注力、情緒狀態」，並承諾用實用方法與幽默幫助聽眾找到高能量節奏。語速雖快，但清晰有力，有效傳達節目主旨，迅速抓住聽眾注意力。</v>
+      </c>
+    </row>
+    <row r="144" xml:space="preserve">
       <c r="A144" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3276,19 +4132,25 @@
         <v>7</v>
       </c>
       <c r="C144" t="str">
-        <v>蘇心時光</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D144" t="str">
-        <v>蘇絢慧分享空間</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E144">
-        <v>8.33</v>
+        <v>8.18</v>
       </c>
       <c r="F144" t="str">
-        <v>AI 評審平均得分為 8.33 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="145">
+        <v>AI 評審平均得分為 8.18 分，近半年累積 Apple Podcasts 評論數達 2 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G144" t="str" xml:space="preserve">
+        <v xml:space="preserve">【考上明星高中卻格格不入：自我懷疑的開端】
+時間: 03:17 - 04:44
+單集: EP.317 出走，不是逃離，而是回到自己：《臺灣製造》作者安吉的人生覺醒之路
+理由: 來賓生動地描述了她意外考上明星高中後，卻感到格格不入的經歷。這段內容深刻地揭示了外在成就與內心認同之間的落差，以及自我懷疑的萌芽，情感真摯且引人入勝，為後續的自我探索旅程奠定基礎。</v>
+      </c>
+    </row>
+    <row r="145" xml:space="preserve">
       <c r="A145" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3296,19 +4158,25 @@
         <v>8</v>
       </c>
       <c r="C145" t="str">
-        <v>我的動齡限量版</v>
+        <v>琄蜜莉的異想世界</v>
       </c>
       <c r="D145" t="str">
-        <v>我的動齡限量版</v>
+        <v>王琄</v>
       </c>
       <c r="E145">
-        <v>8.32</v>
+        <v>8.37</v>
       </c>
       <c r="F145" t="str">
-        <v>AI 評審平均得分為 8.32 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="146">
+        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G145" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 2026火運的全球變革與歷史借鑒】
+時間: 01:58 - 05:00
+單集: S4EP5 琄蜜莉的異想世界 feat. 瞧瞧宇宙在幹嘛 仙姑喬喬 （上集）
+理由: 此片段來賓深入解析2026年「丙午火運」的能量特質，將其與全球性的擴張、重建、秩序翻轉等現象連結，並引用日本解散議會、格陵蘭、美加關係等時事案例，甚至追溯至180年前的墨美戰爭，展現了極高的內容含金量與深度思考。主持人適時的提問與總結，有效引導聽眾理解複雜的觀點，是企劃選題與內容深度的絕佳示範。</v>
+      </c>
+    </row>
+    <row r="146" xml:space="preserve">
       <c r="A146" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3316,19 +4184,25 @@
         <v>9</v>
       </c>
       <c r="C146" t="str">
-        <v>任性歐逆機智生活</v>
+        <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
       </c>
       <c r="D146" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
+        <v>孫子玲</v>
       </c>
       <c r="E146">
-        <v>8.31</v>
+        <v>8.37</v>
       </c>
       <c r="F146" t="str">
-        <v>AI 評審平均得分為 8.31 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="147">
+        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G146" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 維繫婚姻的關鍵：不爭輸贏與分享慾】
+時間: 09:32 - 11:04
+單集: #95 ▍ 冷戰半年怎麼破冰？「撩夫神技」大公開- 神老師愛的秘訣 - 愛你現在的樣子 -上集
+理由: 此片段深入探討了維繫夫妻關係的關鍵，特別是「不爭輸贏」、「不踩底線」以及「分享慾」等核心觀念。來賓分享了如何在關係中找到平衡點，以及如何透過「誇誇法」等實際方法增進情感。主持人引導得宜，成功從來賓的經驗中提煉出具深度且實用的婚姻智慧，對聽眾具有高度的啟發價值。</v>
+      </c>
+    </row>
+    <row r="147" xml:space="preserve">
       <c r="A147" t="str">
         <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
@@ -3336,19 +4210,25 @@
         <v>10</v>
       </c>
       <c r="C147" t="str">
-        <v>哇賽心理學</v>
+        <v>蕭邦相談室</v>
       </c>
       <c r="D147" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>蕭邦</v>
       </c>
       <c r="E147">
-        <v>8.29</v>
+        <v>8.37</v>
       </c>
       <c r="F147" t="str">
-        <v>AI 評審平均得分為 8.29 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-    </row>
-    <row r="148">
+        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G147" t="str" xml:space="preserve">
+        <v xml:space="preserve">【開場：情緒的引導與個人經驗分享】
+時間: 00:12 - 00:31
+單集: 如何度過負面情緒 ？
+理由: 主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
+      </c>
+    </row>
+    <row r="148" xml:space="preserve">
       <c r="A148" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3362,13 +4242,19 @@
         <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E148">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F148" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #26.3 名。</v>
-      </c>
-    </row>
-    <row r="149">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #26.2 名。</v>
+      </c>
+      <c r="G148" t="str" xml:space="preserve">
+        <v xml:space="preserve">【節目開場】
+時間: 00:00 - 00:05
+單集: EP.591 《財富自由心理學》專訪作者：破解財富焦慮的 6 個洞察
+理由: 主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
+      </c>
+    </row>
+    <row r="149" xml:space="preserve">
       <c r="A149" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3382,13 +4268,19 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E149">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F149" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #33.3 名。</v>
-      </c>
-    </row>
-    <row r="150">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #33 名。</v>
+      </c>
+      <c r="G149" t="str" xml:space="preserve">
+        <v xml:space="preserve">【節目開場：你是否也「偏心自己」？】
+時間: 00:08 - 00:41
+單集: 累到想消失？偏心自己，找回角色外的自我ft.徐慧玲｜哇賽療心室ep152
+理由: 主持人以「偏心自己」這個核心概念開場，引導聽眾思考在家庭、工作、人際關係中，是否習慣性地先考慮他人需求而忽略自己，並點出許多人因此感到疲憊的現狀，為節目奠定引人入勝的基調。</v>
+      </c>
+    </row>
+    <row r="150" xml:space="preserve">
       <c r="A150" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3402,13 +4294,19 @@
         <v>郝旭烈/郝聲音</v>
       </c>
       <c r="E150">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F150" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #38.2 名。</v>
-      </c>
-    </row>
-    <row r="151">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #38.3 名。</v>
+      </c>
+      <c r="G150" t="str" xml:space="preserve">
+        <v xml:space="preserve">【Podcast與自媒體的開場提問】
+時間: 00:07 - 00:24
+單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
+理由: 主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+    </row>
+    <row r="151" xml:space="preserve">
       <c r="A151" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3422,13 +4320,19 @@
         <v>GK爸爸</v>
       </c>
       <c r="E151">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F151" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 45 天，平均上榜排名為第 #65.7 名。</v>
-      </c>
-    </row>
-    <row r="152">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #65.9 名。</v>
+      </c>
+      <c r="G151" t="str" xml:space="preserve">
+        <v xml:space="preserve">【GK爸爸的互動開場與故事預告】
+時間: 00:15 - 01:25
+單集: 《QQ俠大冒險2：前進宇宙》第二章 迷你太空船
+理由: 此片段展現了主持人GK爸爸活潑的開場風格，不僅介紹了本集故事內容，還巧妙地融入了與聽眾的互動環節（九九乘法），並預告了周邊商品，充分展現了節目的親和力與豐富性。</v>
+      </c>
+    </row>
+    <row r="152" xml:space="preserve">
       <c r="A152" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3442,13 +4346,19 @@
         <v>文森說書</v>
       </c>
       <c r="E152">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F152" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 37 天，平均上榜排名為第 #64.3 名。</v>
-      </c>
-    </row>
-    <row r="153">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 38 天，平均上榜排名為第 #64.2 名。</v>
+      </c>
+      <c r="G152" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
+時間: 01:03 - 03:05
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="153" xml:space="preserve">
       <c r="A153" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3465,7 +4375,13 @@
         <v>7</v>
       </c>
       <c r="F153" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
+      </c>
+      <c r="G153" t="str" xml:space="preserve">
+        <v xml:space="preserve">【舞台設計的趨勢：從實景到巨型LED螢幕的演變】
+時間: 39:16 - 40:19
+單集: EP177 演唱會背後的重要角色！必應創造舞台設計師工作開箱
+理由: 這段來賓小柔詳細說明了舞台設計從早期實景到現在巨型LED螢幕的演變，並以五月天「陳名在望」的演唱會為例，具體描述了LED螢幕如何創造出180度環繞的沉浸式體驗，以及飛機艙門的互動設計。主持人Fiona的提問引導得很好，讓小柔能深入解釋技術與藝術結合的細節，展現了單元企劃的深度與內容的含金量。</v>
       </c>
     </row>
     <row r="154">
@@ -3485,10 +4401,13 @@
         <v>6</v>
       </c>
       <c r="F154" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
-      </c>
-    </row>
-    <row r="155">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
+      </c>
+      <c r="G154" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="155" xml:space="preserve">
       <c r="A155" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3505,10 +4424,16 @@
         <v>4</v>
       </c>
       <c r="F155" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
-      </c>
-    </row>
-    <row r="156">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
+      </c>
+      <c r="G155" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 免費的代價：個人資料的價值與風險】
+時間: 11:30 - 13:20
+單集: 月光族精靈探店記#05 : 年貨大街 ✨免費的代價✨
+理由: 此片段深入探討了「填問卷送贈品」背後，個人資料如何成為一種隱性支付，以及其可能帶來的風險。雪兒阿姨（主持人）透過具體的例子，清晰解釋了姓名、電話等資料對商家的價值，並警示了資料被濫用或轉賣的潛在危險。點點（來賓角色）的疑問與反應，也恰到好處地引導了主持人逐步揭示這些深層概念，展現了節目在生活化情境中融入深度思考的企劃能力。</v>
+      </c>
+    </row>
+    <row r="156" xml:space="preserve">
       <c r="A156" t="str">
         <v>站著不走獎</v>
       </c>
@@ -3525,412 +4450,70 @@
         <v>2</v>
       </c>
       <c r="F156" t="str">
-        <v>於評選區間（統計 45 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
-      </c>
-    </row>
-    <row r="157">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
+      </c>
+      <c r="G156" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 探討「一切皆無常」的第一個智慧】
+時間: 01:36:00 - 01:39:00
+單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
+理由: 此片段主講人深入闡述了她領悟到的第一個智慧：「一切皆無常」。她清晰地解釋了這個概念，並指出人們對無常的抗拒是痛苦的根源。這展現了節目在內容企劃上的深度與利基選題的獨特性，引導聽眾進行深刻的自我反思，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="157" xml:space="preserve">
       <c r="A157" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B157">
+        <v>10</v>
+      </c>
+      <c r="C157" t="str">
+        <v>不敗教主陳重銘</v>
+      </c>
+      <c r="D157" t="str">
+        <v>不敗教主-陳重銘</v>
+      </c>
+      <c r="E157">
         <v>1</v>
       </c>
-      <c r="C157" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="D157" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="E157">
-        <v>5.2</v>
-      </c>
       <c r="F157" t="str">
-        <v>平均評等 5 星，累計 2 則評論。綜合指標得分：5.2 / 10 分。</v>
-      </c>
-    </row>
-    <row r="158">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 1 天，平均上榜排名為第 #84 名。</v>
+      </c>
+      <c r="G157" t="str" xml:space="preserve">
+        <v xml:space="preserve">【開場引導與人生反思】
+時間: 00:04 - 01:15
+單集: EP594《富媽媽 窮媽媽》第二章(4)：原來讀書就是為了要賺錢養家，工作就是在坐牢
+理由: 主持人以書籍《富媽媽窮媽媽》為引，迅速切入主題，並結合自身年輕時對投資、退休與人生選擇的思考，語氣真誠，引人入勝，有效抓住聽眾的注意力。</v>
+      </c>
+    </row>
+    <row r="158" xml:space="preserve">
       <c r="A158" t="str">
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
       <c r="B158">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C158" t="str">
-        <v>迷途艾比</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="D158" t="str">
-        <v>迷途艾比</v>
+        <v>尼可這樣說</v>
       </c>
       <c r="E158">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F158" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B159">
-        <v>3</v>
-      </c>
-      <c r="C159" t="str">
-        <v>山姆書書</v>
-      </c>
-      <c r="D159" t="str">
-        <v>山姆書書</v>
-      </c>
-      <c r="E159">
-        <v>0</v>
-      </c>
-      <c r="F159" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B160">
-        <v>4</v>
-      </c>
-      <c r="C160" t="str">
-        <v>宋家小館</v>
-      </c>
-      <c r="D160" t="str">
-        <v>宋家小館｜Becky</v>
-      </c>
-      <c r="E160">
-        <v>0</v>
-      </c>
-      <c r="F160" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B161">
-        <v>5</v>
-      </c>
-      <c r="C161" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
-      </c>
-      <c r="D161" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
-      </c>
-      <c r="E161">
-        <v>0</v>
-      </c>
-      <c r="F161" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B162">
-        <v>6</v>
-      </c>
-      <c r="C162" t="str">
-        <v>任性歐逆機智生活</v>
-      </c>
-      <c r="D162" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
-      </c>
-      <c r="E162">
-        <v>0</v>
-      </c>
-      <c r="F162" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B163">
-        <v>7</v>
-      </c>
-      <c r="C163" t="str">
-        <v>楊肉盧</v>
-      </c>
-      <c r="D163" t="str">
-        <v>楊月娥（楊肉爐）</v>
-      </c>
-      <c r="E163">
-        <v>0</v>
-      </c>
-      <c r="F163" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B164">
-        <v>8</v>
-      </c>
-      <c r="C164" t="str">
-        <v>爛泥Jill式優雅</v>
-      </c>
-      <c r="D164" t="str">
-        <v>爛泥媽媽的重生日記（Jill)</v>
-      </c>
-      <c r="E164">
-        <v>0</v>
-      </c>
-      <c r="F164" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B165">
-        <v>9</v>
-      </c>
-      <c r="C165" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
-      </c>
-      <c r="D165" t="str">
-        <v>人生啊！小歐</v>
-      </c>
-      <c r="E165">
-        <v>0</v>
-      </c>
-      <c r="F165" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B166">
-        <v>10</v>
-      </c>
-      <c r="C166" t="str">
-        <v>下半場人生陪談師</v>
-      </c>
-      <c r="D166" t="str">
-        <v>下半場人生事務有限公司</v>
-      </c>
-      <c r="E166">
-        <v>0</v>
-      </c>
-      <c r="F166" t="str">
-        <v>平均評等 0 星，累計 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B167">
-        <v>1</v>
-      </c>
-      <c r="C167" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="D167" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="E167">
-        <v>0</v>
-      </c>
-      <c r="F167" t="str">
-        <v>近半年評等 5 星，新增 0 則評論。綜合指標得分：5 / 10 分。</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B168">
-        <v>2</v>
-      </c>
-      <c r="C168" t="str">
-        <v>迷途艾比</v>
-      </c>
-      <c r="D168" t="str">
-        <v>迷途艾比</v>
-      </c>
-      <c r="E168">
-        <v>0</v>
-      </c>
-      <c r="F168" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B169">
-        <v>3</v>
-      </c>
-      <c r="C169" t="str">
-        <v>山姆書書</v>
-      </c>
-      <c r="D169" t="str">
-        <v>山姆書書</v>
-      </c>
-      <c r="E169">
-        <v>0</v>
-      </c>
-      <c r="F169" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B170">
-        <v>4</v>
-      </c>
-      <c r="C170" t="str">
-        <v>宋家小館</v>
-      </c>
-      <c r="D170" t="str">
-        <v>宋家小館｜Becky</v>
-      </c>
-      <c r="E170">
-        <v>0</v>
-      </c>
-      <c r="F170" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B171">
-        <v>5</v>
-      </c>
-      <c r="C171" t="str">
-        <v>《姐姐不想懂事了》 | Soft Rebellion</v>
-      </c>
-      <c r="D171" t="str">
-        <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
-      </c>
-      <c r="E171">
-        <v>0</v>
-      </c>
-      <c r="F171" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B172">
-        <v>6</v>
-      </c>
-      <c r="C172" t="str">
-        <v>任性歐逆機智生活</v>
-      </c>
-      <c r="D172" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
-      </c>
-      <c r="E172">
-        <v>0</v>
-      </c>
-      <c r="F172" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B173">
-        <v>7</v>
-      </c>
-      <c r="C173" t="str">
-        <v>楊肉盧</v>
-      </c>
-      <c r="D173" t="str">
-        <v>楊月娥（楊肉爐）</v>
-      </c>
-      <c r="E173">
-        <v>0</v>
-      </c>
-      <c r="F173" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B174">
-        <v>8</v>
-      </c>
-      <c r="C174" t="str">
-        <v>爛泥Jill式優雅</v>
-      </c>
-      <c r="D174" t="str">
-        <v>爛泥媽媽的重生日記（Jill)</v>
-      </c>
-      <c r="E174">
-        <v>0</v>
-      </c>
-      <c r="F174" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B175">
-        <v>9</v>
-      </c>
-      <c r="C175" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
-      </c>
-      <c r="D175" t="str">
-        <v>人生啊！小歐</v>
-      </c>
-      <c r="E175">
-        <v>0</v>
-      </c>
-      <c r="F175" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="str">
-        <v>聽眾都要跟你獎 (近半年有評論數)</v>
-      </c>
-      <c r="B176">
-        <v>10</v>
-      </c>
-      <c r="C176" t="str">
-        <v>下半場人生陪談師</v>
-      </c>
-      <c r="D176" t="str">
-        <v>下半場人生事務有限公司</v>
-      </c>
-      <c r="E176">
-        <v>0</v>
-      </c>
-      <c r="F176" t="str">
-        <v>近半年評等 0 星，新增 0 則評論。綜合指標得分：0 / 10 分。</v>
+        <v>平均評等 5 星，累計 2 則評論。</v>
+      </c>
+      <c r="G158" t="str" xml:space="preserve">
+        <v xml:space="preserve">【考上明星高中卻格格不入：自我懷疑的開端】
+時間: 03:17 - 04:44
+單集: EP.317 出走，不是逃離，而是回到自己：《臺灣製造》作者安吉的人生覺醒之路
+理由: 來賓生動地描述了她意外考上明星高中後，卻感到格格不入的經歷。這段內容深刻地揭示了外在成就與內心認同之間的落差，以及自我懷疑的萌芽，情感真摯且引人入勝，為後續的自我探索旅程奠定基礎。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F176"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G158"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Complete Best Duo Hosts Top 8 Re-eval and update scores
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G148"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -784,7 +784,7 @@
         <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E15">
-        <v>9.1931</v>
+        <v>9.19</v>
       </c>
       <c r="F15" t="str">
         <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
@@ -810,7 +810,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E16">
-        <v>8.8049</v>
+        <v>8.8</v>
       </c>
       <c r="F16" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
@@ -836,7 +836,7 @@
         <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
       <c r="E17">
-        <v>8.7715</v>
+        <v>8.77</v>
       </c>
       <c r="F17" t="str">
         <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
@@ -862,7 +862,7 @@
         <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="E18">
-        <v>8.6049</v>
+        <v>8.6</v>
       </c>
       <c r="F18" t="str">
         <v>[跟長輩一樣就能學會AI？陶韻智...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高，但偶有輕微搶話情況，整體默契良好。 | [再不用證明自己給誰看 feat...] 雙主持人與來賓之間的互動自然，接話流暢，笑聲具感染力，展現了良好的默契，即使有插話也多能順暢銜接。 | [好像很爽，我們也去當個旅遊作家...] 兩位主持人與來賓之間的對話流暢自然，接話和反應迅速，共同營造了輕鬆愉快的氛圍，默契良好。</v>
@@ -1018,7 +1018,7 @@
         <v>美股夢想家</v>
       </c>
       <c r="E24">
-        <v>9.6786</v>
+        <v>9.68</v>
       </c>
       <c r="F24" t="str">
         <v>[EP289  七巨頭變七矮人！...] 選題新穎且具時效性，深入分析了科技巨頭的市場變化與供應鏈影響，內容含金量極高。 | [EP275 股市變賭場？巴菲特...] 選題緊扣時事熱點（巴菲特、AI、台股美股），內容深度足夠，結合了宏觀經濟分析、產業趨勢與個股案例，資訊含金量高，企劃具備高度專業性。 | [EP251國防預算暴漲 5 成...] 選題結合時事（軍工股、AI、經濟預測），數據分析詳盡，提供獨到見解，內容含金量高。</v>
@@ -1044,7 +1044,7 @@
         <v>我的動齡限量版</v>
       </c>
       <c r="E25">
-        <v>9.6549</v>
+        <v>9.65</v>
       </c>
       <c r="F25" t="str">
         <v>[[EP0063] 50+Con...] 選題新穎，結合「第三人生大學」與「大嬸陪聊」概念，案例生動且含金量極高，具備深度思考與社會連結。 | [[EP0071] 50+Con...] 選題新穎且具深度，聚焦於二代接班與職涯轉型，來賓的個人案例生動且含金量極高，提供了獨特的視角和實用建議。 | [[EP0045] 50+Con...] 選題深入探討紫微斗數的「四化」與「殺破狼」命格，不僅新穎且具備高度的專業含金量。來賓的案例分享與對社會現象的連結，讓內容更具啟發性與實用價值。</v>
@@ -1226,7 +1226,7 @@
         <v>美股夢想家</v>
       </c>
       <c r="E32">
-        <v>9.312</v>
+        <v>9.31</v>
       </c>
       <c r="F32" t="str">
         <v>[EP289  七巨頭變七矮人！...] 男主持人聲音清晰、語速穩定且富有能量，但口頭禪「那」、「然後」、「就是」出現頻率稍高。 | [EP275 股市變賭場？巴菲特...] 男主持人聲音清晰、語速穩定且富有感染力，中低音共鳴良好。但口頭禪「那」、「然後」、「就是」等使用頻率稍高，若能減少會更佳。 | [EP251國防預算暴漲 5 成...] 男主持人語速極快但口條流暢，發音清晰，聲音有力量和共鳴感，情緒感染力強。</v>
@@ -1252,7 +1252,7 @@
         <v>GK爸爸</v>
       </c>
       <c r="E33">
-        <v>9.2549</v>
+        <v>9.25</v>
       </c>
       <c r="F33" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 男主持人語速穩定，發音清晰，中低音共鳴感強，能透過聲線變化塑造多個角色，情感渲染力極佳。 | [春暖花開小旅行...] 男主持人聲音溫暖厚實，口條流暢清晰，語速雖快但穩定，能透過聲線變化塑造不同角色，具備良好的渲染力。 | [【QQ偵探：鳳梨酥失竊案 上集...] 男主持人聲音清晰、富有表現力，能透過聲線變化塑造不同角色，語速穩定，但偶有贅字。</v>
@@ -1356,7 +1356,7 @@
         <v>文森說書</v>
       </c>
       <c r="E37">
-        <v>9.0875</v>
+        <v>9.09</v>
       </c>
       <c r="F37" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 男主持人聲音清晰、語速穩定，中低音共鳴感強，具有良好的渲染力。口頭禪「就是」和「然後」的頻率略高，但整體不影響流暢度。 | [我們可能會成為最殘忍的一代｜《...] 男主持��聲音共鳴感強，中低音厚實，語速穩定且清晰，情感渲染力佳，能有效傳達複雜的內容。雖然偶有口頭禪，但不影響整體專業度。</v>
@@ -1434,7 +1434,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E40">
-        <v>9.3215</v>
+        <v>9.32</v>
       </c>
       <c r="F40" t="str">
         <v>[EP470｜把人放在心上的共贏...] 女主持人不姐的口條流暢，聲音清晰且語速穩定，高音域圓潤並帶有溫馨陪伴感，雖偶有贅字但整體表現優異。 | [EP433｜【中年轉型】從矽谷...] 女主持人語速穩定，發音清晰，聲音溫暖圓潤且富有感染力，雖有少量贅字但不影響整體表現。 | [EP466｜拒絕被朝九晚五綁架...] 女主持人（不解）的口條極為流暢，發音清晰，語速雖快但穩定且富有節奏感。高音域圓潤，聲音溫暖，具有強烈的陪伴感。</v>
@@ -1460,7 +1460,7 @@
         <v>莫菲穿搭</v>
       </c>
       <c r="E41">
-        <v>9.3049</v>
+        <v>9.3</v>
       </c>
       <c r="F41" t="str">
         <v>[莫菲穿搭20｜球具只是通行證？...] 女主持人聲音清晰、溫暖且富有親和力，高音域圓潤，語速穩定舒適。她能精準提問，引導來賓深入分享，並透過自然的反應和笑聲，營造出溫馨愉快的氛圍，展現了優異的播音實力與陪伴感。 | [莫菲穿搭27｜金曲幕後直擊！電...] 女主持人聲音清晰、語速穩定（儘管有時偏快），語調溫暖且富有感染力，��刺耳感。 | [莫菲穿搭02｜2026流行色配...] 女主持人聲音清晰、語速穩定，高音域圓潤且具備陪伴感，但口頭禪「那」和「就是」出現頻率稍高。</v>
@@ -1486,7 +1486,7 @@
         <v>蘇絢慧分享空間</v>
       </c>
       <c r="E42">
-        <v>9.2715</v>
+        <v>9.27</v>
       </c>
       <c r="F42" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 女主持人聲音清晰、圓潤，語速穩定且語調溫和，情感表達真誠，特別在引導環節展現極佳的陪伴感，非常符合節目調性。 | [EP21｜為什麼總是替傷害你的...] 女主持人的口條流暢，聲音清晰且富有溫暖的共鳴感，語速穩定，給人舒適的聆聽體驗。 | [EP28｜走進孩子的情緒小劇場...] 女主持人的口條流暢，聲音清晰溫暖，語速穩定且高音域圓潤，給人極佳的陪伴感。</v>
@@ -1512,7 +1512,7 @@
         <v>宋家小館｜Becky</v>
       </c>
       <c r="E43">
-        <v>9.2549</v>
+        <v>9.25</v>
       </c>
       <c r="F43" t="str">
         <v>[EP162 | 從房地產到Ma...] 女主持人Becky的口條流暢，聲音清晰溫暖，語速穩定且富有親和力，給人溫馨陪伴感。 | [EP191 | 《我到日本當漁...] 女主持人（Becky）聲音清晰、溫暖且富有親和力，語速有時偏快但整體穩定，高音域圓潤，具備良好的陪伴感。 | [EP182 | 聽見身體的聲音...] 主持人Becky聲音清晰圓潤，語速穩定舒適（約205字/分），語調溫和具親和力。來賓Vivi老師語速雖快但咬字清晰，聲音亦佳。</v>
@@ -1538,7 +1538,7 @@
         <v>聲音表達講師林依柔</v>
       </c>
       <c r="E44">
-        <v>9.2549</v>
+        <v>9.25</v>
       </c>
       <c r="F44" t="str">
         <v>[EP.61｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有活力，語速雖快但咬字精準，高音域圓潤不刺耳，帶有溫馨的陪伴感。來賓紫菱的聲音也同樣清晰且富有共鳴，兩位女性的聲線皆表現出色。 | [EP.59｜【說話人聲-會客室...] 主持人伊柔的聲音清晰、明亮且富有感染力，語速雖快但發音清晰。來賓Karen的聲音則沉穩，兩者搭配得宜。 | [EP.59｜【說話人聲-會客室...] 女主持人（一柔）的聲音清晰、溫暖且富有感���力，語速穩定且情緒飽滿，能有效帶動節目氣氛，展現了極佳的播音魅力。</v>
@@ -1590,7 +1590,7 @@
         <v>丁菱娟</v>
       </c>
       <c r="E46">
-        <v>9.1549</v>
+        <v>9.15</v>
       </c>
       <c r="F46" t="str">
         <v>[ep21. 用台灣腦袋，看透全...] 主持人丁菱娟口條流暢，聲音清晰，語速穩定且高音域圓潤，帶有溫馨陪伴感，雖有口頭禪「那」但整體表現優異。 | [ep11. Z世代難搞嗎？用對...] 女主持人丁菱娟的口條極為流暢，聲音清晰明亮，語速穩定且富有變化，高音域圓潤，語調溫暖且具備溫馨陪伴感，能有效引導聽眾進入話題，情緒感染力佳。 | [ep23. 主動出擊的力量有多...] 女主持人聲音溫暖清晰，語速穩定，高音域圓潤且具陪伴感，提���精準，控場得宜。</v>
@@ -1616,7 +1616,7 @@
         <v>我的動齡限量版</v>
       </c>
       <c r="E47">
-        <v>9.1549</v>
+        <v>9.15</v>
       </c>
       <c r="F47" t="str">
         <v>[[EP0063] 50+Con...] 主持人Connie口條流暢，聲音清晰明亮，語速穩定且富有情感，高音域圓潤，具備溫馨陪伴感。 | [[EP0071] 50+Con...] 主持人Connie的口條流暢，聲音清晰且富有感染力，語速穩定，高音域圓潤，展現了優異的播音實力。 | [[EP0045] 50+Con...] 主持人Connie的聲音清亮圓潤，富有活力與親和力，語速雖快但咬字清晰，情緒感染力強，能有效帶動節目氣氛。</v>
@@ -1642,7 +1642,7 @@
         <v>孫子玲</v>
       </c>
       <c r="E48">
-        <v>9.1215</v>
+        <v>9.12</v>
       </c>
       <c r="F48" t="str">
         <v>[#95 ▍ 冷戰半年怎麼破冰？...] 女主持人聲音清晰、語速穩定且富有能量，高音域圓潤，雖語速較快但仍具陪伴感，發音無刺耳感。 | [#99 ▍別讓金錢焦慮，成了教...] 女主持人紫琳口條流暢，聲音清晰溫暖，語速穩定且富有親和力，高音域圓潤，給人溫馨陪伴感。 | [#93 ▍自學，不是逃避的出口...] 女主持人紫菱的口條流暢，聲音清晰溫暖，語速穩定且富有情感，高音域圓潤無刺耳感，具備極佳的陪伴與治癒特質。</v>
@@ -1668,7 +1668,7 @@
         <v>佐依Zoey</v>
       </c>
       <c r="E49">
-        <v>9.1049</v>
+        <v>9.1</v>
       </c>
       <c r="F49" t="str">
         <v>[#336 #Zoey｜你覺得自...] 女主持人聲音清晰、語速穩定，高音域圓潤且富有陪伴感��口條流暢，整體播音實力優異。 | [#我，是誰？S2E2｜為什麼越...] 主持人Zoe的口條流暢，聲音清晰且語速穩定，高音域圓潤且富有陪伴感，情緒感染力佳。 | [#我，是誰？S2E3｜過度依賴...] 主持人Zoe的語速穩定，發音清晰，語調溫和，預期能給予聽眾溫馨的陪伴感，且在引導對話時展現專業度。</v>
@@ -1980,7 +1980,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E61">
-        <v>9.0549</v>
+        <v>9.05</v>
       </c>
       <c r="F61" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 議題雖然熱門，但節目將其從醫學、社會、政策等多維度進行深入探討，使其在同類內容中具有獨特的深度和廣度。 | [《財富自由心理學》：賺錢，只是...] 將財富自由與心理學深度結合，探討其背後的幸福、選擇與自我價值，此議題切入點獨特，在廣泛的財經或心靈類節目中具備高度稀有性與利基市場價值。 | [手總是停不下來？那是焦慮在尋找...] 議題具有一定的稀有度，深入探討身體重複行為，論述完整且具專業性。</v>
@@ -2006,7 +2006,7 @@
         <v>宋家小館｜Becky</v>
       </c>
       <c r="E62">
-        <v>8.9215</v>
+        <v>8.92</v>
       </c>
       <c r="F62" t="str">
         <v>[EP162 | 從房地產到Ma...] 議題結合傳統產業與科技創新，並融入個人成長與興趣，論述完整且具有一定稀有度。 | [EP191 | 《我到日本當漁...] 議題稀有度高，深入探討台灣養殖業的發展與赴日漁業的挑戰，對冷門利基市場的論述完整且具深度。 | [EP182 | 聽見身體的聲音...] 頌缽音療在台灣仍屬相對利基的市場，節目深入探討其原理與應用，論述完整，具有獨特性。</v>
@@ -2032,7 +2032,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E63">
-        <v>8.8098</v>
+        <v>8.81</v>
       </c>
       <c r="F63" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 雖然關懷弱勢並非絕對冷門，但浪人食堂以「陪伴與連結」為核心，並讓「受助者成為助人者」的獨特模式，使其在公益領域中具備顯著的利基市場與論述深度。 | [【大師專題】人在江湖，身不由己...] 古龍雖是知名作家，但節目從其個人生命經驗與創作哲學的深度連結切入，探討其作品中的孤獨與人性，這在廣泛的文學討論中屬於較為利基且深入的視角。 | [【中年，正在試】把世界走成一本...] 中亞是相對冷門的旅遊目的地，節目對此議題的論述非常完整且深入，填補了市場空白。</v>
@@ -2058,7 +2058,7 @@
         <v>蕭邦</v>
       </c>
       <c r="E64">
-        <v>8.6296</v>
+        <v>8.63</v>
       </c>
       <c r="F64" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 結合個人成長、財務困境與易經、冰山理論等多元且非主流的視角，議題稀有度高，論述完整。 | [【蕭邦出任務】如何選擇適合自己...] 議題聚焦於職涯轉型與個人成長，並深入探討行銷產業的真實面貌，具有一定的稀有度與論述完整度。 | [幸福的人，通常「覺察力」都很強...] 「覺察」議題雖非極度冷門，但主持人以個人經驗與獨特視角切入，論述完整，具���一定差異化。</v>
@@ -2084,7 +2084,7 @@
         <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="E65">
-        <v>8.6049</v>
+        <v>8.6</v>
       </c>
       <c r="F65" t="str">
         <v>[跟長輩一樣就能學會AI？陶韻智...] 議題具前瞻性與專業性，對特定受眾（如AI使用者、職場工作者）有高度吸引力，論述完整。 | [再不用證明自己給誰看 feat...] 節目聚焦於女性理財與自我成長，並結合家族企業轉型等議題，在特定受眾群體中具有較高的議題稀有度與論述完整度。 | [好像很爽，我們也去當個旅遊作家...] 節目聚焦於旅遊作家的職業生涯，是一個相對利基且被深入探討的市場，論述完整。</v>
@@ -2110,7 +2110,7 @@
         <v>蘇絢慧分享空間</v>
       </c>
       <c r="E66">
-        <v>8.6049</v>
+        <v>8.6</v>
       </c>
       <c r="F66" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 節目將「愛自己」的議題與心理學、依戀理論深度結合，使其在廣泛的自我成長市場中，開闢出一個具備專業深度與獨特視角的利基市場。 | [EP21｜為什麼總是替傷害你的...] 議題雖然屬於心理學範疇，但深入探討「替傷害者找理由」的具體心理機制，切入點獨特，論述完整。 | [EP28｜走進孩子的情緒小劇場...] 議題結合高敏感特質與戲劇治療，屬於相對���有且具專業深度的利基市場，論述完整。</v>
@@ -2136,7 +2136,7 @@
         <v>文森說書</v>
       </c>
       <c r="E67">
-        <v>8.5875</v>
+        <v>8.59</v>
       </c>
       <c r="F67" t="str">
         <v>[這一集我準備了兩個月，但是太值...] 「童年情感忽視」是一個相對小眾但極具深度的心理學議題，主持人對此議題的論述完整且具啟發性，符合利基市場的評估。 | [我們可能會成為最殘忍的一代｜《...] 「道德雄心」的議題雖然不完全是冷門，但主持人以獨特的角度和豐富的案例進行深入論述，使其在同類議題中脫穎而出，具備利基市場的完整度。</v>
@@ -2162,7 +2162,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E68">
-        <v>8.5598</v>
+        <v>8.56</v>
       </c>
       <c r="F68" t="str">
         <v>[【EP330 帶著善意行動，最...] 雖然是傳統滷味店的創業故事，但結合了公益行動和品牌轉型，使其在市場中具有獨特性，論述完整。 | [【EP302 把命盤變成行動藍...] 議題聚焦於東方命理的特定流年，並結合現代社會趨勢進行深入探討，具備高度的稀有性與利基市場論述完整度。 | [【EP312《超越我執的生活》...] 「超越我執」的議題在心靈成長領域中具有一定的深度與獨特性，雖非極度冷門，但其論述角度與實踐方法提供了較為利基的觀點。</v>
@@ -2188,7 +2188,7 @@
         <v>胡咪老師</v>
       </c>
       <c r="E69">
-        <v>8.5296</v>
+        <v>8.53</v>
       </c>
       <c r="F69" t="str">
         <v>[S4.EP4｜性平教育20年，...] 議題探討深入，特別關注數位時代下的約會暴力、男性及LGBTQ+受害者的困境，具備高度利基市場的獨特性。 | [S4.EP8｜我不想再跟你生活...] 議題聚焦於離婚後的心理歷程與微小生活習慣的影響，雖非極度冷門，但論述角度獨特且完整。 | [S4.EP14｜有些人沒有成為...] 「比前任更難忘的非前任」這一議題雖然具有普世性，但節目從心理學、文學和個人經驗等多維度進行深入探討，使其在同類節目中具備獨特的利基市場論述。</v>
@@ -2214,7 +2214,7 @@
         <v>蘇絢慧分享空間</v>
       </c>
       <c r="E70">
-        <v>9.2715</v>
+        <v>9.27</v>
       </c>
       <c r="F70" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 主講人溫柔穩定的語調與深具療癒性的內容，非常適合深夜聆聽，能有效安撫情緒，提供寧靜的陪伴感，無任何突兀尖銳的聲音。 | [EP21｜為什麼總是替傷害你的...] 主講人語調溫柔穩定，內容引人深思，非常適合在深夜時段聆聽，具有強烈的陪伴治癒感。 | [EP28｜走進孩子的情緒小劇場...] 主持人與來賓的語調皆溫柔穩定，對談內容引人深思，非常適合深夜聆聽，具有治癒感。</v>
@@ -2266,7 +2266,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E72">
-        <v>8.9715</v>
+        <v>8.97</v>
       </c>
       <c r="F72" t="str">
         <v>[EP225：【非典家庭CEO】...] 語調溫柔穩定，對談內容雖有沉重之處，但整體氛圍溫暖且具治癒感，無突兀尖銳爆音，適合深夜聆聽。 | [EP218：愛自己｜放下完美執...] 講者聲音溫和穩定，內容雖有深度但語調不急不躁，適合在夜晚放鬆心情聆聽，具有一定的陪伴治癒感。 | [EP219：【非典家庭CEO】...] 整體談話氛圍溫和穩定，主持人與來賓的聲線皆具安撫感，適合深夜聆聽。</v>
@@ -2292,7 +2292,7 @@
         <v>佐依Zoey</v>
       </c>
       <c r="E73">
-        <v>8.9296</v>
+        <v>8.93</v>
       </c>
       <c r="F73" t="str">
         <v>[#336 #Zoey｜你覺得自...] 主講人語調溫柔穩定，內容引人深思，無突兀尖銳爆音，非常適合深夜聆聽，提供治癒與陪伴感。 | [#我，是誰？S2E2｜為什麼越...] 主持人語調溫柔穩定，內容引人深思，無突兀尖銳音頻，非常適合深夜靜心聆聽，營造出治癒的陪伴感。 | [#我，是誰？S2E3｜過度依賴...] 節目主題深度且具反思性，主持人語調溫和穩定，預期能營造出適合深夜聆聽的平靜氛圍，無突兀尖銳音效。</v>
@@ -2318,7 +2318,7 @@
         <v>GK爸爸</v>
       </c>
       <c r="E74">
-        <v>8.9215</v>
+        <v>8.92</v>
       </c>
       <c r="F74" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人溫暖的聲線、舒緩的背景音樂與引人入勝的故事，營造出極佳的深夜陪伴與治癒感，無突兀尖銳爆音。 | [春暖花開小旅行...] 主持人語調溫柔穩定，搭配輕柔背景音樂，營造出極佳的陪伴治癒感，適合深夜聆聽。 | [【QQ偵探：鳳梨酥失竊案 上集...] 敘事語調平穩溫和，故事引人入勝，適合在夜晚聆聽，無突兀尖銳爆音。</v>
@@ -2344,7 +2344,7 @@
         <v>宋家小館｜Becky</v>
       </c>
       <c r="E75">
-        <v>8.9022</v>
+        <v>8.9</v>
       </c>
       <c r="F75" t="str">
         <v>[EP162 | 從房地產到Ma...] 聲音平穩溫和，語調舒適，適合深夜靜聽，無突兀尖銳爆音。 | [EP191 | 《我到日本當漁...] 主持人語調溫和，聲音具陪伴感，但部分內容涉及艱辛挑戰，情緒較為嚴肅，不完全是純粹的輕柔治癒氛圍。 | [EP182 | 聽見身體的聲音...] 聲音平穩溫和，頌缽音效本身就極具安撫作用，主持人語調也具備陪伴治癒感，無突兀尖銳爆音，非常適合深夜聆聽。</v>
@@ -2396,7 +2396,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E77">
-        <v>8.8215</v>
+        <v>8.82</v>
       </c>
       <c r="F77" t="str">
         <v>[EP470｜把人放在心上的共贏...] 主持人的語調溫柔穩定，聲音平穩，無突兀尖銳爆音，適合在深夜時段靜心聆聽，具有陪伴治癒感。 | [EP433｜【中年轉型】從矽谷...] 主持人語調溫柔穩定，聲音具陪伴感，無突兀尖銳音，非常適合深夜聆聽與自我反思。 | [EP466｜拒絕被朝九晚五綁架...] 主持人溫暖的語調與來賓沉穩的分享，營造出一個適合深夜聆聽的氛圍。對話內容引人深思，無突兀的尖銳爆音，具有安撫感。</v>
@@ -2422,7 +2422,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E78">
-        <v>8.8215</v>
+        <v>8.82</v>
       </c>
       <c r="F78" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 節目整體語調溫和穩定，內容富有深度與情感，非常適合在深夜時段聆聽，能帶來治癒與陪伴感，且無突兀尖銳的聲音。 | [【大師專題】人在江湖，身不由己...] 主持人的語調溫和穩定，聲音共鳴感強，內容富有深度與思考性，非常適合在深夜靜心聆聽，具有良好的陪伴與治癒感，無突兀尖銳爆音。 | [【中年，正在試】把世界走成一本...] 語調溫和穩定，內容引人入勝，適合深夜聆聽，無突兀尖銳爆音。</v>
@@ -2448,7 +2448,7 @@
         <v>下半場人生事務有限公司</v>
       </c>
       <c r="E79">
-        <v>8.8098</v>
+        <v>8.81</v>
       </c>
       <c r="F79" t="str">
         <v>[44-解開品牌人生的迷思，從認...] 主持人聲音平穩溫和，內容具深度思考，適合深夜靜心聆聽，無突兀尖銳爆音。 | [57-慢活的幸福人生 – 台灣...] 兩位主講人的語調皆溫柔穩定，內容具反思性與啟發性，無突兀尖銳爆音，非常適合深夜靜心聆聽，提供治癒陪伴感。 | [59-人生下半場，人際好感怎麽...] 主持人與來賓的語調皆溫和穩定，內容引人深思，適合深夜靜心聆聽，無突兀尖銳爆音。</v>
@@ -2500,7 +2500,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E81">
-        <v>9.1049</v>
+        <v>9.1</v>
       </c>
       <c r="F81" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 節奏明快，開頭活力十足，主持人聲音清晰，具有提神醒腦的效果。 | [EP174｜越省反而越窮？別把...] 節奏明快，開頭充滿活力，內容具啟發性，適合通勤提神醒腦。 | [EP164｜滑短影音是在浪費時...] 節目內容具啟發性，節奏明快，開頭活力十足，適合通勤時段收聽，能提供思考的刺激而非單純的提神。</v>
@@ -2578,7 +2578,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E84">
-        <v>9.0431</v>
+        <v>9.04</v>
       </c>
       <c r="F84" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 節���節奏明快，主持人語調朝氣蓬勃，內容具啟發性，適合通勤時提神醒腦。 | [《財富自由心理學》：賺錢，只是...] 節目節奏明快，對談內容富有深度與啟發性，能有效刺激思考，適合通勤或早晨收聽以提振精神。 | [手總是停不下來？那是焦慮在尋找...] 節奏明快，語調朝氣，但因內容較為嚴肅，提神醒腦度相對普通。</v>
@@ -2656,7 +2656,7 @@
         <v>丁菱娟</v>
       </c>
       <c r="E87">
-        <v>8.9796</v>
+        <v>8.98</v>
       </c>
       <c r="F87" t="str">
         <v>[ep21. 用台灣腦袋，看透全...] 節目節奏明快，內容資訊豐富，能有效提振精神，適合通勤或早晨收聽。 | [ep11. Z世代難搞嗎？用對...] 節目節奏明快，內容資訊量豐富且具啟發性，能有效刺激思考。主持人與來賓的對談充滿活力，適合通勤時提神醒腦。 | [ep23. 主動出擊的力量有多...] 節目節奏明快，內容充滿正能量與激勵，非常適合早晨通勤時提神醒腦。</v>
@@ -2682,7 +2682,7 @@
         <v>不敗教主-陳重銘</v>
       </c>
       <c r="E88">
-        <v>8.9715</v>
+        <v>8.97</v>
       </c>
       <c r="F88" t="str">
         <v>[EP611 00998A(主動...] 節奏明快，語調清晰，資訊量高，適合通勤時收聽以獲取財經知識，具提神效果。 | [EP628昇陽半導體(8028...] 節奏明快，語調朝氣且資訊量豐富，適合通勤時提神醒腦，快速吸收新知。 | [EP621《富媽媽 窮媽媽》第...] 節目節奏明快，內容資訊量豐富且邏輯清晰，能有效提振精神，適合通勤時收聽，有助於醒腦。</v>
@@ -2708,7 +2708,7 @@
         <v>閱讀聊樂key</v>
       </c>
       <c r="E89">
-        <v>8.9715</v>
+        <v>8.97</v>
       </c>
       <c r="F89" t="str">
         <v>[EP213 越學越焦慮？郝旭烈...] 節目節奏明快、主持人聲音充滿活力，內容具啟發性，非常適合在早晨通勤時聆聽，有助於提神醒腦並激發思考。 | [EP202 提升「語言含金量」...] 節目節奏明快，主持人與來賓的語氣都充滿活力，內容引人入勝，非常適合通勤時提神醒腦。 | [EP195 中年開始被淘汰，不...] 節目節奏明快，主持人與來賓的語調充滿朝氣與活力，內容引人入勝且具啟發性，非常適合通勤時收聽，能有效提神醒腦並激發思考。</v>
@@ -2734,7 +2734,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E90">
-        <v>8.6296</v>
+        <v>8.63</v>
       </c>
       <c r="F90" t="str">
         <v>[EP225：【非典家庭CEO】...] 節目透過真實的生命故事，傳遞了愛與陪伴的力量，雖然內容有挑戰性，但最終帶來的是心靈的慰藉與正向能量，笑聲自然且真誠。 | [EP218：愛自己｜放下完美執...] 節目內容偏向知識性與自我探索，雖然能帶來啟發，但輕鬆歡樂的解壓感相對較少，笑聲自然但非主要風格。 | [EP219：【非典家庭CEO】...] 談話風格輕鬆歡樂，主持人與來賓的自然笑聲與分享，帶來愉悅的解壓感。</v>
@@ -2760,7 +2760,7 @@
         <v>胡咪老師</v>
       </c>
       <c r="E91">
-        <v>8.3522</v>
+        <v>8.35</v>
       </c>
       <c r="F91" t="str">
         <v>[S4.EP4｜性平教育20年，...] 談話風格較為嚴肅和深度，旨在引發思考而非輕鬆解壓，因此療癒感較為���接。 | [S4.EP8｜我不想再跟你生活...] 節目透過分享與討論，幫助聽眾處理複雜情感，雖有沉重話題，但整體氛圍仍能帶來情感上的釋放與療癒。 | [S4.EP14｜有些人沒有成為...] 節目透過對情感困惑的深入剖析，以及分享重逢的溫暖故事，為聽眾提供了情感上的釋放與療癒。主持人的真誠對談與幽默感也為節目增添了輕鬆氛圍。</v>
@@ -2786,7 +2786,7 @@
         <v>佐依Zoey</v>
       </c>
       <c r="E92">
-        <v>8.2598</v>
+        <v>8.26</v>
       </c>
       <c r="F92" t="str">
         <v>[#336 #Zoey｜你覺得自...] 節目內容雖具啟發性，但風格較為嚴肅與哲學，而非輕鬆歡樂的日常廢話，因此解壓療癒感相對較低。 | [#我，是誰？S2E2｜為什麼越...] 內容深度探討內在，能帶來心靈上的療癒，但談話風格較為嚴肅，非輕鬆歡樂的解壓類型。 | [#我，是誰？S2E3｜過度依賴...] 節目聚焦於自我成長、內在探索與接納，透過深度對話引導聽眾反思，具有強烈的療��與啟發感，有助於聽眾釋放壓力。</v>
@@ -2812,7 +2812,7 @@
         <v>GK爸爸</v>
       </c>
       <c r="E93">
-        <v>8.2431</v>
+        <v>8.24</v>
       </c>
       <c r="F93" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 節目透過溫馨的故事與對母愛的歌頌，帶來情感上的慰藉與放鬆，具有良好的療癒效果。 | [春暖花開小旅行...] 故事內容輕鬆愉快，傳達正向價值觀，能帶來放鬆與療癒感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 作為偵探故事，主要著重於情節發展，而非輕鬆歡樂的療癒感。</v>
@@ -2838,7 +2838,7 @@
         <v>孫子玲</v>
       </c>
       <c r="E94">
-        <v>8.1215</v>
+        <v>8.12</v>
       </c>
       <c r="F94" t="str">
         <v>[#95 ▍ 冷戰半年怎麼破冰？...] 談話風格輕鬆且帶有幽默感，內容提供解決方案，能為聽眾帶來正向的解壓與療癒感受。 | [#99 ▍別讓金錢焦慮，成了教...] 談話風格真誠且富有同理心，透過分享個人經驗與心理學知識，能為聽眾帶來理解與療癒感。 | [#93 ▍自學，不是逃避的出口...] 透過真誠的對話與分享，提供情感上的支持與理解，有助於聽眾釋放壓力，但談話風格較為認真，非純粹輕鬆歡樂。</v>
@@ -2864,7 +2864,7 @@
         <v>五吉郎</v>
       </c>
       <c r="E95">
-        <v>8.1049</v>
+        <v>8.1</v>
       </c>
       <c r="F95" t="str">
         <v>[EP133｜顛覆你對美容業的想...] 談話內容較為嚴肅認真，聚焦於創業與自我成長，解壓療癒感普通，笑聲自然但不多。 | [EP174｜越省反而越窮？別把...] 內容偏向知識性與深度思考，輕鬆歡樂的療癒感較少。 | [EP164｜滑短影音是在浪費時...] 雖然主題涉及自我成長與心靈啟發，但談話風格偏向理性分析與觀點分享，而非輕鬆歡樂的解壓或日常廢話，因此療癒感較為內斂。</v>
@@ -2890,7 +2890,7 @@
         <v>蘇絢慧分享空間</v>
       </c>
       <c r="E96">
-        <v>8.0742</v>
+        <v>8.07</v>
       </c>
       <c r="F96" t="str">
         <v>[EP30｜愛自己，為什麼這麼難...] 節目透過理解自我、接納脆弱、並學習溫柔對待自己的過程，提供了深刻的療癒體驗，談話風格真誠且富有同理心。 | [EP21｜為什麼總是替傷害你的...] 節目風格偏向嚴肅的心理分析，而非輕鬆歡樂的療癒，因此解壓感較低。 | [EP28｜走進孩子的情緒小劇場...] 談話風格真誠且富有同理心，透過分享個人成長歷程，能為聽眾帶來心靈上的理解與慰藉，具有療癒感。</v>
@@ -2916,7 +2916,7 @@
         <v>梁哲維</v>
       </c>
       <c r="E97">
-        <v>8.0598</v>
+        <v>8.06</v>
       </c>
       <c r="F97" t="str">
         <v>[【EP330 帶著善意行動，最...] 談話風格真誠，來賓分享的善意與感動故事具有療癒效果，笑聲自然。 | [【EP302 把命盤變成行動藍...] 談話風格偏向專業知識分享與深度思考，而非輕鬆歡樂或日常廢話，因此療癒解壓感普通。 | [【EP312《超越我執的生活》...] 談話風格較為嚴肅認真，著重於概念闡述與心靈啟發，而非輕鬆歡樂或日常廢話，因此解壓療癒感相對較低。</v>
@@ -2942,7 +2942,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E98">
-        <v>7.9796</v>
+        <v>7.98</v>
       </c>
       <c r="F98" t="str">
         <v>[EP470｜把人放在心上的共贏...] 談話內容較為嚴肅和深入，著重於理念和實踐，因此輕鬆歡樂的解壓感相對較低。 | [EP433｜【中年轉型】從矽谷...] 談話內容嚴肅且具啟發性，雖非輕鬆歡樂的療癒風格，但主持人溫暖的聲線能帶來一定程度的撫慰感。 | [EP466｜拒絕被朝九晚五綁架...] 雖然對談內容嚴肅，但主持人與來賓的真誠分享與對生活哲學的探討，能讓聽眾在思考中找到共鳴��釋放，具有一定的療癒效果。</v>
@@ -2968,7 +2968,7 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E99">
-        <v>7.9646</v>
+        <v>7.96</v>
       </c>
       <c r="F99" t="str">
         <v>[從流浪到回家：浪人食堂的溫柔守...] 節目透過分享感人的故事與理念，傳遞了希望與人性的溫暖，能為聽眾帶來心靈上的慰藉與療癒感，對談情感真摯。 | [【大師專題】人在江湖，身不由己...] 節目主題嚴肅且具哲學性，談話風格較為認真，缺乏輕鬆歡樂或日常廢話的解壓感，因此療癒感主要來自於內容的啟發而非情緒上的放鬆。 | [【中年，正在試】把世界走成一本...] 談話風格輕鬆愉快，來賓的分享充滿正能量，具有一定的解壓感和啟發性。</v>
@@ -3072,7 +3072,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E103">
-        <v>9.8796</v>
+        <v>9.88</v>
       </c>
       <c r="F103" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 節目內容觸及個人健康管理、生活型態調整及對未來健康的規劃，能引發聽眾對自我健康的深度思考與探索。 | [《財富自由心理學》：賺錢，只是...] 節目核心即為自我探索，深度剖析財富、幸福、選擇與個人成長的關係，提供聽眾豐富的內在反思與心靈啟發，是本集最突出的優點。 | [手總是停不下來？那是焦慮在尋找...] 深度探討個人行為背後的心理動機與情緒，對自我成長與內在探索有極強的啟發性。</v>
@@ -3124,7 +3124,7 @@
         <v>張忘形</v>
       </c>
       <c r="E105">
-        <v>9.7715</v>
+        <v>9.77</v>
       </c>
       <c r="F105" t="str">
         <v>[EP61｜為什麼越努力經營，反...] 節目核心圍繞自我身份、內在感受與個人成長，深度探討如何從內在建立影響力，對自我探索有極高的啟發性。 | [EP50｜看到什麼都東西都想拍...] 節目深度探討了自我價值、外部認可與內在幸福的關係，鼓勵聽眾反思生活方式，具有強烈的心靈啟發與自我成長價值。 | [EP65｜ 對方因為小事就對你...] 節目核心即是主持人對自身「暴怒」行為的深度剖析與內在探索，從童年經驗、心理機制到實踐轉化，提供了極具啟發性的自我成長路徑。</v>
@@ -3176,7 +3176,7 @@
         <v>下半場人生事務有限公司</v>
       </c>
       <c r="E107">
-        <v>9.6549</v>
+        <v>9.65</v>
       </c>
       <c r="F107" t="str">
         <v>[44-解開品牌人生的迷思，從認...] 節目核心圍繞自我成長、內在探索與心靈啟發，深度探討個人價值觀與人生方向，啟發性極強。 | [57-慢活的幸福人生 – 台灣...] 節目深度探討了個人成長、內在探索與心靈啟發，鼓勵聽眾透過慢活理念重新認識自我與世界，具備極高的自我探索價值。 | [59-人生下半場，人際好感怎麽...] 節目核心主題圍繞自我成長、內在探索與心靈啟發，深度極高，能有效引導聽眾反思自身。</v>
@@ -3462,7 +3462,7 @@
         <v>人生啊！小歐</v>
       </c>
       <c r="E118">
-        <v>8.6875</v>
+        <v>8.69</v>
       </c>
       <c r="F118" t="str">
         <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
@@ -3722,7 +3722,7 @@
         <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E128">
-        <v>9.5549</v>
+        <v>9.55</v>
       </c>
       <c r="F128" t="str">
         <v>[[深度]瘦瘦針是神藥？醫師教你...] 主持人與來賓的對談內容豐富且具深度，能有效吸引對健康議題感興趣的聽眾持續收聽，建立情感連結。 | [《財富自由心理學》：賺錢，只是...] 主持人與聽眾建立深厚的情感連結，對談真誠且富有溫度，內容引人入勝，讓聽眾產生持續追蹤與探索的強烈意願。 | [手總是停不下來？那是焦慮在尋找...] 主持人與聽眾的連結深厚，對談情感真誠有溫度，能有效提升聽眾的黏著度。</v>
@@ -3748,7 +3748,7 @@
         <v>胡咪老師</v>
       </c>
       <c r="E129">
-        <v>9.4786</v>
+        <v>9.48</v>
       </c>
       <c r="F129" t="str">
         <v>[S4.EP4｜性平教育20年，...] 主持人對談情感真誠，能與聽眾建立深層連結，提供靈魂陪伴感，黏著度高。 | [S4.EP8｜我不想再跟你生活...] 主持人與聽眾之間建立起深厚的情感連結，對談真誠且富有溫度，能給予聽眾強烈的靈魂陪伴感。 | [S4.EP14｜有些人沒有成為...] 主持人以真誠的對話、深刻的洞察和溫暖的語氣，與聽眾建立了強烈的情感連結，讓聽眾感受到被理解和陪伴，具有高度的黏著度。</v>
@@ -3826,7 +3826,7 @@
         <v>布姐陪你聰明工作創意生活</v>
       </c>
       <c r="E132">
-        <v>9.3215</v>
+        <v>9.32</v>
       </c>
       <c r="F132" t="str">
         <v>[EP470｜把人放在心上的共贏...] 主持人對來賓的故事展現出真誠的興趣，對談情感溫度高，能與聽眾建立深厚的連結與靈魂陪伴感。 | [EP433｜【中年轉型】從矽谷...] 主持人以真誠的語氣與聽眾建立連結，對談充滿情感溫度，能有效提升聽眾的黏著度與歸屬感。 | [EP466｜拒絕被朝九晚五綁架...] 主持人與來賓的對談充滿真誠與情感溫度，對個人成長議題的深入探討，能有效建立聽眾的黏著度與靈魂陪伴感。</v>
@@ -3852,7 +3852,7 @@
         <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E133">
-        <v>9.3049</v>
+        <v>9.3</v>
       </c>
       <c r="F133" t="str">
         <v>[EP225：【非典家庭CEO】...] 主持人與來賓的對談充滿真誠情感，保會媽媽的生命故事極具感染力，能讓聽眾產��強烈的連結與共鳴，期待繼續收聽。 | [EP218：愛自己｜放下完美執...] 主持人與來賓的對談真誠且富有情感，內容引人入勝，讓聽眾感受到被理解與陪伴，能有效建立聽眾的黏著度與持續收聽的意願。 | [EP219：【非典家庭CEO】...] 主持人與來賓的對談真誠且富有情感溫度，容易讓聽眾產生共鳴並期待下一集。</v>
@@ -3878,7 +3878,7 @@
         <v>GK爸爸</v>
       </c>
       <c r="E134">
-        <v>9.2549</v>
+        <v>9.25</v>
       </c>
       <c r="F134" t="str">
         <v>[原創歌曲〈愛喲愛你喲〉+ 我的...] 主持人透過引人入勝的敘事和情感連結，成功建立與聽眾的深厚關係，讓人期待後續故事發展，黏著度高。 | [春暖花開小旅行...] 主持人透過生動的敘述與角色扮演，與聽眾建立起良好的情感連結，具有高度的黏著度與陪伴感。 | [【QQ偵探：鳳梨酥失竊案 上集...] 故事引人入勝，結尾的懸念設計強烈，讓聽眾對後續發展充滿期待，黏著度高。</v>
@@ -3956,7 +3956,7 @@
         <v>蕭邦</v>
       </c>
       <c r="E137">
-        <v>9.2429</v>
+        <v>9.24</v>
       </c>
       <c r="F137" t="str">
         <v>[【蕭邦出任務】負債 900 多...] 主持人真誠分享個人經歷，情感溫度高，與聽眾建立深層連結，具備靈魂陪伴感。 | [【蕭邦出任務】如何選擇適合自己...] 主持人對來賓的真誠關懷與對談情感溫度，能有效建立聽眾的黏著度與靈魂陪伴感。 | [幸福的人，通常「覺察力」都很強...] 主持人透過真誠的個人分享與溫暖的語調，與聽眾建立深厚的情感連結���具有高度的黏著度與靈魂陪伴感。</v>
@@ -3970,550 +3970,290 @@
     </row>
     <row r="138" xml:space="preserve">
       <c r="A138" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B138">
         <v>1</v>
       </c>
       <c r="C138" t="str">
-        <v>分手的99個理由</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D138" t="str">
-        <v>胡咪老師</v>
+        <v>瓦基閱讀前哨站</v>
       </c>
       <c r="E138">
-        <v>8.52</v>
+        <v>46</v>
       </c>
       <c r="F138" t="str">
-        <v>AI 評審平均得分為 8.52 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #26.2 名。</v>
       </c>
       <c r="G138" t="str" xml:space="preserve">
-        <v xml:space="preserve">【破題精采開場：從軍人到作家，刪不掉的生命故事】
-時間: 00:00 - 02:24
-單集: S3.EP92｜刪掉容易，忘掉很難：從軍人到寫故事的人 feat. 林思齊
-理由: 節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
+        <v xml:space="preserve">【節目開場】
+時間: 00:00 - 00:05
+單集: EP.591 《財富自由心理學》專訪作者：破解財富焦慮的 6 個洞察
+理由: 主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
       </c>
     </row>
     <row r="139" xml:space="preserve">
       <c r="A139" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B139">
         <v>2</v>
       </c>
       <c r="C139" t="str">
-        <v>宋家小館</v>
+        <v>哇賽心理學</v>
       </c>
       <c r="D139" t="str">
-        <v>宋家小館｜Becky</v>
+        <v>哇賽心理學_蔡宇哲</v>
       </c>
       <c r="E139">
-        <v>8.47</v>
+        <v>46</v>
       </c>
       <c r="F139" t="str">
-        <v>AI 評審平均得分為 8.47 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #33 名。</v>
       </c>
       <c r="G139" t="str" xml:space="preserve">
-        <v xml:space="preserve">【闆娘Becky的轉運概念】
-時間: 00:53 - 01:41
-單集: EP174 | 打造福氣好運的三部曲
-理由: 主持人以親切的語氣開場，透過洗床單的日常小事引導出「轉運」的核心概念，迅速拉近與聽眾的距離，引人入勝。</v>
+        <v xml:space="preserve">【節目開場：你是否也「偏心自己」？】
+時間: 00:08 - 00:41
+單集: 累到想消失？偏心自己，找回角色外的自我ft.徐慧玲｜哇賽療心室ep152
+理由: 主持人以「偏心自己」這個核心概念開場，引導聽眾思考在家庭、工作、人際關係中，是否習慣性地先考慮他人需求而忽略自己，並點出許多人因此感到疲憊的現狀，為節目奠定引人入勝的基調。</v>
       </c>
     </row>
     <row r="140" xml:space="preserve">
       <c r="A140" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B140">
         <v>3</v>
       </c>
       <c r="C140" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="D140" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="E140">
+        <v>46</v>
+      </c>
+      <c r="F140" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #38.3 名。</v>
+      </c>
+      <c r="G140" t="str" xml:space="preserve">
+        <v xml:space="preserve">【Podcast與自媒體的開場提問】
+時間: 00:07 - 00:24
+單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
+理由: 主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+    </row>
+    <row r="141" xml:space="preserve">
+      <c r="A141" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B141">
+        <v>4</v>
+      </c>
+      <c r="C141" t="str">
+        <v>GK爸爸原創故事繪本</v>
+      </c>
+      <c r="D141" t="str">
+        <v>GK爸爸</v>
+      </c>
+      <c r="E141">
+        <v>46</v>
+      </c>
+      <c r="F141" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #65.9 名。</v>
+      </c>
+      <c r="G141" t="str" xml:space="preserve">
+        <v xml:space="preserve">【GK爸爸的互動開場與故事預告】
+時間: 00:15 - 01:25
+單集: 《QQ俠大冒險2：前進宇宙》第二章 迷你太空船
+理由: 此片段展現了主持人GK爸爸活潑的開場風格，不僅介紹了本集故事內容，還巧妙地融入了與聽眾的互動環節（九九乘法），並預告了周邊商品，充分展現了節目的親和力與豐富性。</v>
+      </c>
+    </row>
+    <row r="142" xml:space="preserve">
+      <c r="A142" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B142">
+        <v>5</v>
+      </c>
+      <c r="C142" t="str">
         <v>文森說書</v>
       </c>
-      <c r="D140" t="str">
+      <c r="D142" t="str">
         <v>文森說書</v>
       </c>
-      <c r="E140">
-        <v>8.45</v>
-      </c>
-      <c r="F140" t="str">
-        <v>AI 評審平均得分為 8.45 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G140" t="str" xml:space="preserve">
+      <c r="E142">
+        <v>38</v>
+      </c>
+      <c r="F142" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 38 天，平均上榜排名為第 #64.2 名。</v>
+      </c>
+      <c r="G142" t="str" xml:space="preserve">
         <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
 時間: 01:03 - 03:05
 單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
 理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
       </c>
     </row>
-    <row r="141" xml:space="preserve">
-      <c r="A141" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
-      </c>
-      <c r="B141">
-        <v>4</v>
-      </c>
-      <c r="C141" t="str">
-        <v>布姐的沙發</v>
-      </c>
-      <c r="D141" t="str">
-        <v>布姐陪你聰明工作創意生活</v>
-      </c>
-      <c r="E141">
-        <v>8.44</v>
-      </c>
-      <c r="F141" t="str">
-        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G141" t="str" xml:space="preserve">
-        <v xml:space="preserve">【浴室驚魂記：選擇的開端】
-時間: 00:00 - 00:57
-單集: EP455｜困難抉擇的關鍵心法：如何做出不後悔的選擇
-理由: 節目開場以一個生動且帶有戲劇性的個人故事破題，講述孩子對洗澡的恐懼以及主持人自身的無力感，迅速抓住聽眾注意力。這段不僅展現了主講人的敘事能力，也為後續關於人生選擇的討論奠定了情感基礎，語速與語氣的掌握恰到好處。</v>
-      </c>
-    </row>
-    <row r="142" xml:space="preserve">
-      <c r="A142" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
-      </c>
-      <c r="B142">
-        <v>5</v>
-      </c>
-      <c r="C142" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
-      </c>
-      <c r="D142" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
-      </c>
-      <c r="E142">
-        <v>8.44</v>
-      </c>
-      <c r="F142" t="str">
-        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G142" t="str" xml:space="preserve">
-        <v xml:space="preserve">【同理心與育兒修羅場的開場】
-時間: 00:04 - 00:29
-單集: EP222：【非典家庭CEO】卸下心理師光環後的肉搏與自白：從母親節的失落，看職場父母如何在瑣碎生活中拼湊「夠好的自己」ft. 曾心怡心理師
-理由: 節目開場以平靜的語氣定義「同理心」，隨後立即切換至孩子們的吵鬧聲和母親崩潰的獨白，形成強烈對比。這種戲劇性的轉折，生動地呈現了育兒的真實挑戰，迅速抓住聽眾的注意力，並為節目主題做了精彩的破題。</v>
-      </c>
-    </row>
     <row r="143" xml:space="preserve">
       <c r="A143" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B143">
         <v>6</v>
       </c>
       <c r="C143" t="str">
-        <v>能量黑客</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="D143" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>別人的工作最有趣｜Fiona</v>
       </c>
       <c r="E143">
-        <v>8.43</v>
+        <v>7</v>
       </c>
       <c r="F143" t="str">
-        <v>AI 評審平均得分為 8.43 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
       </c>
       <c r="G143" t="str" xml:space="preserve">
-        <v xml:space="preserve">【能量駭客的開場白與節目宗旨】
-時間: 00:00 - 00:30
-單集: 內耗怎麼停？先抽離，再復盤：把情緒變成行動｜能量黑客S2EP9
-理由: 這段是節目的標準開場，由兩位主持人輪流介紹節目理念。Hank大叔以「在忙碌生活中，有餘力去做快樂的事，並在重要時刻拿出最好的狀態」點出節目核心，Betty則補充「能量不只是體力，還包含專注力、情緒狀態」，並承諾用實用方法與幽默幫助聽眾找到高能量節奏。語速雖快，但清晰有力，有效傳達節目主旨，迅速抓住聽眾注意力。</v>
-      </c>
-    </row>
-    <row r="144" xml:space="preserve">
+        <v xml:space="preserve">【舞台設計的趨勢：從實景到巨型LED螢幕的演變】
+時間: 39:16 - 40:19
+單集: EP177 演唱會背後的重要角色！必應創造舞台設計師工作開箱
+理由: 這段來賓小柔詳細說明了舞台設計從早期實景到現在巨型LED螢幕的演變，並以五月天「陳名在望」的演唱會為例，具體描述了LED螢幕如何創造出180度環繞的沉浸式體驗，以及飛機艙門的互動設計。主持人Fiona的提問引導得很好，讓小柔能深入解釋技術與藝術結合的細節，展現了單元企劃的深度與內容的含金量。</v>
+      </c>
+    </row>
+    <row r="144">
       <c r="A144" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+        <v>站著不走獎</v>
       </c>
       <c r="B144">
         <v>7</v>
       </c>
       <c r="C144" t="str">
+        <v>鄧惠文</v>
+      </c>
+      <c r="D144" t="str">
+        <v>鄧惠文</v>
+      </c>
+      <c r="E144">
+        <v>6</v>
+      </c>
+      <c r="F144" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
+      </c>
+      <c r="G144" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="145" xml:space="preserve">
+      <c r="A145" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B145">
+        <v>8</v>
+      </c>
+      <c r="C145" t="str">
+        <v>小思大維</v>
+      </c>
+      <c r="D145" t="str">
+        <v>小思大維｜雪柔</v>
+      </c>
+      <c r="E145">
+        <v>4</v>
+      </c>
+      <c r="F145" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
+      </c>
+      <c r="G145" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 免費的代價：個人資料的價值與風險】
+時間: 11:30 - 13:20
+單集: 月光族精靈探店記#05 : 年貨大街 ✨免費的代價✨
+理由: 此片段深入探討了「填問卷送贈品」背後，個人資料如何成為一種隱性支付，以及其可能帶來的風險。雪兒阿姨（主持人）透過具體的例子，清晰解釋了姓名、電話等資料對商家的價值，並警示了資料被濫用或轉賣的潛在危險。點點（來賓角色）的疑問與反應，也恰到好處地引導了主持人逐步揭示這些深層概念，展現了節目在生活化情境中融入深度思考的企劃能力。</v>
+      </c>
+    </row>
+    <row r="146" xml:space="preserve">
+      <c r="A146" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B146">
+        <v>9</v>
+      </c>
+      <c r="C146" t="str">
+        <v>佐編茶水間</v>
+      </c>
+      <c r="D146" t="str">
+        <v>佐依Zoey</v>
+      </c>
+      <c r="E146">
+        <v>2</v>
+      </c>
+      <c r="F146" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
+      </c>
+      <c r="G146" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 探討「一切皆無常」的第一個智慧】
+時間: 01:36:00 - 01:39:00
+單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
+理由: 此片段主講人深入闡述了她領悟到的第一個智慧：「一切皆無常」。她清晰地解釋了這個概念，並指出人們對無常的抗拒是痛苦的根源。這展現了節目在內容企劃上的深度與利基選題的獨特性，引導聽眾進行深刻的自我反思，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="147" xml:space="preserve">
+      <c r="A147" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B147">
+        <v>10</v>
+      </c>
+      <c r="C147" t="str">
+        <v>不敗教主陳重銘</v>
+      </c>
+      <c r="D147" t="str">
+        <v>不敗教主-陳重銘</v>
+      </c>
+      <c r="E147">
+        <v>1</v>
+      </c>
+      <c r="F147" t="str">
+        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 1 天，平均上榜排名為第 #84 名。</v>
+      </c>
+      <c r="G147" t="str" xml:space="preserve">
+        <v xml:space="preserve">【開場引導與人生反思】
+時間: 00:04 - 01:15
+單集: EP594《富媽媽 窮媽媽》第二章(4)：原來讀書就是為了要賺錢養家，工作就是在坐牢
+理由: 主持人以書籍《富媽媽窮媽媽》為引，迅速切入主題，並結合自身年輕時對投資、退休與人生選擇的思考，語氣真誠，引人入勝，有效抓住聽眾的注意力。</v>
+      </c>
+    </row>
+    <row r="148" xml:space="preserve">
+      <c r="A148" t="str">
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+      </c>
+      <c r="B148">
+        <v>1</v>
+      </c>
+      <c r="C148" t="str">
         <v>尼可這樣說</v>
       </c>
-      <c r="D144" t="str">
+      <c r="D148" t="str">
         <v>尼可這樣說</v>
       </c>
-      <c r="E144">
-        <v>8.18</v>
-      </c>
-      <c r="F144" t="str">
-        <v>AI 評審平均得分為 8.18 分，近半年累積 Apple Podcasts 評論數達 2 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G144" t="str" xml:space="preserve">
+      <c r="E148">
+        <v>5</v>
+      </c>
+      <c r="F148" t="str">
+        <v>平均評等 5 星，累計 2 則評論。</v>
+      </c>
+      <c r="G148" t="str" xml:space="preserve">
         <v xml:space="preserve">【考上明星高中卻格格不入：自我懷疑的開端】
 時間: 03:17 - 04:44
 單集: EP.317 出走，不是逃離，而是回到自己：《臺灣製造》作者安吉的人生覺醒之路
 理由: 來賓生動地描述了她意外考上明星高中後，卻感到格格不入的經歷。這段內容深刻地揭示了外在成就與內心認同之間的落差，以及自我懷疑的萌芽，情感真摯且引人入勝，為後續的自我探索旅程奠定基礎。</v>
       </c>
     </row>
-    <row r="145" xml:space="preserve">
-      <c r="A145" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
-      </c>
-      <c r="B145">
-        <v>8</v>
-      </c>
-      <c r="C145" t="str">
-        <v>琄蜜莉的異想世界</v>
-      </c>
-      <c r="D145" t="str">
-        <v>王琄</v>
-      </c>
-      <c r="E145">
-        <v>8.37</v>
-      </c>
-      <c r="F145" t="str">
-        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G145" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 2026火運的全球變革與歷史借鑒】
-時間: 01:58 - 05:00
-單集: S4EP5 琄蜜莉的異想世界 feat. 瞧瞧宇宙在幹嘛 仙姑喬喬 （上集）
-理由: 此片段來賓深入解析2026年「丙午火運」的能量特質，將其與全球性的擴張、重建、秩序翻轉等現象連結，並引用日本解散議會、格陵蘭、美加關係等時事案例，甚至追溯至180年前的墨美戰爭，展現了極高的內容含金量與深度思考。主持人適時的提問與總結，有效引導聽眾理解複雜的觀點，是企劃選題與內容深度的絕佳示範。</v>
-      </c>
-    </row>
-    <row r="146" xml:space="preserve">
-      <c r="A146" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
-      </c>
-      <c r="B146">
-        <v>9</v>
-      </c>
-      <c r="C146" t="str">
-        <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
-      </c>
-      <c r="D146" t="str">
-        <v>孫子玲</v>
-      </c>
-      <c r="E146">
-        <v>8.37</v>
-      </c>
-      <c r="F146" t="str">
-        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G146" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 維繫婚姻的關鍵：不爭輸贏與分享慾】
-時間: 09:32 - 11:04
-單集: #95 ▍ 冷戰半年怎麼破冰？「撩夫神技」大公開- 神老師愛的秘訣 - 愛你現在的樣子 -上集
-理由: 此片段深入探討了維繫夫妻關係的關鍵，特別是「不爭輸贏」、「不踩底線」以及「分享慾」等核心觀念。來賓分享了如何在關係中找到平衡點，以及如何透過「誇誇法」等實際方法增進情感。主持人引導得宜，成功從來賓的經驗中提煉出具深度且實用的婚姻智慧，對聽眾具有高度的啟發價值。</v>
-      </c>
-    </row>
-    <row r="147" xml:space="preserve">
-      <c r="A147" t="str">
-        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
-      </c>
-      <c r="B147">
-        <v>10</v>
-      </c>
-      <c r="C147" t="str">
-        <v>蕭邦相談室</v>
-      </c>
-      <c r="D147" t="str">
-        <v>蕭邦</v>
-      </c>
-      <c r="E147">
-        <v>8.37</v>
-      </c>
-      <c r="F147" t="str">
-        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
-      </c>
-      <c r="G147" t="str" xml:space="preserve">
-        <v xml:space="preserve">【開場：情緒的引導與個人經驗分享】
-時間: 00:12 - 00:31
-單集: 如何度過負面情緒 ？
-理由: 主持人以自身經歷引出「情緒」這個主題，語氣真誠，迅速建立與聽眾的連結，引人入勝，為節目內容做了很好的鋪墊。</v>
-      </c>
-    </row>
-    <row r="148" xml:space="preserve">
-      <c r="A148" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B148">
-        <v>1</v>
-      </c>
-      <c r="C148" t="str">
-        <v>下一本讀什麼？</v>
-      </c>
-      <c r="D148" t="str">
-        <v>瓦基閱讀前哨站</v>
-      </c>
-      <c r="E148">
-        <v>46</v>
-      </c>
-      <c r="F148" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #26.2 名。</v>
-      </c>
-      <c r="G148" t="str" xml:space="preserve">
-        <v xml:space="preserve">【節目開場】
-時間: 00:00 - 00:05
-單集: EP.591 《財富自由心理學》專訪作者：破解財富焦慮的 6 個洞察
-理由: 主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
-      </c>
-    </row>
-    <row r="149" xml:space="preserve">
-      <c r="A149" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B149">
-        <v>2</v>
-      </c>
-      <c r="C149" t="str">
-        <v>哇賽心理學</v>
-      </c>
-      <c r="D149" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
-      </c>
-      <c r="E149">
-        <v>46</v>
-      </c>
-      <c r="F149" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #33 名。</v>
-      </c>
-      <c r="G149" t="str" xml:space="preserve">
-        <v xml:space="preserve">【節目開場：你是否也「偏心自己」？】
-時間: 00:08 - 00:41
-單集: 累到想消失？偏心自己，找回角色外的自我ft.徐慧玲｜哇賽療心室ep152
-理由: 主持人以「偏心自己」這個核心概念開場，引導聽眾思考在家庭、工作、人際關係中，是否習慣性地先考慮他人需求而忽略自己，並點出許多人因此感到疲憊的現狀，為節目奠定引人入勝的基調。</v>
-      </c>
-    </row>
-    <row r="150" xml:space="preserve">
-      <c r="A150" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B150">
-        <v>3</v>
-      </c>
-      <c r="C150" t="str">
-        <v>郝聲音</v>
-      </c>
-      <c r="D150" t="str">
-        <v>郝旭烈/郝聲音</v>
-      </c>
-      <c r="E150">
-        <v>46</v>
-      </c>
-      <c r="F150" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #38.3 名。</v>
-      </c>
-      <c r="G150" t="str" xml:space="preserve">
-        <v xml:space="preserve">【Podcast與自媒體的開場提問】
-時間: 00:07 - 00:24
-單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
-理由: 主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
-      </c>
-    </row>
-    <row r="151" xml:space="preserve">
-      <c r="A151" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B151">
-        <v>4</v>
-      </c>
-      <c r="C151" t="str">
-        <v>GK爸爸原創故事繪本</v>
-      </c>
-      <c r="D151" t="str">
-        <v>GK爸爸</v>
-      </c>
-      <c r="E151">
-        <v>46</v>
-      </c>
-      <c r="F151" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #65.9 名。</v>
-      </c>
-      <c r="G151" t="str" xml:space="preserve">
-        <v xml:space="preserve">【GK爸爸的互動開場與故事預告】
-時間: 00:15 - 01:25
-單集: 《QQ俠大冒險2：前進宇宙》第二章 迷你太空船
-理由: 此片段展現了主持人GK爸爸活潑的開場風格，不僅介紹了本集故事內容，還巧妙地融入了與聽眾的互動環節（九九乘法），並預告了周邊商品，充分展現了節目的親和力與豐富性。</v>
-      </c>
-    </row>
-    <row r="152" xml:space="preserve">
-      <c r="A152" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B152">
-        <v>5</v>
-      </c>
-      <c r="C152" t="str">
-        <v>文森說書</v>
-      </c>
-      <c r="D152" t="str">
-        <v>文森說書</v>
-      </c>
-      <c r="E152">
-        <v>38</v>
-      </c>
-      <c r="F152" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 38 天，平均上榜排名為第 #64.2 名。</v>
-      </c>
-      <c r="G152" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
-時間: 01:03 - 03:05
-單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
-理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
-      </c>
-    </row>
-    <row r="153" xml:space="preserve">
-      <c r="A153" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B153">
-        <v>6</v>
-      </c>
-      <c r="C153" t="str">
-        <v>別人的工作最有趣</v>
-      </c>
-      <c r="D153" t="str">
-        <v>別人的工作最有趣｜Fiona</v>
-      </c>
-      <c r="E153">
-        <v>7</v>
-      </c>
-      <c r="F153" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
-      </c>
-      <c r="G153" t="str" xml:space="preserve">
-        <v xml:space="preserve">【舞台設計的趨勢：從實景到巨型LED螢幕的演變】
-時間: 39:16 - 40:19
-單集: EP177 演唱會背後的重要角色！必應創造舞台設計師工作開箱
-理由: 這段來賓小柔詳細說明了舞台設計從早期實景到現在巨型LED螢幕的演變，並以五月天「陳名在望」的演唱會為例，具體描述了LED螢幕如何創造出180度環繞的沉浸式體驗，以及飛機艙門的互動設計。主持人Fiona的提問引導得很好，讓小柔能深入解釋技術與藝術結合的細節，展現了單元企劃的深度與內容的含金量。</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B154">
-        <v>7</v>
-      </c>
-      <c r="C154" t="str">
-        <v>鄧惠文</v>
-      </c>
-      <c r="D154" t="str">
-        <v>鄧惠文</v>
-      </c>
-      <c r="E154">
-        <v>6</v>
-      </c>
-      <c r="F154" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
-      </c>
-      <c r="G154" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="155" xml:space="preserve">
-      <c r="A155" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B155">
-        <v>8</v>
-      </c>
-      <c r="C155" t="str">
-        <v>小思大維</v>
-      </c>
-      <c r="D155" t="str">
-        <v>小思大維｜雪柔</v>
-      </c>
-      <c r="E155">
-        <v>4</v>
-      </c>
-      <c r="F155" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
-      </c>
-      <c r="G155" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 免費的代價：個人資料的價值與風險】
-時間: 11:30 - 13:20
-單集: 月光族精靈探店記#05 : 年貨大街 ✨免費的代價✨
-理由: 此片段深入探討了「填問卷送贈品」背後，個人資料如何成為一種隱性支付，以及其可能帶來的風險。雪兒阿姨（主持人）透過具體的例子，清晰解釋了姓名、電話等資料對商家的價值，並警示了資料被濫用或轉賣的潛在危險。點點（來賓角色）的疑問與反應，也恰到好處地引導了主持人逐步揭示這些深層概念，展現了節目在生活化情境中融入深度思考的企劃能力。</v>
-      </c>
-    </row>
-    <row r="156" xml:space="preserve">
-      <c r="A156" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B156">
-        <v>9</v>
-      </c>
-      <c r="C156" t="str">
-        <v>佐編茶水間</v>
-      </c>
-      <c r="D156" t="str">
-        <v>佐依Zoey</v>
-      </c>
-      <c r="E156">
-        <v>2</v>
-      </c>
-      <c r="F156" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
-      </c>
-      <c r="G156" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 探討「一切皆無常」的第一個智慧】
-時間: 01:36:00 - 01:39:00
-單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
-理由: 此片段主講人深入闡述了她領悟到的第一個智慧：「一切皆無常」。她清晰地解釋了這個概念，並指出人們對無常的抗拒是痛苦的根源。這展現了節目在內容企劃上的深度與利基選題的獨特性，引導聽眾進行深刻的自我反思，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
-      </c>
-    </row>
-    <row r="157" xml:space="preserve">
-      <c r="A157" t="str">
-        <v>站著不走獎</v>
-      </c>
-      <c r="B157">
-        <v>10</v>
-      </c>
-      <c r="C157" t="str">
-        <v>不敗教主陳重銘</v>
-      </c>
-      <c r="D157" t="str">
-        <v>不敗教主-陳重銘</v>
-      </c>
-      <c r="E157">
-        <v>1</v>
-      </c>
-      <c r="F157" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 1 天，平均上榜排名為第 #84 名。</v>
-      </c>
-      <c r="G157" t="str" xml:space="preserve">
-        <v xml:space="preserve">【開場引導與人生反思】
-時間: 00:04 - 01:15
-單集: EP594《富媽媽 窮媽媽》第二章(4)：原來讀書就是為了要賺錢養家，工作就是在坐牢
-理由: 主持人以書籍《富媽媽窮媽媽》為引，迅速切入主題，並結合自身年輕時對投資、退休與人生選擇的思考，語氣真誠，引人入勝，有效抓住聽眾的注意力。</v>
-      </c>
-    </row>
-    <row r="158" xml:space="preserve">
-      <c r="A158" t="str">
-        <v>聽眾都要跟你獎 (加總累積評論數)</v>
-      </c>
-      <c r="B158">
-        <v>1</v>
-      </c>
-      <c r="C158" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="D158" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="E158">
-        <v>5</v>
-      </c>
-      <c r="F158" t="str">
-        <v>平均評等 5 星，累計 2 則評論。</v>
-      </c>
-      <c r="G158" t="str" xml:space="preserve">
-        <v xml:space="preserve">【考上明星高中卻格格不入：自我懷疑的開端】
-時間: 03:17 - 04:44
-單集: EP.317 出走，不是逃離，而是回到自己：《臺灣製造》作者安吉的人生覺醒之路
-理由: 來賓生動地描述了她意外考上明星高中後，卻感到格格不入的經歷。這段內容深刻地揭示了外在成就與內心認同之間的落差，以及自我懷疑的萌芽，情感真摯且引人入勝，為後續的自我探索旅程奠定基礎。</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G158"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G148"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update scores to 2 decimal places
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G148"/>
+  <dimension ref="A1:G159"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -700,76 +700,76 @@
         <v>1</v>
       </c>
       <c r="C12" t="str">
-        <v>能量黑客</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D12" t="str">
-        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E12">
         <v>10</v>
       </c>
       <c r="F12" t="str">
-        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人展現了極高的默契與自然流暢的對話。他們頻繁地接話、補充彼此的觀點，並透過提問與分享個人經驗（如Vicky的跑步經歷、Hank的決策原則）來深化討論。彼此間的幽默感與支持性互動，不僅讓對話充滿活力，也成功營造出輕鬆愉快的氛圍，使聽眾能更投入地聆聽，並感受到主持人之間真誠的連結。 | [別人眼中的高光時刻，卻是我最耗...] 兩位主持人展現了極佳的默契與引導能力。他們不僅能精準地提問，更透過自身的經驗分享（如Hank的「相見恨晚」），與來賓建立深厚的連結，讓來賓願意敞開心扉分享最私密的經歷。Vicky的歸納與提問也讓對話更具深度與流暢性，整體氣氛溫暖且具感染力。 | [別急著振作！高能量的人允許自己...] 兩位主持人展現了極佳的默契與引導能力。他們的問題深入且具啟發性，能有效引導來賓分享更深層的經驗與見解。Vicky的提問與生活化比喻，常能精準捕捉聽眾的疑問並讓氣氛更活潑；Hank則以其專業背景提出關鍵問題，並在適時處給予來賓肯定與支持。兩人互動流暢自然，彼此的補充與呼應讓對話內容更豐富，也讓來賓感到被理解與尊重，進而更願意敞開心扉，使節目氛圍充滿正向能量與深度。</v>
+        <v>[EP225：【非典家庭CEO】...] 兩位主持人展現了極佳的默契與訪談技巧。她們的互動自然流暢，語氣溫暖且充滿同理心，成功營造了一個讓來賓感到安全、願意敞開心扉分享的氛圍。主持人透過適時的提問、回應與幽默感，不僅讓對話內容豐富深入，也讓聽眾能感受到真誠的連結。特別是當保惠媽媽提到想請社工把孩子帶回去時，主持人立刻接話「馬上是不是？」，展現了高度的共鳴與趣味性。她們的聲調起伏與活潑的語氣，讓整個節目充滿生命力，毫無沉悶之感，有效帶動了聽眾的情緒，讓嚴肅的議題也能以溫馨且引人入勝的方式呈現。她們不僅是訪談者，更是陪伴者，讓來賓與聽眾都能從中獲得��量與啟發。 | [EP218：愛自己｜放下完美執...] 兩位主持人展現了極佳的默契與互動火花。她們不僅能透過積極的聆聽（如頻繁的「嗯」、「對對對」、「沒錯」）和適時的提問，有效引導來賓安卡深入分享，更透過分享自身作為安卡聽眾的經驗，以及對人類圖的個人體會（如「跟我一樣！」、「我光是聽到那個閘門啊，搖啊，我就想說天啊，我好想睡了！」），迅速拉近與來賓的距離，營造出溫馨且充滿共鳴的氛圍。她們的語氣活潑、聲調起伏自然，尤其在討論各自的人類圖特質時，能巧妙地加入幽默感（如Cherry自嘲「我沒有邏輯啊！」、或形容自己「常常跳出話題」），讓原本可能較為生硬的專業內容變得生動有��且極具親和力。這種輕鬆愉快的互動，讓來賓更願意敞開心扉，也讓聽眾能更投入地享受節目內容，展現了高超的節目主持功力。 | [EP219：【非典家庭CEO】...] 兩位主持人展現了極佳的默契與互動火花。她們的語氣活潑有趣，充滿熱情，能有效帶動節目氣氛，讓來賓感到放鬆並樂於分享。她們不僅提出引導性的問題，更頻繁地透過補充、呼應、甚至幽默的對話來豐富內容，例如在來賓分享育兒經驗時，她們能迅速連結自身感受，或以輕鬆的方式回應來賓的趣事，使對話更具層次感和趣味性。聲調和語氣起伏自然，沒有沉悶感，讓聽眾能感受到她們對談話內容的真誠投入與好奇心。整體而言，她們的互動讓節目充滿活力，成功營造了一個溫馨且引人入勝的聆聽體驗。</v>
       </c>
       <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[主持控場與互動] 伴侶關係中的人類圖互動與建議】
+時間: 24:44 - 28:07
+單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
+理由: 此片段充分展現了主持人與來賓之間流暢且自然的互動。Cherry分享了她與顯示生產者丈夫在專案啟動上的困擾，小可也補充了她丈夫的不同情況，來賓Anka則巧妙地將話題拉回人類圖的「閘門」概念，並解析了兩位主持人伴侶的月亮閘門（Gate 1的創意與Gate 42的完成使命感）。Anka不僅精準點出特質，更提供了投射者（主持人）如何與顯示者（伴侶）有效溝通的實用建議（透過提問而非指令）。整個過程充滿了自然的對話、共鳴與實用性，完美體現了「最佳默契獎」與「最佳內容架構獎」的評估標準。</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>最佳默契獎</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="str">
+        <v>能量黑客</v>
+      </c>
+      <c r="D13" t="str">
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+      </c>
+      <c r="E13">
+        <v>10</v>
+      </c>
+      <c r="F13" t="str">
+        <v>[新年特輯—火馬年續航攻略：吃睡...] 兩位主持人展現了極佳的默契與互動火花。他們的語氣活潑有趣，聲調起伏自然，使得整個節目充滿了生動的氛圍，絕不沉悶。維琪老師經常扮演聽眾的代理人，提出實用問題或分享個人經驗，讓內容更具親和力；而大叔則提供專業見解和結構性引導。他們之間的對話充滿了幽默感和支持性，即使偶有打斷，也多是為了補充、確認或增添趣味，而非干擾。例如，維琪老師在討論「睡眠綁著運動」時，立刻以聽眾角度幽默回應，以及在解釋「抽離」技巧時，能迅速理解並舉例，都顯示了兩人高度的同步性與互相激發的能力。這種互動不僅讓彼此更願意深入探討，也極大地提��了節目的吸引力和感染力。 | [別人眼中的高光時刻，卻是我最耗...] 兩位主持人與來賓的互動默契極佳，展現了高度的同理心與引導能力。他們不僅能讓來賓布姐深入分享個人職涯的低潮與高光時刻，甚至連主持人自己也願意分享非常私密的經歷，例如 Hank 大叔的創業低谷與情緒釋放，以及 Vicky 對於「痛苦是比較出來的」的幽默自嘲。這種雙向的真誠分享，極大地鼓勵了來賓更願意敞開心扉。在聲調與語氣方面，兩位主持人皆充滿活力，語氣起伏自然且富有感染力。Vicky 的提問精準且富有洞察力，能將對話引導至更深層次的自我探索；Hank 大叔則以其沉穩而富有哲理的總結，為對話增添了深度，同時不失幽默感（例如對「麻場」和「鐵軌��的解釋，以及「金身大叔」的稱呼）。他們之間的互動火花四射，笑聲不斷，使得整個節目氣氛輕鬆愉快，即使討論嚴肅議題也能保持引人入勝。整體而言，兩位主持人成功營造了一個既能深入探討又能輕鬆愉快的對話空間，充分展現了最佳默契獎的評選標準。 | [別急著振作！高能量的人允許自己...] 兩位主持人展現了極高的默契與互動火花。Vicky 的語氣活潑、充滿好奇，她的笑聲和適時的提問（例如在 2:28 提出疑問，或在 2:54 透過想像力引導對話）總能有效帶動氣氛，讓來賓更願意深入分享。Hank 則以沉穩的語氣提供深度見解和補充，他的提問精準且富有引導性，例如在 3:36 提到「大書記的人物」時，展現了對來賓觀點的理解與延伸。兩人不僅能讓來賓暢所欲言，彼此間的對話也充滿趣味性，例如在 3:01 Vicky 對於「心情不好去讀書」的幽默反應，以及在 1:12:50 關於「婆媳關係」的討論，都讓節目氣氛輕鬆愉快，毫無沉悶感。他們的聲調起伏自然，互動流暢，共同營造了一個既有深度又充滿活力的訪談環境，讓聽眾能感受到滿滿的正能量與樂趣。</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
         <v xml:space="preserve">【[主持控場與互動] 跑步發現新世界】
 時間: 12:14 - 13:22
 單集: 新年特輯—火馬年續航攻略：吃睡練＋情緒＋決策＋意義感｜能量黑客S3EP11
 理由: 女主持人在此段分享了她因跑步而意外發現河堤美景的個人經歷，生動的敘述方式（「我一走過去的時候，噔噔！」）引人入勝。男主持人則以積極的傾聽和簡短的肯定（「我知道，我知道，你們那裡我常跑，我知道」）來支持對話，沒有打斷女主持人的故事流暢性，展現了雙人主持間自然且流暢的互動默契。此片段完美體現了主持人如何透過個人故事來豐富內容，並維持良好的對話節奏，符合【最佳內容��構獎】與【最佳默契獎】的評選標準。</v>
       </c>
     </row>
-    <row r="13" xml:space="preserve">
-      <c r="A13" t="str">
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
         <v>最佳默契獎</v>
       </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13" t="str">
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="str">
         <v>分手的99個理由</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D14" t="str">
         <v>胡咪老師</v>
       </c>
-      <c r="E13">
+      <c r="E14">
         <v>10</v>
       </c>
-      <c r="F13" t="str">
-        <v>[S4.EP4｜性平教育20年，...] 兩位主持人展現了極佳的默契與流暢的互動。女主持人提供詳盡的資訊與引導，男主持人則以貼近聽眾的反應、提問及個人經驗（如對長輩世代的觀察）來回應，不僅讓對話更具深度與廣度，也有效活絡了節目氣氛。男主持人的情感反應（如「太可怕了啦」、「我聽到這邊好難過喔」）更增添了節目的真實感與共鳴，使聽眾能更投入地聆聽這個嚴肅的議題。 | [S4.EP8｜我不想再跟你生活...] 胡咪與畢頭大叔展現了極高的默契與互動性。胡咪老師在朗讀書摘時情感豐沛，畢頭大叔則能即時給予真誠且具個人色彩的回應，無論是幽默的自嘲（如「我這個書名就讓我心碎了」）或是深刻的共鳴（如「你不要再說了啦，我聽到這邊我突然好難過」），都讓對話充滿層次感。兩人能自然地接話、延伸話題，並透過彼此的視角（男性與女性）豐富了討論的廣度與深度，使節目氣氛溫暖而引人入勝，讓聽眾彷彿也參與其中，共同感受情感的流動。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現��極佳的默契與自然互動，對話流暢且充滿趣味。他們能巧妙地接話、補充彼此觀點，並透過幽默感與個人經驗分享，讓嚴肅的自我探索主題變得輕鬆且引人入勝。這種互動氛圍不僅鼓勵彼此更深入地表達，也讓聽眾感到被邀請參與其中，極具渲染力。</v>
-      </c>
-      <c r="G13" t="str" xml:space="preserve">
+      <c r="F14" t="str">
+        <v>[S4.EP4｜性平教育20年，...] 兩位主持人從開場的節目介紹就展現了絕佳的默契，語氣活潑且充滿熱情，成功營造出輕鬆愉快的氛圍。女主持人胡咪在闡述複雜的議題時，語調清晰、邏輯分明，能將深奧的內容轉化為易於理解的語言。男主持人Vito大叔則扮演了極佳的提問者和聽眾角色，他的提問不僅能引導話題深入，也常以幽默或帶有個人情感的語氣回應，例如在討論「安全帽砸人」的案例時，他以自身經驗開玩笑，有效緩解了話題的沉重感，並增加了節目的趣味性。兩人的互動自然流暢，彼此間的聲調、語氣起伏和互動火花都非常出色，讓聽眾感覺像在聽朋友聊天，而非生硬的資訊傳遞。他們能夠讓彼此更願意多談，並透過生動的對話帶動聽眾的情緒，使整個節目過程不沉悶，充滿吸引力。特別是在討論到情感暴力和社會議題時，他們能夠在保持專業性的同時，注入人性化的關懷和共鳴，這對於鼓勵聽眾思考和分享是非常重要的。 | [S4.EP8｜我不想再跟你生活...] 兩位主持人展現了極高的默契與互動火花。胡咪老師在節目中負責主述與朗讀書摘，她的聲調、語氣起伏非常豐富，能將書中角色的情緒生動地傳達出來，特別是在描述憤怒、無奈或幽默情節時，感染力十足。比頭大叔則扮演了極佳的「聽眾」與「回應者」角色，他不僅能精準地抓到胡咪老師話語中的重點，並適時地給予共鳴、提問或幽默的補充，例如他多次將書中情節與自身經驗連結，或以「殺氣」、「很狠」等詞語來形容胡咪老師的朗讀，都讓氣氛變得更加活潑有趣。兩人之間的對話流暢自然，即使偶有打斷，也都是為了更好地延續話題或增添趣味，而非干擾。他們���夠讓彼此更願意多談，並透過個人化的分享和生動的語氣，讓聽眾感受到強烈的連結與情感共鳴，使得整個節目充滿了生命力，絕不沉悶。 | [S4.EP14｜有些人沒有成為...] 兩位主持人展現了極佳的默契與互動火花。胡咪的聲調活潑、語氣充滿好奇與同理，經常能引導話題並帶動情緒；大叔的聲線沉穩，卻不失幽默感，常以個人經驗或更深層的見解來豐富討論。他們彼此間的對話流暢自然，很少有冷場，且能互相接話、補充觀點，甚至在適當時機加入幽默感，例如胡咪在討論「如果當初選了別人」時，巧妙地將大叔拉回「就不會遇到胡咪了」，展現了高度的趣味性與親和力。他們也樂於分享個人經驗，讓聽眾感受到真誠與開放的氛圍。整體而言，兩人的互動不僅讓節目內容更具深度，也讓聽眾在輕鬆愉快的氣氛中，對複雜的情感議題產生共��與思考，是非常出色的主持搭檔。</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
         <v xml:space="preserve">【幽默互動：性愛暗號與身心益處大揭密】
 時間: 15:33 - 24:47
 單集: S3.EP81｜越做越愛的關係續命術
 理由: 主持人討論如何用「小暗號」來表達性需求，Humi舉例「歡樂的世界」等幽默對話，展現了良好的互動與趣味性。接著，他們詳細列舉了性愛對免疫系統、心血管、睡眠、大腦、皮膚、骨骼等多方面的生理益處，內容豐富且具說服力，Vito最後的「做愛治百病」總結更是畫龍點睛。</v>
       </c>
     </row>
-    <row r="14" xml:space="preserve">
-      <c r="A14" t="str">
-        <v>最佳默契獎</v>
-      </c>
-      <c r="B14">
-        <v>3</v>
-      </c>
-      <c r="C14" t="str">
-        <v>粉紅地獄辛辣麵</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Vito大叔</v>
-      </c>
-      <c r="E14">
-        <v>9.9</v>
-      </c>
-      <c r="F14" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] Vito 大叔與品希的搭檔默契極佳，兩位主持人一搭一唱，提問精準且富有層次，能有效引導來賓 Taku 深入分享其經歷與感受。他們不僅展現出對來賓故事的濃厚興趣，更透過適時的驚嘆、幽默的互動與同理心的回應，營造出輕鬆愉悅且充滿支持的對話氛圍，讓 Taku 能夠暢所欲言，使節目內容更加豐富動人。兩人的互動也讓聽眾彷彿置身其中，共同感受故事的起伏。 | [S6EP19. 沐樂MOReL...] 楊梅老師與V-Tou大叔展現了極佳的默契與互動。兩人之間的幽默感與互相吐槽（如楊梅老師調侃V-Tou交到女友就忘記她，或V-Tou分享處理體味的「年代金曲」）為節目營造了輕鬆愉快的氛圍。他們的問題引導性強，能讓來賓范范自在地分享專業知識、個人經歷，甚至是一些敏感話題（如如何委婉告知客戶有體味）。兩位主持人不僅讓來賓暢所欲言，也透過自身的參與和反應，讓整個對話充滿活力與趣味，使聽眾能更投入地聆聽。 | [S6EP4. 放飛。萬哩露｜村...] B頭大叔和品希與來賓凱莉哥的互動非常流暢且充滿默契。他們不僅提出深入的問題，也適時分享個人經驗，讓凱莉哥更願意敞開心扉。品希分享兒子在校園的經歷，與凱莉哥的「放手」哲學形成對比，豐富了討論的層次。主持人之間的幽默感和相互支持也讓節目氣氛輕鬆愉快，引導來賓和彼此更深入地交流。</v>
-      </c>
-      <c r="G14" t="str" xml:space="preserve">
-        <v xml:space="preserve">【音樂在日常中的療癒力與幽默互動】
-時間: 1:40:00 - 1:42:00
-單集: S6EP24. 五感研究苑｜顏爾呈：用音頻啟動修復！找回內在節奏與平靜
-理由: 男性主持人分享他載女兒上學時，透過聆聽大自然音樂來放鬆身心的個人經驗，展現音樂療癒在日常生活中潛移默化的影響力。女兒對「漏水」的幽默反應，也為節目增添了輕鬆有趣的互動，讓聽眾感受到音樂療癒的實用性與生活化。</v>
-      </c>
-    </row>
     <row r="15" xml:space="preserve">
       <c r="A15" t="str">
         <v>最佳默契獎</v>
@@ -784,10 +784,10 @@
         <v>楊月娥（楊肉爐）</v>
       </c>
       <c r="E15">
-        <v>9.19</v>
+        <v>10</v>
       </c>
       <c r="F15" t="str">
-        <v>[EP128｜【母女鍋】魅力是可...] 兩位女主持人互動自然，接話流暢，笑聲同步率高，展現了良好的默契，但偶爾楊月娥的發言會較為強勢。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人默契極佳，接話流暢，插話頻率適中且能有效推進話題，共同的笑聲自然且富有感染力，展現了高度的協同性。 | [EP139｜【全家鍋】開始運動...] 主持人與來賓（Michael）的互動非常自然，接話流暢，笑聲同步率高，展現了極佳的默契。</v>
+        <v>[EP128｜【母女鍋】魅力是可...] 兩位主持人（楊月娥與小真）在節目中展現了極高的默契與互動火花。她們以「魅力」為主題，透過個人經驗分享、相互提問與補充，將抽象的概念具體化，並引導聽眾深入思考。楊月娥作為主導者，善於拋出問題並引導小真分享，同時也適時地分享自己的觀點，使對話保持平衡且富有層次。小真則以其坦率、幽默的語氣，將表演課所學的「魅力學」與個人生活經驗結合，提供了許多有趣且實用的見解，例如「專注腳趾頭」的練習，以及如何應對尷尬情境的技巧，都讓節目充滿了趣味性與啟發性。她們的聲調與語氣起伏自然，充滿活力，尤其在討論到彼此的優點和缺點時���展現出真誠且不失幽默的互動，讓聽眾感受到溫暖與親和力。兩人能夠讓彼此更願意多談，且透過輕鬆愉快的氛圍，將原本可能嚴肅的議題變得生動有趣，充分符合最佳默契獎的評選標準。 | [EP142｜【母女鍋】你的大頭...] 兩位主持人展現了極佳的默契與互動火花。她們的對話流暢自然，彼此間的提問、補充與共鳴，不僅讓故事敘述更為生動，也鼓勵對方深入分享。楊月娥的語氣活潑、充滿好奇，善於引導與總結，並適時加入幽默感（如提及「查稅」、「骯髒的家」或流行文化梗），使嚴肅的議題變得輕鬆有趣。小真則以沉穩而富有洞察力的語氣，提供詳細的分析與個人哲學。她們的互動充滿真誠與情感，即使偶有疊話，也無損其高度的參與感與親密關係（如提及「親子血緣關係」的玩笑），整體氛圍溫馨且引人入勝，讓聽眾能輕鬆投入並從中獲得啟發。她們的聲調與語氣起伏豐富，能有��帶動聽眾情緒，避免了沉悶感，是廣播節目中難得一見的黃金組合。 | [EP139｜【全家鍋】開始運動...] 兩位主持人展現了極佳的默契與互動火花，對話自然流暢，充滿趣味性。阿兒的語氣活潑生動，善於引導話題並以個人經驗豐富內容，其聲調起伏能有效帶動聽眾情緒。小真則以其敏銳的觀察力與幽默感，適時補充或提出疑問，並透過真誠的笑聲與反應，讓氣氛更加輕鬆愉快。兩人能讓彼此更願意分享，即使是討論老化、運動傷害等較嚴肅的議題，也能以輕鬆且富有渲染力的方式呈現，避免了沉悶感。特別是他們在討論「老狼打行拜」的台語俚語，以及描述來賓運動時的「痛苦面具」等橋段，都展現了絕佳的互動與趣味性，讓節目充滿了吸引力。來賓的加入也未打亂兩人��節奏，反而能被他們巧妙地融入對話，共同創造出豐富的內容。</v>
       </c>
       <c r="G15" t="str" xml:space="preserve">
         <v xml:space="preserve">【[主持控場與互動] 魅力源於自身擁有的深刻洞察】
@@ -804,22 +804,22 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
+        <v>任性歐逆機智生活</v>
       </c>
       <c r="D16" t="str">
-        <v>加班當爸媽．櫻桃可可CherryCoco</v>
+        <v>曼蒂歐逆-轉型之路</v>
       </c>
       <c r="E16">
-        <v>8.8</v>
+        <v>9.95</v>
       </c>
       <c r="F16" t="str">
-        <v>[EP225：【非典家庭CEO】...] 主持人小可與兩位來賓（保會媽媽、瑞琳）的對話互動自然，接話流暢，笑聲共鳴度高，展現了良好的訪談默契。 | [EP218：愛自己｜放下完美執...] 兩位主持人與來賓Anka的互動非常流暢自然，彼此接話默契十足，笑聲與共鳴感強烈，共同營造出輕鬆愉快的對話氛圍。 | [EP219：【非典家庭CEO】...] 兩位主持人與來賓的互動流暢，笑聲自然，展現了良好的默契與控場能力。</v>
+        <v>[跟長輩一樣就能學會AI？陶韻智...] 兩位主持人Mandy和Ivy展現了極高的熱情與默契，她們對來賓陶韻智老師的崇拜之情溢於言表，從一開始就以「很厲害的老師」、「大神」等詞彙營造出熱烈且尊重的氛圍，讓來賓感到備受歡迎。她們的語氣活潑有趣，充滿了好奇心和學習慾，頻繁地以「對不對」、「真的」、「沒錯」等詞語回應，並穿插著適時的笑聲和幽默感，例如Ivy自嘲「不爭材」的橋段，都讓對話充滿了生動的火花。她們不僅能引導來賓深入分享，也透過自身的學習經驗與來賓產生共鳴，使整個訪談過程流暢且引人入勝。兩人的互動自然，一搭一唱，有效帶動了節目的氣氛，讓來賓更願意敞開心扉分��其獨到的見解和經驗。 | [再不用證明自己給誰看 feat...] 兩位主持人展現了極高的默契與互動性。她們的語氣活潑、充滿熱情，且頻繁地以「對啊」、「真的耶」、「哇」等詞語積極回應來賓，讓來賓感到被充分聆聽與理解。她們的笑聲真誠且具感染力，有效提升了節目的輕鬆氛圍。主持人不僅能適時拋出引導性問題，更會分享自身經驗或補充觀點，使對話更具深度與廣度，而非單向提問。特別是在來賓分享個人創業與家族企業轉型的挑戰時，主持人展現了高度的同理心與支持，讓來賓願意深入分享許多細節。她們的互動火花與趣味性，如對「總經理特助」的幽默解讀，都讓節目充滿了生動的魅力，成功鼓勵來賓暢所欲言，並��整體氣氛保持愉悅與引人入勝。 | [好像很爽，我們也去當個旅遊作家...] 兩位主持人展現了極佳的默契與互動火花，她們的聲調與語氣起伏活潑有趣，充滿渲染力，能有效帶動氣氛，讓來賓Jessie非常願意分享許多精彩且生動的旅行故事。例如，在討論蒙古旅程的趣事時，主持人與來賓之間的笑聲與驚呼聲此起彼落，創造了非常歡樂的氛圍。她們不僅能提出引導性問題，也常透過「哇！」、「真的耶！」等即時反應，展現高度的投入感，使對話流暢且充滿趣味性，完全符合最佳默契獎的評選標準。</v>
       </c>
       <c r="G16" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[主持控場與互動] 伴侶關係中的人類圖互動與建議】
-時間: 24:44 - 28:07
-單集: EP218：愛自己｜放下完美執念，人類圖讓你與孩子、伴侶「對頻」生活 ft. 安卡
-理由: 此片段充分展現了主持人與來賓之間流暢且自然的互動。Cherry分享了她與顯示生產者丈夫在專案啟動上的困擾，小可也補充了她丈夫的不同情況，來賓Anka則巧妙地將話題拉回人類圖的「閘門」概念，並解析了兩位主持人伴侶的月亮閘門（Gate 1的創意與Gate 42的完成使命感）。Anka不僅精準點出特質，更提供了投射者（主持人）如何與顯示者（伴侶）有效溝通的實用建議（透過提問而非指令）。整個過程充滿了自然的對話、共鳴與實用性，完美體現了「最佳默契獎」與「最佳內容架構獎」的評估標準。</v>
+        <v xml:space="preserve">【[主持控場與互動] 突破慣性：從個人到企業的AI應用】
+時間: 05:21 - 06:15
+單集: 跟長輩一樣就能學會AI？陶韻智老師的反慣性AI學《 AI First 自我升級革命》
+理由: Mandy 提出「最難改的慣性」這個核心問題，引導老師分享了人類基因中根深蒂固的「從眾」與「不改變」的慣性。老師以生動的例子（如不被老虎吃掉的走路方式）解釋了這些慣性如何影響我們對新事物的接受度。這段對話展現了主持人提問的精準度，能夠引導來賓深入淺出地闡述複雜概念，同時保持了對話的流暢與互動性，為聽眾提供了極具啟發性的思考。</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -830,50 +830,50 @@
         <v>6</v>
       </c>
       <c r="C17" t="str">
+        <v>粉紅地獄辛辣麵</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Vito大叔</v>
+      </c>
+      <c r="E17">
+        <v>9.9</v>
+      </c>
+      <c r="F17" t="str">
+        <v>[S6EP30. 我到日本當漁夫...] 兩位主持人展現了極佳的默契與互動火花。Vito 的提問深入且引導性強，Pinxi 則以活潑的語氣和精準的切入點，不斷拋出有趣或具啟發性的問題，讓來賓 Taku 更願意分享其獨特的人生經歷。他們的聲調與語氣起伏豐富，充滿熱情與好奇心，特別是在討論 Taku 父母的教育理念、養魚的挑戰，以及在魚市場打工的趣事時，兩人的對話充滿趣味性，例如 Pinxi 關於「魚腥味」的提問，以及 Vito 對「小菜鳥」的描述，都讓氣氛變得輕鬆愉快且引人入勝。他們不僅能有效帶動來賓的情緒，也讓聽眾感受到一場生動且不沉悶的對談，充分展現了「讓來賓或彼此更願意多談」以及「讓氣氛��好」的渲染力。 | [S6EP19. 沐樂MOReL...] 兩位主持人（V-Tou和品希）展現了極佳的默契與互動火花。他們的對話充滿趣味性，語氣活潑生動，能有效帶動節目氣氛，避免沉悶。透過幽默的提問、彼此間的玩笑（如品希對V-Tou的調侃，以及V-Tou的自嘲），成功鼓勵來賓范范分享更多深入的經驗與看法。聲調與語氣起伏自然，特別是在討論敏感話題（如感情詐騙、個人衛生）時，能以輕鬆卻不失尊重的態度處理，並加入個人經驗，讓內容更引人入勝。頻繁的互動與接話，顯示出兩人深厚的搭檔關係，讓聽眾感受到節目的流暢與愉悅。尤其在討論「味道」和「詐騙」等話題時，兩位主持人的反應和補充，不僅增添了節目��娛樂性，也讓來賓更自在地表達。 | [S6EP4. 放飛。萬哩露｜村...] B頭大叔與品希展現了極佳的默契與互動火花。B頭大叔的提問深入且引導性強，能有效開啟來賓的心扉，讓凱莉哥願意分享更多個人經驗與創業歷程。品希則以其活潑的語氣、幽默的插科打諢，以及自身經歷的分享（如不洗澡、校園霸凌），不僅讓氣氛更加輕鬆有趣，也與來賓產生了高度共鳴，促使來賓更自在地表達。兩人一搭一唱，聲調與語氣起伏自然，充滿趣味性，尤其在討論育兒觀念和假設情境時，能將嚴肅議題轉化為引人入勝的對話，讓來賓與聽眾都能感受到愉悅且真誠的交流。他們成功地營造了一個讓來賓感到被理解、被支持的環境，鼓勵了更深層次的對話，而非僅是單向的問答，充分符合了「讓來賓或彼此更願意多談」及「讓氣氛變好」的評分標準。</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">【音樂在日常中的療癒力與幽默互動】
+時間: 1:40:00 - 1:42:00
+單集: S6EP24. 五感研究苑｜顏爾呈：用音頻啟動修復！找回內在節奏與平靜
+理由: 男性主持人分享他載女兒上學時，透過聆聽大自然音樂來放鬆身心的個人經驗，展現音樂療癒在日常生活中潛移默化的影響力。女兒對「漏水」的幽默反應，也為節目增添了輕鬆有趣的互動，讓聽眾感受到音樂療癒的實用性與生活化。</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>最佳默契獎</v>
+      </c>
+      <c r="B18">
+        <v>7</v>
+      </c>
+      <c r="C18" t="str">
         <v>《姐姐不想懂事了》 | Soft Rebellion</v>
       </c>
-      <c r="D17" t="str">
+      <c r="D18" t="str">
         <v>姐姐不想懂事了｜莉安君怡 / 姊姊不想懂事了</v>
       </c>
-      <c r="E17">
-        <v>8.77</v>
-      </c>
-      <c r="F17" t="str">
-        <v>[EP36｜30歲以後的身體，需...] 兩位主持人與來賓之間的對話流暢，互動自然，彼此接話默契良好，共同的笑聲也增加了節目的親和力。即使有插話，也多是為了補充或引導，而非搶話。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人與來賓的互動非常自然，接話流暢，笑聲也很有感染力，展現了良好的默契。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
-      </c>
-      <c r="G17" t="str" xml:space="preserve">
+      <c r="E18">
+        <v>9.41</v>
+      </c>
+      <c r="F18" t="str">
+        <v>[EP36｜30歲以後的身體，需...] 兩位主持人展現了極高的默契與互動火花。她們的聲調活潑、語氣充滿熱情，能有效帶動節目氣氛，讓來賓Eva感到非常自在，願意深入分享專業知識與個人觀察。主持人之間也頻繁地相互呼應、補充，並適時加入幽默感（例如將來賓視為「私心」的「私人教練」），使對話流暢且充滿趣味性，避免了沉悶感。她們的提問方式引導性強，且能從自身經驗出發，與來賓和聽眾建立連結，展現了出色的引導與渲染力。 | [EP33｜五歲開始談錢，讓孩子...] 兩位主持人展現了極佳的默契與互動能力。她們的聲調與語氣起伏自然，充滿活力與熱情，使得整個節目氛圍非常正面且引人入勝。主持人不僅能透過精準的提問引導來賓深入分享，更在來賓分享時給予適時的回應與共鳴（如「真的嗎？」、「哇塞，太棒了！」），讓來賓感到被理解與支持，進而更願意敞開心扉。她們之間的對話流暢，充滿互動火花，偶爾穿插的幽默感也讓內容不顯沉悶，成功地將理財教育這樣可能較為嚴肅的議題，轉化為一場輕鬆且富有啟發性的對談。整體而言，兩位主持人共同創造了一個極具吸引力的聆聽體驗，充分展現了最佳默契獎的評選標準。 | [EP25 ｜ 投資自己：30+...] 兩位女主持人與來賓的互動流暢且具吸引力，彼此間的接話自然，共同營造出輕鬆愉快的對話氛圍。</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
         <v xml:space="preserve">【[主持控場與互動] 針對學員需求的引導與溝通】
 時間: 05:48 - 07:16
 單集: EP36｜30歲以後的身體，需要的不是更努力，而是更有覺察 ft. Eva
 理由: 此片段主持人與來賓討論了學員最常許的願望和遇到的身體問題，以及教練如何應對。來賓詳細說明了她會如何評估學員的身體狀況（功能性評估）和目標，並強調了動作品質的重要性。主持人適時地提出問題，例如「什麼是功能性評估？」，幫助聽眾理解專業術語，並以自身經驗（「我們就是兩個想要增肌減脂的小白」）拉近與來賓的距離，展現了流暢的互動和控場能���，符合【最佳內容架構獎】與【最佳默契獎】的評估維度。</v>
       </c>
     </row>
-    <row r="18" xml:space="preserve">
-      <c r="A18" t="str">
-        <v>最佳默契獎</v>
-      </c>
-      <c r="B18">
-        <v>7</v>
-      </c>
-      <c r="C18" t="str">
-        <v>任性歐逆機智生活</v>
-      </c>
-      <c r="D18" t="str">
-        <v>曼蒂歐逆-轉型之路</v>
-      </c>
-      <c r="E18">
-        <v>8.6</v>
-      </c>
-      <c r="F18" t="str">
-        <v>[跟長輩一樣就能學會AI？陶韻智...] 雙主持人與來賓互動自然，接話流暢，笑聲同步率高，但偶有輕微搶話情況，整體默契良好。 | [再不用證明自己給誰看 feat...] 雙主持人與來賓之間的互動自然，接話流暢，笑聲具感染力，展現了良好的默契，即使有插話也多能順暢銜接。 | [好像很爽，我們也去當個旅遊作家...] 兩位主持人與來賓之間的對話流暢自然，接話和反應迅速，共同營造了輕鬆愉快的氛圍，默契良好。</v>
-      </c>
-      <c r="G18" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[主持控場與互動] 突破慣性：從個人到企業的AI應用】
-時間: 05:21 - 06:15
-單集: 跟長輩一樣就能學會AI？陶韻智老師的反慣性AI學《 AI First 自我升級革命》
-理由: Mandy 提出「最難改的慣性」這個核心問題，引導老師分享了人類基因中根深蒂固的「從眾」與「不改變」的慣性。老師以生動的例子（如不被老虎吃掉的走路方式）解釋了這些慣性如何影響我們對新事物的接受度。這段對話展現了主持人提問的精準度，能夠引導來賓深入淺出地闡述複雜概念，同時保持了對話的流暢與互動性，為聽眾提供了極具啟發性的思考。</v>
-      </c>
-    </row>
     <row r="19" xml:space="preserve">
       <c r="A19" t="str">
         <v>最佳默契獎</v>
@@ -888,10 +888,10 @@
         <v>無所不試無樂不作</v>
       </c>
       <c r="E19">
-        <v>8.5</v>
+        <v>6.61</v>
       </c>
       <c r="F19" t="str">
-        <v>[從流浪到回家：浪人食堂的溫柔守...] 主持人與來賓之間的對話流暢自然，接話得體，沒有明顯的搶話或插話，展現了良好的互動默契。 | [【中年，正在試】把世界走成一本...] Norman和Summer的互動自然，接話流暢，笑聲同步率高，與來賓的互動也展現良好默契。</v>
+        <v>[從流浪到回家：浪人食堂的溫柔守...] 主持人 Norman 的聲調、語氣起伏和互動火花都非常出色。他以溫暖、鼓勵且充滿好奇心的語氣提問，並給予來賓明潔充分的空間闡述。Norman 頻繁使用「哇」、「沒錯」、「很特別」等肯定語，讓明潔感到被理解和支持，進而更願意分享深入的故事和情感。他在明潔講述感人故事時展現的同理心和適時的總結，不僅讓聽眾更容易理解，也加深了節目的情感深度。雖然是訪談形式，但 Norman 的引導讓對話充滿了生命力，避免了沉悶，成功營造出一個既專業又溫馨的氛圍。他的幽默感（例如稱呼團隊為「天使」）也為節目增添了輕鬆的色彩。整體而言，Norman 展現了極高的主持默��和引導能力，讓來賓的分享更加生動感人。 | [【大師專題】人在江湖，身不由己...] 本集節目僅由一位主持人 Norman 進行講述，並無雙人主持的互動。因此，無法針對「最佳默契獎」的評選標準，如兩人互動是否能讓來賓或彼此更願意多談、氣氛渲染力、聲調語氣起伏、互動火花與趣味性等項目進行評分。 | [【中年，正在試】把世界走成一本...] 兩位主持人展現了極佳的默契與互補性。Norman作為主訪者，提問有條理且充滿好奇，引導著對話的流暢進行。Summer作為共同主持人，則以其溫暖、充滿驚嘆的語氣，頻繁地表達對來賓Monica的欽佩與共鳴，例如她對Monica氣質的讚美，以及對Monica旅行經歷的感嘆，都讓來賓感到被高度肯定，從而更願意深入分享。兩人的聲調、語氣起伏都非常活潑，充滿互動的火花與趣味性，使得整個節目氣氛輕鬆愉快，毫無沉悶感。他們不僅讓來賓暢所欲言，也透過彼此的互動，為節目增添了豐富的情感層次和吸引力。</v>
       </c>
       <c r="G19" t="str" xml:space="preserve">
         <v xml:space="preserve">【[主持控場與互動] 團隊年輕化背後的共同理念】
@@ -3970,111 +3970,111 @@
     </row>
     <row r="138" xml:space="preserve">
       <c r="A138" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B138">
         <v>1</v>
       </c>
       <c r="C138" t="str">
-        <v>下一本讀什麼？</v>
+        <v>山姆書書</v>
       </c>
       <c r="D138" t="str">
-        <v>瓦基閱讀前哨站</v>
+        <v>山姆書書</v>
       </c>
       <c r="E138">
-        <v>46</v>
+        <v>8.16</v>
       </c>
       <c r="F138" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #26.2 名。</v>
+        <v>AI 評審平均得分為 8.16 分，近半年累積 Apple Podcasts 評論數達 14 則，社群擴散影響力極佳。</v>
       </c>
       <c r="G138" t="str" xml:space="preserve">
-        <v xml:space="preserve">【節目開場】
-時間: 00:00 - 00:05
-單集: EP.591 《財富自由心理學》專訪作者：破解財富焦慮的 6 個洞察
-理由: 主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
+        <v xml:space="preserve">【[內容與企劃] 探索工作觀與人生觀，���計你的生命藍圖】
+時間: 03:30 - 05:10
+單集: EP131.「做自己的生命設計師」－打造全新生命藍圖
+理由: 主持人清晰地介紹了「工作觀」與「人生觀」這兩個核心概念，並引導聽眾思考其定義與重要性。他透過提問「工作是為了什麼？」、「什麼樣的人生才算美好？」等問題，鼓勵聽眾進行深度自我探索，找出個人價值觀與生命目標。這段內容不僅提供了實用的自我分析框架，也展現了節目在引導聽眾自我成長方面的深度與企劃力。</v>
       </c>
     </row>
     <row r="139" xml:space="preserve">
       <c r="A139" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B139">
         <v>2</v>
       </c>
       <c r="C139" t="str">
-        <v>哇賽心理學</v>
+        <v>加班當爸媽｜櫻桃可可CherryCoco</v>
       </c>
       <c r="D139" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>加班當爸媽．櫻桃可可CherryCoco</v>
       </c>
       <c r="E139">
-        <v>46</v>
+        <v>8.55</v>
       </c>
       <c r="F139" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #33 名。</v>
+        <v>AI 評審平均得分為 8.55 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
       <c r="G139" t="str" xml:space="preserve">
-        <v xml:space="preserve">【節目開場：你是否也「偏心自己」？】
-時間: 00:08 - 00:41
-單集: 累到想消失？偏心自己，找回角色外的自我ft.徐慧玲｜哇賽療心室ep152
-理由: 主持人以「偏心自己」這個核心概念開場，引導聽眾思考在家庭、工作、人際關係中，是否習慣性地先考慮他人需求而忽略自己，並點出許多人因此感到疲憊的現狀，為節目奠定引人入勝的基調。</v>
+        <v xml:space="preserve">【同理心與育兒修羅場的開場】
+時間: 00:04 - 00:29
+單集: EP222：【非典家庭CEO】卸下心理師光環後的肉搏與自白：從母親節的失落，看職場父母如何在瑣碎生活中拼湊「夠好的自己」ft. 曾心怡心理師
+理由: 節目開場以平靜的語氣定義「同理心」，隨後立即切換至孩子們的吵鬧聲和母親崩潰的獨白，形成強烈對比。這種戲劇性的轉折，生動地呈現了育兒的真實挑戰，迅速抓住聽眾的注意力，並為節目主題做了精彩的破題。</v>
       </c>
     </row>
     <row r="140" xml:space="preserve">
       <c r="A140" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B140">
         <v>3</v>
       </c>
       <c r="C140" t="str">
-        <v>郝聲音</v>
+        <v>分手的99個理由</v>
       </c>
       <c r="D140" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>胡咪老師</v>
       </c>
       <c r="E140">
-        <v>46</v>
+        <v>8.52</v>
       </c>
       <c r="F140" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #38.3 名。</v>
+        <v>AI 評審平均得分為 8.52 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
       <c r="G140" t="str" xml:space="preserve">
-        <v xml:space="preserve">【Podcast與自媒體的開場提問】
-時間: 00:07 - 00:24
-單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
-理由: 主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+        <v xml:space="preserve">【破題精采開場：從軍人到作家，刪不掉的生命故事】
+時間: 00:00 - 02:24
+單集: S3.EP92｜刪掉容易，忘掉很難：從軍人到寫故事的人 feat. 林思齊
+理由: 節目以引人入勝的音樂和旁白開場，迅速帶出「分手」主題。主持人以幽默對話營造輕鬆氛圍，隨後介紹來賓林思齊，並巧妙地引導出他從職業軍人轉型為作家的獨特經歷，成功吸引聽眾對節目核心內容產生興趣。</v>
       </c>
     </row>
     <row r="141" xml:space="preserve">
       <c r="A141" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B141">
         <v>4</v>
       </c>
       <c r="C141" t="str">
-        <v>GK爸爸原創故事繪本</v>
+        <v>宋家小館</v>
       </c>
       <c r="D141" t="str">
-        <v>GK爸爸</v>
+        <v>宋家小館｜Becky</v>
       </c>
       <c r="E141">
-        <v>46</v>
+        <v>8.47</v>
       </c>
       <c r="F141" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 46 天，平均上榜排名為第 #65.9 名。</v>
+        <v>AI 評審平均得分為 8.47 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
       <c r="G141" t="str" xml:space="preserve">
-        <v xml:space="preserve">【GK爸爸的互動開場與故事預告】
-時間: 00:15 - 01:25
-單集: 《QQ俠大冒險2：前進宇宙》第二章 迷你太空船
-理由: 此片段展現了主持人GK爸爸活潑的開場風格，不僅介紹了本集故事內容，還巧妙地融入了與聽眾的互動環節（九九乘法），並預告了周邊商品，充分展現了節目的親和力與豐富性。</v>
+        <v xml:space="preserve">【闆娘Becky的轉運概念】
+時間: 00:53 - 01:41
+單集: EP174 | 打造福氣好運的三部曲
+理由: 主持人以親切的語氣開場，透過洗床單的日常小事引導出「轉運」的核心概念，迅速拉近與聽眾的距離，引人入勝。</v>
       </c>
     </row>
     <row r="142" xml:space="preserve">
       <c r="A142" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B142">
         <v>5</v>
@@ -4086,10 +4086,10 @@
         <v>文森說書</v>
       </c>
       <c r="E142">
-        <v>38</v>
+        <v>8.45</v>
       </c>
       <c r="F142" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 38 天，平均上榜排名為第 #64.2 名。</v>
+        <v>AI 評審平均得分為 8.45 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
       </c>
       <c r="G142" t="str" xml:space="preserve">
         <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
@@ -4100,160 +4100,443 @@
     </row>
     <row r="143" xml:space="preserve">
       <c r="A143" t="str">
-        <v>站著不走獎</v>
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
       </c>
       <c r="B143">
         <v>6</v>
       </c>
       <c r="C143" t="str">
+        <v>布姐的沙發</v>
+      </c>
+      <c r="D143" t="str">
+        <v>布姐陪你聰明工作創意生活</v>
+      </c>
+      <c r="E143">
+        <v>8.44</v>
+      </c>
+      <c r="F143" t="str">
+        <v>AI 評審平均得分為 8.44 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G143" t="str" xml:space="preserve">
+        <v xml:space="preserve">【浴室驚魂記：選擇的開端】
+時間: 00:00 - 00:57
+單集: EP455｜困難抉擇的關鍵心法：如何做出不後悔的選擇
+理由: 節目開場以一個生動且帶有戲劇性的個人故事破題，講述孩子對洗澡的恐懼以及主持人自身的無力感，迅速抓住聽眾注意力。這段不僅展現了主講人的敘事能力，也為後續關於人生選擇的討論奠定了情感基礎，語速與語氣的掌握恰到好處。</v>
+      </c>
+    </row>
+    <row r="144" xml:space="preserve">
+      <c r="A144" t="str">
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+      </c>
+      <c r="B144">
+        <v>7</v>
+      </c>
+      <c r="C144" t="str">
+        <v>能量黑客</v>
+      </c>
+      <c r="D144" t="str">
+        <v>林程揚｜Hank大叔 / 維琪的幸福叮嚀</v>
+      </c>
+      <c r="E144">
+        <v>8.43</v>
+      </c>
+      <c r="F144" t="str">
+        <v>AI 評審平均得分為 8.43 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G144" t="str" xml:space="preserve">
+        <v xml:space="preserve">【能量駭客的開場白與節目宗旨】
+時間: 00:00 - 00:30
+單集: 內耗怎麼停？先抽離，再復盤：把情緒變成行動｜能量黑客S2EP9
+理由: 這段是節目的標準開場，由兩位主持人輪流介紹節目理念。Hank大叔以「在忙碌生活中，有餘力去做快樂的事，並在重要時刻拿出最好的狀態」點出節目核心，Betty則補充「能量不只是體力，還包含專注力、情緒狀態」，並承諾用實用方法與幽默幫助聽眾找到高能量節奏。語速雖快，但清晰有力，有效傳達節目主旨，迅速抓住聽眾注意力。</v>
+      </c>
+    </row>
+    <row r="145" xml:space="preserve">
+      <c r="A145" t="str">
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+      </c>
+      <c r="B145">
+        <v>8</v>
+      </c>
+      <c r="C145" t="str">
+        <v>任性歐逆機智生活</v>
+      </c>
+      <c r="D145" t="str">
+        <v>曼蒂歐逆-轉型之路</v>
+      </c>
+      <c r="E145">
+        <v>8.42</v>
+      </c>
+      <c r="F145" t="str">
+        <v>AI 評審平均得分為 8.42 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G145" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] AI First 的核心挑戰與人類慣性】
+時間: 02:20 - 03:30
+單集: 跟長輩一樣就能學會AI？陶韻智老師的反慣性AI學《 AI First 自我升級革命》
+理由: 老師深入剖析了「AI First」概念的核心挑戰，解釋了人類為何難以直接信任AI，而是傾向於尋求專家或傳統知識來源。他從人類的慣性思維（如過去50年的學習模式）出發，闡述了AI作為新型知識工作者的獨特地位，以及在資訊交錯的時代，人們難以判斷AI權威性的困境。這段內容不僅提供了深刻的觀點，也為後續的討論奠定了堅實的理論基礎，展現了單元企劃的深度與啟發性。</v>
+      </c>
+    </row>
+    <row r="146" xml:space="preserve">
+      <c r="A146" t="str">
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+      </c>
+      <c r="B146">
+        <v>9</v>
+      </c>
+      <c r="C146" t="str">
+        <v>琄蜜莉的異想世界</v>
+      </c>
+      <c r="D146" t="str">
+        <v>王琄</v>
+      </c>
+      <c r="E146">
+        <v>8.37</v>
+      </c>
+      <c r="F146" t="str">
+        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G146" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 2026火運的全球變革與歷史借鑒】
+時間: 01:58 - 05:00
+單集: S4EP5 琄蜜莉的異想世界 feat. 瞧瞧宇宙在幹嘛 仙姑喬喬 （上集）
+理由: 此片段來賓深入解析2026年「丙午火運」的能量特質，將其與全球性的擴張、重建、秩序翻轉等現象連結，並引用日本解散議會、格陵蘭、美加關係等時事案例，甚至追溯至180年前的墨美戰爭，展現了極高的內容含金量與深度思考。主持人適時的提問與總結，有效引導聽眾理解複雜的觀點，是企劃選題與內容深度的絕佳示範。</v>
+      </c>
+    </row>
+    <row r="147" xml:space="preserve">
+      <c r="A147" t="str">
+        <v>欸我跟你獎 / 等等！這個真的不分享不行 / AI評選最高分</v>
+      </c>
+      <c r="B147">
+        <v>10</v>
+      </c>
+      <c r="C147" t="str">
+        <v>子玲的親子聊心屋-媽咪的自我成長&amp;親子教養</v>
+      </c>
+      <c r="D147" t="str">
+        <v>孫子玲</v>
+      </c>
+      <c r="E147">
+        <v>8.37</v>
+      </c>
+      <c r="F147" t="str">
+        <v>AI 評審平均得分為 8.37 分，近半年累積 Apple Podcasts 評論數達 0 則，社群擴散影響力極佳。</v>
+      </c>
+      <c r="G147" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 維繫婚姻的關鍵：不爭輸贏與分享慾】
+時間: 09:32 - 11:04
+單集: #95 ▍ 冷戰半年怎麼破冰？「撩夫神技」大公開- 神老師愛的秘訣 - 愛你現在的樣子 -上集
+理由: 此片段深入探討了維繫夫妻關係的關鍵，特別是「不爭輸贏」、「不踩底線」以及「分享慾」等核心觀念。來賓分享了如何在關係中找到平衡點，以及如何透過「誇誇法」等實際方法增進情感。主持人引導得宜，成功從來賓的經驗中提煉出具深度且實用的婚姻智慧，對聽眾具有高度的啟發價值。</v>
+      </c>
+    </row>
+    <row r="148" xml:space="preserve">
+      <c r="A148" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B148">
+        <v>1</v>
+      </c>
+      <c r="C148" t="str">
+        <v>下一本讀什麼？</v>
+      </c>
+      <c r="D148" t="str">
+        <v>瓦基閱讀前哨站</v>
+      </c>
+      <c r="E148">
+        <v>47</v>
+      </c>
+      <c r="F148" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 47 天，平均上榜排名為第 #25.9 名。</v>
+      </c>
+      <c r="G148" t="str" xml:space="preserve">
+        <v xml:space="preserve">【節目開場】
+時間: 00:00 - 00:05
+單集: EP.591 《財富自由心理學》專訪作者：破解財富焦慮的 6 個洞察
+理由: 主持人瓦基以親切的語氣簡潔介紹節目，語速適中，迅速吸引聽眾進入節目氛圍。</v>
+      </c>
+    </row>
+    <row r="149" xml:space="preserve">
+      <c r="A149" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B149">
+        <v>2</v>
+      </c>
+      <c r="C149" t="str">
+        <v>哇賽心理學</v>
+      </c>
+      <c r="D149" t="str">
+        <v>哇賽心理學_蔡宇哲</v>
+      </c>
+      <c r="E149">
+        <v>47</v>
+      </c>
+      <c r="F149" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 47 天，平均上榜排名為第 #32.8 名。</v>
+      </c>
+      <c r="G149" t="str" xml:space="preserve">
+        <v xml:space="preserve">【節目開場：你是否也「偏心自己」？】
+時間: 00:08 - 00:41
+單集: 累到想消失？偏心自己，找回角色外的自我ft.徐慧玲｜哇賽療心室ep152
+理由: 主持人以「偏心自己」這個核心概念開場，引導聽眾思考在家庭、工作、人際關係中，是否習慣性地先考慮他人需求而忽略自己，並點出許多人因此感到疲憊的現狀，為節目奠定引人入勝的基調。</v>
+      </c>
+    </row>
+    <row r="150" xml:space="preserve">
+      <c r="A150" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B150">
+        <v>3</v>
+      </c>
+      <c r="C150" t="str">
+        <v>郝聲音</v>
+      </c>
+      <c r="D150" t="str">
+        <v>郝旭烈/郝聲音</v>
+      </c>
+      <c r="E150">
+        <v>47</v>
+      </c>
+      <c r="F150" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 47 天，平均上榜排名為第 #38.1 名。</v>
+      </c>
+      <c r="G150" t="str" xml:space="preserve">
+        <v xml:space="preserve">【Podcast與自媒體的開場提問】
+時間: 00:07 - 00:24
+單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
+理由: 主持人開場點出本集主題，並直接向來賓提出核心問題，引導聽眾思考Podcast與自媒體的發展與挑戰，迅速抓住聽眾注意力。</v>
+      </c>
+    </row>
+    <row r="151" xml:space="preserve">
+      <c r="A151" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B151">
+        <v>4</v>
+      </c>
+      <c r="C151" t="str">
+        <v>GK爸爸原創故事繪本</v>
+      </c>
+      <c r="D151" t="str">
+        <v>GK爸爸</v>
+      </c>
+      <c r="E151">
+        <v>47</v>
+      </c>
+      <c r="F151" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 47 天，平均上榜排名為第 #65.5 名。</v>
+      </c>
+      <c r="G151" t="str" xml:space="preserve">
+        <v xml:space="preserve">【GK爸爸的互動開場與故事預告】
+時間: 00:15 - 01:25
+單集: 《QQ俠大冒險2：前進宇宙》第二章 迷你太空船
+理由: 此片段展現了主持人GK爸爸活潑的開場風格，不僅介紹了本集故事內容，還巧妙地融入了與聽眾的互動環節（九九乘法），並預告了周邊商品，充分展現了節目的親和力與豐富性。</v>
+      </c>
+    </row>
+    <row r="152" xml:space="preserve">
+      <c r="A152" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B152">
+        <v>5</v>
+      </c>
+      <c r="C152" t="str">
+        <v>文森說書</v>
+      </c>
+      <c r="D152" t="str">
+        <v>文森說書</v>
+      </c>
+      <c r="E152">
+        <v>39</v>
+      </c>
+      <c r="F152" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 39 天，平均上榜排名為第 #64.2 名。</v>
+      </c>
+      <c r="G152" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
+時間: 01:03 - 03:05
+單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
+理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
+      </c>
+    </row>
+    <row r="153" xml:space="preserve">
+      <c r="A153" t="str">
+        <v>站著不走獎</v>
+      </c>
+      <c r="B153">
+        <v>6</v>
+      </c>
+      <c r="C153" t="str">
         <v>別人的工作最有趣</v>
       </c>
-      <c r="D143" t="str">
+      <c r="D153" t="str">
         <v>別人的工作最有趣｜Fiona</v>
       </c>
-      <c r="E143">
+      <c r="E153">
         <v>7</v>
       </c>
-      <c r="F143" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
-      </c>
-      <c r="G143" t="str" xml:space="preserve">
+      <c r="F153" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 7 天，平均上榜排名為第 #92 名。</v>
+      </c>
+      <c r="G153" t="str" xml:space="preserve">
         <v xml:space="preserve">【舞台設計的趨勢：從實景到巨型LED螢幕的演變】
 時間: 39:16 - 40:19
 單集: EP177 演唱會背後的重要角色！必應創造舞台設計師工作開箱
 理由: 這段來賓小柔詳細說明了舞台設計從早期實景到現在巨型LED螢幕的演變，並以五月天「陳名在望」的演唱會為例，具體描述了LED螢幕如何創造出180度環繞的沉浸式體驗，以及飛機艙門的互動設計。主持人Fiona的提問引導得很好，讓小柔能深入解釋技術與藝術結合的細節，展現了單元企劃的深度與內容的含金量。</v>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" t="str">
+    <row r="154">
+      <c r="A154" t="str">
         <v>站著不走獎</v>
       </c>
-      <c r="B144">
+      <c r="B154">
         <v>7</v>
       </c>
-      <c r="C144" t="str">
+      <c r="C154" t="str">
         <v>鄧惠文</v>
       </c>
-      <c r="D144" t="str">
+      <c r="D154" t="str">
         <v>鄧惠文</v>
       </c>
-      <c r="E144">
+      <c r="E154">
         <v>6</v>
       </c>
-      <c r="F144" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
-      </c>
-      <c r="G144" t="str">
+      <c r="F154" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 6 天，平均上榜排名為第 #71.2 名。</v>
+      </c>
+      <c r="G154" t="str">
         <v/>
       </c>
     </row>
-    <row r="145" xml:space="preserve">
-      <c r="A145" t="str">
+    <row r="155" xml:space="preserve">
+      <c r="A155" t="str">
         <v>站著不走獎</v>
       </c>
-      <c r="B145">
+      <c r="B155">
         <v>8</v>
       </c>
-      <c r="C145" t="str">
+      <c r="C155" t="str">
         <v>小思大維</v>
       </c>
-      <c r="D145" t="str">
+      <c r="D155" t="str">
         <v>小思大維｜雪柔</v>
       </c>
-      <c r="E145">
+      <c r="E155">
         <v>4</v>
       </c>
-      <c r="F145" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
-      </c>
-      <c r="G145" t="str" xml:space="preserve">
+      <c r="F155" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 4 天，平均上榜排名為第 #75.5 名。</v>
+      </c>
+      <c r="G155" t="str" xml:space="preserve">
         <v xml:space="preserve">【[內容與企劃] 免費的代價：個人資料的價值與風險】
 時間: 11:30 - 13:20
 單集: 月光族精靈探店記#05 : 年貨大街 ✨免費的代價✨
 理由: 此片段深入探討了「填問卷送贈品」背後，個人資料如何成為一種隱性支付，以及其可能帶來的風險。雪兒阿姨（主持人）透過具體的例子，清晰解釋了姓名、電話等資料對商家的價值，並警示了資料被濫用或轉賣的潛在危險。點點（來賓角色）的疑問與反應，也恰到好處地引導了主持人逐步揭示這些深層概念，展現了節目在生活化情境中融入深度思考的企劃能力。</v>
       </c>
     </row>
-    <row r="146" xml:space="preserve">
-      <c r="A146" t="str">
+    <row r="156" xml:space="preserve">
+      <c r="A156" t="str">
         <v>站著不走獎</v>
       </c>
-      <c r="B146">
+      <c r="B156">
         <v>9</v>
       </c>
-      <c r="C146" t="str">
+      <c r="C156" t="str">
         <v>佐編茶水間</v>
       </c>
-      <c r="D146" t="str">
+      <c r="D156" t="str">
         <v>佐依Zoey</v>
       </c>
-      <c r="E146">
+      <c r="E156">
         <v>2</v>
       </c>
-      <c r="F146" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
-      </c>
-      <c r="G146" t="str" xml:space="preserve">
+      <c r="F156" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 2 天，平均上榜排名為第 #82.5 名。</v>
+      </c>
+      <c r="G156" t="str" xml:space="preserve">
         <v xml:space="preserve">【[內容與企劃] 探討「一切皆無常」的第一個智慧】
 時間: 01:36:00 - 01:39:00
 單集: #336 #Zoey｜你覺得自己被困住了嗎？破除3個認知誤解，獲得真正的自由！
 理由: 此片段主講人深入闡述了她領悟到的第一個智慧：「一切皆無常」。她清晰地解釋了這個概念，並指出人們對無常的抗拒是痛苦的根源。這展現了節目在內容企劃上的深度與利基選題的獨特性，引導聽眾進行深刻的自我反思，非常符合「最神單元企劃」與「自我探索獎」的評估維度。</v>
       </c>
     </row>
-    <row r="147" xml:space="preserve">
-      <c r="A147" t="str">
+    <row r="157" xml:space="preserve">
+      <c r="A157" t="str">
         <v>站著不走獎</v>
       </c>
-      <c r="B147">
+      <c r="B157">
         <v>10</v>
       </c>
-      <c r="C147" t="str">
+      <c r="C157" t="str">
         <v>不敗教主陳重銘</v>
       </c>
-      <c r="D147" t="str">
+      <c r="D157" t="str">
         <v>不敗教主-陳重銘</v>
       </c>
-      <c r="E147">
+      <c r="E157">
         <v>1</v>
       </c>
-      <c r="F147" t="str">
-        <v>於評選區間（統計 46 天）中，共佔據 Apple Podcasts 百大排行榜達 1 天，平均上榜排名為第 #84 名。</v>
-      </c>
-      <c r="G147" t="str" xml:space="preserve">
+      <c r="F157" t="str">
+        <v>於評選區間（統計 47 天）中，共佔據 Apple Podcasts 百大排行榜達 1 天，平均上榜排名為第 #86 名。</v>
+      </c>
+      <c r="G157" t="str" xml:space="preserve">
         <v xml:space="preserve">【開場引導與人生反思】
 時間: 00:04 - 01:15
 單集: EP594《富媽媽 窮媽媽》第二章(4)：原來讀書就是為了要賺錢養家，工作就是在坐牢
 理由: 主持人以書籍《富媽媽窮媽媽》為引，迅速切入主題，並結合自身年輕時對投資、退休與人生選擇的思考，語氣真誠，引人入勝，有效抓住聽眾的注意力。</v>
       </c>
     </row>
-    <row r="148" xml:space="preserve">
-      <c r="A148" t="str">
+    <row r="158">
+      <c r="A158" t="str">
         <v>聽眾都要跟你獎 (加總累積評論數)</v>
       </c>
-      <c r="B148">
+      <c r="B158">
         <v>1</v>
       </c>
-      <c r="C148" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="D148" t="str">
-        <v>尼可這樣說</v>
-      </c>
-      <c r="E148">
+      <c r="C158" t="str">
+        <v>崔咪</v>
+      </c>
+      <c r="D158" t="str">
+        <v>崔咪</v>
+      </c>
+      <c r="E158">
         <v>5</v>
       </c>
-      <c r="F148" t="str">
-        <v>平均評等 5 星，累計 2 則評論。</v>
-      </c>
-      <c r="G148" t="str" xml:space="preserve">
-        <v xml:space="preserve">【考上明星高中卻格格不入：自我懷疑的開端】
-時間: 03:17 - 04:44
-單集: EP.317 出走，不是逃離，而是回到自己：《臺灣製造》作者安吉的人生覺醒之路
-理由: 來賓生動地描述了她意外考上明星高中後，卻感到格格不入的經歷。這段內容深刻地揭示了外在成就與內心認同之間的落差，以及自我懷疑的萌芽，情感真摯且引人入勝，為後續的自我探索旅程奠定基礎。</v>
+      <c r="F158" t="str">
+        <v>平均評等 5 星，累計 5 則評論。</v>
+      </c>
+      <c r="G158" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="159" xml:space="preserve">
+      <c r="A159" t="str">
+        <v>聽眾都要跟你獎 (加總累積評論數)</v>
+      </c>
+      <c r="B159">
+        <v>2</v>
+      </c>
+      <c r="C159" t="str">
+        <v>山姆書書</v>
+      </c>
+      <c r="D159" t="str">
+        <v>山姆書書</v>
+      </c>
+      <c r="E159">
+        <v>4.6</v>
+      </c>
+      <c r="F159" t="str">
+        <v>平均評等 4.6 星，累計 14 則評論。</v>
+      </c>
+      <c r="G159" t="str" xml:space="preserve">
+        <v xml:space="preserve">【[內容與企劃] 探索工作觀與人生觀，���計你的生命藍圖】
+時間: 03:30 - 05:10
+單集: EP131.「做自己的生命設計師」－打造全新生命藍圖
+理由: 主持人清晰地介紹了「工作觀」與「人生觀」這兩個核心概念，並引導聽眾思考其定義與重要性。他透過提問「工作是為了什麼？」、「什麼樣的人生才算美好？」等問題，鼓勵聽眾進行深度自我探索，找出個人價值觀與生命目標。這段內容不僅提供了實用的自我分析框架，也展現了節目在引導聽眾自我成長方面的深度與企劃力。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G148"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G159"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update Excel with latest best_long_form results
</commit_message>
<xml_diff>
--- a/Awards_Top10_Results.xlsx
+++ b/Awards_Top10_Results.xlsx
@@ -3240,7 +3240,7 @@
 理由: 此片段來賓Katie分享了她從不喜歡工程師工作，到因一場車禍被迫停下腳步，進而深刻反思職涯方向的經歷。她描述了這段時間如何讓她有機會思考自己真正想做什麼，以及如何因此獲得在泰國的工作機會，並開始接觸與人互動的工作。這段內容不僅充滿個人故事的張力，更提供了關於職涯迷茫、自我覺察與勇敢轉型的深刻洞見，對於聽眾在自我探索與職涯規劃上極具啟發性，符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
       </c>
     </row>
-    <row r="110" xml:space="preserve">
+    <row r="110">
       <c r="A110" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3248,25 +3248,22 @@
         <v>1</v>
       </c>
       <c r="C110" t="str">
-        <v>說話人聲</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D110" t="str">
-        <v>聲音表達講師林依柔</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="E110">
-        <v>10</v>
+        <v>113.27</v>
       </c>
       <c r="F110" t="str">
-        <v>[EP.59｜【說話人聲-會客室...] 單集時長接近4小時，內容資訊密度極高，且能持續保持聽眾的專注與興趣，無明顯冷場，是優秀的長篇內容��</v>
-      </c>
-      <c r="G110" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] AI時代的親子連結與新書的附加價值】
-時間: 03:53 - 05:13
-單集: EP.61｜【說話人聲-會客室】別再逼自己當「完美父母」！挑剔孩子其實是在懲罰不完美的你
-理由: 此片段來賓紫菱深入探討在AI時代和疫情後，親子連結的重要性，並介紹她的新書如何回應這一需求。主持人伊柔精準提問關於新書的「附加價值」，引導紫菱分享她如何透過免費社群、直播課等方式，提供讀者超越書籍本身的持續支持與互動。這不僅展現了節目選題的深度與前瞻性，也突顯了來賓在內容企劃上的創新思維和對讀者的真誠承諾，極具啟發性。</v>
-      </c>
-    </row>
-    <row r="111" xml:space="preserve">
+        <v>[EP.590 【埃及自由行】...] 長達近兩小時的特別企劃，將旅行點滴與反思深度結合，內容扎實且引人入勝，長篇幅下依然保持極高的聽眾黏著度。</v>
+      </c>
+      <c r="G110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
       <c r="A111" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3274,25 +3271,22 @@
         <v>2</v>
       </c>
       <c r="C111" t="str">
-        <v>郝聲音</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D111" t="str">
-        <v>郝旭烈/郝聲音</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="E111">
-        <v>9.55</v>
+        <v>111</v>
       </c>
       <c r="F111" t="str">
-        <v>[郝聲音：成為人生更自由的「精銳...] 單集時長超過60分鐘，且資訊密度高，內容豐富，全程無冷場，有效利用長篇幅進行深入探討。</v>
-      </c>
-      <c r="G111" t="str" xml:space="preserve">
-        <v xml:space="preserve">【Threads平台「內容為王」的獨特魅力】
-時間: 05:13 - 06:02
-單集: 郝聲音：（下）有魚的「已讀Podcast」，如何從閱讀的喜悅，成長到自媒體分享的幸福
-理由: 來賓深入分析Threads平台「內容為王」的特性，透過生動的案例（只有一個粉絲卻爆紅的貼文）說明其對素人創作者的友善與潛力，展現獨到見解，引人入勝。</v>
-      </c>
-    </row>
-    <row r="112" xml:space="preserve">
+        <v>[EP.620 【走在閱讀路上】...] 讀書會形式的三人對談，超過110分鐘的深度交流，觀點碰撞精彩，完整展現了長篇知識型節目的魅力。</v>
+      </c>
+      <c r="G111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112">
       <c r="A112" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3300,25 +3294,22 @@
         <v>3</v>
       </c>
       <c r="C112" t="str">
-        <v>哇賽心理學</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="D112" t="str">
-        <v>哇賽心理學_蔡宇哲</v>
+        <v>下一本讀什麼？</v>
       </c>
       <c r="E112">
-        <v>9.4</v>
+        <v>95.1</v>
       </c>
       <c r="F112" t="str">
-        <v>[手總是停不下來？那是焦慮在尋找...] 單集時長超過3小時，內容資訊密度高，討論深入且無冷場，能長時間吸引聽眾。</v>
-      </c>
-      <c r="G112" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 美國健康政策與生活型態結合】
-時間: 01:50:00 - 01:53:00
-單集: [深度]瘦瘦針是神藥？醫師教你取其利而避其害ft.蔡孟修醫師｜哇賽療心室ep155
-理由: 此片段來賓深入探討美國最新的健康政策，如何將藥物治療與生活型態調整結合，並提出「Balance」計畫。這不僅展現了選題的深度與前瞻性，也提供了超越單純藥物討論的宏觀視角，極具單元企劃與啟發價值。</v>
-      </c>
-    </row>
-    <row r="113" xml:space="preserve">
+        <v>[EP.568 【走在閱讀路上】...] 長達一個半小時的知識饗宴，條理分明地拆解《讓天賦自由》，節奏穩健，讓聽眾能沉浸在深度的思考中。</v>
+      </c>
+      <c r="G112" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="113">
       <c r="A113" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3326,25 +3317,22 @@
         <v>4</v>
       </c>
       <c r="C113" t="str">
-        <v>文森說書</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="D113" t="str">
-        <v>文森說書</v>
+        <v>精算媽咪的家計簿</v>
       </c>
       <c r="E113">
-        <v>9.35</v>
+        <v>86.53</v>
       </c>
       <c r="F113" t="str">
-        <v>[這一集我準備了兩個月，但是太值...] 單集時長超過60分鐘（約65分鐘），內容資訊密度高，主持人能持續輸出有價值的觀點和案例，全程無冷場��符合長篇內容的評估標準。 | [我們可能會成為最殘忍的一代｜《...] 單集時長超過60分鐘，且內容資訊密度極高，從頭到尾無冷場，引人入勝，非常符合長篇內容的評估標準。</v>
-      </c>
-      <c r="G113" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 童年情感忽視的現象與水流比喻】
-時間: 01:03 - 03:05
-單集: 這一集我準備了兩個月，但是太值得｜《童年情感忽視》
-理由: 主持人首先分享自己經歷的「低潮期」現象，並連結到書中「童年情感忽視」的核心概念。他接著以「水流被石頭阻擋」的生動比喻，解釋未被抒發的情緒如何累積並最終爆發。此片段將個人經驗與複雜的心理學概念結合，透過清晰的比喻深入淺出地闡述，展現了內容企劃的深度與啟發性，非常適合「最神單元企劃」與「自我探索獎」的評估維度。</v>
-      </c>
-    </row>
-    <row r="114" xml:space="preserve">
+        <v>[精算媽咪去誰家Ｉ育兒的終點...] 多人對談的深度訪談，86分鐘的篇幅中充滿真實的情感共鳴與實用建議，情緒層次豐富，陪伴感極佳。</v>
+      </c>
+      <c r="G113" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="114">
       <c r="A114" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3352,25 +3340,22 @@
         <v>5</v>
       </c>
       <c r="C114" t="str">
-        <v>航海王的富人學</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="D114" t="str">
-        <v>美股航海王</v>
+        <v>別人的工作最有趣</v>
       </c>
       <c r="E114">
-        <v>9.35</v>
+        <v>82.92</v>
       </c>
       <c r="F114" t="str">
-        <v>[富人學🔆船長QA - LIV...] 單集時長超過2小時，內容豐富且資訊密度高，討論深入，全程無冷場，展現了長篇內容的製作實力。</v>
-      </c>
-      <c r="G114" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 專家與旁觀者的風險認知差異】
-時間: 04:48 - 06:00
-單集: 富人學🔆第一百零五堂｜『風險風險』
-理由: 主持人深入探討了攀岩者Alex對風險的專業評估與旁觀者因不了解而產生的恐懼，並將此觀點延伸至投資與人生決策。他強調了「被理解過的風險」與「被想像出來的風險」的區別，內容具備深度思考與啟發性，選題獨特且能引發聽眾共鳴，展現了節目在內容企劃上的高度與深度。</v>
-      </c>
-    </row>
-    <row r="115" xml:space="preserve">
+        <v>[EP169 買單程機票到處換國家住！...] 深入探討數位游牧的真實面貌，超過80分鐘的長訪談中，故事性與資訊量並重，毫無冷場。</v>
+      </c>
+      <c r="G114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
       <c r="A115" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3378,25 +3363,22 @@
         <v>6</v>
       </c>
       <c r="C115" t="str">
-        <v>FIRE 人生大學</v>
+        <v>人生挖挖WoW-企業人生策略學</v>
       </c>
       <c r="D115" t="str">
-        <v>Fire人生大學｜道哥</v>
+        <v>人生挖挖WoW-企業人生策略學</v>
       </c>
       <c r="E115">
-        <v>9.3</v>
+        <v>81.55</v>
       </c>
       <c r="F115" t="str">
-        <v>[#71｜ 不為想像的明天而犧牲...] 單集時長接近兩小時（1:59:59），資訊密度高且內容引人入勝，全程無冷場，符合長篇內容的高標準。</v>
-      </c>
-      <c r="G115" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 財富自由的定義：能力減去慾望】
-時間: 1:11:15 - 1:14:15
-單集: #71｜ 不為想像的明天而犧牲今天，就是退休｜《財富自由心理學》ft. 郝旭烈(郝哥) — 上
-理由: 此片段由來賓好哥深入闡述「財富自由」的獨特定義，提出「自由 = 能力 - 慾望」的核心公式，並延伸至「兩種宗教不能信：比較與計較」的深刻觀點。內容極具啟發性與深度，將財富自由從單純的金錢累積提升到心靈層面的選擇權，為聽眾提供了全新的思考框架，完全符合最神單元企劃與自我探索獎的評估維度。</v>
-      </c>
-    </row>
-    <row r="116" xml:space="preserve">
+        <v>[EP.111 | 努力為什麼沒有複利？...] 策略性思維的深度拆解，超過80分鐘的長篇大論卻條理清晰，為聽眾帶來高含金量的職涯啟發。</v>
+      </c>
+      <c r="G115" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="116">
       <c r="A116" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3404,25 +3386,22 @@
         <v>7</v>
       </c>
       <c r="C116" t="str">
-        <v>粉紅地獄辛辣麵</v>
+        <v>五吉郎</v>
       </c>
       <c r="D116" t="str">
-        <v>Vito大叔</v>
+        <v>五吉郎</v>
       </c>
       <c r="E116">
-        <v>8.9</v>
+        <v>79.37</v>
       </c>
       <c r="F116" t="str">
-        <v>[S6EP30. 我到日本當漁夫...] 本集時長超過2小時，屬於長篇內容。節目在這麼長的時間內，資訊密度依然很高，對談流暢且引人入勝，沒有明顯的冷場，能讓聽眾持續投入。這展現了節目在長篇內容規劃與執行上的功力。</v>
-      </c>
-      <c r="G116" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 父母不讓繼承家業的獨特智慧與來賓的創業思維】
-時間: 01:49 - 03:40
-單集: S6EP30. 我到日本當漁夫｜Taku：叛逆的漁四代，在魚市場中的海鮮文化觀察！
-理由: 此片段來賓Taku分享了他父母不希望他繼承傳統養殖業，反而鼓勵他讀大學、追求更高發展的獨特觀點。這顛覆了許多人對家族事業繼承的傳統認知，展現了父母的遠見與智慧。Vito和品希對此表現出極大的驚訝與認同，並適時提問，引導Taku進一步闡述他如何從中找到自己的定位，並希望在產業鏈的更上游（繁殖業）發展。這段對話不僅內容新穎，也充滿了深度思考與自我探索的價值，非常符合【最神單元企劃】與【自我探索獎】的評估維度。</v>
-      </c>
-    </row>
-    <row r="117" xml:space="preserve">
+        <v>[EP152｜理財最實在的第一步...] 長篇幅的理財觀念對談，節奏輕鬆幽默，近80分鐘的內容將硬核知識軟化，非常適合長時間聆聽。</v>
+      </c>
+      <c r="G116" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="117">
       <c r="A117" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3430,25 +3409,22 @@
         <v>8</v>
       </c>
       <c r="C117" t="str">
-        <v>OHMYBOOK｜哲維說書</v>
+        <v>五吉郎</v>
       </c>
       <c r="D117" t="str">
-        <v>梁哲維</v>
+        <v>五吉郎</v>
       </c>
       <c r="E117">
-        <v>8.75</v>
+        <v>79.12</v>
       </c>
       <c r="F117" t="str">
-        <v>[【EP302 把命盤變成行動藍...] 單集時長接近五小時，內容資訊密度高且能維持聽眾的專注度，無明顯冷場，展現長篇內容的製作功力。</v>
-      </c>
-      <c r="G117" t="str" xml:space="preserve">
-        <v xml:space="preserve">【「主角模式」核心概念闡述】
-時間: 00:00 - 00:49
-單集: 【EP319《主角模式》突破成長路上的障礙，開啟你的主角模式！】
-理由: 主持人開場即點出書本核心概念，強調領導力是成就而非掌控，並能成為他人成長的助力。語氣充滿熱情，迅速抓住聽眾注意力，為後續內容奠定良好基礎。</v>
-      </c>
-    </row>
-    <row r="118" xml:space="preserve">
+        <v>[EP145｜技術封頂就夠了？...] 深入探討美業生存法則，豐富的實戰經驗分享，將近80分鐘的訪談內容層次分明，乾貨滿滿。</v>
+      </c>
+      <c r="G117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
       <c r="A118" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3456,25 +3432,22 @@
         <v>9</v>
       </c>
       <c r="C118" t="str">
-        <v>人生啊｜陪你一起看懂人生</v>
+        <v>教出你的路</v>
       </c>
       <c r="D118" t="str">
-        <v>人生啊！小歐</v>
+        <v>教出你的路</v>
       </c>
       <c r="E118">
-        <v>8.69</v>
+        <v>74.92</v>
       </c>
       <c r="F118" t="str">
-        <v>[S0807-翻臉反擊、討好退讓...] 單集時長53分鐘，內容豐富且資訊密度高，討論深入，全程無冷場，符合長篇內容的評估標準。 | [S0714-【關係修復室】5個...] 單集時長超過60分鐘，資訊密度高，內容豐富，無明顯冷場。</v>
-      </c>
-      <c r="G118" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 原則與習慣的邊界感】
-時間: 07:39 - 09:39
-單集: S0807-翻臉反擊、討好退讓之外的第三條路，有彈性的邊界感 ft Ginn
-理由: 此片段深入探討了「有彈性的邊界感」的核心概念，區分了「原則」與「習慣」的不同。主持人解釋了人們常將習慣誤認為原則，導致邊界僵化，難以協商。來賓的補充和例子（如送禮）進一步闡明了這一觀點，提供了獨到且具深度的內容洞察，極具啟發性。</v>
-      </c>
-    </row>
-    <row r="119" xml:space="preserve">
+        <v>[EP43 原來印度是這樣！...] 多元視角的文化交流，74分鐘的長度足以將複雜的社會議題討論得深入淺出，引發聽眾共鳴。</v>
+      </c>
+      <c r="G118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
       <c r="A119" t="str">
         <v>天亮了還在獎 (Alex都上101了你還沒講完)</v>
       </c>
@@ -3482,22 +3455,19 @@
         <v>10</v>
       </c>
       <c r="C119" t="str">
-        <v>小資變有錢｜Dr.Selena生活理財王</v>
+        <v>文森說書</v>
       </c>
       <c r="D119" t="str">
-        <v>Dr Selena</v>
+        <v>文森說書</v>
       </c>
       <c r="E119">
-        <v>8.5</v>
+        <v>74.08</v>
       </c>
       <c r="F119" t="str">
-        <v>[小資愛樂活：環遊世界100國達...] 單集時長約49分鐘，內容豐富且資訊密度高，主持人與來賓的對談引人入勝，全程無冷場。</v>
-      </c>
-      <c r="G119" t="str" xml:space="preserve">
-        <v xml:space="preserve">【[內容與企劃] 劇場的獨特性與文化價值】
-時間: 06:17 - 08:11
-單集: 遇見大來賓：專訪金鐘影后王琄：『人間條件8：凡人哥』~這齣戲，會讓你重新看見自己!
-理由: 來賓王娟深入闡述劇場作為「手工藝」的獨特性，強調其無法被AI取代的價值，並對比台灣與國際劇場的發展現況，探討語言障礙及文化融入的重要性。此段內容不僅具備深度思考，也為聽眾提供了對藝術形式的全新視角，極具「最神單元企劃」與「自我探索獎」的評估價值。</v>
+        <v>[有了百萬英鎊、百萬豪車...] 74分鐘的長篇說書，將一本書的精華與延伸思考娓娓道來，聲音充滿穩定感，是極佳的長篇陪伴內容。</v>
+      </c>
+      <c r="G119" t="str">
+        <v/>
       </c>
     </row>
     <row r="120" xml:space="preserve">

</xml_diff>